<commit_message>
update realisasi 1 agst 11.00
coba update, karena sisa ralisasi 51 tgl 25 antara F16 detail (20M) beda dengan sheet realisasi SP2D per timja (23M)
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -601,7 +601,7 @@
       <c r="A3" s="4" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">Periode Juli 2025</t>
+            <t xml:space="preserve">Periode Agustus 2025</t>
           </r>
         </is>
       </c>
@@ -979,22 +979,22 @@
       <c r="U9" s="10" t="inlineStr"/>
       <c r="V9" s="10" t="inlineStr"/>
       <c r="W9" s="11" t="n">
-        <v>5.4924374881E10</v>
+        <v>6.1530207365E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>6.595922484E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>6.1520297365E10</v>
+        <v>6.1530207365E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.7236762548405614</v>
+        <v>0.7237928282641735</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>2.3490502635E10</v>
+        <v>2.3480592635E10</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1042,10 +1042,10 @@
       <c r="U10" s="14" t="inlineStr"/>
       <c r="V10" s="14" t="inlineStr"/>
       <c r="W10" s="14" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X10" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y10" s="14" t="inlineStr"/>
       <c r="Z10" s="14" t="n">
@@ -1105,10 +1105,10 @@
       <c r="U11" s="14" t="inlineStr"/>
       <c r="V11" s="14" t="inlineStr"/>
       <c r="W11" s="14" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X11" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y11" s="14" t="inlineStr"/>
       <c r="Z11" s="14" t="n">
@@ -1168,10 +1168,10 @@
       <c r="U12" s="17" t="inlineStr"/>
       <c r="V12" s="17" t="inlineStr"/>
       <c r="W12" s="17" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X12" s="17" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y12" s="17" t="inlineStr"/>
       <c r="Z12" s="17" t="n">
@@ -1231,10 +1231,10 @@
       <c r="U13" s="21" t="inlineStr"/>
       <c r="V13" s="21" t="inlineStr"/>
       <c r="W13" s="22" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X13" s="22" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y13" s="22" t="inlineStr"/>
       <c r="Z13" s="21" t="n">
@@ -1294,10 +1294,10 @@
       <c r="U14" s="25" t="inlineStr"/>
       <c r="V14" s="25" t="inlineStr"/>
       <c r="W14" s="25" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X14" s="25" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y14" s="25" t="inlineStr"/>
       <c r="Z14" s="25" t="n">
@@ -1357,10 +1357,10 @@
       <c r="U15" s="14" t="inlineStr"/>
       <c r="V15" s="14" t="inlineStr"/>
       <c r="W15" s="14" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X15" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y15" s="14" t="inlineStr"/>
       <c r="Z15" s="14" t="n">
@@ -1420,10 +1420,10 @@
       <c r="U16" s="14" t="inlineStr"/>
       <c r="V16" s="14" t="inlineStr"/>
       <c r="W16" s="14" t="n">
-        <v>3.52885832E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="X16" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y16" s="14" t="inlineStr"/>
       <c r="Z16" s="14" t="n">
@@ -1477,10 +1477,10 @@
       <c r="U17" s="14" t="inlineStr"/>
       <c r="V17" s="14" t="inlineStr"/>
       <c r="W17" s="14" t="n">
-        <v>3.024E8</v>
+        <v>3.456E8</v>
       </c>
       <c r="X17" s="14" t="n">
-        <v>4.32E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y17" s="14" t="inlineStr"/>
       <c r="Z17" s="14" t="n">
@@ -1534,10 +1534,10 @@
       <c r="U18" s="14" t="inlineStr"/>
       <c r="V18" s="14" t="inlineStr"/>
       <c r="W18" s="14" t="n">
-        <v>3.1122E9</v>
+        <v>3.5568E9</v>
       </c>
       <c r="X18" s="14" t="n">
-        <v>4.446E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y18" s="14" t="inlineStr"/>
       <c r="Z18" s="14" t="n">
@@ -1591,10 +1591,10 @@
       <c r="U19" s="14" t="inlineStr"/>
       <c r="V19" s="14" t="inlineStr"/>
       <c r="W19" s="14" t="n">
-        <v>9.8E7</v>
+        <v>1.12E8</v>
       </c>
       <c r="X19" s="14" t="n">
-        <v>1.4E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y19" s="14" t="inlineStr"/>
       <c r="Z19" s="14" t="n">
@@ -1648,10 +1648,10 @@
       <c r="U20" s="14" t="inlineStr"/>
       <c r="V20" s="14" t="inlineStr"/>
       <c r="W20" s="14" t="n">
-        <v>1.625832E7</v>
+        <v>1.896804E7</v>
       </c>
       <c r="X20" s="14" t="n">
-        <v>2709720.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y20" s="14" t="inlineStr"/>
       <c r="Z20" s="14" t="n">
@@ -1711,23 +1711,23 @@
       <c r="U21" s="14" t="inlineStr"/>
       <c r="V21" s="14" t="inlineStr"/>
       <c r="W21" s="14" t="n">
-        <v>5.1395516561E10</v>
+        <v>5.7496839325E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>6.091412764E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>5.7486929325E10</v>
+        <v>5.7496839325E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.7189023584783437</v>
+        <v>0.7190262879081493</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>2.2477934675E10</v>
+        <v>2.2468024675E10</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1774,23 +1774,23 @@
       <c r="U22" s="14" t="inlineStr"/>
       <c r="V22" s="14" t="inlineStr"/>
       <c r="W22" s="14" t="n">
-        <v>5.1395516561E10</v>
+        <v>5.7496839325E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>6.091412764E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>5.7486929325E10</v>
+        <v>5.7496839325E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.7189023584783437</v>
+        <v>0.7190262879081493</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>2.2477934675E10</v>
+        <v>2.2468024675E10</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1837,23 +1837,23 @@
       <c r="U23" s="17" t="inlineStr"/>
       <c r="V23" s="17" t="inlineStr"/>
       <c r="W23" s="17" t="n">
-        <v>5.1394916561E10</v>
+        <v>5.7496239325E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>6.091412764E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>5.7486329325E10</v>
+        <v>5.7496239325E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.718900249303864</v>
+        <v>0.7190241796635557</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>2.2477934675E10</v>
+        <v>2.2468024675E10</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -2561,10 +2561,10 @@
       <c r="U35" s="21" t="inlineStr"/>
       <c r="V35" s="21" t="inlineStr"/>
       <c r="W35" s="22" t="n">
-        <v>3949100.0</v>
+        <v>9686100.0</v>
       </c>
       <c r="X35" s="22" t="n">
-        <v>5737000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y35" s="22" t="inlineStr"/>
       <c r="Z35" s="21" t="n">
@@ -2624,10 +2624,10 @@
       <c r="U36" s="25" t="inlineStr"/>
       <c r="V36" s="25" t="inlineStr"/>
       <c r="W36" s="25" t="n">
-        <v>3949100.0</v>
+        <v>9686100.0</v>
       </c>
       <c r="X36" s="25" t="n">
-        <v>5737000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y36" s="25" t="inlineStr"/>
       <c r="Z36" s="25" t="n">
@@ -2687,10 +2687,10 @@
       <c r="U37" s="14" t="inlineStr"/>
       <c r="V37" s="14" t="inlineStr"/>
       <c r="W37" s="14" t="n">
-        <v>600000.0</v>
+        <v>2400000.0</v>
       </c>
       <c r="X37" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y37" s="14" t="inlineStr"/>
       <c r="Z37" s="14" t="n">
@@ -2750,10 +2750,10 @@
       <c r="U38" s="14" t="inlineStr"/>
       <c r="V38" s="14" t="inlineStr"/>
       <c r="W38" s="14" t="n">
-        <v>0.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="X38" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y38" s="14" t="inlineStr"/>
       <c r="Z38" s="14" t="n">
@@ -2807,10 +2807,10 @@
       <c r="U39" s="14" t="inlineStr"/>
       <c r="V39" s="14" t="inlineStr"/>
       <c r="W39" s="14" t="n">
-        <v>0.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="X39" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y39" s="14" t="inlineStr"/>
       <c r="Z39" s="14" t="n">
@@ -2990,10 +2990,10 @@
       <c r="U42" s="14" t="inlineStr"/>
       <c r="V42" s="14" t="inlineStr"/>
       <c r="W42" s="14" t="n">
-        <v>3349100.0</v>
+        <v>7286100.0</v>
       </c>
       <c r="X42" s="14" t="n">
-        <v>3937000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y42" s="14" t="inlineStr"/>
       <c r="Z42" s="14" t="n">
@@ -3053,10 +3053,10 @@
       <c r="U43" s="14" t="inlineStr"/>
       <c r="V43" s="14" t="inlineStr"/>
       <c r="W43" s="14" t="n">
-        <v>3349100.0</v>
+        <v>7286100.0</v>
       </c>
       <c r="X43" s="14" t="n">
-        <v>3937000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y43" s="14" t="inlineStr"/>
       <c r="Z43" s="14" t="n">
@@ -3110,10 +3110,10 @@
       <c r="U44" s="14" t="inlineStr"/>
       <c r="V44" s="14" t="inlineStr"/>
       <c r="W44" s="14" t="n">
-        <v>2600000.0</v>
+        <v>6537000.0</v>
       </c>
       <c r="X44" s="14" t="n">
-        <v>3937000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y44" s="14" t="inlineStr"/>
       <c r="Z44" s="14" t="n">
@@ -3230,23 +3230,23 @@
       <c r="U46" s="21" t="inlineStr"/>
       <c r="V46" s="21" t="inlineStr"/>
       <c r="W46" s="22" t="n">
-        <v>5.1389917461E10</v>
+        <v>5.7485503225E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>6.085675764E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>5.7475593225E10</v>
+        <v>5.7485503225E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.7189325852583954</v>
+        <v>0.7190565443429414</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>2.2470140775E10</v>
+        <v>2.2460230775E10</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3293,10 +3293,10 @@
       <c r="U47" s="25" t="inlineStr"/>
       <c r="V47" s="25" t="inlineStr"/>
       <c r="W47" s="25" t="n">
-        <v>4.7473912316E10</v>
+        <v>5.3329786245E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>5.855873929E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
@@ -3356,10 +3356,10 @@
       <c r="U48" s="14" t="inlineStr"/>
       <c r="V48" s="14" t="inlineStr"/>
       <c r="W48" s="14" t="n">
-        <v>3.772450364E9</v>
+        <v>4.187549504E9</v>
       </c>
       <c r="X48" s="14" t="n">
-        <v>4.1509914E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y48" s="14" t="inlineStr"/>
       <c r="Z48" s="14" t="n">
@@ -3419,10 +3419,10 @@
       <c r="U49" s="14" t="inlineStr"/>
       <c r="V49" s="14" t="inlineStr"/>
       <c r="W49" s="14" t="n">
-        <v>1.4858101E9</v>
+        <v>1.6503171E9</v>
       </c>
       <c r="X49" s="14" t="n">
-        <v>1.64507E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y49" s="14" t="inlineStr"/>
       <c r="Z49" s="14" t="n">
@@ -3476,10 +3476,10 @@
       <c r="U50" s="14" t="inlineStr"/>
       <c r="V50" s="14" t="inlineStr"/>
       <c r="W50" s="14" t="n">
-        <v>1.1556297E9</v>
+        <v>1.3201367E9</v>
       </c>
       <c r="X50" s="14" t="n">
-        <v>1.64507E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y50" s="14" t="inlineStr"/>
       <c r="Z50" s="14" t="n">
@@ -3653,10 +3653,10 @@
       <c r="U53" s="14" t="inlineStr"/>
       <c r="V53" s="14" t="inlineStr"/>
       <c r="W53" s="14" t="n">
-        <v>17822.0</v>
+        <v>19549.0</v>
       </c>
       <c r="X53" s="14" t="n">
-        <v>1727.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y53" s="14" t="inlineStr"/>
       <c r="Z53" s="14" t="n">
@@ -3710,10 +3710,10 @@
       <c r="U54" s="14" t="inlineStr"/>
       <c r="V54" s="14" t="inlineStr"/>
       <c r="W54" s="14" t="n">
-        <v>13240.0</v>
+        <v>14967.0</v>
       </c>
       <c r="X54" s="14" t="n">
-        <v>1727.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y54" s="14" t="inlineStr"/>
       <c r="Z54" s="14" t="n">
@@ -3887,10 +3887,10 @@
       <c r="U57" s="14" t="inlineStr"/>
       <c r="V57" s="14" t="inlineStr"/>
       <c r="W57" s="14" t="n">
-        <v>1.1333796E8</v>
+        <v>1.2585432E8</v>
       </c>
       <c r="X57" s="14" t="n">
-        <v>1.251636E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y57" s="14" t="inlineStr"/>
       <c r="Z57" s="14" t="n">
@@ -3944,10 +3944,10 @@
       <c r="U58" s="14" t="inlineStr"/>
       <c r="V58" s="14" t="inlineStr"/>
       <c r="W58" s="14" t="n">
-        <v>8.813964E7</v>
+        <v>1.00656E8</v>
       </c>
       <c r="X58" s="14" t="n">
-        <v>1.251636E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y58" s="14" t="inlineStr"/>
       <c r="Z58" s="14" t="n">
@@ -4164,10 +4164,10 @@
       <c r="U62" s="14" t="inlineStr"/>
       <c r="V62" s="14" t="inlineStr"/>
       <c r="W62" s="14" t="n">
-        <v>3.4441812E7</v>
+        <v>3.8237084E7</v>
       </c>
       <c r="X62" s="14" t="n">
-        <v>3795272.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y62" s="14" t="inlineStr"/>
       <c r="Z62" s="14" t="n">
@@ -4221,10 +4221,10 @@
       <c r="U63" s="14" t="inlineStr"/>
       <c r="V63" s="14" t="inlineStr"/>
       <c r="W63" s="14" t="n">
-        <v>2.6765754E7</v>
+        <v>3.0561026E7</v>
       </c>
       <c r="X63" s="14" t="n">
-        <v>3795272.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y63" s="14" t="inlineStr"/>
       <c r="Z63" s="14" t="n">
@@ -4398,10 +4398,10 @@
       <c r="U66" s="14" t="inlineStr"/>
       <c r="V66" s="14" t="inlineStr"/>
       <c r="W66" s="14" t="n">
-        <v>1.62E7</v>
+        <v>1.8E7</v>
       </c>
       <c r="X66" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y66" s="14" t="inlineStr"/>
       <c r="Z66" s="14" t="n">
@@ -4455,10 +4455,10 @@
       <c r="U67" s="14" t="inlineStr"/>
       <c r="V67" s="14" t="inlineStr"/>
       <c r="W67" s="14" t="n">
-        <v>1.26E7</v>
+        <v>1.44E7</v>
       </c>
       <c r="X67" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y67" s="14" t="inlineStr"/>
       <c r="Z67" s="14" t="n">
@@ -4632,10 +4632,10 @@
       <c r="U70" s="14" t="inlineStr"/>
       <c r="V70" s="14" t="inlineStr"/>
       <c r="W70" s="14" t="n">
-        <v>1.06486E8</v>
+        <v>1.1796E8</v>
       </c>
       <c r="X70" s="14" t="n">
-        <v>1.1474E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y70" s="14" t="inlineStr"/>
       <c r="Z70" s="14" t="n">
@@ -4689,10 +4689,10 @@
       <c r="U71" s="14" t="inlineStr"/>
       <c r="V71" s="14" t="inlineStr"/>
       <c r="W71" s="14" t="n">
-        <v>8.2458E7</v>
+        <v>9.3932E7</v>
       </c>
       <c r="X71" s="14" t="n">
-        <v>1.1474E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y71" s="14" t="inlineStr"/>
       <c r="Z71" s="14" t="n">
@@ -4866,10 +4866,10 @@
       <c r="U74" s="14" t="inlineStr"/>
       <c r="V74" s="14" t="inlineStr"/>
       <c r="W74" s="14" t="n">
-        <v>1.9186331E7</v>
+        <v>1.9384414E7</v>
       </c>
       <c r="X74" s="14" t="n">
-        <v>198083.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y74" s="14" t="inlineStr"/>
       <c r="Z74" s="14" t="n">
@@ -4923,10 +4923,10 @@
       <c r="U75" s="14" t="inlineStr"/>
       <c r="V75" s="14" t="inlineStr"/>
       <c r="W75" s="14" t="n">
-        <v>1655315.0</v>
+        <v>1853398.0</v>
       </c>
       <c r="X75" s="14" t="n">
-        <v>198083.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y75" s="14" t="inlineStr"/>
       <c r="Z75" s="14" t="n">
@@ -5100,10 +5100,10 @@
       <c r="U78" s="14" t="inlineStr"/>
       <c r="V78" s="14" t="inlineStr"/>
       <c r="W78" s="14" t="n">
-        <v>7.864812E7</v>
+        <v>8.72661E7</v>
       </c>
       <c r="X78" s="14" t="n">
-        <v>8617980.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y78" s="14" t="inlineStr"/>
       <c r="Z78" s="14" t="n">
@@ -5157,10 +5157,10 @@
       <c r="U79" s="14" t="inlineStr"/>
       <c r="V79" s="14" t="inlineStr"/>
       <c r="W79" s="14" t="n">
-        <v>6.112248E7</v>
+        <v>6.974046E7</v>
       </c>
       <c r="X79" s="14" t="n">
-        <v>8617980.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y79" s="14" t="inlineStr"/>
       <c r="Z79" s="14" t="n">
@@ -5334,10 +5334,10 @@
       <c r="U82" s="14" t="inlineStr"/>
       <c r="V82" s="14" t="inlineStr"/>
       <c r="W82" s="14" t="n">
-        <v>1.28383E8</v>
+        <v>1.54008E8</v>
       </c>
       <c r="X82" s="14" t="n">
-        <v>2.5625E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y82" s="14" t="inlineStr"/>
       <c r="Z82" s="14" t="n">
@@ -5391,10 +5391,10 @@
       <c r="U83" s="14" t="inlineStr"/>
       <c r="V83" s="14" t="inlineStr"/>
       <c r="W83" s="14" t="n">
-        <v>8260000.0</v>
+        <v>9450000.0</v>
       </c>
       <c r="X83" s="14" t="n">
-        <v>1190000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y83" s="14" t="inlineStr"/>
       <c r="Z83" s="14" t="n">
@@ -5448,10 +5448,10 @@
       <c r="U84" s="14" t="inlineStr"/>
       <c r="V84" s="14" t="inlineStr"/>
       <c r="W84" s="14" t="n">
-        <v>1.05117E8</v>
+        <v>1.25985E8</v>
       </c>
       <c r="X84" s="14" t="n">
-        <v>2.0868E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y84" s="14" t="inlineStr"/>
       <c r="Z84" s="14" t="n">
@@ -5505,10 +5505,10 @@
       <c r="U85" s="14" t="inlineStr"/>
       <c r="V85" s="14" t="inlineStr"/>
       <c r="W85" s="14" t="n">
-        <v>1.5006E7</v>
+        <v>1.8573E7</v>
       </c>
       <c r="X85" s="14" t="n">
-        <v>3567000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y85" s="14" t="inlineStr"/>
       <c r="Z85" s="14" t="n">
@@ -5568,10 +5568,10 @@
       <c r="U86" s="14" t="inlineStr"/>
       <c r="V86" s="14" t="inlineStr"/>
       <c r="W86" s="14" t="n">
-        <v>3.637E7</v>
+        <v>4.044E7</v>
       </c>
       <c r="X86" s="14" t="n">
-        <v>4070000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y86" s="14" t="inlineStr"/>
       <c r="Z86" s="14" t="n">
@@ -5625,10 +5625,10 @@
       <c r="U87" s="14" t="inlineStr"/>
       <c r="V87" s="14" t="inlineStr"/>
       <c r="W87" s="14" t="n">
-        <v>2.844E7</v>
+        <v>3.251E7</v>
       </c>
       <c r="X87" s="14" t="n">
-        <v>4070000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y87" s="14" t="inlineStr"/>
       <c r="Z87" s="14" t="n">
@@ -5845,10 +5845,10 @@
       <c r="U91" s="14" t="inlineStr"/>
       <c r="V91" s="14" t="inlineStr"/>
       <c r="W91" s="14" t="n">
-        <v>1.753569219E9</v>
+        <v>1.936062937E9</v>
       </c>
       <c r="X91" s="14" t="n">
-        <v>1.82493718E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y91" s="14" t="inlineStr"/>
       <c r="Z91" s="14" t="n">
@@ -5902,10 +5902,10 @@
       <c r="U92" s="14" t="inlineStr"/>
       <c r="V92" s="14" t="inlineStr"/>
       <c r="W92" s="14" t="n">
-        <v>1.310954427E9</v>
+        <v>1.493448145E9</v>
       </c>
       <c r="X92" s="14" t="n">
-        <v>1.82493718E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y92" s="14" t="inlineStr"/>
       <c r="Z92" s="14" t="n">
@@ -7943,10 +7943,10 @@
       <c r="U127" s="14" t="inlineStr"/>
       <c r="V127" s="14" t="inlineStr"/>
       <c r="W127" s="14" t="n">
-        <v>3.169917513E10</v>
+        <v>3.5544999187E10</v>
       </c>
       <c r="X127" s="14" t="n">
-        <v>3.845824057E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y127" s="14" t="inlineStr"/>
       <c r="Z127" s="14" t="n">
@@ -8006,10 +8006,10 @@
       <c r="U128" s="14" t="inlineStr"/>
       <c r="V128" s="14" t="inlineStr"/>
       <c r="W128" s="14" t="n">
-        <v>1.11880769E10</v>
+        <v>1.23832303E10</v>
       </c>
       <c r="X128" s="14" t="n">
-        <v>1.1951534E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y128" s="14" t="inlineStr"/>
       <c r="Z128" s="14" t="n">
@@ -8063,10 +8063,10 @@
       <c r="U129" s="14" t="inlineStr"/>
       <c r="V129" s="14" t="inlineStr"/>
       <c r="W129" s="14" t="n">
-        <v>8.6973235E9</v>
+        <v>9.8924769E9</v>
       </c>
       <c r="X129" s="14" t="n">
-        <v>1.1951534E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y129" s="14" t="inlineStr"/>
       <c r="Z129" s="14" t="n">
@@ -8240,10 +8240,10 @@
       <c r="U132" s="14" t="inlineStr"/>
       <c r="V132" s="14" t="inlineStr"/>
       <c r="W132" s="14" t="n">
-        <v>152199.0</v>
+        <v>168114.0</v>
       </c>
       <c r="X132" s="14" t="n">
-        <v>15915.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y132" s="14" t="inlineStr"/>
       <c r="Z132" s="14" t="n">
@@ -8297,10 +8297,10 @@
       <c r="U133" s="14" t="inlineStr"/>
       <c r="V133" s="14" t="inlineStr"/>
       <c r="W133" s="14" t="n">
-        <v>118425.0</v>
+        <v>134340.0</v>
       </c>
       <c r="X133" s="14" t="n">
-        <v>15915.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y133" s="14" t="inlineStr"/>
       <c r="Z133" s="14" t="n">
@@ -8474,10 +8474,10 @@
       <c r="U136" s="14" t="inlineStr"/>
       <c r="V136" s="14" t="inlineStr"/>
       <c r="W136" s="14" t="n">
-        <v>8.786895E8</v>
+        <v>9.7329066E8</v>
       </c>
       <c r="X136" s="14" t="n">
-        <v>9.460116E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y136" s="14" t="inlineStr"/>
       <c r="Z136" s="14" t="n">
@@ -8531,10 +8531,10 @@
       <c r="U137" s="14" t="inlineStr"/>
       <c r="V137" s="14" t="inlineStr"/>
       <c r="W137" s="14" t="n">
-        <v>6.8370444E8</v>
+        <v>7.783056E8</v>
       </c>
       <c r="X137" s="14" t="n">
-        <v>9.460116E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y137" s="14" t="inlineStr"/>
       <c r="Z137" s="14" t="n">
@@ -8708,10 +8708,10 @@
       <c r="U140" s="14" t="inlineStr"/>
       <c r="V140" s="14" t="inlineStr"/>
       <c r="W140" s="14" t="n">
-        <v>2.7256082E8</v>
+        <v>3.02306822E8</v>
       </c>
       <c r="X140" s="14" t="n">
-        <v>2.9746002E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y140" s="14" t="inlineStr"/>
       <c r="Z140" s="14" t="n">
@@ -8765,10 +8765,10 @@
       <c r="U141" s="14" t="inlineStr"/>
       <c r="V141" s="14" t="inlineStr"/>
       <c r="W141" s="14" t="n">
-        <v>2.12169964E8</v>
+        <v>2.41915966E8</v>
       </c>
       <c r="X141" s="14" t="n">
-        <v>2.9746002E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y141" s="14" t="inlineStr"/>
       <c r="Z141" s="14" t="n">
@@ -8942,10 +8942,10 @@
       <c r="U144" s="14" t="inlineStr"/>
       <c r="V144" s="14" t="inlineStr"/>
       <c r="W144" s="14" t="n">
-        <v>2.41703E9</v>
+        <v>2.67431E9</v>
       </c>
       <c r="X144" s="14" t="n">
-        <v>2.5728E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y144" s="14" t="inlineStr"/>
       <c r="Z144" s="14" t="n">
@@ -9042,10 +9042,10 @@
       <c r="U146" s="14" t="inlineStr"/>
       <c r="V146" s="14" t="inlineStr"/>
       <c r="W146" s="14" t="n">
-        <v>1.87877E9</v>
+        <v>2.13605E9</v>
       </c>
       <c r="X146" s="14" t="n">
-        <v>2.5728E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y146" s="14" t="inlineStr"/>
       <c r="Z146" s="14" t="n">
@@ -9219,10 +9219,10 @@
       <c r="U149" s="14" t="inlineStr"/>
       <c r="V149" s="14" t="inlineStr"/>
       <c r="W149" s="14" t="n">
-        <v>2.14257962E8</v>
+        <v>2.17635496E8</v>
       </c>
       <c r="X149" s="14" t="n">
-        <v>3377534.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y149" s="14" t="inlineStr"/>
       <c r="Z149" s="14" t="n">
@@ -9276,10 +9276,10 @@
       <c r="U150" s="14" t="inlineStr"/>
       <c r="V150" s="14" t="inlineStr"/>
       <c r="W150" s="14" t="n">
-        <v>2.8801831E7</v>
+        <v>3.2179365E7</v>
       </c>
       <c r="X150" s="14" t="n">
-        <v>3377534.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y150" s="14" t="inlineStr"/>
       <c r="Z150" s="14" t="n">
@@ -9453,10 +9453,10 @@
       <c r="U153" s="14" t="inlineStr"/>
       <c r="V153" s="14" t="inlineStr"/>
       <c r="W153" s="14" t="n">
-        <v>6.133974E8</v>
+        <v>6.7995138E8</v>
       </c>
       <c r="X153" s="14" t="n">
-        <v>6.655398E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y153" s="14" t="inlineStr"/>
       <c r="Z153" s="14" t="n">
@@ -9510,10 +9510,10 @@
       <c r="U154" s="14" t="inlineStr"/>
       <c r="V154" s="14" t="inlineStr"/>
       <c r="W154" s="14" t="n">
-        <v>4.7666844E8</v>
+        <v>5.4322242E8</v>
       </c>
       <c r="X154" s="14" t="n">
-        <v>6.655398E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y154" s="14" t="inlineStr"/>
       <c r="Z154" s="14" t="n">
@@ -9687,10 +9687,10 @@
       <c r="U157" s="14" t="inlineStr"/>
       <c r="V157" s="14" t="inlineStr"/>
       <c r="W157" s="14" t="n">
-        <v>1.046634E9</v>
+        <v>1.249247E9</v>
       </c>
       <c r="X157" s="14" t="n">
-        <v>2.02613E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y157" s="14" t="inlineStr"/>
       <c r="Z157" s="14" t="n">
@@ -9744,10 +9744,10 @@
       <c r="U158" s="14" t="inlineStr"/>
       <c r="V158" s="14" t="inlineStr"/>
       <c r="W158" s="14" t="n">
-        <v>9.1E7</v>
+        <v>1.09165E8</v>
       </c>
       <c r="X158" s="14" t="n">
-        <v>1.8165E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y158" s="14" t="inlineStr"/>
       <c r="Z158" s="14" t="n">
@@ -9801,10 +9801,10 @@
       <c r="U159" s="14" t="inlineStr"/>
       <c r="V159" s="14" t="inlineStr"/>
       <c r="W159" s="14" t="n">
-        <v>7.40999E8</v>
+        <v>8.87112E8</v>
       </c>
       <c r="X159" s="14" t="n">
-        <v>1.46113E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y159" s="14" t="inlineStr"/>
       <c r="Z159" s="14" t="n">
@@ -9858,10 +9858,10 @@
       <c r="U160" s="14" t="inlineStr"/>
       <c r="V160" s="14" t="inlineStr"/>
       <c r="W160" s="14" t="n">
-        <v>2.14635E8</v>
+        <v>2.5297E8</v>
       </c>
       <c r="X160" s="14" t="n">
-        <v>3.8335E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y160" s="14" t="inlineStr"/>
       <c r="Z160" s="14" t="n">
@@ -9921,10 +9921,10 @@
       <c r="U161" s="14" t="inlineStr"/>
       <c r="V161" s="14" t="inlineStr"/>
       <c r="W161" s="14" t="n">
-        <v>2035000.0</v>
+        <v>2220000.0</v>
       </c>
       <c r="X161" s="14" t="n">
-        <v>185000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y161" s="14" t="inlineStr"/>
       <c r="Z161" s="14" t="n">
@@ -9978,10 +9978,10 @@
       <c r="U162" s="14" t="inlineStr"/>
       <c r="V162" s="14" t="inlineStr"/>
       <c r="W162" s="14" t="n">
-        <v>1480000.0</v>
+        <v>1665000.0</v>
       </c>
       <c r="X162" s="14" t="n">
-        <v>185000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y162" s="14" t="inlineStr"/>
       <c r="Z162" s="14" t="n">
@@ -10155,10 +10155,10 @@
       <c r="U165" s="14" t="inlineStr"/>
       <c r="V165" s="14" t="inlineStr"/>
       <c r="W165" s="14" t="n">
-        <v>1.5066341349E10</v>
+        <v>1.7062639415E10</v>
       </c>
       <c r="X165" s="14" t="n">
-        <v>1.996298066E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y165" s="14" t="inlineStr"/>
       <c r="Z165" s="14" t="n">
@@ -10212,10 +10212,10 @@
       <c r="U166" s="14" t="inlineStr"/>
       <c r="V166" s="14" t="inlineStr"/>
       <c r="W166" s="14" t="n">
-        <v>1.0293742797E10</v>
+        <v>1.2285354215E10</v>
       </c>
       <c r="X166" s="14" t="n">
-        <v>1.991611418E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y166" s="14" t="inlineStr"/>
       <c r="Z166" s="14" t="n">
@@ -10269,10 +10269,10 @@
       <c r="U167" s="14" t="inlineStr"/>
       <c r="V167" s="14" t="inlineStr"/>
       <c r="W167" s="14" t="n">
-        <v>2.362459773E9</v>
+        <v>2.367146421E9</v>
       </c>
       <c r="X167" s="14" t="n">
-        <v>4686648.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y167" s="14" t="inlineStr"/>
       <c r="Z167" s="14" t="n">
@@ -10389,10 +10389,10 @@
       <c r="U169" s="14" t="inlineStr"/>
       <c r="V169" s="14" t="inlineStr"/>
       <c r="W169" s="14" t="n">
-        <v>1.2002286822E10</v>
+        <v>1.3597237554E10</v>
       </c>
       <c r="X169" s="14" t="n">
-        <v>1.594950732E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y169" s="14" t="inlineStr"/>
       <c r="Z169" s="14" t="n">
@@ -10452,10 +10452,10 @@
       <c r="U170" s="14" t="inlineStr"/>
       <c r="V170" s="14" t="inlineStr"/>
       <c r="W170" s="14" t="n">
-        <v>4.762388866E9</v>
+        <v>5.311759666E9</v>
       </c>
       <c r="X170" s="14" t="n">
-        <v>5.493708E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y170" s="14" t="inlineStr"/>
       <c r="Z170" s="14" t="n">
@@ -10509,10 +10509,10 @@
       <c r="U171" s="14" t="inlineStr"/>
       <c r="V171" s="14" t="inlineStr"/>
       <c r="W171" s="14" t="n">
-        <v>3.6732752E9</v>
+        <v>4.222646E9</v>
       </c>
       <c r="X171" s="14" t="n">
-        <v>5.493708E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y171" s="14" t="inlineStr"/>
       <c r="Z171" s="14" t="n">
@@ -10729,10 +10729,10 @@
       <c r="U175" s="14" t="inlineStr"/>
       <c r="V175" s="14" t="inlineStr"/>
       <c r="W175" s="14" t="n">
-        <v>91671.0</v>
+        <v>101733.0</v>
       </c>
       <c r="X175" s="14" t="n">
-        <v>10062.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y175" s="14" t="inlineStr"/>
       <c r="Z175" s="14" t="n">
@@ -10786,10 +10786,10 @@
       <c r="U176" s="14" t="inlineStr"/>
       <c r="V176" s="14" t="inlineStr"/>
       <c r="W176" s="14" t="n">
-        <v>78551.0</v>
+        <v>88613.0</v>
       </c>
       <c r="X176" s="14" t="n">
-        <v>10062.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y176" s="14" t="inlineStr"/>
       <c r="Z176" s="14" t="n">
@@ -10963,10 +10963,10 @@
       <c r="U179" s="14" t="inlineStr"/>
       <c r="V179" s="14" t="inlineStr"/>
       <c r="W179" s="14" t="n">
-        <v>3.2254353E8</v>
+        <v>3.5985017E8</v>
       </c>
       <c r="X179" s="14" t="n">
-        <v>3.730664E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y179" s="14" t="inlineStr"/>
       <c r="Z179" s="14" t="n">
@@ -11020,10 +11020,10 @@
       <c r="U180" s="14" t="inlineStr"/>
       <c r="V180" s="14" t="inlineStr"/>
       <c r="W180" s="14" t="n">
-        <v>2.4881876E8</v>
+        <v>2.861254E8</v>
       </c>
       <c r="X180" s="14" t="n">
-        <v>3.730664E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y180" s="14" t="inlineStr"/>
       <c r="Z180" s="14" t="n">
@@ -11197,10 +11197,10 @@
       <c r="U183" s="14" t="inlineStr"/>
       <c r="V183" s="14" t="inlineStr"/>
       <c r="W183" s="14" t="n">
-        <v>9.6747576E7</v>
+        <v>1.07733296E8</v>
       </c>
       <c r="X183" s="14" t="n">
-        <v>1.098572E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y183" s="14" t="inlineStr"/>
       <c r="Z183" s="14" t="n">
@@ -11254,10 +11254,10 @@
       <c r="U184" s="14" t="inlineStr"/>
       <c r="V184" s="14" t="inlineStr"/>
       <c r="W184" s="14" t="n">
-        <v>7.4864992E7</v>
+        <v>8.5850712E7</v>
       </c>
       <c r="X184" s="14" t="n">
-        <v>1.098572E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y184" s="14" t="inlineStr"/>
       <c r="Z184" s="14" t="n">
@@ -11431,10 +11431,10 @@
       <c r="U187" s="14" t="inlineStr"/>
       <c r="V187" s="14" t="inlineStr"/>
       <c r="W187" s="14" t="n">
-        <v>7.7817E8</v>
+        <v>8.6691E8</v>
       </c>
       <c r="X187" s="14" t="n">
-        <v>8.874E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y187" s="14" t="inlineStr"/>
       <c r="Z187" s="14" t="n">
@@ -11488,10 +11488,10 @@
       <c r="U188" s="14" t="inlineStr"/>
       <c r="V188" s="14" t="inlineStr"/>
       <c r="W188" s="14" t="n">
-        <v>6.0036E8</v>
+        <v>6.891E8</v>
       </c>
       <c r="X188" s="14" t="n">
-        <v>8.874E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y188" s="14" t="inlineStr"/>
       <c r="Z188" s="14" t="n">
@@ -11665,10 +11665,10 @@
       <c r="U191" s="14" t="inlineStr"/>
       <c r="V191" s="14" t="inlineStr"/>
       <c r="W191" s="14" t="n">
-        <v>2.9241989E8</v>
+        <v>3.2558825E8</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>3.316836E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
@@ -11722,10 +11722,10 @@
       <c r="U192" s="14" t="inlineStr"/>
       <c r="V192" s="14" t="inlineStr"/>
       <c r="W192" s="14" t="n">
-        <v>2.2587798E8</v>
+        <v>2.5904634E8</v>
       </c>
       <c r="X192" s="14" t="n">
-        <v>3.316836E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y192" s="14" t="inlineStr"/>
       <c r="Z192" s="14" t="n">
@@ -11899,10 +11899,10 @@
       <c r="U195" s="14" t="inlineStr"/>
       <c r="V195" s="14" t="inlineStr"/>
       <c r="W195" s="14" t="n">
-        <v>5.34431E8</v>
+        <v>6.44264E8</v>
       </c>
       <c r="X195" s="14" t="n">
-        <v>1.09833E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y195" s="14" t="inlineStr"/>
       <c r="Z195" s="14" t="n">
@@ -11956,10 +11956,10 @@
       <c r="U196" s="14" t="inlineStr"/>
       <c r="V196" s="14" t="inlineStr"/>
       <c r="W196" s="14" t="n">
-        <v>5.11E7</v>
+        <v>6.181E7</v>
       </c>
       <c r="X196" s="14" t="n">
-        <v>1.071E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y196" s="14" t="inlineStr"/>
       <c r="Z196" s="14" t="n">
@@ -12013,10 +12013,10 @@
       <c r="U197" s="14" t="inlineStr"/>
       <c r="V197" s="14" t="inlineStr"/>
       <c r="W197" s="14" t="n">
-        <v>4.83331E8</v>
+        <v>5.82454E8</v>
       </c>
       <c r="X197" s="14" t="n">
-        <v>9.9123E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y197" s="14" t="inlineStr"/>
       <c r="Z197" s="14" t="n">
@@ -12076,10 +12076,10 @@
       <c r="U198" s="14" t="inlineStr"/>
       <c r="V198" s="14" t="inlineStr"/>
       <c r="W198" s="14" t="n">
-        <v>5.215494289E9</v>
+        <v>5.981030439E9</v>
       </c>
       <c r="X198" s="14" t="n">
-        <v>7.6553615E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y198" s="14" t="inlineStr"/>
       <c r="Z198" s="14" t="n">
@@ -12133,10 +12133,10 @@
       <c r="U199" s="14" t="inlineStr"/>
       <c r="V199" s="14" t="inlineStr"/>
       <c r="W199" s="14" t="n">
-        <v>3.641050913E9</v>
+        <v>4.406587063E9</v>
       </c>
       <c r="X199" s="14" t="n">
-        <v>7.6553615E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y199" s="14" t="inlineStr"/>
       <c r="Z199" s="14" t="n">
@@ -12353,23 +12353,23 @@
       <c r="U203" s="25" t="inlineStr"/>
       <c r="V203" s="25" t="inlineStr"/>
       <c r="W203" s="25" t="n">
-        <v>3.916005145E9</v>
+        <v>4.15571698E9</v>
       </c>
       <c r="X203" s="25" t="n">
-        <v>2.29801835E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y203" s="25" t="inlineStr"/>
       <c r="Z203" s="25" t="n">
-        <v>4.14580698E9</v>
+        <v>4.15571698E9</v>
       </c>
       <c r="AA203" s="25" t="inlineStr"/>
       <c r="AB203" s="25" t="inlineStr"/>
       <c r="AC203" s="26" t="n">
-        <v>0.7330226853324455</v>
+        <v>0.7347748785355271</v>
       </c>
       <c r="AD203" s="26" t="inlineStr"/>
       <c r="AE203" s="25" t="n">
-        <v>1.50996202E9</v>
+        <v>1.50005202E9</v>
       </c>
       <c r="AF203" s="25" t="inlineStr"/>
       <c r="AG203" s="25" t="inlineStr"/>
@@ -12416,10 +12416,10 @@
       <c r="U204" s="14" t="inlineStr"/>
       <c r="V204" s="14" t="inlineStr"/>
       <c r="W204" s="14" t="n">
-        <v>3.114927616E9</v>
+        <v>3.258757999E9</v>
       </c>
       <c r="X204" s="14" t="n">
-        <v>1.43830383E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y204" s="14" t="inlineStr"/>
       <c r="Z204" s="14" t="n">
@@ -12479,10 +12479,10 @@
       <c r="U205" s="14" t="inlineStr"/>
       <c r="V205" s="14" t="inlineStr"/>
       <c r="W205" s="14" t="n">
-        <v>4.77118356E8</v>
+        <v>5.46628803E8</v>
       </c>
       <c r="X205" s="14" t="n">
-        <v>6.9510447E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y205" s="14" t="inlineStr"/>
       <c r="Z205" s="14" t="n">
@@ -12536,10 +12536,10 @@
       <c r="U206" s="14" t="inlineStr"/>
       <c r="V206" s="14" t="inlineStr"/>
       <c r="W206" s="14" t="n">
-        <v>4.48E8</v>
+        <v>5.115E8</v>
       </c>
       <c r="X206" s="14" t="n">
-        <v>6.35E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y206" s="14" t="inlineStr"/>
       <c r="Z206" s="14" t="n">
@@ -12593,10 +12593,10 @@
       <c r="U207" s="14" t="inlineStr"/>
       <c r="V207" s="14" t="inlineStr"/>
       <c r="W207" s="14" t="n">
-        <v>2076300.0</v>
+        <v>2419200.0</v>
       </c>
       <c r="X207" s="14" t="n">
-        <v>342900.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y207" s="14" t="inlineStr"/>
       <c r="Z207" s="14" t="n">
@@ -12650,10 +12650,10 @@
       <c r="U208" s="14" t="inlineStr"/>
       <c r="V208" s="14" t="inlineStr"/>
       <c r="W208" s="14" t="n">
-        <v>2.7042056E7</v>
+        <v>3.2709603E7</v>
       </c>
       <c r="X208" s="14" t="n">
-        <v>5667547.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y208" s="14" t="inlineStr"/>
       <c r="Z208" s="14" t="n">
@@ -12713,10 +12713,10 @@
       <c r="U209" s="14" t="inlineStr"/>
       <c r="V209" s="14" t="inlineStr"/>
       <c r="W209" s="14" t="n">
-        <v>4157000.0</v>
+        <v>5144000.0</v>
       </c>
       <c r="X209" s="14" t="n">
-        <v>987000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y209" s="14" t="inlineStr"/>
       <c r="Z209" s="14" t="n">
@@ -12770,10 +12770,10 @@
       <c r="U210" s="14" t="inlineStr"/>
       <c r="V210" s="14" t="inlineStr"/>
       <c r="W210" s="14" t="n">
-        <v>2137000.0</v>
+        <v>2720000.0</v>
       </c>
       <c r="X210" s="14" t="n">
-        <v>583000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y210" s="14" t="inlineStr"/>
       <c r="Z210" s="14" t="n">
@@ -12827,10 +12827,10 @@
       <c r="U211" s="14" t="inlineStr"/>
       <c r="V211" s="14" t="inlineStr"/>
       <c r="W211" s="14" t="n">
-        <v>2020000.0</v>
+        <v>2424000.0</v>
       </c>
       <c r="X211" s="14" t="n">
-        <v>404000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y211" s="14" t="inlineStr"/>
       <c r="Z211" s="14" t="n">
@@ -12890,10 +12890,10 @@
       <c r="U212" s="14" t="inlineStr"/>
       <c r="V212" s="14" t="inlineStr"/>
       <c r="W212" s="14" t="n">
-        <v>8622580.0</v>
+        <v>1.280558E7</v>
       </c>
       <c r="X212" s="14" t="n">
-        <v>4183000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y212" s="14" t="inlineStr"/>
       <c r="Z212" s="14" t="n">
@@ -12947,10 +12947,10 @@
       <c r="U213" s="14" t="inlineStr"/>
       <c r="V213" s="14" t="inlineStr"/>
       <c r="W213" s="14" t="n">
-        <v>8622580.0</v>
+        <v>1.280558E7</v>
       </c>
       <c r="X213" s="14" t="n">
-        <v>4183000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y213" s="14" t="inlineStr"/>
       <c r="Z213" s="14" t="n">
@@ -13130,10 +13130,10 @@
       <c r="U216" s="14" t="inlineStr"/>
       <c r="V216" s="14" t="inlineStr"/>
       <c r="W216" s="14" t="n">
-        <v>2.62303968E9</v>
+        <v>2.692189616E9</v>
       </c>
       <c r="X216" s="14" t="n">
-        <v>6.9149936E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y216" s="14" t="inlineStr"/>
       <c r="Z216" s="14" t="n">
@@ -13187,10 +13187,10 @@
       <c r="U217" s="14" t="inlineStr"/>
       <c r="V217" s="14" t="inlineStr"/>
       <c r="W217" s="14" t="n">
-        <v>2.4455968E8</v>
+        <v>2.85881376E8</v>
       </c>
       <c r="X217" s="14" t="n">
-        <v>4.1321696E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y217" s="14" t="inlineStr"/>
       <c r="Z217" s="14" t="n">
@@ -13244,10 +13244,10 @@
       <c r="U218" s="14" t="inlineStr"/>
       <c r="V218" s="14" t="inlineStr"/>
       <c r="W218" s="14" t="n">
-        <v>5.597624E7</v>
+        <v>6.5444768E7</v>
       </c>
       <c r="X218" s="14" t="n">
-        <v>9468528.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y218" s="14" t="inlineStr"/>
       <c r="Z218" s="14" t="n">
@@ -13301,10 +13301,10 @@
       <c r="U219" s="14" t="inlineStr"/>
       <c r="V219" s="14" t="inlineStr"/>
       <c r="W219" s="14" t="n">
-        <v>8.129932E7</v>
+        <v>9.5029104E7</v>
       </c>
       <c r="X219" s="14" t="n">
-        <v>1.3729784E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y219" s="14" t="inlineStr"/>
       <c r="Z219" s="14" t="n">
@@ -13358,10 +13358,10 @@
       <c r="U220" s="14" t="inlineStr"/>
       <c r="V220" s="14" t="inlineStr"/>
       <c r="W220" s="14" t="n">
-        <v>2.736644E7</v>
+        <v>3.1996368E7</v>
       </c>
       <c r="X220" s="14" t="n">
-        <v>4629928.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y220" s="14" t="inlineStr"/>
       <c r="Z220" s="14" t="n">
@@ -13478,10 +13478,10 @@
       <c r="U222" s="14" t="inlineStr"/>
       <c r="V222" s="14" t="inlineStr"/>
       <c r="W222" s="14" t="n">
-        <v>3.80681131E8</v>
+        <v>4.32620013E8</v>
       </c>
       <c r="X222" s="14" t="n">
-        <v>5.1938882E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y222" s="14" t="inlineStr"/>
       <c r="Z222" s="14" t="n">
@@ -13541,10 +13541,10 @@
       <c r="U223" s="14" t="inlineStr"/>
       <c r="V223" s="14" t="inlineStr"/>
       <c r="W223" s="14" t="n">
-        <v>2.73406741E8</v>
+        <v>3.10883859E8</v>
       </c>
       <c r="X223" s="14" t="n">
-        <v>3.7477118E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y223" s="14" t="inlineStr"/>
       <c r="Z223" s="14" t="n">
@@ -13598,10 +13598,10 @@
       <c r="U224" s="14" t="inlineStr"/>
       <c r="V224" s="14" t="inlineStr"/>
       <c r="W224" s="14" t="n">
-        <v>2.73406741E8</v>
+        <v>3.10883859E8</v>
       </c>
       <c r="X224" s="14" t="n">
-        <v>3.7477118E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y224" s="14" t="inlineStr"/>
       <c r="Z224" s="14" t="n">
@@ -13661,10 +13661,10 @@
       <c r="U225" s="14" t="inlineStr"/>
       <c r="V225" s="14" t="inlineStr"/>
       <c r="W225" s="14" t="n">
-        <v>4161834.0</v>
+        <v>4425348.0</v>
       </c>
       <c r="X225" s="14" t="n">
-        <v>263514.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y225" s="14" t="inlineStr"/>
       <c r="Z225" s="14" t="n">
@@ -13718,10 +13718,10 @@
       <c r="U226" s="14" t="inlineStr"/>
       <c r="V226" s="14" t="inlineStr"/>
       <c r="W226" s="14" t="n">
-        <v>4161834.0</v>
+        <v>4425348.0</v>
       </c>
       <c r="X226" s="14" t="n">
-        <v>263514.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y226" s="14" t="inlineStr"/>
       <c r="Z226" s="14" t="n">
@@ -13781,10 +13781,10 @@
       <c r="U227" s="14" t="inlineStr"/>
       <c r="V227" s="14" t="inlineStr"/>
       <c r="W227" s="14" t="n">
-        <v>2.13328E7</v>
+        <v>2.48451E7</v>
       </c>
       <c r="X227" s="14" t="n">
-        <v>3512300.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y227" s="14" t="inlineStr"/>
       <c r="Z227" s="14" t="n">
@@ -13881,10 +13881,10 @@
       <c r="U229" s="14" t="inlineStr"/>
       <c r="V229" s="14" t="inlineStr"/>
       <c r="W229" s="14" t="n">
-        <v>2.13328E7</v>
+        <v>2.48451E7</v>
       </c>
       <c r="X229" s="14" t="n">
-        <v>3512300.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y229" s="14" t="inlineStr"/>
       <c r="Z229" s="14" t="n">
@@ -13944,10 +13944,10 @@
       <c r="U230" s="14" t="inlineStr"/>
       <c r="V230" s="14" t="inlineStr"/>
       <c r="W230" s="14" t="n">
-        <v>8.1779756E7</v>
+        <v>9.2465706E7</v>
       </c>
       <c r="X230" s="14" t="n">
-        <v>1.068595E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y230" s="14" t="inlineStr"/>
       <c r="Z230" s="14" t="n">
@@ -14001,10 +14001,10 @@
       <c r="U231" s="14" t="inlineStr"/>
       <c r="V231" s="14" t="inlineStr"/>
       <c r="W231" s="14" t="n">
-        <v>5.607995E7</v>
+        <v>6.58569E7</v>
       </c>
       <c r="X231" s="14" t="n">
-        <v>9776950.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y231" s="14" t="inlineStr"/>
       <c r="Z231" s="14" t="n">
@@ -14058,10 +14058,10 @@
       <c r="U232" s="14" t="inlineStr"/>
       <c r="V232" s="14" t="inlineStr"/>
       <c r="W232" s="14" t="n">
-        <v>2.5699806E7</v>
+        <v>2.6608806E7</v>
       </c>
       <c r="X232" s="14" t="n">
-        <v>909000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y232" s="14" t="inlineStr"/>
       <c r="Z232" s="14" t="n">
@@ -14121,10 +14121,10 @@
       <c r="U233" s="14" t="inlineStr"/>
       <c r="V233" s="14" t="inlineStr"/>
       <c r="W233" s="14" t="n">
-        <v>3.51036398E8</v>
+        <v>3.84588968E8</v>
       </c>
       <c r="X233" s="14" t="n">
-        <v>3.355257E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y233" s="14" t="inlineStr"/>
       <c r="Z233" s="14" t="n">
@@ -14481,10 +14481,10 @@
       <c r="U239" s="14" t="inlineStr"/>
       <c r="V239" s="14" t="inlineStr"/>
       <c r="W239" s="14" t="n">
-        <v>9.0095326E7</v>
+        <v>1.10331326E8</v>
       </c>
       <c r="X239" s="14" t="n">
-        <v>2.0236E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y239" s="14" t="inlineStr"/>
       <c r="Z239" s="14" t="n">
@@ -14538,10 +14538,10 @@
       <c r="U240" s="14" t="inlineStr"/>
       <c r="V240" s="14" t="inlineStr"/>
       <c r="W240" s="14" t="n">
-        <v>1.5716622E7</v>
+        <v>1.6931622E7</v>
       </c>
       <c r="X240" s="14" t="n">
-        <v>1215000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y240" s="14" t="inlineStr"/>
       <c r="Z240" s="14" t="n">
@@ -14595,10 +14595,10 @@
       <c r="U241" s="14" t="inlineStr"/>
       <c r="V241" s="14" t="inlineStr"/>
       <c r="W241" s="14" t="n">
-        <v>1.0101299E7</v>
+        <v>1.1156299E7</v>
       </c>
       <c r="X241" s="14" t="n">
-        <v>1055000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y241" s="14" t="inlineStr"/>
       <c r="Z241" s="14" t="n">
@@ -14652,10 +14652,10 @@
       <c r="U242" s="14" t="inlineStr"/>
       <c r="V242" s="14" t="inlineStr"/>
       <c r="W242" s="14" t="n">
-        <v>1.155E7</v>
+        <v>2.5327E7</v>
       </c>
       <c r="X242" s="14" t="n">
-        <v>1.3777E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y242" s="14" t="inlineStr"/>
       <c r="Z242" s="14" t="n">
@@ -15108,10 +15108,10 @@
       <c r="U250" s="14" t="inlineStr"/>
       <c r="V250" s="14" t="inlineStr"/>
       <c r="W250" s="14" t="n">
-        <v>1.1095E7</v>
+        <v>1.5284E7</v>
       </c>
       <c r="X250" s="14" t="n">
-        <v>4189000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y250" s="14" t="inlineStr"/>
       <c r="Z250" s="14" t="n">
@@ -15285,10 +15285,10 @@
       <c r="U253" s="14" t="inlineStr"/>
       <c r="V253" s="14" t="inlineStr"/>
       <c r="W253" s="14" t="n">
-        <v>8.3881357E7</v>
+        <v>8.8386927E7</v>
       </c>
       <c r="X253" s="14" t="n">
-        <v>4505570.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y253" s="14" t="inlineStr"/>
       <c r="Z253" s="14" t="n">
@@ -15556,10 +15556,10 @@
       <c r="U258" s="14" t="inlineStr"/>
       <c r="V258" s="14" t="inlineStr"/>
       <c r="W258" s="14" t="n">
-        <v>6.3191077E7</v>
+        <v>6.6116077E7</v>
       </c>
       <c r="X258" s="14" t="n">
-        <v>2925000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y258" s="14" t="inlineStr"/>
       <c r="Z258" s="14" t="n">
@@ -15613,10 +15613,10 @@
       <c r="U259" s="14" t="inlineStr"/>
       <c r="V259" s="14" t="inlineStr"/>
       <c r="W259" s="14" t="n">
-        <v>2027000.0</v>
+        <v>2177000.0</v>
       </c>
       <c r="X259" s="14" t="n">
-        <v>150000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y259" s="14" t="inlineStr"/>
       <c r="Z259" s="14" t="n">
@@ -15670,10 +15670,10 @@
       <c r="U260" s="14" t="inlineStr"/>
       <c r="V260" s="14" t="inlineStr"/>
       <c r="W260" s="14" t="n">
-        <v>4686025.0</v>
+        <v>4737535.0</v>
       </c>
       <c r="X260" s="14" t="n">
-        <v>51510.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y260" s="14" t="inlineStr"/>
       <c r="Z260" s="14" t="n">
@@ -15841,10 +15841,10 @@
       <c r="U263" s="14" t="inlineStr"/>
       <c r="V263" s="14" t="inlineStr"/>
       <c r="W263" s="14" t="n">
-        <v>2597953.0</v>
+        <v>3707013.0</v>
       </c>
       <c r="X263" s="14" t="n">
-        <v>1109060.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y263" s="14" t="inlineStr"/>
       <c r="Z263" s="14" t="n">
@@ -16012,10 +16012,10 @@
       <c r="U266" s="14" t="inlineStr"/>
       <c r="V266" s="14" t="inlineStr"/>
       <c r="W266" s="14" t="n">
-        <v>0.0</v>
+        <v>270000.0</v>
       </c>
       <c r="X266" s="14" t="n">
-        <v>270000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y266" s="14" t="inlineStr"/>
       <c r="Z266" s="14" t="n">
@@ -16075,10 +16075,10 @@
       <c r="U267" s="14" t="inlineStr"/>
       <c r="V267" s="14" t="inlineStr"/>
       <c r="W267" s="14" t="n">
-        <v>5.2605E7</v>
+        <v>6.1416E7</v>
       </c>
       <c r="X267" s="14" t="n">
-        <v>8811000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y267" s="14" t="inlineStr"/>
       <c r="Z267" s="14" t="n">
@@ -16246,10 +16246,10 @@
       <c r="U270" s="14" t="inlineStr"/>
       <c r="V270" s="14" t="inlineStr"/>
       <c r="W270" s="14" t="n">
-        <v>1965000.0</v>
+        <v>1.0776E7</v>
       </c>
       <c r="X270" s="14" t="n">
-        <v>8811000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y270" s="14" t="inlineStr"/>
       <c r="Z270" s="14" t="n">
@@ -16309,23 +16309,23 @@
       <c r="U271" s="14" t="inlineStr"/>
       <c r="V271" s="14" t="inlineStr"/>
       <c r="W271" s="14" t="n">
-        <v>6.936E7</v>
+        <v>7.975E7</v>
       </c>
       <c r="X271" s="14" t="n">
-        <v>480000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y271" s="14" t="inlineStr"/>
       <c r="Z271" s="14" t="n">
-        <v>6.984E7</v>
+        <v>7.975E7</v>
       </c>
       <c r="AA271" s="14" t="inlineStr"/>
       <c r="AB271" s="14" t="inlineStr"/>
       <c r="AC271" s="15" t="n">
-        <v>0.5283704039945529</v>
+        <v>0.6033439249508247</v>
       </c>
       <c r="AD271" s="15" t="inlineStr"/>
       <c r="AE271" s="14" t="n">
-        <v>6.234E7</v>
+        <v>5.243E7</v>
       </c>
       <c r="AF271" s="14" t="inlineStr"/>
       <c r="AG271" s="14" t="inlineStr"/>
@@ -16372,23 +16372,23 @@
       <c r="U272" s="14" t="inlineStr"/>
       <c r="V272" s="14" t="inlineStr"/>
       <c r="W272" s="14" t="n">
-        <v>6.186E7</v>
+        <v>7.225E7</v>
       </c>
       <c r="X272" s="14" t="n">
-        <v>480000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y272" s="14" t="inlineStr"/>
       <c r="Z272" s="14" t="n">
-        <v>6.234E7</v>
+        <v>7.225E7</v>
       </c>
       <c r="AA272" s="14" t="inlineStr"/>
       <c r="AB272" s="14" t="inlineStr"/>
       <c r="AC272" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5794834777029195</v>
       </c>
       <c r="AD272" s="15" t="inlineStr"/>
       <c r="AE272" s="14" t="n">
-        <v>6.234E7</v>
+        <v>5.243E7</v>
       </c>
       <c r="AF272" s="14" t="inlineStr"/>
       <c r="AG272" s="14" t="inlineStr"/>
@@ -16429,23 +16429,23 @@
       <c r="U273" s="14" t="inlineStr"/>
       <c r="V273" s="14" t="inlineStr"/>
       <c r="W273" s="14" t="n">
-        <v>1.53E7</v>
+        <v>1.785E7</v>
       </c>
       <c r="X273" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y273" s="14" t="inlineStr"/>
       <c r="Z273" s="14" t="n">
-        <v>1.53E7</v>
+        <v>1.785E7</v>
       </c>
       <c r="AA273" s="14" t="inlineStr"/>
       <c r="AB273" s="14" t="inlineStr"/>
       <c r="AC273" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD273" s="15" t="inlineStr"/>
       <c r="AE273" s="14" t="n">
-        <v>1.53E7</v>
+        <v>1.275E7</v>
       </c>
       <c r="AF273" s="14" t="inlineStr"/>
       <c r="AG273" s="14" t="inlineStr"/>
@@ -16486,23 +16486,23 @@
       <c r="U274" s="14" t="inlineStr"/>
       <c r="V274" s="14" t="inlineStr"/>
       <c r="W274" s="14" t="n">
-        <v>1.488E7</v>
+        <v>1.736E7</v>
       </c>
       <c r="X274" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y274" s="14" t="inlineStr"/>
       <c r="Z274" s="14" t="n">
-        <v>1.488E7</v>
+        <v>1.736E7</v>
       </c>
       <c r="AA274" s="14" t="inlineStr"/>
       <c r="AB274" s="14" t="inlineStr"/>
       <c r="AC274" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD274" s="15" t="inlineStr"/>
       <c r="AE274" s="14" t="n">
-        <v>1.488E7</v>
+        <v>1.24E7</v>
       </c>
       <c r="AF274" s="14" t="inlineStr"/>
       <c r="AG274" s="14" t="inlineStr"/>
@@ -16543,23 +16543,23 @@
       <c r="U275" s="14" t="inlineStr"/>
       <c r="V275" s="14" t="inlineStr"/>
       <c r="W275" s="14" t="n">
-        <v>7380000.0</v>
+        <v>8610000.0</v>
       </c>
       <c r="X275" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y275" s="14" t="inlineStr"/>
       <c r="Z275" s="14" t="n">
-        <v>7380000.0</v>
+        <v>8610000.0</v>
       </c>
       <c r="AA275" s="14" t="inlineStr"/>
       <c r="AB275" s="14" t="inlineStr"/>
       <c r="AC275" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD275" s="15" t="inlineStr"/>
       <c r="AE275" s="14" t="n">
-        <v>7380000.0</v>
+        <v>6150000.0</v>
       </c>
       <c r="AF275" s="14" t="inlineStr"/>
       <c r="AG275" s="14" t="inlineStr"/>
@@ -16600,23 +16600,23 @@
       <c r="U276" s="14" t="inlineStr"/>
       <c r="V276" s="14" t="inlineStr"/>
       <c r="W276" s="14" t="n">
-        <v>6420000.0</v>
+        <v>7490000.0</v>
       </c>
       <c r="X276" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y276" s="14" t="inlineStr"/>
       <c r="Z276" s="14" t="n">
-        <v>6420000.0</v>
+        <v>7490000.0</v>
       </c>
       <c r="AA276" s="14" t="inlineStr"/>
       <c r="AB276" s="14" t="inlineStr"/>
       <c r="AC276" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD276" s="15" t="inlineStr"/>
       <c r="AE276" s="14" t="n">
-        <v>6420000.0</v>
+        <v>5350000.0</v>
       </c>
       <c r="AF276" s="14" t="inlineStr"/>
       <c r="AG276" s="14" t="inlineStr"/>
@@ -16657,23 +16657,23 @@
       <c r="U277" s="14" t="inlineStr"/>
       <c r="V277" s="14" t="inlineStr"/>
       <c r="W277" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.68E7</v>
       </c>
       <c r="X277" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y277" s="14" t="inlineStr"/>
       <c r="Z277" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.68E7</v>
       </c>
       <c r="AA277" s="14" t="inlineStr"/>
       <c r="AB277" s="14" t="inlineStr"/>
       <c r="AC277" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD277" s="15" t="inlineStr"/>
       <c r="AE277" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.2E7</v>
       </c>
       <c r="AF277" s="14" t="inlineStr"/>
       <c r="AG277" s="14" t="inlineStr"/>
@@ -16714,10 +16714,10 @@
       <c r="U278" s="14" t="inlineStr"/>
       <c r="V278" s="14" t="inlineStr"/>
       <c r="W278" s="14" t="n">
-        <v>1500000.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="X278" s="14" t="n">
-        <v>300000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y278" s="14" t="inlineStr"/>
       <c r="Z278" s="14" t="n">
@@ -16771,23 +16771,23 @@
       <c r="U279" s="14" t="inlineStr"/>
       <c r="V279" s="14" t="inlineStr"/>
       <c r="W279" s="14" t="n">
-        <v>1980000.0</v>
+        <v>2340000.0</v>
       </c>
       <c r="X279" s="14" t="n">
-        <v>180000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y279" s="14" t="inlineStr"/>
       <c r="Z279" s="14" t="n">
-        <v>2160000.0</v>
+        <v>2340000.0</v>
       </c>
       <c r="AA279" s="14" t="inlineStr"/>
       <c r="AB279" s="14" t="inlineStr"/>
       <c r="AC279" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="AD279" s="15" t="inlineStr"/>
       <c r="AE279" s="14" t="n">
-        <v>2160000.0</v>
+        <v>1980000.0</v>
       </c>
       <c r="AF279" s="14" t="inlineStr"/>
       <c r="AG279" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
Realisasi per 6 Agustus
Realisasi per 6 Agustus
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>6.1530207365E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>6.1530207365E10</v>
+        <v>6.1530855165E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.7237928282641735</v>
+        <v>0.7238004484724294</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>2.3480592635E10</v>
+        <v>2.3479944835E10</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>5.7496839325E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>5.7496839325E10</v>
+        <v>5.7497487125E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.7190262879081493</v>
+        <v>0.7190343889661339</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>2.2468024675E10</v>
+        <v>2.2467376875E10</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>5.7496839325E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>5.7496839325E10</v>
+        <v>5.7497487125E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.7190262879081493</v>
+        <v>0.7190343889661339</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>2.2468024675E10</v>
+        <v>2.2467376875E10</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>5.7496239325E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>5.7496239325E10</v>
+        <v>5.7496887125E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.7190241796635557</v>
+        <v>0.7190322807823255</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>2.2468024675E10</v>
+        <v>2.2467376875E10</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>5.7485503225E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>5.7485503225E10</v>
+        <v>5.7486151025E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.7190565443429414</v>
+        <v>0.7190646473394064</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>2.2460230775E10</v>
+        <v>2.2459582975E10</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -12356,20 +12356,20 @@
         <v>4.15571698E9</v>
       </c>
       <c r="X203" s="25" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y203" s="25" t="inlineStr"/>
       <c r="Z203" s="25" t="n">
-        <v>4.15571698E9</v>
+        <v>4.15636478E9</v>
       </c>
       <c r="AA203" s="25" t="inlineStr"/>
       <c r="AB203" s="25" t="inlineStr"/>
       <c r="AC203" s="26" t="n">
-        <v>0.7347748785355271</v>
+        <v>0.7348894164524753</v>
       </c>
       <c r="AD203" s="26" t="inlineStr"/>
       <c r="AE203" s="25" t="n">
-        <v>1.50005202E9</v>
+        <v>1.49940422E9</v>
       </c>
       <c r="AF203" s="25" t="inlineStr"/>
       <c r="AG203" s="25" t="inlineStr"/>
@@ -13481,20 +13481,20 @@
         <v>4.32620013E8</v>
       </c>
       <c r="X222" s="14" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y222" s="14" t="inlineStr"/>
       <c r="Z222" s="14" t="n">
-        <v>4.32620013E8</v>
+        <v>4.33267813E8</v>
       </c>
       <c r="AA222" s="14" t="inlineStr"/>
       <c r="AB222" s="14" t="inlineStr"/>
       <c r="AC222" s="15" t="n">
-        <v>0.4647829963472282</v>
+        <v>0.4654789568113451</v>
       </c>
       <c r="AD222" s="15" t="inlineStr"/>
       <c r="AE222" s="14" t="n">
-        <v>4.98179987E8</v>
+        <v>4.97532187E8</v>
       </c>
       <c r="AF222" s="14" t="inlineStr"/>
       <c r="AG222" s="14" t="inlineStr"/>
@@ -13784,20 +13784,20 @@
         <v>2.48451E7</v>
       </c>
       <c r="X227" s="14" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y227" s="14" t="inlineStr"/>
       <c r="Z227" s="14" t="n">
-        <v>2.48451E7</v>
+        <v>2.54929E7</v>
       </c>
       <c r="AA227" s="14" t="inlineStr"/>
       <c r="AB227" s="14" t="inlineStr"/>
       <c r="AC227" s="15" t="n">
-        <v>0.6274015151515151</v>
+        <v>0.6437601010101011</v>
       </c>
       <c r="AD227" s="15" t="inlineStr"/>
       <c r="AE227" s="14" t="n">
-        <v>1.47549E7</v>
+        <v>1.41071E7</v>
       </c>
       <c r="AF227" s="14" t="inlineStr"/>
       <c r="AG227" s="14" t="inlineStr"/>
@@ -13884,20 +13884,20 @@
         <v>2.48451E7</v>
       </c>
       <c r="X229" s="14" t="n">
-        <v>0.0</v>
+        <v>647800.0</v>
       </c>
       <c r="Y229" s="14" t="inlineStr"/>
       <c r="Z229" s="14" t="n">
-        <v>2.48451E7</v>
+        <v>2.54929E7</v>
       </c>
       <c r="AA229" s="14" t="inlineStr"/>
       <c r="AB229" s="14" t="inlineStr"/>
       <c r="AC229" s="15" t="n">
-        <v>0.6274015151515151</v>
+        <v>0.6437601010101011</v>
       </c>
       <c r="AD229" s="15" t="inlineStr"/>
       <c r="AE229" s="14" t="n">
-        <v>1.47549E7</v>
+        <v>1.41071E7</v>
       </c>
       <c r="AF229" s="14" t="inlineStr"/>
       <c r="AG229" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
Update realiasi per 12 Agustus
Update realiasi per 12 Agustus, untuk ngecek yang minus 51 apa aja
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>6.1530207365E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>647800.0</v>
+        <v>2.980475502E9</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>6.1530855165E10</v>
+        <v>6.4510682867E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.7238004484724294</v>
+        <v>0.7588527912571109</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>2.3479944835E10</v>
+        <v>2.0500117133E10</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>5.7496839325E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>647800.0</v>
+        <v>2.980475502E9</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>5.7497487125E10</v>
+        <v>6.0477314827E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.7190343889661339</v>
+        <v>0.7562986016833594</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>2.2467376875E10</v>
+        <v>1.9487549173E10</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>5.7496839325E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>647800.0</v>
+        <v>2.980475502E9</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>5.7497487125E10</v>
+        <v>6.0477314827E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.7190343889661339</v>
+        <v>0.7562986016833594</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>2.2467376875E10</v>
+        <v>1.9487549173E10</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>5.7496239325E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>647800.0</v>
+        <v>2.980475502E9</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>5.7496887125E10</v>
+        <v>6.0476714827E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.7190322807823255</v>
+        <v>0.7562967731060465</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>2.2467376875E10</v>
+        <v>1.9487549173E10</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>5.7485503225E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>647800.0</v>
+        <v>2.980475502E9</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>5.7486151025E10</v>
+        <v>6.0465978727E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.7190646473394064</v>
+        <v>0.7563377769100225</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>2.2459582975E10</v>
+        <v>1.9479755273E10</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3296,20 +3296,20 @@
         <v>5.3329786245E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>0.0</v>
+        <v>2.81070658E9</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
-        <v>5.3329786245E10</v>
+        <v>5.6140492825E10</v>
       </c>
       <c r="AA47" s="25" t="inlineStr"/>
       <c r="AB47" s="25" t="inlineStr"/>
       <c r="AC47" s="26" t="n">
-        <v>0.7178598919113772</v>
+        <v>0.755694161721573</v>
       </c>
       <c r="AD47" s="26" t="inlineStr"/>
       <c r="AE47" s="25" t="n">
-        <v>2.0960178755E10</v>
+        <v>1.8149472175E10</v>
       </c>
       <c r="AF47" s="25" t="inlineStr"/>
       <c r="AG47" s="25" t="inlineStr"/>
@@ -3359,20 +3359,20 @@
         <v>4.187549504E9</v>
       </c>
       <c r="X48" s="14" t="n">
-        <v>0.0</v>
+        <v>5.4407639E7</v>
       </c>
       <c r="Y48" s="14" t="inlineStr"/>
       <c r="Z48" s="14" t="n">
-        <v>4.187549504E9</v>
+        <v>4.241957143E9</v>
       </c>
       <c r="AA48" s="14" t="inlineStr"/>
       <c r="AB48" s="14" t="inlineStr"/>
       <c r="AC48" s="15" t="n">
-        <v>0.6536032120530656</v>
+        <v>0.662095292582897</v>
       </c>
       <c r="AD48" s="15" t="inlineStr"/>
       <c r="AE48" s="14" t="n">
-        <v>2.219318496E9</v>
+        <v>2.164910857E9</v>
       </c>
       <c r="AF48" s="14" t="inlineStr"/>
       <c r="AG48" s="14" t="inlineStr"/>
@@ -3422,20 +3422,20 @@
         <v>1.6503171E9</v>
       </c>
       <c r="X49" s="14" t="n">
-        <v>0.0</v>
+        <v>1.62007E7</v>
       </c>
       <c r="Y49" s="14" t="inlineStr"/>
       <c r="Z49" s="14" t="n">
-        <v>1.6503171E9</v>
+        <v>1.6665178E9</v>
       </c>
       <c r="AA49" s="14" t="inlineStr"/>
       <c r="AB49" s="14" t="inlineStr"/>
       <c r="AC49" s="15" t="n">
-        <v>0.5888925167213339</v>
+        <v>0.5946735093533847</v>
       </c>
       <c r="AD49" s="15" t="inlineStr"/>
       <c r="AE49" s="14" t="n">
-        <v>1.1520909E9</v>
+        <v>1.1358902E9</v>
       </c>
       <c r="AF49" s="14" t="inlineStr"/>
       <c r="AG49" s="14" t="inlineStr"/>
@@ -3479,20 +3479,20 @@
         <v>1.3201367E9</v>
       </c>
       <c r="X50" s="14" t="n">
-        <v>0.0</v>
+        <v>1.62007E7</v>
       </c>
       <c r="Y50" s="14" t="inlineStr"/>
       <c r="Z50" s="14" t="n">
-        <v>1.3201367E9</v>
+        <v>1.3363374E9</v>
       </c>
       <c r="AA50" s="14" t="inlineStr"/>
       <c r="AB50" s="14" t="inlineStr"/>
       <c r="AC50" s="15" t="n">
-        <v>0.5369028387831463</v>
+        <v>0.5434917032698877</v>
       </c>
       <c r="AD50" s="15" t="inlineStr"/>
       <c r="AE50" s="14" t="n">
-        <v>1.1386633E9</v>
+        <v>1.1224626E9</v>
       </c>
       <c r="AF50" s="14" t="inlineStr"/>
       <c r="AG50" s="14" t="inlineStr"/>
@@ -3656,20 +3656,20 @@
         <v>19549.0</v>
       </c>
       <c r="X53" s="14" t="n">
-        <v>0.0</v>
+        <v>121.0</v>
       </c>
       <c r="Y53" s="14" t="inlineStr"/>
       <c r="Z53" s="14" t="n">
-        <v>19549.0</v>
+        <v>19670.0</v>
       </c>
       <c r="AA53" s="14" t="inlineStr"/>
       <c r="AB53" s="14" t="inlineStr"/>
       <c r="AC53" s="15" t="n">
-        <v>0.6516333333333333</v>
+        <v>0.6556666666666666</v>
       </c>
       <c r="AD53" s="15" t="inlineStr"/>
       <c r="AE53" s="14" t="n">
-        <v>10451.0</v>
+        <v>10330.0</v>
       </c>
       <c r="AF53" s="14" t="inlineStr"/>
       <c r="AG53" s="14" t="inlineStr"/>
@@ -3713,20 +3713,20 @@
         <v>14967.0</v>
       </c>
       <c r="X54" s="14" t="n">
-        <v>0.0</v>
+        <v>121.0</v>
       </c>
       <c r="Y54" s="14" t="inlineStr"/>
       <c r="Z54" s="14" t="n">
-        <v>14967.0</v>
+        <v>15088.0</v>
       </c>
       <c r="AA54" s="14" t="inlineStr"/>
       <c r="AB54" s="14" t="inlineStr"/>
       <c r="AC54" s="15" t="n">
-        <v>0.623625</v>
+        <v>0.6286666666666667</v>
       </c>
       <c r="AD54" s="15" t="inlineStr"/>
       <c r="AE54" s="14" t="n">
-        <v>9033.0</v>
+        <v>8912.0</v>
       </c>
       <c r="AF54" s="14" t="inlineStr"/>
       <c r="AG54" s="14" t="inlineStr"/>
@@ -3890,20 +3890,20 @@
         <v>1.2585432E8</v>
       </c>
       <c r="X57" s="14" t="n">
-        <v>0.0</v>
+        <v>1620070.0</v>
       </c>
       <c r="Y57" s="14" t="inlineStr"/>
       <c r="Z57" s="14" t="n">
-        <v>1.2585432E8</v>
+        <v>1.2747439E8</v>
       </c>
       <c r="AA57" s="14" t="inlineStr"/>
       <c r="AB57" s="14" t="inlineStr"/>
       <c r="AC57" s="15" t="n">
-        <v>0.6915072527472528</v>
+        <v>0.7004087362637362</v>
       </c>
       <c r="AD57" s="15" t="inlineStr"/>
       <c r="AE57" s="14" t="n">
-        <v>5.614568E7</v>
+        <v>5.452561E7</v>
       </c>
       <c r="AF57" s="14" t="inlineStr"/>
       <c r="AG57" s="14" t="inlineStr"/>
@@ -3947,20 +3947,20 @@
         <v>1.00656E8</v>
       </c>
       <c r="X58" s="14" t="n">
-        <v>0.0</v>
+        <v>1620070.0</v>
       </c>
       <c r="Y58" s="14" t="inlineStr"/>
       <c r="Z58" s="14" t="n">
-        <v>1.00656E8</v>
+        <v>1.0227607E8</v>
       </c>
       <c r="AA58" s="14" t="inlineStr"/>
       <c r="AB58" s="14" t="inlineStr"/>
       <c r="AC58" s="15" t="n">
-        <v>0.6452307692307693</v>
+        <v>0.6556158333333333</v>
       </c>
       <c r="AD58" s="15" t="inlineStr"/>
       <c r="AE58" s="14" t="n">
-        <v>5.5344E7</v>
+        <v>5.372393E7</v>
       </c>
       <c r="AF58" s="14" t="inlineStr"/>
       <c r="AG58" s="14" t="inlineStr"/>
@@ -4167,20 +4167,20 @@
         <v>3.8237084E7</v>
       </c>
       <c r="X62" s="14" t="n">
-        <v>0.0</v>
+        <v>648028.0</v>
       </c>
       <c r="Y62" s="14" t="inlineStr"/>
       <c r="Z62" s="14" t="n">
-        <v>3.8237084E7</v>
+        <v>3.8885112E7</v>
       </c>
       <c r="AA62" s="14" t="inlineStr"/>
       <c r="AB62" s="14" t="inlineStr"/>
       <c r="AC62" s="15" t="n">
-        <v>0.6828050714285714</v>
+        <v>0.694377</v>
       </c>
       <c r="AD62" s="15" t="inlineStr"/>
       <c r="AE62" s="14" t="n">
-        <v>1.7762916E7</v>
+        <v>1.7114888E7</v>
       </c>
       <c r="AF62" s="14" t="inlineStr"/>
       <c r="AG62" s="14" t="inlineStr"/>
@@ -4224,20 +4224,20 @@
         <v>3.0561026E7</v>
       </c>
       <c r="X63" s="14" t="n">
-        <v>0.0</v>
+        <v>648028.0</v>
       </c>
       <c r="Y63" s="14" t="inlineStr"/>
       <c r="Z63" s="14" t="n">
-        <v>3.0561026E7</v>
+        <v>3.1209054E7</v>
       </c>
       <c r="AA63" s="14" t="inlineStr"/>
       <c r="AB63" s="14" t="inlineStr"/>
       <c r="AC63" s="15" t="n">
-        <v>0.6366880416666667</v>
+        <v>0.650188625</v>
       </c>
       <c r="AD63" s="15" t="inlineStr"/>
       <c r="AE63" s="14" t="n">
-        <v>1.7438974E7</v>
+        <v>1.6790946E7</v>
       </c>
       <c r="AF63" s="14" t="inlineStr"/>
       <c r="AG63" s="14" t="inlineStr"/>
@@ -4401,20 +4401,20 @@
         <v>1.8E7</v>
       </c>
       <c r="X66" s="14" t="n">
-        <v>0.0</v>
+        <v>540000.0</v>
       </c>
       <c r="Y66" s="14" t="inlineStr"/>
       <c r="Z66" s="14" t="n">
-        <v>1.8E7</v>
+        <v>1.854E7</v>
       </c>
       <c r="AA66" s="14" t="inlineStr"/>
       <c r="AB66" s="14" t="inlineStr"/>
       <c r="AC66" s="15" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7357142857142858</v>
       </c>
       <c r="AD66" s="15" t="inlineStr"/>
       <c r="AE66" s="14" t="n">
-        <v>7200000.0</v>
+        <v>6660000.0</v>
       </c>
       <c r="AF66" s="14" t="inlineStr"/>
       <c r="AG66" s="14" t="inlineStr"/>
@@ -4458,20 +4458,20 @@
         <v>1.44E7</v>
       </c>
       <c r="X67" s="14" t="n">
-        <v>0.0</v>
+        <v>540000.0</v>
       </c>
       <c r="Y67" s="14" t="inlineStr"/>
       <c r="Z67" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.494E7</v>
       </c>
       <c r="AA67" s="14" t="inlineStr"/>
       <c r="AB67" s="14" t="inlineStr"/>
       <c r="AC67" s="15" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6916666666666667</v>
       </c>
       <c r="AD67" s="15" t="inlineStr"/>
       <c r="AE67" s="14" t="n">
-        <v>7200000.0</v>
+        <v>6660000.0</v>
       </c>
       <c r="AF67" s="14" t="inlineStr"/>
       <c r="AG67" s="14" t="inlineStr"/>
@@ -4635,20 +4635,20 @@
         <v>1.1796E8</v>
       </c>
       <c r="X70" s="14" t="n">
-        <v>0.0</v>
+        <v>1100000.0</v>
       </c>
       <c r="Y70" s="14" t="inlineStr"/>
       <c r="Z70" s="14" t="n">
-        <v>1.1796E8</v>
+        <v>1.1906E8</v>
       </c>
       <c r="AA70" s="14" t="inlineStr"/>
       <c r="AB70" s="14" t="inlineStr"/>
       <c r="AC70" s="15" t="n">
-        <v>0.8134387024701063</v>
+        <v>0.8210241769760162</v>
       </c>
       <c r="AD70" s="15" t="inlineStr"/>
       <c r="AE70" s="14" t="n">
-        <v>2.7054E7</v>
+        <v>2.5954E7</v>
       </c>
       <c r="AF70" s="14" t="inlineStr"/>
       <c r="AG70" s="14" t="inlineStr"/>
@@ -4692,20 +4692,20 @@
         <v>9.3932E7</v>
       </c>
       <c r="X71" s="14" t="n">
-        <v>0.0</v>
+        <v>1100000.0</v>
       </c>
       <c r="Y71" s="14" t="inlineStr"/>
       <c r="Z71" s="14" t="n">
-        <v>9.3932E7</v>
+        <v>9.5032E7</v>
       </c>
       <c r="AA71" s="14" t="inlineStr"/>
       <c r="AB71" s="14" t="inlineStr"/>
       <c r="AC71" s="15" t="n">
-        <v>0.7827666666666667</v>
+        <v>0.7919333333333334</v>
       </c>
       <c r="AD71" s="15" t="inlineStr"/>
       <c r="AE71" s="14" t="n">
-        <v>2.6068E7</v>
+        <v>2.4968E7</v>
       </c>
       <c r="AF71" s="14" t="inlineStr"/>
       <c r="AG71" s="14" t="inlineStr"/>
@@ -5103,20 +5103,20 @@
         <v>8.72661E7</v>
       </c>
       <c r="X78" s="14" t="n">
-        <v>0.0</v>
+        <v>1158720.0</v>
       </c>
       <c r="Y78" s="14" t="inlineStr"/>
       <c r="Z78" s="14" t="n">
-        <v>8.72661E7</v>
+        <v>8.842482E7</v>
       </c>
       <c r="AA78" s="14" t="inlineStr"/>
       <c r="AB78" s="14" t="inlineStr"/>
       <c r="AC78" s="15" t="n">
-        <v>0.6925880952380953</v>
+        <v>0.7017842857142857</v>
       </c>
       <c r="AD78" s="15" t="inlineStr"/>
       <c r="AE78" s="14" t="n">
-        <v>3.87339E7</v>
+        <v>3.757518E7</v>
       </c>
       <c r="AF78" s="14" t="inlineStr"/>
       <c r="AG78" s="14" t="inlineStr"/>
@@ -5160,20 +5160,20 @@
         <v>6.974046E7</v>
       </c>
       <c r="X79" s="14" t="n">
-        <v>0.0</v>
+        <v>1158720.0</v>
       </c>
       <c r="Y79" s="14" t="inlineStr"/>
       <c r="Z79" s="14" t="n">
-        <v>6.974046E7</v>
+        <v>7.089918E7</v>
       </c>
       <c r="AA79" s="14" t="inlineStr"/>
       <c r="AB79" s="14" t="inlineStr"/>
       <c r="AC79" s="15" t="n">
-        <v>0.645745</v>
+        <v>0.6564738888888889</v>
       </c>
       <c r="AD79" s="15" t="inlineStr"/>
       <c r="AE79" s="14" t="n">
-        <v>3.825954E7</v>
+        <v>3.710082E7</v>
       </c>
       <c r="AF79" s="14" t="inlineStr"/>
       <c r="AG79" s="14" t="inlineStr"/>
@@ -5337,20 +5337,20 @@
         <v>1.54008E8</v>
       </c>
       <c r="X82" s="14" t="n">
-        <v>0.0</v>
+        <v>3.2765E7</v>
       </c>
       <c r="Y82" s="14" t="inlineStr"/>
       <c r="Z82" s="14" t="n">
-        <v>1.54008E8</v>
+        <v>1.86773E8</v>
       </c>
       <c r="AA82" s="14" t="inlineStr"/>
       <c r="AB82" s="14" t="inlineStr"/>
       <c r="AC82" s="15" t="n">
-        <v>0.4913852515506547</v>
+        <v>0.5959268193072466</v>
       </c>
       <c r="AD82" s="15" t="inlineStr"/>
       <c r="AE82" s="14" t="n">
-        <v>1.59408E8</v>
+        <v>1.26643E8</v>
       </c>
       <c r="AF82" s="14" t="inlineStr"/>
       <c r="AG82" s="14" t="inlineStr"/>
@@ -5394,20 +5394,20 @@
         <v>9450000.0</v>
       </c>
       <c r="X83" s="14" t="n">
-        <v>0.0</v>
+        <v>1610000.0</v>
       </c>
       <c r="Y83" s="14" t="inlineStr"/>
       <c r="Z83" s="14" t="n">
-        <v>9450000.0</v>
+        <v>1.106E7</v>
       </c>
       <c r="AA83" s="14" t="inlineStr"/>
       <c r="AB83" s="14" t="inlineStr"/>
       <c r="AC83" s="15" t="n">
-        <v>0.3125</v>
+        <v>0.36574074074074076</v>
       </c>
       <c r="AD83" s="15" t="inlineStr"/>
       <c r="AE83" s="14" t="n">
-        <v>2.079E7</v>
+        <v>1.918E7</v>
       </c>
       <c r="AF83" s="14" t="inlineStr"/>
       <c r="AG83" s="14" t="inlineStr"/>
@@ -5451,20 +5451,20 @@
         <v>1.25985E8</v>
       </c>
       <c r="X84" s="14" t="n">
-        <v>0.0</v>
+        <v>2.6973E7</v>
       </c>
       <c r="Y84" s="14" t="inlineStr"/>
       <c r="Z84" s="14" t="n">
-        <v>1.25985E8</v>
+        <v>1.52958E8</v>
       </c>
       <c r="AA84" s="14" t="inlineStr"/>
       <c r="AB84" s="14" t="inlineStr"/>
       <c r="AC84" s="15" t="n">
-        <v>0.5085125448028673</v>
+        <v>0.6173835125448028</v>
       </c>
       <c r="AD84" s="15" t="inlineStr"/>
       <c r="AE84" s="14" t="n">
-        <v>1.21767E8</v>
+        <v>9.4794E7</v>
       </c>
       <c r="AF84" s="14" t="inlineStr"/>
       <c r="AG84" s="14" t="inlineStr"/>
@@ -5508,20 +5508,20 @@
         <v>1.8573E7</v>
       </c>
       <c r="X85" s="14" t="n">
-        <v>0.0</v>
+        <v>4182000.0</v>
       </c>
       <c r="Y85" s="14" t="inlineStr"/>
       <c r="Z85" s="14" t="n">
-        <v>1.8573E7</v>
+        <v>2.2755E7</v>
       </c>
       <c r="AA85" s="14" t="inlineStr"/>
       <c r="AB85" s="14" t="inlineStr"/>
       <c r="AC85" s="15" t="n">
-        <v>0.5243055555555556</v>
+        <v>0.6423611111111112</v>
       </c>
       <c r="AD85" s="15" t="inlineStr"/>
       <c r="AE85" s="14" t="n">
-        <v>1.6851E7</v>
+        <v>1.2669E7</v>
       </c>
       <c r="AF85" s="14" t="inlineStr"/>
       <c r="AG85" s="14" t="inlineStr"/>
@@ -5571,20 +5571,20 @@
         <v>4.044E7</v>
       </c>
       <c r="X86" s="14" t="n">
-        <v>0.0</v>
+        <v>375000.0</v>
       </c>
       <c r="Y86" s="14" t="inlineStr"/>
       <c r="Z86" s="14" t="n">
-        <v>4.044E7</v>
+        <v>4.0815E7</v>
       </c>
       <c r="AA86" s="14" t="inlineStr"/>
       <c r="AB86" s="14" t="inlineStr"/>
       <c r="AC86" s="15" t="n">
-        <v>0.6419047619047619</v>
+        <v>0.6478571428571429</v>
       </c>
       <c r="AD86" s="15" t="inlineStr"/>
       <c r="AE86" s="14" t="n">
-        <v>2.256E7</v>
+        <v>2.2185E7</v>
       </c>
       <c r="AF86" s="14" t="inlineStr"/>
       <c r="AG86" s="14" t="inlineStr"/>
@@ -5628,20 +5628,20 @@
         <v>3.251E7</v>
       </c>
       <c r="X87" s="14" t="n">
-        <v>0.0</v>
+        <v>375000.0</v>
       </c>
       <c r="Y87" s="14" t="inlineStr"/>
       <c r="Z87" s="14" t="n">
-        <v>3.251E7</v>
+        <v>3.2885E7</v>
       </c>
       <c r="AA87" s="14" t="inlineStr"/>
       <c r="AB87" s="14" t="inlineStr"/>
       <c r="AC87" s="15" t="n">
-        <v>0.602037037037037</v>
+        <v>0.6089814814814815</v>
       </c>
       <c r="AD87" s="15" t="inlineStr"/>
       <c r="AE87" s="14" t="n">
-        <v>2.149E7</v>
+        <v>2.1115E7</v>
       </c>
       <c r="AF87" s="14" t="inlineStr"/>
       <c r="AG87" s="14" t="inlineStr"/>
@@ -7946,20 +7946,20 @@
         <v>3.5544999187E10</v>
       </c>
       <c r="X127" s="14" t="n">
-        <v>0.0</v>
+        <v>1.897709787E9</v>
       </c>
       <c r="Y127" s="14" t="inlineStr"/>
       <c r="Z127" s="14" t="n">
-        <v>3.5544999187E10</v>
+        <v>3.7442708974E10</v>
       </c>
       <c r="AA127" s="14" t="inlineStr"/>
       <c r="AB127" s="14" t="inlineStr"/>
       <c r="AC127" s="15" t="n">
-        <v>0.672068230837679</v>
+        <v>0.7079492404976508</v>
       </c>
       <c r="AD127" s="15" t="inlineStr"/>
       <c r="AE127" s="14" t="n">
-        <v>1.7343974813E10</v>
+        <v>1.5446265026E10</v>
       </c>
       <c r="AF127" s="14" t="inlineStr"/>
       <c r="AG127" s="14" t="inlineStr"/>
@@ -8009,20 +8009,20 @@
         <v>1.23832303E10</v>
       </c>
       <c r="X128" s="14" t="n">
-        <v>0.0</v>
+        <v>1.190934E9</v>
       </c>
       <c r="Y128" s="14" t="inlineStr"/>
       <c r="Z128" s="14" t="n">
-        <v>1.23832303E10</v>
+        <v>1.35741643E10</v>
       </c>
       <c r="AA128" s="14" t="inlineStr"/>
       <c r="AB128" s="14" t="inlineStr"/>
       <c r="AC128" s="15" t="n">
-        <v>0.9416393177101017</v>
+        <v>1.0321997168975223</v>
       </c>
       <c r="AD128" s="15" t="inlineStr"/>
       <c r="AE128" s="14" t="n">
-        <v>7.674847E8</v>
+        <v>-4.234493E8</v>
       </c>
       <c r="AF128" s="14" t="inlineStr"/>
       <c r="AG128" s="14" t="inlineStr"/>
@@ -8066,20 +8066,20 @@
         <v>9.8924769E9</v>
       </c>
       <c r="X129" s="14" t="n">
-        <v>0.0</v>
+        <v>1.190934E9</v>
       </c>
       <c r="Y129" s="14" t="inlineStr"/>
       <c r="Z129" s="14" t="n">
-        <v>9.8924769E9</v>
+        <v>1.10834109E10</v>
       </c>
       <c r="AA129" s="14" t="inlineStr"/>
       <c r="AB129" s="14" t="inlineStr"/>
       <c r="AC129" s="15" t="n">
-        <v>0.933490665920816</v>
+        <v>1.0458715978113662</v>
       </c>
       <c r="AD129" s="15" t="inlineStr"/>
       <c r="AE129" s="14" t="n">
-        <v>7.048191E8</v>
+        <v>-4.861149E8</v>
       </c>
       <c r="AF129" s="14" t="inlineStr"/>
       <c r="AG129" s="14" t="inlineStr"/>
@@ -8243,20 +8243,20 @@
         <v>168114.0</v>
       </c>
       <c r="X132" s="14" t="n">
-        <v>0.0</v>
+        <v>15731.0</v>
       </c>
       <c r="Y132" s="14" t="inlineStr"/>
       <c r="Z132" s="14" t="n">
-        <v>168114.0</v>
+        <v>183845.0</v>
       </c>
       <c r="AA132" s="14" t="inlineStr"/>
       <c r="AB132" s="14" t="inlineStr"/>
       <c r="AC132" s="15" t="n">
-        <v>0.7063613445378151</v>
+        <v>0.7724579831932773</v>
       </c>
       <c r="AD132" s="15" t="inlineStr"/>
       <c r="AE132" s="14" t="n">
-        <v>69886.0</v>
+        <v>54155.0</v>
       </c>
       <c r="AF132" s="14" t="inlineStr"/>
       <c r="AG132" s="14" t="inlineStr"/>
@@ -8300,20 +8300,20 @@
         <v>134340.0</v>
       </c>
       <c r="X133" s="14" t="n">
-        <v>0.0</v>
+        <v>15731.0</v>
       </c>
       <c r="Y133" s="14" t="inlineStr"/>
       <c r="Z133" s="14" t="n">
-        <v>134340.0</v>
+        <v>150071.0</v>
       </c>
       <c r="AA133" s="14" t="inlineStr"/>
       <c r="AB133" s="14" t="inlineStr"/>
       <c r="AC133" s="15" t="n">
-        <v>0.6585294117647059</v>
+        <v>0.7356421568627451</v>
       </c>
       <c r="AD133" s="15" t="inlineStr"/>
       <c r="AE133" s="14" t="n">
-        <v>69660.0</v>
+        <v>53929.0</v>
       </c>
       <c r="AF133" s="14" t="inlineStr"/>
       <c r="AG133" s="14" t="inlineStr"/>
@@ -8477,20 +8477,20 @@
         <v>9.7329066E8</v>
       </c>
       <c r="X136" s="14" t="n">
-        <v>0.0</v>
+        <v>9.414094E7</v>
       </c>
       <c r="Y136" s="14" t="inlineStr"/>
       <c r="Z136" s="14" t="n">
-        <v>9.7329066E8</v>
+        <v>1.0674316E9</v>
       </c>
       <c r="AA136" s="14" t="inlineStr"/>
       <c r="AB136" s="14" t="inlineStr"/>
       <c r="AC136" s="15" t="n">
-        <v>0.7096282745798549</v>
+        <v>0.7782666326419015</v>
       </c>
       <c r="AD136" s="15" t="inlineStr"/>
       <c r="AE136" s="14" t="n">
-        <v>3.9825934E8</v>
+        <v>3.041184E8</v>
       </c>
       <c r="AF136" s="14" t="inlineStr"/>
       <c r="AG136" s="14" t="inlineStr"/>
@@ -8534,20 +8534,20 @@
         <v>7.783056E8</v>
       </c>
       <c r="X137" s="14" t="n">
-        <v>0.0</v>
+        <v>9.414094E7</v>
       </c>
       <c r="Y137" s="14" t="inlineStr"/>
       <c r="Z137" s="14" t="n">
-        <v>7.783056E8</v>
+        <v>8.7244654E8</v>
       </c>
       <c r="AA137" s="14" t="inlineStr"/>
       <c r="AB137" s="14" t="inlineStr"/>
       <c r="AC137" s="15" t="n">
-        <v>0.6618244897959183</v>
+        <v>0.7418763095238096</v>
       </c>
       <c r="AD137" s="15" t="inlineStr"/>
       <c r="AE137" s="14" t="n">
-        <v>3.976944E8</v>
+        <v>3.0355346E8</v>
       </c>
       <c r="AF137" s="14" t="inlineStr"/>
       <c r="AG137" s="14" t="inlineStr"/>
@@ -8711,20 +8711,20 @@
         <v>3.02306822E8</v>
       </c>
       <c r="X140" s="14" t="n">
-        <v>0.0</v>
+        <v>2.9613198E7</v>
       </c>
       <c r="Y140" s="14" t="inlineStr"/>
       <c r="Z140" s="14" t="n">
-        <v>3.02306822E8</v>
+        <v>3.3192002E8</v>
       </c>
       <c r="AA140" s="14" t="inlineStr"/>
       <c r="AB140" s="14" t="inlineStr"/>
       <c r="AC140" s="15" t="n">
-        <v>0.6977540397500791</v>
+        <v>0.7661042291295929</v>
       </c>
       <c r="AD140" s="15" t="inlineStr"/>
       <c r="AE140" s="14" t="n">
-        <v>1.30950178E8</v>
+        <v>1.0133698E8</v>
       </c>
       <c r="AF140" s="14" t="inlineStr"/>
       <c r="AG140" s="14" t="inlineStr"/>
@@ -8768,20 +8768,20 @@
         <v>2.41915966E8</v>
       </c>
       <c r="X141" s="14" t="n">
-        <v>0.0</v>
+        <v>2.9613198E7</v>
       </c>
       <c r="Y141" s="14" t="inlineStr"/>
       <c r="Z141" s="14" t="n">
-        <v>2.41915966E8</v>
+        <v>2.71529164E8</v>
       </c>
       <c r="AA141" s="14" t="inlineStr"/>
       <c r="AB141" s="14" t="inlineStr"/>
       <c r="AC141" s="15" t="n">
-        <v>0.6503117365591398</v>
+        <v>0.7299171075268818</v>
       </c>
       <c r="AD141" s="15" t="inlineStr"/>
       <c r="AE141" s="14" t="n">
-        <v>1.30084034E8</v>
+        <v>1.00470836E8</v>
       </c>
       <c r="AF141" s="14" t="inlineStr"/>
       <c r="AG141" s="14" t="inlineStr"/>
@@ -8945,20 +8945,20 @@
         <v>2.67431E9</v>
       </c>
       <c r="X144" s="14" t="n">
-        <v>0.0</v>
+        <v>2.5602E8</v>
       </c>
       <c r="Y144" s="14" t="inlineStr"/>
       <c r="Z144" s="14" t="n">
-        <v>2.67431E9</v>
+        <v>2.93033E9</v>
       </c>
       <c r="AA144" s="14" t="inlineStr"/>
       <c r="AB144" s="14" t="inlineStr"/>
       <c r="AC144" s="15" t="n">
-        <v>0.694625974025974</v>
+        <v>0.7611246753246753</v>
       </c>
       <c r="AD144" s="15" t="inlineStr"/>
       <c r="AE144" s="14" t="n">
-        <v>1.17569E9</v>
+        <v>9.1967E8</v>
       </c>
       <c r="AF144" s="14" t="inlineStr"/>
       <c r="AG144" s="14" t="inlineStr"/>
@@ -9045,20 +9045,20 @@
         <v>2.13605E9</v>
       </c>
       <c r="X146" s="14" t="n">
-        <v>0.0</v>
+        <v>2.5602E8</v>
       </c>
       <c r="Y146" s="14" t="inlineStr"/>
       <c r="Z146" s="14" t="n">
-        <v>2.13605E9</v>
+        <v>2.39207E9</v>
       </c>
       <c r="AA146" s="14" t="inlineStr"/>
       <c r="AB146" s="14" t="inlineStr"/>
       <c r="AC146" s="15" t="n">
-        <v>0.6472878787878787</v>
+        <v>0.7248696969696969</v>
       </c>
       <c r="AD146" s="15" t="inlineStr"/>
       <c r="AE146" s="14" t="n">
-        <v>1.16395E9</v>
+        <v>9.0793E8</v>
       </c>
       <c r="AF146" s="14" t="inlineStr"/>
       <c r="AG146" s="14" t="inlineStr"/>
@@ -9222,20 +9222,20 @@
         <v>2.17635496E8</v>
       </c>
       <c r="X149" s="14" t="n">
-        <v>0.0</v>
+        <v>3343198.0</v>
       </c>
       <c r="Y149" s="14" t="inlineStr"/>
       <c r="Z149" s="14" t="n">
-        <v>2.17635496E8</v>
+        <v>2.20978694E8</v>
       </c>
       <c r="AA149" s="14" t="inlineStr"/>
       <c r="AB149" s="14" t="inlineStr"/>
       <c r="AC149" s="15" t="n">
-        <v>0.885669214178163</v>
+        <v>0.8992743824522851</v>
       </c>
       <c r="AD149" s="15" t="inlineStr"/>
       <c r="AE149" s="14" t="n">
-        <v>2.8094504E7</v>
+        <v>2.4751306E7</v>
       </c>
       <c r="AF149" s="14" t="inlineStr"/>
       <c r="AG149" s="14" t="inlineStr"/>
@@ -9279,20 +9279,20 @@
         <v>3.2179365E7</v>
       </c>
       <c r="X150" s="14" t="n">
-        <v>0.0</v>
+        <v>3343198.0</v>
       </c>
       <c r="Y150" s="14" t="inlineStr"/>
       <c r="Z150" s="14" t="n">
-        <v>3.2179365E7</v>
+        <v>3.5522563E7</v>
       </c>
       <c r="AA150" s="14" t="inlineStr"/>
       <c r="AB150" s="14" t="inlineStr"/>
       <c r="AC150" s="15" t="n">
-        <v>0.53632275</v>
+        <v>0.5920427166666666</v>
       </c>
       <c r="AD150" s="15" t="inlineStr"/>
       <c r="AE150" s="14" t="n">
-        <v>2.7820635E7</v>
+        <v>2.4477437E7</v>
       </c>
       <c r="AF150" s="14" t="inlineStr"/>
       <c r="AG150" s="14" t="inlineStr"/>
@@ -9456,20 +9456,20 @@
         <v>6.7995138E8</v>
       </c>
       <c r="X153" s="14" t="n">
-        <v>0.0</v>
+        <v>6.633672E7</v>
       </c>
       <c r="Y153" s="14" t="inlineStr"/>
       <c r="Z153" s="14" t="n">
-        <v>6.7995138E8</v>
+        <v>7.462881E8</v>
       </c>
       <c r="AA153" s="14" t="inlineStr"/>
       <c r="AB153" s="14" t="inlineStr"/>
       <c r="AC153" s="15" t="n">
-        <v>0.6938279387755102</v>
+        <v>0.7615184693877551</v>
       </c>
       <c r="AD153" s="15" t="inlineStr"/>
       <c r="AE153" s="14" t="n">
-        <v>3.0004862E8</v>
+        <v>2.337119E8</v>
       </c>
       <c r="AF153" s="14" t="inlineStr"/>
       <c r="AG153" s="14" t="inlineStr"/>
@@ -9513,20 +9513,20 @@
         <v>5.4322242E8</v>
       </c>
       <c r="X154" s="14" t="n">
-        <v>0.0</v>
+        <v>6.633672E7</v>
       </c>
       <c r="Y154" s="14" t="inlineStr"/>
       <c r="Z154" s="14" t="n">
-        <v>5.4322242E8</v>
+        <v>6.0955914E8</v>
       </c>
       <c r="AA154" s="14" t="inlineStr"/>
       <c r="AB154" s="14" t="inlineStr"/>
       <c r="AC154" s="15" t="n">
-        <v>0.6466933571428571</v>
+        <v>0.7256656428571429</v>
       </c>
       <c r="AD154" s="15" t="inlineStr"/>
       <c r="AE154" s="14" t="n">
-        <v>2.9677758E8</v>
+        <v>2.3044086E8</v>
       </c>
       <c r="AF154" s="14" t="inlineStr"/>
       <c r="AG154" s="14" t="inlineStr"/>
@@ -9690,20 +9690,20 @@
         <v>1.249247E9</v>
       </c>
       <c r="X157" s="14" t="n">
-        <v>0.0</v>
+        <v>2.57121E8</v>
       </c>
       <c r="Y157" s="14" t="inlineStr"/>
       <c r="Z157" s="14" t="n">
-        <v>1.249247E9</v>
+        <v>1.506368E9</v>
       </c>
       <c r="AA157" s="14" t="inlineStr"/>
       <c r="AB157" s="14" t="inlineStr"/>
       <c r="AC157" s="15" t="n">
-        <v>0.47821654753811194</v>
+        <v>0.5766434534418658</v>
       </c>
       <c r="AD157" s="15" t="inlineStr"/>
       <c r="AE157" s="14" t="n">
-        <v>1.363057E9</v>
+        <v>1.105936E9</v>
       </c>
       <c r="AF157" s="14" t="inlineStr"/>
       <c r="AG157" s="14" t="inlineStr"/>
@@ -9747,20 +9747,20 @@
         <v>1.09165E8</v>
       </c>
       <c r="X158" s="14" t="n">
-        <v>0.0</v>
+        <v>2.3555E7</v>
       </c>
       <c r="Y158" s="14" t="inlineStr"/>
       <c r="Z158" s="14" t="n">
-        <v>1.09165E8</v>
+        <v>1.3272E8</v>
       </c>
       <c r="AA158" s="14" t="inlineStr"/>
       <c r="AB158" s="14" t="inlineStr"/>
       <c r="AC158" s="15" t="n">
-        <v>0.4247004357298475</v>
+        <v>0.5163398692810458</v>
       </c>
       <c r="AD158" s="15" t="inlineStr"/>
       <c r="AE158" s="14" t="n">
-        <v>1.47875E8</v>
+        <v>1.2432E8</v>
       </c>
       <c r="AF158" s="14" t="inlineStr"/>
       <c r="AG158" s="14" t="inlineStr"/>
@@ -9804,20 +9804,20 @@
         <v>8.87112E8</v>
       </c>
       <c r="X159" s="14" t="n">
-        <v>0.0</v>
+        <v>1.84038E8</v>
       </c>
       <c r="Y159" s="14" t="inlineStr"/>
       <c r="Z159" s="14" t="n">
-        <v>8.87112E8</v>
+        <v>1.07115E9</v>
       </c>
       <c r="AA159" s="14" t="inlineStr"/>
       <c r="AB159" s="14" t="inlineStr"/>
       <c r="AC159" s="15" t="n">
-        <v>0.4911504424778761</v>
+        <v>0.5930432645034415</v>
       </c>
       <c r="AD159" s="15" t="inlineStr"/>
       <c r="AE159" s="14" t="n">
-        <v>9.1908E8</v>
+        <v>7.35042E8</v>
       </c>
       <c r="AF159" s="14" t="inlineStr"/>
       <c r="AG159" s="14" t="inlineStr"/>
@@ -9861,20 +9861,20 @@
         <v>2.5297E8</v>
       </c>
       <c r="X160" s="14" t="n">
-        <v>0.0</v>
+        <v>4.9528E7</v>
       </c>
       <c r="Y160" s="14" t="inlineStr"/>
       <c r="Z160" s="14" t="n">
-        <v>2.5297E8</v>
+        <v>3.02498E8</v>
       </c>
       <c r="AA160" s="14" t="inlineStr"/>
       <c r="AB160" s="14" t="inlineStr"/>
       <c r="AC160" s="15" t="n">
-        <v>0.46072281959378736</v>
+        <v>0.5509259259259259</v>
       </c>
       <c r="AD160" s="15" t="inlineStr"/>
       <c r="AE160" s="14" t="n">
-        <v>2.96102E8</v>
+        <v>2.46574E8</v>
       </c>
       <c r="AF160" s="14" t="inlineStr"/>
       <c r="AG160" s="14" t="inlineStr"/>
@@ -9924,20 +9924,20 @@
         <v>2220000.0</v>
       </c>
       <c r="X161" s="14" t="n">
-        <v>0.0</v>
+        <v>185000.0</v>
       </c>
       <c r="Y161" s="14" t="inlineStr"/>
       <c r="Z161" s="14" t="n">
-        <v>2220000.0</v>
+        <v>2405000.0</v>
       </c>
       <c r="AA161" s="14" t="inlineStr"/>
       <c r="AB161" s="14" t="inlineStr"/>
       <c r="AC161" s="15" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.4642857142857143</v>
       </c>
       <c r="AD161" s="15" t="inlineStr"/>
       <c r="AE161" s="14" t="n">
-        <v>2960000.0</v>
+        <v>2775000.0</v>
       </c>
       <c r="AF161" s="14" t="inlineStr"/>
       <c r="AG161" s="14" t="inlineStr"/>
@@ -9981,20 +9981,20 @@
         <v>1665000.0</v>
       </c>
       <c r="X162" s="14" t="n">
-        <v>0.0</v>
+        <v>185000.0</v>
       </c>
       <c r="Y162" s="14" t="inlineStr"/>
       <c r="Z162" s="14" t="n">
-        <v>1665000.0</v>
+        <v>1850000.0</v>
       </c>
       <c r="AA162" s="14" t="inlineStr"/>
       <c r="AB162" s="14" t="inlineStr"/>
       <c r="AC162" s="15" t="n">
-        <v>0.375</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="AD162" s="15" t="inlineStr"/>
       <c r="AE162" s="14" t="n">
-        <v>2775000.0</v>
+        <v>2590000.0</v>
       </c>
       <c r="AF162" s="14" t="inlineStr"/>
       <c r="AG162" s="14" t="inlineStr"/>
@@ -10392,20 +10392,20 @@
         <v>1.3597237554E10</v>
       </c>
       <c r="X169" s="14" t="n">
-        <v>0.0</v>
+        <v>8.58589154E8</v>
       </c>
       <c r="Y169" s="14" t="inlineStr"/>
       <c r="Z169" s="14" t="n">
-        <v>1.3597237554E10</v>
+        <v>1.4455826708E10</v>
       </c>
       <c r="AA169" s="14" t="inlineStr"/>
       <c r="AB169" s="14" t="inlineStr"/>
       <c r="AC169" s="15" t="n">
-        <v>0.9068459674637595</v>
+        <v>0.9641081950979286</v>
       </c>
       <c r="AD169" s="15" t="inlineStr"/>
       <c r="AE169" s="14" t="n">
-        <v>1.396750446E9</v>
+        <v>5.38161292E8</v>
       </c>
       <c r="AF169" s="14" t="inlineStr"/>
       <c r="AG169" s="14" t="inlineStr"/>
@@ -10455,20 +10455,20 @@
         <v>5.311759666E9</v>
       </c>
       <c r="X170" s="14" t="n">
-        <v>0.0</v>
+        <v>5.493708E8</v>
       </c>
       <c r="Y170" s="14" t="inlineStr"/>
       <c r="Z170" s="14" t="n">
-        <v>5.311759666E9</v>
+        <v>5.861130466E9</v>
       </c>
       <c r="AA170" s="14" t="inlineStr"/>
       <c r="AB170" s="14" t="inlineStr"/>
       <c r="AC170" s="15" t="n">
-        <v>1.1913573489125906</v>
+        <v>1.3145739439794482</v>
       </c>
       <c r="AD170" s="15" t="inlineStr"/>
       <c r="AE170" s="14" t="n">
-        <v>-8.53181666E8</v>
+        <v>-1.402552466E9</v>
       </c>
       <c r="AF170" s="14" t="inlineStr"/>
       <c r="AG170" s="14" t="inlineStr"/>
@@ -10512,20 +10512,20 @@
         <v>4.222646E9</v>
       </c>
       <c r="X171" s="14" t="n">
-        <v>0.0</v>
+        <v>5.493708E8</v>
       </c>
       <c r="Y171" s="14" t="inlineStr"/>
       <c r="Z171" s="14" t="n">
-        <v>4.222646E9</v>
+        <v>4.7720168E9</v>
       </c>
       <c r="AA171" s="14" t="inlineStr"/>
       <c r="AB171" s="14" t="inlineStr"/>
       <c r="AC171" s="15" t="n">
-        <v>1.2542045959477153</v>
+        <v>1.4173779669192512</v>
       </c>
       <c r="AD171" s="15" t="inlineStr"/>
       <c r="AE171" s="14" t="n">
-        <v>-8.55854E8</v>
+        <v>-1.4052248E9</v>
       </c>
       <c r="AF171" s="14" t="inlineStr"/>
       <c r="AG171" s="14" t="inlineStr"/>
@@ -10732,20 +10732,20 @@
         <v>101733.0</v>
       </c>
       <c r="X175" s="14" t="n">
-        <v>0.0</v>
+        <v>10038.0</v>
       </c>
       <c r="Y175" s="14" t="inlineStr"/>
       <c r="Z175" s="14" t="n">
-        <v>101733.0</v>
+        <v>111771.0</v>
       </c>
       <c r="AA175" s="14" t="inlineStr"/>
       <c r="AB175" s="14" t="inlineStr"/>
       <c r="AC175" s="15" t="n">
-        <v>0.643879746835443</v>
+        <v>0.7074113924050633</v>
       </c>
       <c r="AD175" s="15" t="inlineStr"/>
       <c r="AE175" s="14" t="n">
-        <v>56267.0</v>
+        <v>46229.0</v>
       </c>
       <c r="AF175" s="14" t="inlineStr"/>
       <c r="AG175" s="14" t="inlineStr"/>
@@ -10789,20 +10789,20 @@
         <v>88613.0</v>
       </c>
       <c r="X176" s="14" t="n">
-        <v>0.0</v>
+        <v>10038.0</v>
       </c>
       <c r="Y176" s="14" t="inlineStr"/>
       <c r="Z176" s="14" t="n">
-        <v>88613.0</v>
+        <v>98651.0</v>
       </c>
       <c r="AA176" s="14" t="inlineStr"/>
       <c r="AB176" s="14" t="inlineStr"/>
       <c r="AC176" s="15" t="n">
-        <v>0.6153680555555555</v>
+        <v>0.6850763888888889</v>
       </c>
       <c r="AD176" s="15" t="inlineStr"/>
       <c r="AE176" s="14" t="n">
-        <v>55387.0</v>
+        <v>45349.0</v>
       </c>
       <c r="AF176" s="14" t="inlineStr"/>
       <c r="AG176" s="14" t="inlineStr"/>
@@ -10966,20 +10966,20 @@
         <v>3.5985017E8</v>
       </c>
       <c r="X179" s="14" t="n">
-        <v>0.0</v>
+        <v>3.730664E7</v>
       </c>
       <c r="Y179" s="14" t="inlineStr"/>
       <c r="Z179" s="14" t="n">
-        <v>3.5985017E8</v>
+        <v>3.9715681E8</v>
       </c>
       <c r="AA179" s="14" t="inlineStr"/>
       <c r="AB179" s="14" t="inlineStr"/>
       <c r="AC179" s="15" t="n">
-        <v>0.9966326654960589</v>
+        <v>1.0999562683830657</v>
       </c>
       <c r="AD179" s="15" t="inlineStr"/>
       <c r="AE179" s="14" t="n">
-        <v>1215830.0</v>
+        <v>-3.609081E7</v>
       </c>
       <c r="AF179" s="14" t="inlineStr"/>
       <c r="AG179" s="14" t="inlineStr"/>
@@ -11023,20 +11023,20 @@
         <v>2.861254E8</v>
       </c>
       <c r="X180" s="14" t="n">
-        <v>0.0</v>
+        <v>3.730664E7</v>
       </c>
       <c r="Y180" s="14" t="inlineStr"/>
       <c r="Z180" s="14" t="n">
-        <v>2.861254E8</v>
+        <v>3.2343204E8</v>
       </c>
       <c r="AA180" s="14" t="inlineStr"/>
       <c r="AB180" s="14" t="inlineStr"/>
       <c r="AC180" s="15" t="n">
-        <v>0.9934909722222223</v>
+        <v>1.1230279166666666</v>
       </c>
       <c r="AD180" s="15" t="inlineStr"/>
       <c r="AE180" s="14" t="n">
-        <v>1874600.0</v>
+        <v>-3.543204E7</v>
       </c>
       <c r="AF180" s="14" t="inlineStr"/>
       <c r="AG180" s="14" t="inlineStr"/>
@@ -11200,20 +11200,20 @@
         <v>1.07733296E8</v>
       </c>
       <c r="X183" s="14" t="n">
-        <v>0.0</v>
+        <v>1.1042896E7</v>
       </c>
       <c r="Y183" s="14" t="inlineStr"/>
       <c r="Z183" s="14" t="n">
-        <v>1.07733296E8</v>
+        <v>1.18776192E8</v>
       </c>
       <c r="AA183" s="14" t="inlineStr"/>
       <c r="AB183" s="14" t="inlineStr"/>
       <c r="AC183" s="15" t="n">
-        <v>0.9613207695327837</v>
+        <v>1.0598582289324339</v>
       </c>
       <c r="AD183" s="15" t="inlineStr"/>
       <c r="AE183" s="14" t="n">
-        <v>4334704.0</v>
+        <v>-6708192.0</v>
       </c>
       <c r="AF183" s="14" t="inlineStr"/>
       <c r="AG183" s="14" t="inlineStr"/>
@@ -11257,20 +11257,20 @@
         <v>8.5850712E7</v>
       </c>
       <c r="X184" s="14" t="n">
-        <v>0.0</v>
+        <v>1.1042896E7</v>
       </c>
       <c r="Y184" s="14" t="inlineStr"/>
       <c r="Z184" s="14" t="n">
-        <v>8.5850712E7</v>
+        <v>9.6893608E7</v>
       </c>
       <c r="AA184" s="14" t="inlineStr"/>
       <c r="AB184" s="14" t="inlineStr"/>
       <c r="AC184" s="15" t="n">
-        <v>0.9538968</v>
+        <v>1.0765956444444444</v>
       </c>
       <c r="AD184" s="15" t="inlineStr"/>
       <c r="AE184" s="14" t="n">
-        <v>4149288.0</v>
+        <v>-6893608.0</v>
       </c>
       <c r="AF184" s="14" t="inlineStr"/>
       <c r="AG184" s="14" t="inlineStr"/>
@@ -11434,20 +11434,20 @@
         <v>8.6691E8</v>
       </c>
       <c r="X187" s="14" t="n">
-        <v>0.0</v>
+        <v>8.874E7</v>
       </c>
       <c r="Y187" s="14" t="inlineStr"/>
       <c r="Z187" s="14" t="n">
-        <v>8.6691E8</v>
+        <v>9.5565E8</v>
       </c>
       <c r="AA187" s="14" t="inlineStr"/>
       <c r="AB187" s="14" t="inlineStr"/>
       <c r="AC187" s="15" t="n">
-        <v>0.9652281381521812</v>
+        <v>1.064032333489211</v>
       </c>
       <c r="AD187" s="15" t="inlineStr"/>
       <c r="AE187" s="14" t="n">
-        <v>3.123E7</v>
+        <v>-5.751E7</v>
       </c>
       <c r="AF187" s="14" t="inlineStr"/>
       <c r="AG187" s="14" t="inlineStr"/>
@@ -11491,20 +11491,20 @@
         <v>6.891E8</v>
       </c>
       <c r="X188" s="14" t="n">
-        <v>0.0</v>
+        <v>8.874E7</v>
       </c>
       <c r="Y188" s="14" t="inlineStr"/>
       <c r="Z188" s="14" t="n">
-        <v>6.891E8</v>
+        <v>7.7784E8</v>
       </c>
       <c r="AA188" s="14" t="inlineStr"/>
       <c r="AB188" s="14" t="inlineStr"/>
       <c r="AC188" s="15" t="n">
-        <v>0.9570833333333333</v>
+        <v>1.0803333333333334</v>
       </c>
       <c r="AD188" s="15" t="inlineStr"/>
       <c r="AE188" s="14" t="n">
-        <v>3.09E7</v>
+        <v>-5.784E7</v>
       </c>
       <c r="AF188" s="14" t="inlineStr"/>
       <c r="AG188" s="14" t="inlineStr"/>
@@ -11668,20 +11668,20 @@
         <v>3.2558825E8</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>0.0</v>
+        <v>3.324078E7</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
-        <v>3.2558825E8</v>
+        <v>3.5882903E8</v>
       </c>
       <c r="AA191" s="14" t="inlineStr"/>
       <c r="AB191" s="14" t="inlineStr"/>
       <c r="AC191" s="15" t="n">
-        <v>0.9843997544958699</v>
+        <v>1.0849015867064955</v>
       </c>
       <c r="AD191" s="15" t="inlineStr"/>
       <c r="AE191" s="14" t="n">
-        <v>5159750.0</v>
+        <v>-2.808103E7</v>
       </c>
       <c r="AF191" s="14" t="inlineStr"/>
       <c r="AG191" s="14" t="inlineStr"/>
@@ -11725,20 +11725,20 @@
         <v>2.5904634E8</v>
       </c>
       <c r="X192" s="14" t="n">
-        <v>0.0</v>
+        <v>3.324078E7</v>
       </c>
       <c r="Y192" s="14" t="inlineStr"/>
       <c r="Z192" s="14" t="n">
-        <v>2.5904634E8</v>
+        <v>2.9228712E8</v>
       </c>
       <c r="AA192" s="14" t="inlineStr"/>
       <c r="AB192" s="14" t="inlineStr"/>
       <c r="AC192" s="15" t="n">
-        <v>0.9812361363636364</v>
+        <v>1.1071481818181819</v>
       </c>
       <c r="AD192" s="15" t="inlineStr"/>
       <c r="AE192" s="14" t="n">
-        <v>4953660.0</v>
+        <v>-2.828712E7</v>
       </c>
       <c r="AF192" s="14" t="inlineStr"/>
       <c r="AG192" s="14" t="inlineStr"/>
@@ -11902,20 +11902,20 @@
         <v>6.44264E8</v>
       </c>
       <c r="X195" s="14" t="n">
-        <v>0.0</v>
+        <v>1.38878E8</v>
       </c>
       <c r="Y195" s="14" t="inlineStr"/>
       <c r="Z195" s="14" t="n">
-        <v>6.44264E8</v>
+        <v>7.83142E8</v>
       </c>
       <c r="AA195" s="14" t="inlineStr"/>
       <c r="AB195" s="14" t="inlineStr"/>
       <c r="AC195" s="15" t="n">
-        <v>0.6347678726255221</v>
+        <v>0.7715988807440687</v>
       </c>
       <c r="AD195" s="15" t="inlineStr"/>
       <c r="AE195" s="14" t="n">
-        <v>3.70696E8</v>
+        <v>2.31818E8</v>
       </c>
       <c r="AF195" s="14" t="inlineStr"/>
       <c r="AG195" s="14" t="inlineStr"/>
@@ -11959,20 +11959,20 @@
         <v>6.181E7</v>
       </c>
       <c r="X196" s="14" t="n">
-        <v>0.0</v>
+        <v>1.33E7</v>
       </c>
       <c r="Y196" s="14" t="inlineStr"/>
       <c r="Z196" s="14" t="n">
-        <v>6.181E7</v>
+        <v>7.511E7</v>
       </c>
       <c r="AA196" s="14" t="inlineStr"/>
       <c r="AB196" s="14" t="inlineStr"/>
       <c r="AC196" s="15" t="n">
-        <v>0.566025641025641</v>
+        <v>0.6878205128205128</v>
       </c>
       <c r="AD196" s="15" t="inlineStr"/>
       <c r="AE196" s="14" t="n">
-        <v>4.739E7</v>
+        <v>3.409E7</v>
       </c>
       <c r="AF196" s="14" t="inlineStr"/>
       <c r="AG196" s="14" t="inlineStr"/>
@@ -12016,20 +12016,20 @@
         <v>5.82454E8</v>
       </c>
       <c r="X197" s="14" t="n">
-        <v>0.0</v>
+        <v>1.25578E8</v>
       </c>
       <c r="Y197" s="14" t="inlineStr"/>
       <c r="Z197" s="14" t="n">
-        <v>5.82454E8</v>
+        <v>7.08032E8</v>
       </c>
       <c r="AA197" s="14" t="inlineStr"/>
       <c r="AB197" s="14" t="inlineStr"/>
       <c r="AC197" s="15" t="n">
-        <v>0.6430555555555556</v>
+        <v>0.7816993464052288</v>
       </c>
       <c r="AD197" s="15" t="inlineStr"/>
       <c r="AE197" s="14" t="n">
-        <v>3.23306E8</v>
+        <v>1.97728E8</v>
       </c>
       <c r="AF197" s="14" t="inlineStr"/>
       <c r="AG197" s="14" t="inlineStr"/>
@@ -12356,20 +12356,20 @@
         <v>4.15571698E9</v>
       </c>
       <c r="X203" s="25" t="n">
-        <v>647800.0</v>
+        <v>1.69768922E8</v>
       </c>
       <c r="Y203" s="25" t="inlineStr"/>
       <c r="Z203" s="25" t="n">
-        <v>4.15636478E9</v>
+        <v>4.325485902E9</v>
       </c>
       <c r="AA203" s="25" t="inlineStr"/>
       <c r="AB203" s="25" t="inlineStr"/>
       <c r="AC203" s="26" t="n">
-        <v>0.7348894164524753</v>
+        <v>0.7647918261866777</v>
       </c>
       <c r="AD203" s="26" t="inlineStr"/>
       <c r="AE203" s="25" t="n">
-        <v>1.49940422E9</v>
+        <v>1.330283098E9</v>
       </c>
       <c r="AF203" s="25" t="inlineStr"/>
       <c r="AG203" s="25" t="inlineStr"/>
@@ -12419,20 +12419,20 @@
         <v>3.258757999E9</v>
       </c>
       <c r="X204" s="14" t="n">
-        <v>0.0</v>
+        <v>7.5668436E7</v>
       </c>
       <c r="Y204" s="14" t="inlineStr"/>
       <c r="Z204" s="14" t="n">
-        <v>3.258757999E9</v>
+        <v>3.334426435E9</v>
       </c>
       <c r="AA204" s="14" t="inlineStr"/>
       <c r="AB204" s="14" t="inlineStr"/>
       <c r="AC204" s="15" t="n">
-        <v>0.8388798587982353</v>
+        <v>0.8583586684940281</v>
       </c>
       <c r="AD204" s="15" t="inlineStr"/>
       <c r="AE204" s="14" t="n">
-        <v>6.25896001E8</v>
+        <v>5.50227565E8</v>
       </c>
       <c r="AF204" s="14" t="inlineStr"/>
       <c r="AG204" s="14" t="inlineStr"/>
@@ -12482,20 +12482,20 @@
         <v>5.46628803E8</v>
       </c>
       <c r="X205" s="14" t="n">
-        <v>0.0</v>
+        <v>2017000.0</v>
       </c>
       <c r="Y205" s="14" t="inlineStr"/>
       <c r="Z205" s="14" t="n">
-        <v>5.46628803E8</v>
+        <v>5.48645803E8</v>
       </c>
       <c r="AA205" s="14" t="inlineStr"/>
       <c r="AB205" s="14" t="inlineStr"/>
       <c r="AC205" s="15" t="n">
-        <v>0.7439991221109624</v>
+        <v>0.7467443968221777</v>
       </c>
       <c r="AD205" s="15" t="inlineStr"/>
       <c r="AE205" s="14" t="n">
-        <v>1.88088197E8</v>
+        <v>1.86071197E8</v>
       </c>
       <c r="AF205" s="14" t="inlineStr"/>
       <c r="AG205" s="14" t="inlineStr"/>
@@ -12653,20 +12653,20 @@
         <v>3.2709603E7</v>
       </c>
       <c r="X208" s="14" t="n">
-        <v>0.0</v>
+        <v>2017000.0</v>
       </c>
       <c r="Y208" s="14" t="inlineStr"/>
       <c r="Z208" s="14" t="n">
-        <v>3.2709603E7</v>
+        <v>3.4726603E7</v>
       </c>
       <c r="AA208" s="14" t="inlineStr"/>
       <c r="AB208" s="14" t="inlineStr"/>
       <c r="AC208" s="15" t="n">
-        <v>0.6339070348837209</v>
+        <v>0.6729961821705427</v>
       </c>
       <c r="AD208" s="15" t="inlineStr"/>
       <c r="AE208" s="14" t="n">
-        <v>1.8890397E7</v>
+        <v>1.6873397E7</v>
       </c>
       <c r="AF208" s="14" t="inlineStr"/>
       <c r="AG208" s="14" t="inlineStr"/>
@@ -12716,20 +12716,20 @@
         <v>5144000.0</v>
       </c>
       <c r="X209" s="14" t="n">
-        <v>0.0</v>
+        <v>222500.0</v>
       </c>
       <c r="Y209" s="14" t="inlineStr"/>
       <c r="Z209" s="14" t="n">
-        <v>5144000.0</v>
+        <v>5366500.0</v>
       </c>
       <c r="AA209" s="14" t="inlineStr"/>
       <c r="AB209" s="14" t="inlineStr"/>
       <c r="AC209" s="15" t="n">
-        <v>0.3956923076923077</v>
+        <v>0.4128076923076923</v>
       </c>
       <c r="AD209" s="15" t="inlineStr"/>
       <c r="AE209" s="14" t="n">
-        <v>7856000.0</v>
+        <v>7633500.0</v>
       </c>
       <c r="AF209" s="14" t="inlineStr"/>
       <c r="AG209" s="14" t="inlineStr"/>
@@ -12773,20 +12773,20 @@
         <v>2720000.0</v>
       </c>
       <c r="X210" s="14" t="n">
-        <v>0.0</v>
+        <v>222500.0</v>
       </c>
       <c r="Y210" s="14" t="inlineStr"/>
       <c r="Z210" s="14" t="n">
-        <v>2720000.0</v>
+        <v>2942500.0</v>
       </c>
       <c r="AA210" s="14" t="inlineStr"/>
       <c r="AB210" s="14" t="inlineStr"/>
       <c r="AC210" s="15" t="n">
-        <v>0.4689655172413793</v>
+        <v>0.5073275862068966</v>
       </c>
       <c r="AD210" s="15" t="inlineStr"/>
       <c r="AE210" s="14" t="n">
-        <v>3080000.0</v>
+        <v>2857500.0</v>
       </c>
       <c r="AF210" s="14" t="inlineStr"/>
       <c r="AG210" s="14" t="inlineStr"/>
@@ -12893,20 +12893,20 @@
         <v>1.280558E7</v>
       </c>
       <c r="X212" s="14" t="n">
-        <v>0.0</v>
+        <v>4279000.0</v>
       </c>
       <c r="Y212" s="14" t="inlineStr"/>
       <c r="Z212" s="14" t="n">
-        <v>1.280558E7</v>
+        <v>1.708458E7</v>
       </c>
       <c r="AA212" s="14" t="inlineStr"/>
       <c r="AB212" s="14" t="inlineStr"/>
       <c r="AC212" s="15" t="n">
-        <v>0.73178924509972</v>
+        <v>0.9763175038573633</v>
       </c>
       <c r="AD212" s="15" t="inlineStr"/>
       <c r="AE212" s="14" t="n">
-        <v>4693420.0</v>
+        <v>414420.0</v>
       </c>
       <c r="AF212" s="14" t="inlineStr"/>
       <c r="AG212" s="14" t="inlineStr"/>
@@ -12950,20 +12950,20 @@
         <v>1.280558E7</v>
       </c>
       <c r="X213" s="14" t="n">
-        <v>0.0</v>
+        <v>4279000.0</v>
       </c>
       <c r="Y213" s="14" t="inlineStr"/>
       <c r="Z213" s="14" t="n">
-        <v>1.280558E7</v>
+        <v>1.708458E7</v>
       </c>
       <c r="AA213" s="14" t="inlineStr"/>
       <c r="AB213" s="14" t="inlineStr"/>
       <c r="AC213" s="15" t="n">
-        <v>0.73178924509972</v>
+        <v>0.9763175038573633</v>
       </c>
       <c r="AD213" s="15" t="inlineStr"/>
       <c r="AE213" s="14" t="n">
-        <v>4693420.0</v>
+        <v>414420.0</v>
       </c>
       <c r="AF213" s="14" t="inlineStr"/>
       <c r="AG213" s="14" t="inlineStr"/>
@@ -13133,20 +13133,20 @@
         <v>2.692189616E9</v>
       </c>
       <c r="X216" s="14" t="n">
-        <v>0.0</v>
+        <v>6.9149936E7</v>
       </c>
       <c r="Y216" s="14" t="inlineStr"/>
       <c r="Z216" s="14" t="n">
-        <v>2.692189616E9</v>
+        <v>2.761339552E9</v>
       </c>
       <c r="AA216" s="14" t="inlineStr"/>
       <c r="AB216" s="14" t="inlineStr"/>
       <c r="AC216" s="15" t="n">
-        <v>0.8638675359496965</v>
+        <v>0.8860563091580836</v>
       </c>
       <c r="AD216" s="15" t="inlineStr"/>
       <c r="AE216" s="14" t="n">
-        <v>4.24248384E8</v>
+        <v>3.55098448E8</v>
       </c>
       <c r="AF216" s="14" t="inlineStr"/>
       <c r="AG216" s="14" t="inlineStr"/>
@@ -13190,20 +13190,20 @@
         <v>2.85881376E8</v>
       </c>
       <c r="X217" s="14" t="n">
-        <v>0.0</v>
+        <v>4.1321696E7</v>
       </c>
       <c r="Y217" s="14" t="inlineStr"/>
       <c r="Z217" s="14" t="n">
-        <v>2.85881376E8</v>
+        <v>3.27203072E8</v>
       </c>
       <c r="AA217" s="14" t="inlineStr"/>
       <c r="AB217" s="14" t="inlineStr"/>
       <c r="AC217" s="15" t="n">
-        <v>0.5294099555555556</v>
+        <v>0.6059316148148148</v>
       </c>
       <c r="AD217" s="15" t="inlineStr"/>
       <c r="AE217" s="14" t="n">
-        <v>2.54118624E8</v>
+        <v>2.12796928E8</v>
       </c>
       <c r="AF217" s="14" t="inlineStr"/>
       <c r="AG217" s="14" t="inlineStr"/>
@@ -13247,20 +13247,20 @@
         <v>6.5444768E7</v>
       </c>
       <c r="X218" s="14" t="n">
-        <v>0.0</v>
+        <v>9468528.0</v>
       </c>
       <c r="Y218" s="14" t="inlineStr"/>
       <c r="Z218" s="14" t="n">
-        <v>6.5444768E7</v>
+        <v>7.4913296E7</v>
       </c>
       <c r="AA218" s="14" t="inlineStr"/>
       <c r="AB218" s="14" t="inlineStr"/>
       <c r="AC218" s="15" t="n">
-        <v>0.5338072430668842</v>
+        <v>0.6110383034257749</v>
       </c>
       <c r="AD218" s="15" t="inlineStr"/>
       <c r="AE218" s="14" t="n">
-        <v>5.7155232E7</v>
+        <v>4.7686704E7</v>
       </c>
       <c r="AF218" s="14" t="inlineStr"/>
       <c r="AG218" s="14" t="inlineStr"/>
@@ -13304,20 +13304,20 @@
         <v>9.5029104E7</v>
       </c>
       <c r="X219" s="14" t="n">
-        <v>0.0</v>
+        <v>1.3729784E7</v>
       </c>
       <c r="Y219" s="14" t="inlineStr"/>
       <c r="Z219" s="14" t="n">
-        <v>9.5029104E7</v>
+        <v>1.08758888E8</v>
       </c>
       <c r="AA219" s="14" t="inlineStr"/>
       <c r="AB219" s="14" t="inlineStr"/>
       <c r="AC219" s="15" t="n">
-        <v>0.5279394666666667</v>
+        <v>0.6042160444444444</v>
       </c>
       <c r="AD219" s="15" t="inlineStr"/>
       <c r="AE219" s="14" t="n">
-        <v>8.4970896E7</v>
+        <v>7.1241112E7</v>
       </c>
       <c r="AF219" s="14" t="inlineStr"/>
       <c r="AG219" s="14" t="inlineStr"/>
@@ -13361,20 +13361,20 @@
         <v>3.1996368E7</v>
       </c>
       <c r="X220" s="14" t="n">
-        <v>0.0</v>
+        <v>4629928.0</v>
       </c>
       <c r="Y220" s="14" t="inlineStr"/>
       <c r="Z220" s="14" t="n">
-        <v>3.1996368E7</v>
+        <v>3.6626296E7</v>
       </c>
       <c r="AA220" s="14" t="inlineStr"/>
       <c r="AB220" s="14" t="inlineStr"/>
       <c r="AC220" s="15" t="n">
-        <v>0.5332728</v>
+        <v>0.6104382666666667</v>
       </c>
       <c r="AD220" s="15" t="inlineStr"/>
       <c r="AE220" s="14" t="n">
-        <v>2.8003632E7</v>
+        <v>2.3373704E7</v>
       </c>
       <c r="AF220" s="14" t="inlineStr"/>
       <c r="AG220" s="14" t="inlineStr"/>
@@ -13481,20 +13481,20 @@
         <v>4.32620013E8</v>
       </c>
       <c r="X222" s="14" t="n">
-        <v>647800.0</v>
+        <v>5.1920911E7</v>
       </c>
       <c r="Y222" s="14" t="inlineStr"/>
       <c r="Z222" s="14" t="n">
-        <v>4.33267813E8</v>
+        <v>4.84540924E8</v>
       </c>
       <c r="AA222" s="14" t="inlineStr"/>
       <c r="AB222" s="14" t="inlineStr"/>
       <c r="AC222" s="15" t="n">
-        <v>0.4654789568113451</v>
+        <v>0.5205639492909325</v>
       </c>
       <c r="AD222" s="15" t="inlineStr"/>
       <c r="AE222" s="14" t="n">
-        <v>4.97532187E8</v>
+        <v>4.46259076E8</v>
       </c>
       <c r="AF222" s="14" t="inlineStr"/>
       <c r="AG222" s="14" t="inlineStr"/>
@@ -13544,20 +13544,20 @@
         <v>3.10883859E8</v>
       </c>
       <c r="X223" s="14" t="n">
-        <v>0.0</v>
+        <v>4.1758847E7</v>
       </c>
       <c r="Y223" s="14" t="inlineStr"/>
       <c r="Z223" s="14" t="n">
-        <v>3.10883859E8</v>
+        <v>3.52642706E8</v>
       </c>
       <c r="AA223" s="14" t="inlineStr"/>
       <c r="AB223" s="14" t="inlineStr"/>
       <c r="AC223" s="15" t="n">
-        <v>0.42470472540983606</v>
+        <v>0.4817523306010929</v>
       </c>
       <c r="AD223" s="15" t="inlineStr"/>
       <c r="AE223" s="14" t="n">
-        <v>4.21116141E8</v>
+        <v>3.79357294E8</v>
       </c>
       <c r="AF223" s="14" t="inlineStr"/>
       <c r="AG223" s="14" t="inlineStr"/>
@@ -13601,20 +13601,20 @@
         <v>3.10883859E8</v>
       </c>
       <c r="X224" s="14" t="n">
-        <v>0.0</v>
+        <v>4.1758847E7</v>
       </c>
       <c r="Y224" s="14" t="inlineStr"/>
       <c r="Z224" s="14" t="n">
-        <v>3.10883859E8</v>
+        <v>3.52642706E8</v>
       </c>
       <c r="AA224" s="14" t="inlineStr"/>
       <c r="AB224" s="14" t="inlineStr"/>
       <c r="AC224" s="15" t="n">
-        <v>0.42470472540983606</v>
+        <v>0.4817523306010929</v>
       </c>
       <c r="AD224" s="15" t="inlineStr"/>
       <c r="AE224" s="14" t="n">
-        <v>4.21116141E8</v>
+        <v>3.79357294E8</v>
       </c>
       <c r="AF224" s="14" t="inlineStr"/>
       <c r="AG224" s="14" t="inlineStr"/>
@@ -13664,20 +13664,20 @@
         <v>4425348.0</v>
       </c>
       <c r="X225" s="14" t="n">
-        <v>0.0</v>
+        <v>263514.0</v>
       </c>
       <c r="Y225" s="14" t="inlineStr"/>
       <c r="Z225" s="14" t="n">
-        <v>4425348.0</v>
+        <v>4688862.0</v>
       </c>
       <c r="AA225" s="14" t="inlineStr"/>
       <c r="AB225" s="14" t="inlineStr"/>
       <c r="AC225" s="15" t="n">
-        <v>0.9219475</v>
+        <v>0.97684625</v>
       </c>
       <c r="AD225" s="15" t="inlineStr"/>
       <c r="AE225" s="14" t="n">
-        <v>374652.0</v>
+        <v>111138.0</v>
       </c>
       <c r="AF225" s="14" t="inlineStr"/>
       <c r="AG225" s="14" t="inlineStr"/>
@@ -13721,20 +13721,20 @@
         <v>4425348.0</v>
       </c>
       <c r="X226" s="14" t="n">
-        <v>0.0</v>
+        <v>263514.0</v>
       </c>
       <c r="Y226" s="14" t="inlineStr"/>
       <c r="Z226" s="14" t="n">
-        <v>4425348.0</v>
+        <v>4688862.0</v>
       </c>
       <c r="AA226" s="14" t="inlineStr"/>
       <c r="AB226" s="14" t="inlineStr"/>
       <c r="AC226" s="15" t="n">
-        <v>0.9219475</v>
+        <v>0.97684625</v>
       </c>
       <c r="AD226" s="15" t="inlineStr"/>
       <c r="AE226" s="14" t="n">
-        <v>374652.0</v>
+        <v>111138.0</v>
       </c>
       <c r="AF226" s="14" t="inlineStr"/>
       <c r="AG226" s="14" t="inlineStr"/>
@@ -13947,20 +13947,20 @@
         <v>9.2465706E7</v>
       </c>
       <c r="X230" s="14" t="n">
-        <v>0.0</v>
+        <v>9250750.0</v>
       </c>
       <c r="Y230" s="14" t="inlineStr"/>
       <c r="Z230" s="14" t="n">
-        <v>9.2465706E7</v>
+        <v>1.01716456E8</v>
       </c>
       <c r="AA230" s="14" t="inlineStr"/>
       <c r="AB230" s="14" t="inlineStr"/>
       <c r="AC230" s="15" t="n">
-        <v>0.5988711528497409</v>
+        <v>0.6587853367875648</v>
       </c>
       <c r="AD230" s="15" t="inlineStr"/>
       <c r="AE230" s="14" t="n">
-        <v>6.1934294E7</v>
+        <v>5.2683544E7</v>
       </c>
       <c r="AF230" s="14" t="inlineStr"/>
       <c r="AG230" s="14" t="inlineStr"/>
@@ -14004,20 +14004,20 @@
         <v>6.58569E7</v>
       </c>
       <c r="X231" s="14" t="n">
-        <v>0.0</v>
+        <v>9250750.0</v>
       </c>
       <c r="Y231" s="14" t="inlineStr"/>
       <c r="Z231" s="14" t="n">
-        <v>6.58569E7</v>
+        <v>7.510765E7</v>
       </c>
       <c r="AA231" s="14" t="inlineStr"/>
       <c r="AB231" s="14" t="inlineStr"/>
       <c r="AC231" s="15" t="n">
-        <v>0.5189669030732861</v>
+        <v>0.5918648542159181</v>
       </c>
       <c r="AD231" s="15" t="inlineStr"/>
       <c r="AE231" s="14" t="n">
-        <v>6.10431E7</v>
+        <v>5.179235E7</v>
       </c>
       <c r="AF231" s="14" t="inlineStr"/>
       <c r="AG231" s="14" t="inlineStr"/>
@@ -14124,20 +14124,20 @@
         <v>3.84588968E8</v>
       </c>
       <c r="X233" s="14" t="n">
-        <v>0.0</v>
+        <v>4.2179575E7</v>
       </c>
       <c r="Y233" s="14" t="inlineStr"/>
       <c r="Z233" s="14" t="n">
-        <v>3.84588968E8</v>
+        <v>4.26768543E8</v>
       </c>
       <c r="AA233" s="14" t="inlineStr"/>
       <c r="AB233" s="14" t="inlineStr"/>
       <c r="AC233" s="15" t="n">
-        <v>0.543101199630014</v>
+        <v>0.6026655129318562</v>
       </c>
       <c r="AD233" s="15" t="inlineStr"/>
       <c r="AE233" s="14" t="n">
-        <v>3.23546032E8</v>
+        <v>2.81366457E8</v>
       </c>
       <c r="AF233" s="14" t="inlineStr"/>
       <c r="AG233" s="14" t="inlineStr"/>
@@ -14187,20 +14187,20 @@
         <v>9.9195E7</v>
       </c>
       <c r="X234" s="14" t="n">
-        <v>0.0</v>
+        <v>3.474E7</v>
       </c>
       <c r="Y234" s="14" t="inlineStr"/>
       <c r="Z234" s="14" t="n">
-        <v>9.9195E7</v>
+        <v>1.33935E8</v>
       </c>
       <c r="AA234" s="14" t="inlineStr"/>
       <c r="AB234" s="14" t="inlineStr"/>
       <c r="AC234" s="15" t="n">
-        <v>0.495975</v>
+        <v>0.669675</v>
       </c>
       <c r="AD234" s="15" t="inlineStr"/>
       <c r="AE234" s="14" t="n">
-        <v>1.00805E8</v>
+        <v>6.6065E7</v>
       </c>
       <c r="AF234" s="14" t="inlineStr"/>
       <c r="AG234" s="14" t="inlineStr"/>
@@ -14244,20 +14244,20 @@
         <v>8.8315E7</v>
       </c>
       <c r="X235" s="14" t="n">
-        <v>0.0</v>
+        <v>2.5625E7</v>
       </c>
       <c r="Y235" s="14" t="inlineStr"/>
       <c r="Z235" s="14" t="n">
-        <v>8.8315E7</v>
+        <v>1.1394E8</v>
       </c>
       <c r="AA235" s="14" t="inlineStr"/>
       <c r="AB235" s="14" t="inlineStr"/>
       <c r="AC235" s="15" t="n">
-        <v>0.4906388888888889</v>
+        <v>0.633</v>
       </c>
       <c r="AD235" s="15" t="inlineStr"/>
       <c r="AE235" s="14" t="n">
-        <v>9.1685E7</v>
+        <v>6.606E7</v>
       </c>
       <c r="AF235" s="14" t="inlineStr"/>
       <c r="AG235" s="14" t="inlineStr"/>
@@ -14301,20 +14301,20 @@
         <v>1.088E7</v>
       </c>
       <c r="X236" s="14" t="n">
-        <v>0.0</v>
+        <v>9115000.0</v>
       </c>
       <c r="Y236" s="14" t="inlineStr"/>
       <c r="Z236" s="14" t="n">
-        <v>1.088E7</v>
+        <v>1.9995E7</v>
       </c>
       <c r="AA236" s="14" t="inlineStr"/>
       <c r="AB236" s="14" t="inlineStr"/>
       <c r="AC236" s="15" t="n">
-        <v>0.544</v>
+        <v>0.99975</v>
       </c>
       <c r="AD236" s="15" t="inlineStr"/>
       <c r="AE236" s="14" t="n">
-        <v>9120000.0</v>
+        <v>5000.0</v>
       </c>
       <c r="AF236" s="14" t="inlineStr"/>
       <c r="AG236" s="14" t="inlineStr"/>
@@ -14484,20 +14484,20 @@
         <v>1.10331326E8</v>
       </c>
       <c r="X239" s="14" t="n">
-        <v>0.0</v>
+        <v>750000.0</v>
       </c>
       <c r="Y239" s="14" t="inlineStr"/>
       <c r="Z239" s="14" t="n">
-        <v>1.10331326E8</v>
+        <v>1.11081326E8</v>
       </c>
       <c r="AA239" s="14" t="inlineStr"/>
       <c r="AB239" s="14" t="inlineStr"/>
       <c r="AC239" s="15" t="n">
-        <v>0.5574682363640957</v>
+        <v>0.5612577419599323</v>
       </c>
       <c r="AD239" s="15" t="inlineStr"/>
       <c r="AE239" s="14" t="n">
-        <v>8.7583674E7</v>
+        <v>8.6833674E7</v>
       </c>
       <c r="AF239" s="14" t="inlineStr"/>
       <c r="AG239" s="14" t="inlineStr"/>
@@ -14598,20 +14598,20 @@
         <v>1.1156299E7</v>
       </c>
       <c r="X241" s="14" t="n">
-        <v>0.0</v>
+        <v>750000.0</v>
       </c>
       <c r="Y241" s="14" t="inlineStr"/>
       <c r="Z241" s="14" t="n">
-        <v>1.1156299E7</v>
+        <v>1.1906299E7</v>
       </c>
       <c r="AA241" s="14" t="inlineStr"/>
       <c r="AB241" s="14" t="inlineStr"/>
       <c r="AC241" s="15" t="n">
-        <v>0.7083364444444444</v>
+        <v>0.7559554920634921</v>
       </c>
       <c r="AD241" s="15" t="inlineStr"/>
       <c r="AE241" s="14" t="n">
-        <v>4593701.0</v>
+        <v>3843701.0</v>
       </c>
       <c r="AF241" s="14" t="inlineStr"/>
       <c r="AG241" s="14" t="inlineStr"/>
@@ -15288,20 +15288,20 @@
         <v>8.8386927E7</v>
       </c>
       <c r="X253" s="14" t="n">
-        <v>0.0</v>
+        <v>6689575.0</v>
       </c>
       <c r="Y253" s="14" t="inlineStr"/>
       <c r="Z253" s="14" t="n">
-        <v>8.8386927E7</v>
+        <v>9.5076502E7</v>
       </c>
       <c r="AA253" s="14" t="inlineStr"/>
       <c r="AB253" s="14" t="inlineStr"/>
       <c r="AC253" s="15" t="n">
-        <v>0.43356679584028257</v>
+        <v>0.4663813499460414</v>
       </c>
       <c r="AD253" s="15" t="inlineStr"/>
       <c r="AE253" s="14" t="n">
-        <v>1.15473073E8</v>
+        <v>1.08783498E8</v>
       </c>
       <c r="AF253" s="14" t="inlineStr"/>
       <c r="AG253" s="14" t="inlineStr"/>
@@ -15345,20 +15345,20 @@
         <v>4080000.0</v>
       </c>
       <c r="X254" s="14" t="n">
-        <v>0.0</v>
+        <v>4845000.0</v>
       </c>
       <c r="Y254" s="14" t="inlineStr"/>
       <c r="Z254" s="14" t="n">
-        <v>4080000.0</v>
+        <v>8925000.0</v>
       </c>
       <c r="AA254" s="14" t="inlineStr"/>
       <c r="AB254" s="14" t="inlineStr"/>
       <c r="AC254" s="15" t="n">
-        <v>0.3813084112149533</v>
+        <v>0.8341121495327103</v>
       </c>
       <c r="AD254" s="15" t="inlineStr"/>
       <c r="AE254" s="14" t="n">
-        <v>6620000.0</v>
+        <v>1775000.0</v>
       </c>
       <c r="AF254" s="14" t="inlineStr"/>
       <c r="AG254" s="14" t="inlineStr"/>
@@ -15559,20 +15559,20 @@
         <v>6.6116077E7</v>
       </c>
       <c r="X258" s="14" t="n">
-        <v>0.0</v>
+        <v>1225000.0</v>
       </c>
       <c r="Y258" s="14" t="inlineStr"/>
       <c r="Z258" s="14" t="n">
-        <v>6.6116077E7</v>
+        <v>6.7341077E7</v>
       </c>
       <c r="AA258" s="14" t="inlineStr"/>
       <c r="AB258" s="14" t="inlineStr"/>
       <c r="AC258" s="15" t="n">
-        <v>0.530626621187801</v>
+        <v>0.5404580818619583</v>
       </c>
       <c r="AD258" s="15" t="inlineStr"/>
       <c r="AE258" s="14" t="n">
-        <v>5.8483923E7</v>
+        <v>5.7258923E7</v>
       </c>
       <c r="AF258" s="14" t="inlineStr"/>
       <c r="AG258" s="14" t="inlineStr"/>
@@ -15616,20 +15616,20 @@
         <v>2177000.0</v>
       </c>
       <c r="X259" s="14" t="n">
-        <v>0.0</v>
+        <v>233875.0</v>
       </c>
       <c r="Y259" s="14" t="inlineStr"/>
       <c r="Z259" s="14" t="n">
-        <v>2177000.0</v>
+        <v>2410875.0</v>
       </c>
       <c r="AA259" s="14" t="inlineStr"/>
       <c r="AB259" s="14" t="inlineStr"/>
       <c r="AC259" s="15" t="n">
-        <v>0.7256666666666667</v>
+        <v>0.803625</v>
       </c>
       <c r="AD259" s="15" t="inlineStr"/>
       <c r="AE259" s="14" t="n">
-        <v>823000.0</v>
+        <v>589125.0</v>
       </c>
       <c r="AF259" s="14" t="inlineStr"/>
       <c r="AG259" s="14" t="inlineStr"/>
@@ -15844,20 +15844,20 @@
         <v>3707013.0</v>
       </c>
       <c r="X263" s="14" t="n">
-        <v>0.0</v>
+        <v>385700.0</v>
       </c>
       <c r="Y263" s="14" t="inlineStr"/>
       <c r="Z263" s="14" t="n">
-        <v>3707013.0</v>
+        <v>4092713.0</v>
       </c>
       <c r="AA263" s="14" t="inlineStr"/>
       <c r="AB263" s="14" t="inlineStr"/>
       <c r="AC263" s="15" t="n">
-        <v>0.3707013</v>
+        <v>0.4092713</v>
       </c>
       <c r="AD263" s="15" t="inlineStr"/>
       <c r="AE263" s="14" t="n">
-        <v>6292987.0</v>
+        <v>5907287.0</v>
       </c>
       <c r="AF263" s="14" t="inlineStr"/>
       <c r="AG263" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
up date realisasi 4 nov pkl 11.12
up date realisasi 4 nov pkl 11.12
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E641CD86-4225-48BE-AEB5-582BCEAA2324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB7EA93A-EAC6-4995-96BE-75B0C8D3B4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
update realisasi per 5 nov pkl 15.00
update realisasi per 5 nov pkl 15.00
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB7EA93A-EAC6-4995-96BE-75B0C8D3B4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D0373B4-E131-4C64-B601-FC1934E016AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2155,19 +2155,19 @@
         <v>80919905375</v>
       </c>
       <c r="X9" s="4">
-        <v>0</v>
+        <v>1938614197</v>
       </c>
       <c r="Y9" s="18">
-        <v>80919905375</v>
+        <v>82858519572</v>
       </c>
       <c r="Z9" s="18"/>
       <c r="AA9" s="18"/>
       <c r="AB9" s="18"/>
       <c r="AC9" s="5">
-        <v>0.95187794227321709</v>
+        <v>0.97468227062914359</v>
       </c>
       <c r="AD9" s="18">
-        <v>4090894625</v>
+        <v>2152280428</v>
       </c>
       <c r="AE9" s="18"/>
       <c r="AF9" s="18"/>
@@ -2807,20 +2807,20 @@
         <v>76886537335</v>
       </c>
       <c r="X21" s="20">
-        <v>0</v>
+        <v>1938614197</v>
       </c>
       <c r="Y21" s="20"/>
       <c r="Z21" s="20">
-        <v>76886537335</v>
+        <v>78825151532</v>
       </c>
       <c r="AA21" s="20"/>
       <c r="AB21" s="20"/>
       <c r="AC21" s="21">
-        <v>0.9494814273488652</v>
+        <v>0.97342161556187279</v>
       </c>
       <c r="AD21" s="21"/>
       <c r="AE21" s="20">
-        <v>4090862665</v>
+        <v>2152248468</v>
       </c>
       <c r="AF21" s="20"/>
       <c r="AG21" s="20"/>
@@ -2862,20 +2862,20 @@
         <v>76886537335</v>
       </c>
       <c r="X22" s="20">
-        <v>0</v>
+        <v>1938614197</v>
       </c>
       <c r="Y22" s="20"/>
       <c r="Z22" s="20">
-        <v>76886537335</v>
+        <v>78825151532</v>
       </c>
       <c r="AA22" s="20"/>
       <c r="AB22" s="20"/>
       <c r="AC22" s="21">
-        <v>0.9494814273488652</v>
+        <v>0.97342161556187279</v>
       </c>
       <c r="AD22" s="21"/>
       <c r="AE22" s="20">
-        <v>4090862665</v>
+        <v>2152248468</v>
       </c>
       <c r="AF22" s="20"/>
       <c r="AG22" s="20"/>
@@ -2917,20 +2917,20 @@
         <v>76885937335</v>
       </c>
       <c r="X23" s="23">
-        <v>0</v>
+        <v>1938614197</v>
       </c>
       <c r="Y23" s="23"/>
       <c r="Z23" s="23">
-        <v>76885937335</v>
+        <v>78824551532</v>
       </c>
       <c r="AA23" s="23"/>
       <c r="AB23" s="23"/>
       <c r="AC23" s="24">
-        <v>0.94948105303000363</v>
+        <v>0.97342141862854548</v>
       </c>
       <c r="AD23" s="24"/>
       <c r="AE23" s="23">
-        <v>4090862665</v>
+        <v>2152248468</v>
       </c>
       <c r="AF23" s="23"/>
       <c r="AG23" s="23"/>
@@ -4154,20 +4154,20 @@
         <v>76870226283</v>
       </c>
       <c r="X46" s="28">
-        <v>0</v>
+        <v>1938614197</v>
       </c>
       <c r="Y46" s="28"/>
       <c r="Z46" s="27">
-        <v>76870226283</v>
+        <v>78808840480</v>
       </c>
       <c r="AA46" s="27"/>
       <c r="AB46" s="27"/>
       <c r="AC46" s="29">
-        <v>0.94950430985000045</v>
+        <v>0.97345015499960663</v>
       </c>
       <c r="AD46" s="29"/>
       <c r="AE46" s="27">
-        <v>4088043717</v>
+        <v>2149429520</v>
       </c>
       <c r="AF46" s="27"/>
       <c r="AG46" s="27"/>
@@ -4209,20 +4209,20 @@
         <v>70952227437</v>
       </c>
       <c r="X47" s="31">
-        <v>0</v>
+        <v>1929165877</v>
       </c>
       <c r="Y47" s="31"/>
       <c r="Z47" s="31">
-        <v>70952227437</v>
+        <v>72881393314</v>
       </c>
       <c r="AA47" s="31"/>
       <c r="AB47" s="31"/>
       <c r="AC47" s="32">
-        <v>0.95507148828243493</v>
+        <v>0.98103954301230323</v>
       </c>
       <c r="AD47" s="32"/>
       <c r="AE47" s="31">
-        <v>3337737563</v>
+        <v>1408571686</v>
       </c>
       <c r="AF47" s="31"/>
       <c r="AG47" s="31"/>
@@ -4264,20 +4264,20 @@
         <v>5428525892</v>
       </c>
       <c r="X48" s="20">
-        <v>0</v>
+        <v>202138903</v>
       </c>
       <c r="Y48" s="20"/>
       <c r="Z48" s="20">
-        <v>5428525892</v>
+        <v>5630664795</v>
       </c>
       <c r="AA48" s="20"/>
       <c r="AB48" s="20"/>
       <c r="AC48" s="21">
-        <v>0.84729791405098409</v>
+        <v>0.87884826017954487</v>
       </c>
       <c r="AD48" s="21"/>
       <c r="AE48" s="20">
-        <v>978342108</v>
+        <v>776203205</v>
       </c>
       <c r="AF48" s="20"/>
       <c r="AG48" s="20"/>
@@ -4319,20 +4319,20 @@
         <v>2140015700</v>
       </c>
       <c r="X49" s="20">
-        <v>0</v>
+        <v>161230800</v>
       </c>
       <c r="Y49" s="20"/>
       <c r="Z49" s="20">
-        <v>2140015700</v>
+        <v>2301246500</v>
       </c>
       <c r="AA49" s="20"/>
       <c r="AB49" s="20"/>
       <c r="AC49" s="21">
-        <v>0.76363459567628977</v>
+        <v>0.82116754591051699</v>
       </c>
       <c r="AD49" s="21"/>
       <c r="AE49" s="20">
-        <v>662392300</v>
+        <v>501161500</v>
       </c>
       <c r="AF49" s="20"/>
       <c r="AG49" s="20"/>
@@ -4372,20 +4372,20 @@
         <v>1809835300</v>
       </c>
       <c r="X50" s="20">
-        <v>0</v>
+        <v>161230800</v>
       </c>
       <c r="Y50" s="20"/>
       <c r="Z50" s="20">
-        <v>1809835300</v>
+        <v>1971066100</v>
       </c>
       <c r="AA50" s="20"/>
       <c r="AB50" s="20"/>
       <c r="AC50" s="21">
-        <v>0.73207005374934875</v>
+        <v>0.79728717070029476</v>
       </c>
       <c r="AD50" s="21"/>
       <c r="AE50" s="20">
-        <v>662380700</v>
+        <v>501149900</v>
       </c>
       <c r="AF50" s="20"/>
       <c r="AG50" s="20"/>
@@ -4533,20 +4533,20 @@
         <v>25093</v>
       </c>
       <c r="X53" s="20">
-        <v>0</v>
+        <v>1803</v>
       </c>
       <c r="Y53" s="20"/>
       <c r="Z53" s="20">
-        <v>25093</v>
+        <v>26896</v>
       </c>
       <c r="AA53" s="20"/>
       <c r="AB53" s="20"/>
       <c r="AC53" s="21">
-        <v>0.83643333333333336</v>
+        <v>0.89653333333333329</v>
       </c>
       <c r="AD53" s="21"/>
       <c r="AE53" s="20">
-        <v>4907</v>
+        <v>3104</v>
       </c>
       <c r="AF53" s="20"/>
       <c r="AG53" s="20"/>
@@ -4586,20 +4586,20 @@
         <v>20511</v>
       </c>
       <c r="X54" s="20">
-        <v>0</v>
+        <v>1803</v>
       </c>
       <c r="Y54" s="20"/>
       <c r="Z54" s="20">
-        <v>20511</v>
+        <v>22314</v>
       </c>
       <c r="AA54" s="20"/>
       <c r="AB54" s="20"/>
       <c r="AC54" s="21">
-        <v>0.85462499999999997</v>
+        <v>0.92974999999999997</v>
       </c>
       <c r="AD54" s="21"/>
       <c r="AE54" s="20">
-        <v>3489</v>
+        <v>1686</v>
       </c>
       <c r="AF54" s="20"/>
       <c r="AG54" s="20"/>
@@ -4747,20 +4747,20 @@
         <v>163021160</v>
       </c>
       <c r="X57" s="20">
-        <v>0</v>
+        <v>12175610</v>
       </c>
       <c r="Y57" s="20"/>
       <c r="Z57" s="20">
-        <v>163021160</v>
+        <v>175196770</v>
       </c>
       <c r="AA57" s="20"/>
       <c r="AB57" s="20"/>
       <c r="AC57" s="21">
-        <v>0.89572065934065936</v>
+        <v>0.96261961538461538</v>
       </c>
       <c r="AD57" s="21"/>
       <c r="AE57" s="20">
-        <v>18978840</v>
+        <v>6803230</v>
       </c>
       <c r="AF57" s="20"/>
       <c r="AG57" s="20"/>
@@ -4800,20 +4800,20 @@
         <v>137822840</v>
       </c>
       <c r="X58" s="20">
-        <v>0</v>
+        <v>12175610</v>
       </c>
       <c r="Y58" s="20"/>
       <c r="Z58" s="20">
-        <v>137822840</v>
+        <v>149998450</v>
       </c>
       <c r="AA58" s="20"/>
       <c r="AB58" s="20"/>
       <c r="AC58" s="21">
-        <v>0.8790170416858003</v>
+        <v>0.95667157763151178</v>
       </c>
       <c r="AD58" s="21"/>
       <c r="AE58" s="20">
-        <v>18969160</v>
+        <v>6793550</v>
       </c>
       <c r="AF58" s="20"/>
       <c r="AG58" s="20"/>
@@ -5000,20 +5000,20 @@
         <v>49459528</v>
       </c>
       <c r="X62" s="20">
-        <v>0</v>
+        <v>3650984</v>
       </c>
       <c r="Y62" s="20"/>
       <c r="Z62" s="20">
-        <v>49459528</v>
+        <v>53110512</v>
       </c>
       <c r="AA62" s="20"/>
       <c r="AB62" s="20"/>
       <c r="AC62" s="21">
-        <v>0.88320585714285715</v>
+        <v>0.94840199999999997</v>
       </c>
       <c r="AD62" s="21"/>
       <c r="AE62" s="20">
-        <v>6540472</v>
+        <v>2889488</v>
       </c>
       <c r="AF62" s="20"/>
       <c r="AG62" s="20"/>
@@ -5053,20 +5053,20 @@
         <v>41783470</v>
       </c>
       <c r="X63" s="20">
-        <v>0</v>
+        <v>3650984</v>
       </c>
       <c r="Y63" s="20"/>
       <c r="Z63" s="20">
-        <v>41783470</v>
+        <v>45434454</v>
       </c>
       <c r="AA63" s="20"/>
       <c r="AB63" s="20"/>
       <c r="AC63" s="21">
-        <v>0.86486732074846828</v>
+        <v>0.94043827620466969</v>
       </c>
       <c r="AD63" s="21"/>
       <c r="AE63" s="20">
-        <v>6528530</v>
+        <v>2877546</v>
       </c>
       <c r="AF63" s="20"/>
       <c r="AG63" s="20"/>
@@ -5214,20 +5214,20 @@
         <v>23400000</v>
       </c>
       <c r="X66" s="20">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y66" s="20"/>
       <c r="Z66" s="20">
-        <v>23400000</v>
+        <v>25200000</v>
       </c>
       <c r="AA66" s="20"/>
       <c r="AB66" s="20"/>
       <c r="AC66" s="21">
-        <v>0.9285714285714286</v>
+        <v>1</v>
       </c>
       <c r="AD66" s="21"/>
       <c r="AE66" s="20">
-        <v>1800000</v>
+        <v>0</v>
       </c>
       <c r="AF66" s="20"/>
       <c r="AG66" s="20"/>
@@ -5267,20 +5267,20 @@
         <v>19800000</v>
       </c>
       <c r="X67" s="20">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y67" s="20"/>
       <c r="Z67" s="20">
-        <v>19800000</v>
+        <v>21600000</v>
       </c>
       <c r="AA67" s="20"/>
       <c r="AB67" s="20"/>
       <c r="AC67" s="21">
-        <v>0.91666666666666663</v>
+        <v>1</v>
       </c>
       <c r="AD67" s="21"/>
       <c r="AE67" s="20">
-        <v>1800000</v>
+        <v>0</v>
       </c>
       <c r="AF67" s="20"/>
       <c r="AG67" s="20"/>
@@ -5428,20 +5428,20 @@
         <v>149682000</v>
       </c>
       <c r="X70" s="20">
-        <v>0</v>
+        <v>10394000</v>
       </c>
       <c r="Y70" s="20"/>
       <c r="Z70" s="20">
-        <v>149682000</v>
+        <v>160076000</v>
       </c>
       <c r="AA70" s="20"/>
       <c r="AB70" s="20"/>
       <c r="AC70" s="21">
-        <v>1.0321899954487153</v>
+        <v>1.1038658336436482</v>
       </c>
       <c r="AD70" s="21"/>
       <c r="AE70" s="20">
-        <v>-4668000</v>
+        <v>-15062000</v>
       </c>
       <c r="AF70" s="20"/>
       <c r="AG70" s="20"/>
@@ -5481,20 +5481,20 @@
         <v>125654000</v>
       </c>
       <c r="X71" s="20">
-        <v>0</v>
+        <v>10394000</v>
       </c>
       <c r="Y71" s="20"/>
       <c r="Z71" s="20">
-        <v>125654000</v>
+        <v>136048000</v>
       </c>
       <c r="AA71" s="20"/>
       <c r="AB71" s="20"/>
       <c r="AC71" s="21">
-        <v>1.0386001454737817</v>
+        <v>1.1245123322092176</v>
       </c>
       <c r="AD71" s="21"/>
       <c r="AE71" s="20">
-        <v>-4670000</v>
+        <v>-15064000</v>
       </c>
       <c r="AF71" s="20"/>
       <c r="AG71" s="20"/>
@@ -5642,20 +5642,20 @@
         <v>19962339</v>
       </c>
       <c r="X74" s="20">
-        <v>0</v>
+        <v>307406</v>
       </c>
       <c r="Y74" s="20"/>
       <c r="Z74" s="20">
-        <v>19962339</v>
+        <v>20269745</v>
       </c>
       <c r="AA74" s="20"/>
       <c r="AB74" s="20"/>
       <c r="AC74" s="21">
-        <v>1.0081989393939395</v>
+        <v>1.023724494949495</v>
       </c>
       <c r="AD74" s="21"/>
       <c r="AE74" s="20">
-        <v>-162339</v>
+        <v>-469745</v>
       </c>
       <c r="AF74" s="20"/>
       <c r="AG74" s="20"/>
@@ -5695,20 +5695,20 @@
         <v>2431323</v>
       </c>
       <c r="X75" s="20">
-        <v>0</v>
+        <v>307406</v>
       </c>
       <c r="Y75" s="20"/>
       <c r="Z75" s="20">
-        <v>2431323</v>
+        <v>2738729</v>
       </c>
       <c r="AA75" s="20"/>
       <c r="AB75" s="20"/>
       <c r="AC75" s="21">
-        <v>1.0777140957446809</v>
+        <v>1.213975620567376</v>
       </c>
       <c r="AD75" s="21"/>
       <c r="AE75" s="20">
-        <v>-175323</v>
+        <v>-482729</v>
       </c>
       <c r="AF75" s="20"/>
       <c r="AG75" s="20"/>
@@ -5856,20 +5856,20 @@
         <v>112830360</v>
       </c>
       <c r="X78" s="20">
-        <v>0</v>
+        <v>8328300</v>
       </c>
       <c r="Y78" s="20"/>
       <c r="Z78" s="20">
-        <v>112830360</v>
+        <v>121158660</v>
       </c>
       <c r="AA78" s="20"/>
       <c r="AB78" s="20"/>
       <c r="AC78" s="21">
-        <v>0.89547904761904762</v>
+        <v>0.96157666666666664</v>
       </c>
       <c r="AD78" s="21"/>
       <c r="AE78" s="20">
-        <v>13169640</v>
+        <v>4841340</v>
       </c>
       <c r="AF78" s="20"/>
       <c r="AG78" s="20"/>
@@ -5909,20 +5909,20 @@
         <v>95304720</v>
       </c>
       <c r="X79" s="20">
-        <v>0</v>
+        <v>8328300</v>
       </c>
       <c r="Y79" s="20"/>
       <c r="Z79" s="20">
-        <v>95304720</v>
+        <v>103633020</v>
       </c>
       <c r="AA79" s="20"/>
       <c r="AB79" s="20"/>
       <c r="AC79" s="21">
-        <v>0.87864365527160082</v>
+        <v>0.95542482575506138</v>
       </c>
       <c r="AD79" s="21"/>
       <c r="AE79" s="20">
-        <v>13163280</v>
+        <v>4834980</v>
       </c>
       <c r="AF79" s="20"/>
       <c r="AG79" s="20"/>
@@ -6284,20 +6284,20 @@
         <v>53385000</v>
       </c>
       <c r="X86" s="20">
-        <v>0</v>
+        <v>4250000</v>
       </c>
       <c r="Y86" s="20"/>
       <c r="Z86" s="20">
-        <v>53385000</v>
+        <v>57635000</v>
       </c>
       <c r="AA86" s="20"/>
       <c r="AB86" s="20"/>
       <c r="AC86" s="21">
-        <v>0.84738095238095235</v>
+        <v>0.91484126984126979</v>
       </c>
       <c r="AD86" s="21"/>
       <c r="AE86" s="20">
-        <v>9615000</v>
+        <v>5365000</v>
       </c>
       <c r="AF86" s="20"/>
       <c r="AG86" s="20"/>
@@ -6337,20 +6337,20 @@
         <v>45455000</v>
       </c>
       <c r="X87" s="20">
-        <v>0</v>
+        <v>4250000</v>
       </c>
       <c r="Y87" s="20"/>
       <c r="Z87" s="20">
-        <v>45455000</v>
+        <v>49705000</v>
       </c>
       <c r="AA87" s="20"/>
       <c r="AB87" s="20"/>
       <c r="AC87" s="21">
-        <v>0.8261541257724464</v>
+        <v>0.90339876408578701</v>
       </c>
       <c r="AD87" s="21"/>
       <c r="AE87" s="20">
-        <v>9565000</v>
+        <v>5315000</v>
       </c>
       <c r="AF87" s="20"/>
       <c r="AG87" s="20"/>
@@ -6751,20 +6751,20 @@
         <v>136865920</v>
       </c>
       <c r="X95" s="20">
-        <v>0</v>
+        <v>136865920</v>
       </c>
       <c r="Y95" s="20"/>
       <c r="Z95" s="20">
-        <v>136865920</v>
+        <v>273731840</v>
       </c>
       <c r="AA95" s="20"/>
       <c r="AB95" s="20"/>
       <c r="AC95" s="21">
-        <v>1013.8216296296297</v>
+        <v>2027.6432592592594</v>
       </c>
       <c r="AD95" s="21"/>
       <c r="AE95" s="20">
-        <v>-136730920</v>
+        <v>-273596840</v>
       </c>
       <c r="AF95" s="20"/>
       <c r="AG95" s="20"/>
@@ -6806,20 +6806,20 @@
         <v>112205200</v>
       </c>
       <c r="X96" s="20">
-        <v>0</v>
+        <v>112205200</v>
       </c>
       <c r="Y96" s="20"/>
       <c r="Z96" s="20">
-        <v>112205200</v>
+        <v>224410400</v>
       </c>
       <c r="AA96" s="20"/>
       <c r="AB96" s="20"/>
       <c r="AC96" s="21">
-        <v>8014.6571428571433</v>
+        <v>16029.314285714287</v>
       </c>
       <c r="AD96" s="21"/>
       <c r="AE96" s="20">
-        <v>-112191200</v>
+        <v>-224396400</v>
       </c>
       <c r="AF96" s="20"/>
       <c r="AG96" s="20"/>
@@ -6859,20 +6859,20 @@
         <v>112205200</v>
       </c>
       <c r="X97" s="20">
-        <v>0</v>
+        <v>112205200</v>
       </c>
       <c r="Y97" s="20"/>
       <c r="Z97" s="20">
-        <v>112205200</v>
+        <v>224410400</v>
       </c>
       <c r="AA97" s="20"/>
       <c r="AB97" s="20"/>
       <c r="AC97" s="21">
-        <v>9350.4333333333325</v>
+        <v>18700.866666666665</v>
       </c>
       <c r="AD97" s="21"/>
       <c r="AE97" s="20">
-        <v>-112193200</v>
+        <v>-224398400</v>
       </c>
       <c r="AF97" s="20"/>
       <c r="AG97" s="20"/>
@@ -7020,20 +7020,20 @@
         <v>2086</v>
       </c>
       <c r="X100" s="20">
-        <v>0</v>
+        <v>2086</v>
       </c>
       <c r="Y100" s="20"/>
       <c r="Z100" s="20">
-        <v>2086</v>
+        <v>4172</v>
       </c>
       <c r="AA100" s="20"/>
       <c r="AB100" s="20"/>
       <c r="AC100" s="21">
-        <v>0.14899999999999999</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="AD100" s="21"/>
       <c r="AE100" s="20">
-        <v>11914</v>
+        <v>9828</v>
       </c>
       <c r="AF100" s="20"/>
       <c r="AG100" s="20"/>
@@ -7073,20 +7073,20 @@
         <v>2086</v>
       </c>
       <c r="X101" s="20">
-        <v>0</v>
+        <v>2086</v>
       </c>
       <c r="Y101" s="20"/>
       <c r="Z101" s="20">
-        <v>2086</v>
+        <v>4172</v>
       </c>
       <c r="AA101" s="20"/>
       <c r="AB101" s="20"/>
       <c r="AC101" s="21">
-        <v>0.17383333333333334</v>
+        <v>0.34766666666666668</v>
       </c>
       <c r="AD101" s="21"/>
       <c r="AE101" s="20">
-        <v>9914</v>
+        <v>7828</v>
       </c>
       <c r="AF101" s="20"/>
       <c r="AG101" s="20"/>
@@ -7234,20 +7234,20 @@
         <v>7571670</v>
       </c>
       <c r="X104" s="20">
-        <v>0</v>
+        <v>7571670</v>
       </c>
       <c r="Y104" s="20"/>
       <c r="Z104" s="20">
-        <v>7571670</v>
+        <v>15143340</v>
       </c>
       <c r="AA104" s="20"/>
       <c r="AB104" s="20"/>
       <c r="AC104" s="21">
-        <v>540.83357142857142</v>
+        <v>1081.6671428571428</v>
       </c>
       <c r="AD104" s="21"/>
       <c r="AE104" s="20">
-        <v>-7557670</v>
+        <v>-15129340</v>
       </c>
       <c r="AF104" s="20"/>
       <c r="AG104" s="20"/>
@@ -7287,20 +7287,20 @@
         <v>7571670</v>
       </c>
       <c r="X105" s="20">
-        <v>0</v>
+        <v>7571670</v>
       </c>
       <c r="Y105" s="20"/>
       <c r="Z105" s="20">
-        <v>7571670</v>
+        <v>15143340</v>
       </c>
       <c r="AA105" s="20"/>
       <c r="AB105" s="20"/>
       <c r="AC105" s="21">
-        <v>630.97249999999997</v>
+        <v>1261.9449999999999</v>
       </c>
       <c r="AD105" s="21"/>
       <c r="AE105" s="20">
-        <v>-7559670</v>
+        <v>-15131340</v>
       </c>
       <c r="AF105" s="20"/>
       <c r="AG105" s="20"/>
@@ -7448,20 +7448,20 @@
         <v>2630444</v>
       </c>
       <c r="X108" s="20">
-        <v>0</v>
+        <v>2630444</v>
       </c>
       <c r="Y108" s="20"/>
       <c r="Z108" s="20">
-        <v>2630444</v>
+        <v>5260888</v>
       </c>
       <c r="AA108" s="20"/>
       <c r="AB108" s="20"/>
       <c r="AC108" s="21">
-        <v>187.88885714285715</v>
+        <v>375.7777142857143</v>
       </c>
       <c r="AD108" s="21"/>
       <c r="AE108" s="20">
-        <v>-2616444</v>
+        <v>-5246888</v>
       </c>
       <c r="AF108" s="20"/>
       <c r="AG108" s="20"/>
@@ -7501,20 +7501,20 @@
         <v>2630444</v>
       </c>
       <c r="X109" s="20">
-        <v>0</v>
+        <v>2630444</v>
       </c>
       <c r="Y109" s="20"/>
       <c r="Z109" s="20">
-        <v>2630444</v>
+        <v>5260888</v>
       </c>
       <c r="AA109" s="20"/>
       <c r="AB109" s="20"/>
       <c r="AC109" s="21">
-        <v>219.20366666666666</v>
+        <v>438.40733333333333</v>
       </c>
       <c r="AD109" s="21"/>
       <c r="AE109" s="20">
-        <v>-2618444</v>
+        <v>-5248888</v>
       </c>
       <c r="AF109" s="20"/>
       <c r="AG109" s="20"/>
@@ -7662,20 +7662,20 @@
         <v>7676520</v>
       </c>
       <c r="X112" s="20">
-        <v>0</v>
+        <v>7676520</v>
       </c>
       <c r="Y112" s="20"/>
       <c r="Z112" s="20">
-        <v>7676520</v>
+        <v>15353040</v>
       </c>
       <c r="AA112" s="20"/>
       <c r="AB112" s="20"/>
       <c r="AC112" s="21">
-        <v>548.32285714285717</v>
+        <v>1096.6457142857143</v>
       </c>
       <c r="AD112" s="21"/>
       <c r="AE112" s="20">
-        <v>-7662520</v>
+        <v>-15339040</v>
       </c>
       <c r="AF112" s="20"/>
       <c r="AG112" s="20"/>
@@ -7715,20 +7715,20 @@
         <v>7676520</v>
       </c>
       <c r="X113" s="20">
-        <v>0</v>
+        <v>7676520</v>
       </c>
       <c r="Y113" s="20"/>
       <c r="Z113" s="20">
-        <v>7676520</v>
+        <v>15353040</v>
       </c>
       <c r="AA113" s="20"/>
       <c r="AB113" s="20"/>
       <c r="AC113" s="21">
-        <v>639.71</v>
+        <v>1279.42</v>
       </c>
       <c r="AD113" s="21"/>
       <c r="AE113" s="20">
-        <v>-7664520</v>
+        <v>-15341040</v>
       </c>
       <c r="AF113" s="20"/>
       <c r="AG113" s="20"/>
@@ -8023,20 +8023,20 @@
         <v>6780000</v>
       </c>
       <c r="X119" s="20">
-        <v>0</v>
+        <v>6780000</v>
       </c>
       <c r="Y119" s="20"/>
       <c r="Z119" s="20">
-        <v>6780000</v>
+        <v>13560000</v>
       </c>
       <c r="AA119" s="20"/>
       <c r="AB119" s="20"/>
       <c r="AC119" s="21">
-        <v>484.28571428571428</v>
+        <v>968.57142857142856</v>
       </c>
       <c r="AD119" s="21"/>
       <c r="AE119" s="20">
-        <v>-6766000</v>
+        <v>-13546000</v>
       </c>
       <c r="AF119" s="20"/>
       <c r="AG119" s="20"/>
@@ -8076,20 +8076,20 @@
         <v>6780000</v>
       </c>
       <c r="X120" s="20">
-        <v>0</v>
+        <v>6780000</v>
       </c>
       <c r="Y120" s="20"/>
       <c r="Z120" s="20">
-        <v>6780000</v>
+        <v>13560000</v>
       </c>
       <c r="AA120" s="20"/>
       <c r="AB120" s="20"/>
       <c r="AC120" s="21">
-        <v>565</v>
+        <v>1130</v>
       </c>
       <c r="AD120" s="21"/>
       <c r="AE120" s="20">
-        <v>-6768000</v>
+        <v>-13548000</v>
       </c>
       <c r="AF120" s="20"/>
       <c r="AG120" s="20"/>
@@ -8451,20 +8451,20 @@
         <v>46945779107</v>
       </c>
       <c r="X127" s="20">
-        <v>0</v>
+        <v>1590161054</v>
       </c>
       <c r="Y127" s="20"/>
       <c r="Z127" s="20">
-        <v>46945779107</v>
+        <v>48535940161</v>
       </c>
       <c r="AA127" s="20"/>
       <c r="AB127" s="20"/>
       <c r="AC127" s="21">
-        <v>0.89664757938202799</v>
+        <v>0.92701908640605513</v>
       </c>
       <c r="AD127" s="21"/>
       <c r="AE127" s="20">
-        <v>5411222893</v>
+        <v>3821061839</v>
       </c>
       <c r="AF127" s="20"/>
       <c r="AG127" s="20"/>
@@ -8506,20 +8506,20 @@
         <v>15933147500</v>
       </c>
       <c r="X128" s="20">
-        <v>0</v>
+        <v>1154795300</v>
       </c>
       <c r="Y128" s="20"/>
       <c r="Z128" s="20">
-        <v>15933147500</v>
+        <v>17087942800</v>
       </c>
       <c r="AA128" s="20"/>
       <c r="AB128" s="20"/>
       <c r="AC128" s="21">
-        <v>1.2115804130482952</v>
+        <v>1.2993927782172132</v>
       </c>
       <c r="AD128" s="21"/>
       <c r="AE128" s="20">
-        <v>-2782433500</v>
+        <v>-3937228800</v>
       </c>
       <c r="AF128" s="20"/>
       <c r="AG128" s="20"/>
@@ -8559,20 +8559,20 @@
         <v>13442394100</v>
       </c>
       <c r="X129" s="20">
-        <v>0</v>
+        <v>1154795300</v>
       </c>
       <c r="Y129" s="20"/>
       <c r="Z129" s="20">
-        <v>13442394100</v>
+        <v>14597189400</v>
       </c>
       <c r="AA129" s="20"/>
       <c r="AB129" s="20"/>
       <c r="AC129" s="21">
-        <v>1.2610173115096117</v>
+        <v>1.3693474834802382</v>
       </c>
       <c r="AD129" s="21"/>
       <c r="AE129" s="20">
-        <v>-2782434100</v>
+        <v>-3937229400</v>
       </c>
       <c r="AF129" s="20"/>
       <c r="AG129" s="20"/>
@@ -8720,20 +8720,20 @@
         <v>215018</v>
       </c>
       <c r="X132" s="20">
-        <v>0</v>
+        <v>15003</v>
       </c>
       <c r="Y132" s="20"/>
       <c r="Z132" s="20">
-        <v>215018</v>
+        <v>230021</v>
       </c>
       <c r="AA132" s="20"/>
       <c r="AB132" s="20"/>
       <c r="AC132" s="21">
-        <v>0.89965690376569041</v>
+        <v>0.96243096234309622</v>
       </c>
       <c r="AD132" s="21"/>
       <c r="AE132" s="20">
-        <v>23982</v>
+        <v>8979</v>
       </c>
       <c r="AF132" s="20"/>
       <c r="AG132" s="20"/>
@@ -8773,20 +8773,20 @@
         <v>181244</v>
       </c>
       <c r="X133" s="20">
-        <v>0</v>
+        <v>15003</v>
       </c>
       <c r="Y133" s="20"/>
       <c r="Z133" s="20">
-        <v>181244</v>
+        <v>196247</v>
       </c>
       <c r="AA133" s="20"/>
       <c r="AB133" s="20"/>
       <c r="AC133" s="21">
-        <v>0.88845098039215686</v>
+        <v>0.96199509803921568</v>
       </c>
       <c r="AD133" s="21"/>
       <c r="AE133" s="20">
-        <v>22756</v>
+        <v>7753</v>
       </c>
       <c r="AF133" s="20"/>
       <c r="AG133" s="20"/>
@@ -8934,20 +8934,20 @@
         <v>1253308570</v>
       </c>
       <c r="X136" s="20">
-        <v>0</v>
+        <v>91064390</v>
       </c>
       <c r="Y136" s="20"/>
       <c r="Z136" s="20">
-        <v>1253308570</v>
+        <v>1344372960</v>
       </c>
       <c r="AA136" s="20"/>
       <c r="AB136" s="20"/>
       <c r="AC136" s="21">
-        <v>0.9137899238088294</v>
+        <v>0.98018516277204626</v>
       </c>
       <c r="AD136" s="21"/>
       <c r="AE136" s="20">
-        <v>118241430</v>
+        <v>27177040</v>
       </c>
       <c r="AF136" s="20"/>
       <c r="AG136" s="20"/>
@@ -8987,20 +8987,20 @@
         <v>1058323510</v>
       </c>
       <c r="X137" s="20">
-        <v>0</v>
+        <v>91064390</v>
       </c>
       <c r="Y137" s="20"/>
       <c r="Z137" s="20">
-        <v>1058323510</v>
+        <v>1149387900</v>
       </c>
       <c r="AA137" s="20"/>
       <c r="AB137" s="20"/>
       <c r="AC137" s="21">
-        <v>0.89950356291710443</v>
+        <v>0.97690214896937189</v>
       </c>
       <c r="AD137" s="21"/>
       <c r="AE137" s="20">
-        <v>118240490</v>
+        <v>27176100</v>
       </c>
       <c r="AF137" s="20"/>
       <c r="AG137" s="20"/>
@@ -9148,20 +9148,20 @@
         <v>391175896</v>
       </c>
       <c r="X140" s="20">
-        <v>0</v>
+        <v>29286128</v>
       </c>
       <c r="Y140" s="20"/>
       <c r="Z140" s="20">
-        <v>391175896</v>
+        <v>420462024</v>
       </c>
       <c r="AA140" s="20"/>
       <c r="AB140" s="20"/>
       <c r="AC140" s="21">
-        <v>0.90287265064384414</v>
+        <v>0.9704679301199981</v>
       </c>
       <c r="AD140" s="21"/>
       <c r="AE140" s="20">
-        <v>42081104</v>
+        <v>12794976</v>
       </c>
       <c r="AF140" s="20"/>
       <c r="AG140" s="20"/>
@@ -9201,20 +9201,20 @@
         <v>330785040</v>
       </c>
       <c r="X141" s="20">
-        <v>0</v>
+        <v>29286128</v>
       </c>
       <c r="Y141" s="20"/>
       <c r="Z141" s="20">
-        <v>330785040</v>
+        <v>360071168</v>
       </c>
       <c r="AA141" s="20"/>
       <c r="AB141" s="20"/>
       <c r="AC141" s="21">
-        <v>0.88714662718846549</v>
+        <v>0.96569035358736699</v>
       </c>
       <c r="AD141" s="21"/>
       <c r="AE141" s="20">
-        <v>42078960</v>
+        <v>12792832</v>
       </c>
       <c r="AF141" s="20"/>
       <c r="AG141" s="20"/>
@@ -9362,20 +9362,20 @@
         <v>3435770000</v>
       </c>
       <c r="X144" s="20">
-        <v>0</v>
+        <v>247680000</v>
       </c>
       <c r="Y144" s="20"/>
       <c r="Z144" s="20">
-        <v>3435770000</v>
+        <v>3683450000</v>
       </c>
       <c r="AA144" s="20"/>
       <c r="AB144" s="20"/>
       <c r="AC144" s="21">
-        <v>0.89240779220779221</v>
+        <v>0.95674025974025978</v>
       </c>
       <c r="AD144" s="21"/>
       <c r="AE144" s="20">
-        <v>414230000</v>
+        <v>166550000</v>
       </c>
       <c r="AF144" s="20"/>
       <c r="AG144" s="20"/>
@@ -9454,20 +9454,20 @@
         <v>2897510000</v>
       </c>
       <c r="X146" s="20">
-        <v>0</v>
+        <v>247680000</v>
       </c>
       <c r="Y146" s="20"/>
       <c r="Z146" s="20">
-        <v>2897510000</v>
+        <v>3145190000</v>
       </c>
       <c r="AA146" s="20"/>
       <c r="AB146" s="20"/>
       <c r="AC146" s="21">
-        <v>0.87492179328303943</v>
+        <v>0.94971036338645354</v>
       </c>
       <c r="AD146" s="21"/>
       <c r="AE146" s="20">
-        <v>414226000</v>
+        <v>166546000</v>
       </c>
       <c r="AF146" s="20"/>
       <c r="AG146" s="20"/>
@@ -9615,20 +9615,20 @@
         <v>227374624</v>
       </c>
       <c r="X149" s="20">
-        <v>0</v>
+        <v>2029653</v>
       </c>
       <c r="Y149" s="20"/>
       <c r="Z149" s="20">
-        <v>227374624</v>
+        <v>229404277</v>
       </c>
       <c r="AA149" s="20"/>
       <c r="AB149" s="20"/>
       <c r="AC149" s="21">
-        <v>0.92530266552720464</v>
+        <v>0.93356235298905299</v>
       </c>
       <c r="AD149" s="21"/>
       <c r="AE149" s="20">
-        <v>18355376</v>
+        <v>16325723</v>
       </c>
       <c r="AF149" s="20"/>
       <c r="AG149" s="20"/>
@@ -9668,20 +9668,20 @@
         <v>41918493</v>
       </c>
       <c r="X150" s="20">
-        <v>0</v>
+        <v>2029653</v>
       </c>
       <c r="Y150" s="20"/>
       <c r="Z150" s="20">
-        <v>41918493</v>
+        <v>43948146</v>
       </c>
       <c r="AA150" s="20"/>
       <c r="AB150" s="20"/>
       <c r="AC150" s="21">
-        <v>0.6955809936280366</v>
+        <v>0.729260354440462</v>
       </c>
       <c r="AD150" s="21"/>
       <c r="AE150" s="20">
-        <v>18345507</v>
+        <v>16315854</v>
       </c>
       <c r="AF150" s="20"/>
       <c r="AG150" s="20"/>
@@ -9829,20 +9829,20 @@
         <v>877947660</v>
       </c>
       <c r="X153" s="20">
-        <v>0</v>
+        <v>65105580</v>
       </c>
       <c r="Y153" s="20"/>
       <c r="Z153" s="20">
-        <v>877947660</v>
+        <v>943053240</v>
       </c>
       <c r="AA153" s="20"/>
       <c r="AB153" s="20"/>
       <c r="AC153" s="21">
-        <v>0.89586495918367348</v>
+        <v>0.96229922448979588</v>
       </c>
       <c r="AD153" s="21"/>
       <c r="AE153" s="20">
-        <v>102052340</v>
+        <v>36946760</v>
       </c>
       <c r="AF153" s="20"/>
       <c r="AG153" s="20"/>
@@ -9882,20 +9882,20 @@
         <v>741218700</v>
       </c>
       <c r="X154" s="20">
-        <v>0</v>
+        <v>65105580</v>
       </c>
       <c r="Y154" s="20"/>
       <c r="Z154" s="20">
-        <v>741218700</v>
+        <v>806324280</v>
       </c>
       <c r="AA154" s="20"/>
       <c r="AB154" s="20"/>
       <c r="AC154" s="21">
-        <v>0.87898771914845175</v>
+        <v>0.95619435906193073</v>
       </c>
       <c r="AD154" s="21"/>
       <c r="AE154" s="20">
-        <v>102045300</v>
+        <v>36939720</v>
       </c>
       <c r="AF154" s="20"/>
       <c r="AG154" s="20"/>
@@ -10257,20 +10257,20 @@
         <v>2775000</v>
       </c>
       <c r="X161" s="20">
-        <v>0</v>
+        <v>185000</v>
       </c>
       <c r="Y161" s="20"/>
       <c r="Z161" s="20">
-        <v>2775000</v>
+        <v>2960000</v>
       </c>
       <c r="AA161" s="20"/>
       <c r="AB161" s="20"/>
       <c r="AC161" s="21">
-        <v>0.5357142857142857</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="AD161" s="21"/>
       <c r="AE161" s="20">
-        <v>2405000</v>
+        <v>2220000</v>
       </c>
       <c r="AF161" s="20"/>
       <c r="AG161" s="20"/>
@@ -10310,20 +10310,20 @@
         <v>2220000</v>
       </c>
       <c r="X162" s="20">
-        <v>0</v>
+        <v>185000</v>
       </c>
       <c r="Y162" s="20"/>
       <c r="Z162" s="20">
-        <v>2220000</v>
+        <v>2405000</v>
       </c>
       <c r="AA162" s="20"/>
       <c r="AB162" s="20"/>
       <c r="AC162" s="21">
-        <v>0.48051948051948051</v>
+        <v>0.52056277056277056</v>
       </c>
       <c r="AD162" s="21"/>
       <c r="AE162" s="20">
-        <v>2400000</v>
+        <v>2215000</v>
       </c>
       <c r="AF162" s="20"/>
       <c r="AG162" s="20"/>
@@ -12477,20 +12477,20 @@
         <v>5917998846</v>
       </c>
       <c r="X203" s="31">
-        <v>0</v>
+        <v>9448320</v>
       </c>
       <c r="Y203" s="31"/>
       <c r="Z203" s="31">
-        <v>5917998846</v>
+        <v>5927447166</v>
       </c>
       <c r="AA203" s="31"/>
       <c r="AB203" s="31"/>
       <c r="AC203" s="32">
-        <v>0.88748172826527882</v>
+        <v>0.8888986280621537</v>
       </c>
       <c r="AD203" s="32"/>
       <c r="AE203" s="31">
-        <v>750306154</v>
+        <v>740857834</v>
       </c>
       <c r="AF203" s="31"/>
       <c r="AG203" s="31"/>
@@ -14554,20 +14554,20 @@
         <v>560645387</v>
       </c>
       <c r="X242" s="20">
-        <v>0</v>
+        <v>9448320</v>
       </c>
       <c r="Y242" s="20"/>
       <c r="Z242" s="20">
-        <v>560645387</v>
+        <v>570093707</v>
       </c>
       <c r="AA242" s="20"/>
       <c r="AB242" s="20"/>
       <c r="AC242" s="21">
-        <v>0.73765732762307001</v>
+        <v>0.75008875512311934</v>
       </c>
       <c r="AD242" s="21"/>
       <c r="AE242" s="20">
-        <v>199389613</v>
+        <v>189941293</v>
       </c>
       <c r="AF242" s="20"/>
       <c r="AG242" s="20"/>
@@ -15714,20 +15714,20 @@
         <v>158031069</v>
       </c>
       <c r="X264" s="20">
-        <v>0</v>
+        <v>9448320</v>
       </c>
       <c r="Y264" s="20"/>
       <c r="Z264" s="20">
-        <v>158031069</v>
+        <v>167479389</v>
       </c>
       <c r="AA264" s="20"/>
       <c r="AB264" s="20"/>
       <c r="AC264" s="21">
-        <v>0.68721111932510004</v>
+        <v>0.72829791702904856</v>
       </c>
       <c r="AD264" s="21"/>
       <c r="AE264" s="20">
-        <v>71928931</v>
+        <v>62480611</v>
       </c>
       <c r="AF264" s="20"/>
       <c r="AG264" s="20"/>
@@ -16032,20 +16032,20 @@
         <v>4737535</v>
       </c>
       <c r="X270" s="20">
-        <v>0</v>
+        <v>9448320</v>
       </c>
       <c r="Y270" s="20"/>
       <c r="Z270" s="20">
-        <v>4737535</v>
+        <v>14185855</v>
       </c>
       <c r="AA270" s="20"/>
       <c r="AB270" s="20"/>
       <c r="AC270" s="21">
-        <v>0.32672655172413795</v>
+        <v>0.97833482758620693</v>
       </c>
       <c r="AD270" s="21"/>
       <c r="AE270" s="20">
-        <v>9762465</v>
+        <v>314145</v>
       </c>
       <c r="AF270" s="20"/>
       <c r="AG270" s="20"/>

</xml_diff>

<commit_message>
up date realisasi 11 nov 25
up date realisasi 11 nov 25
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D0373B4-E131-4C64-B601-FC1934E016AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{876B2871-EC8D-49A7-9027-8C23F5BD8716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="45" windowWidth="14925" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GLP039_LAPORAN REALISASI SUPER " sheetId="1" r:id="rId1"/>
@@ -2155,19 +2155,19 @@
         <v>80919905375</v>
       </c>
       <c r="X9" s="4">
-        <v>1938614197</v>
+        <v>3695933614</v>
       </c>
       <c r="Y9" s="18">
-        <v>82858519572</v>
+        <v>84615838989</v>
       </c>
       <c r="Z9" s="18"/>
       <c r="AA9" s="18"/>
       <c r="AB9" s="18"/>
       <c r="AC9" s="5">
-        <v>0.97468227062914359</v>
+        <v>0.99535399018712911</v>
       </c>
       <c r="AD9" s="18">
-        <v>2152280428</v>
+        <v>394961011</v>
       </c>
       <c r="AE9" s="18"/>
       <c r="AF9" s="18"/>
@@ -2807,20 +2807,20 @@
         <v>76886537335</v>
       </c>
       <c r="X21" s="20">
-        <v>1938614197</v>
+        <v>3695933614</v>
       </c>
       <c r="Y21" s="20"/>
       <c r="Z21" s="20">
-        <v>78825151532</v>
+        <v>80582470949</v>
       </c>
       <c r="AA21" s="20"/>
       <c r="AB21" s="20"/>
       <c r="AC21" s="21">
-        <v>0.97342161556187279</v>
+        <v>0.9951229719526683</v>
       </c>
       <c r="AD21" s="21"/>
       <c r="AE21" s="20">
-        <v>2152248468</v>
+        <v>394929051</v>
       </c>
       <c r="AF21" s="20"/>
       <c r="AG21" s="20"/>
@@ -2862,20 +2862,20 @@
         <v>76886537335</v>
       </c>
       <c r="X22" s="20">
-        <v>1938614197</v>
+        <v>3695933614</v>
       </c>
       <c r="Y22" s="20"/>
       <c r="Z22" s="20">
-        <v>78825151532</v>
+        <v>80582470949</v>
       </c>
       <c r="AA22" s="20"/>
       <c r="AB22" s="20"/>
       <c r="AC22" s="21">
-        <v>0.97342161556187279</v>
+        <v>0.9951229719526683</v>
       </c>
       <c r="AD22" s="21"/>
       <c r="AE22" s="20">
-        <v>2152248468</v>
+        <v>394929051</v>
       </c>
       <c r="AF22" s="20"/>
       <c r="AG22" s="20"/>
@@ -2917,20 +2917,20 @@
         <v>76885937335</v>
       </c>
       <c r="X23" s="23">
-        <v>1938614197</v>
+        <v>3695933614</v>
       </c>
       <c r="Y23" s="23"/>
       <c r="Z23" s="23">
-        <v>78824551532</v>
+        <v>80581870949</v>
       </c>
       <c r="AA23" s="23"/>
       <c r="AB23" s="23"/>
       <c r="AC23" s="24">
-        <v>0.97342141862854548</v>
+        <v>0.99512293581618438</v>
       </c>
       <c r="AD23" s="24"/>
       <c r="AE23" s="23">
-        <v>2152248468</v>
+        <v>394929051</v>
       </c>
       <c r="AF23" s="23"/>
       <c r="AG23" s="23"/>
@@ -3557,20 +3557,20 @@
         <v>14661052</v>
       </c>
       <c r="X35" s="28">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y35" s="28"/>
       <c r="Z35" s="27">
-        <v>14661052</v>
+        <v>16461052</v>
       </c>
       <c r="AA35" s="27"/>
       <c r="AB35" s="27"/>
       <c r="AC35" s="29">
-        <v>0.83873295194508013</v>
+        <v>0.94170778032036617</v>
       </c>
       <c r="AD35" s="29"/>
       <c r="AE35" s="27">
-        <v>2818948</v>
+        <v>1018948</v>
       </c>
       <c r="AF35" s="27"/>
       <c r="AG35" s="27"/>
@@ -3612,20 +3612,20 @@
         <v>14661052</v>
       </c>
       <c r="X36" s="31">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y36" s="31"/>
       <c r="Z36" s="31">
-        <v>14661052</v>
+        <v>16461052</v>
       </c>
       <c r="AA36" s="31"/>
       <c r="AB36" s="31"/>
       <c r="AC36" s="32">
-        <v>0.83873295194508013</v>
+        <v>0.94170778032036617</v>
       </c>
       <c r="AD36" s="32"/>
       <c r="AE36" s="31">
-        <v>2818948</v>
+        <v>1018948</v>
       </c>
       <c r="AF36" s="31"/>
       <c r="AG36" s="31"/>
@@ -3938,20 +3938,20 @@
         <v>12261052</v>
       </c>
       <c r="X42" s="20">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y42" s="20"/>
       <c r="Z42" s="20">
-        <v>12261052</v>
+        <v>14061052</v>
       </c>
       <c r="AA42" s="20"/>
       <c r="AB42" s="20"/>
       <c r="AC42" s="21">
-        <v>0.81306710875331567</v>
+        <v>0.9324305039787798</v>
       </c>
       <c r="AD42" s="21"/>
       <c r="AE42" s="20">
-        <v>2818948</v>
+        <v>1018948</v>
       </c>
       <c r="AF42" s="20"/>
       <c r="AG42" s="20"/>
@@ -3993,20 +3993,20 @@
         <v>12261052</v>
       </c>
       <c r="X43" s="20">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y43" s="20"/>
       <c r="Z43" s="20">
-        <v>12261052</v>
+        <v>14061052</v>
       </c>
       <c r="AA43" s="20"/>
       <c r="AB43" s="20"/>
       <c r="AC43" s="21">
-        <v>0.81306710875331567</v>
+        <v>0.9324305039787798</v>
       </c>
       <c r="AD43" s="21"/>
       <c r="AE43" s="20">
-        <v>2818948</v>
+        <v>1018948</v>
       </c>
       <c r="AF43" s="20"/>
       <c r="AG43" s="20"/>
@@ -4046,20 +4046,20 @@
         <v>11511952</v>
       </c>
       <c r="X44" s="20">
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Y44" s="20"/>
       <c r="Z44" s="20">
-        <v>11511952</v>
+        <v>13311952</v>
       </c>
       <c r="AA44" s="20"/>
       <c r="AB44" s="20"/>
       <c r="AC44" s="21">
-        <v>0.8366244186046512</v>
+        <v>0.9674383720930233</v>
       </c>
       <c r="AD44" s="21"/>
       <c r="AE44" s="20">
-        <v>2248048</v>
+        <v>448048</v>
       </c>
       <c r="AF44" s="20"/>
       <c r="AG44" s="20"/>
@@ -4154,20 +4154,20 @@
         <v>76870226283</v>
       </c>
       <c r="X46" s="28">
-        <v>1938614197</v>
+        <v>3694133614</v>
       </c>
       <c r="Y46" s="28"/>
       <c r="Z46" s="27">
-        <v>78808840480</v>
+        <v>80564359897</v>
       </c>
       <c r="AA46" s="27"/>
       <c r="AB46" s="27"/>
       <c r="AC46" s="29">
-        <v>0.97345015499960663</v>
+        <v>0.99513440562650368</v>
       </c>
       <c r="AD46" s="29"/>
       <c r="AE46" s="27">
-        <v>2149429520</v>
+        <v>393910103</v>
       </c>
       <c r="AF46" s="27"/>
       <c r="AG46" s="27"/>
@@ -4209,20 +4209,20 @@
         <v>70952227437</v>
       </c>
       <c r="X47" s="31">
-        <v>1929165877</v>
+        <v>3610829713</v>
       </c>
       <c r="Y47" s="31"/>
       <c r="Z47" s="31">
-        <v>72881393314</v>
+        <v>74563057150</v>
       </c>
       <c r="AA47" s="31"/>
       <c r="AB47" s="31"/>
       <c r="AC47" s="32">
-        <v>0.98103954301230323</v>
+        <v>1.0036760301340835</v>
       </c>
       <c r="AD47" s="32"/>
       <c r="AE47" s="31">
-        <v>1408571686</v>
+        <v>-273092150</v>
       </c>
       <c r="AF47" s="31"/>
       <c r="AG47" s="31"/>
@@ -4264,20 +4264,20 @@
         <v>5428525892</v>
       </c>
       <c r="X48" s="20">
-        <v>202138903</v>
+        <v>233886903</v>
       </c>
       <c r="Y48" s="20"/>
       <c r="Z48" s="20">
-        <v>5630664795</v>
+        <v>5662412795</v>
       </c>
       <c r="AA48" s="20"/>
       <c r="AB48" s="20"/>
       <c r="AC48" s="21">
-        <v>0.87884826017954487</v>
+        <v>0.88380356751536004</v>
       </c>
       <c r="AD48" s="21"/>
       <c r="AE48" s="20">
-        <v>776203205</v>
+        <v>744455205</v>
       </c>
       <c r="AF48" s="20"/>
       <c r="AG48" s="20"/>
@@ -6070,20 +6070,20 @@
         <v>245993000</v>
       </c>
       <c r="X82" s="20">
-        <v>0</v>
+        <v>31748000</v>
       </c>
       <c r="Y82" s="20"/>
       <c r="Z82" s="20">
-        <v>245993000</v>
+        <v>277741000</v>
       </c>
       <c r="AA82" s="20"/>
       <c r="AB82" s="20"/>
       <c r="AC82" s="21">
-        <v>0.78487696862955303</v>
+        <v>0.88617364780355823</v>
       </c>
       <c r="AD82" s="21"/>
       <c r="AE82" s="20">
-        <v>67423000</v>
+        <v>35675000</v>
       </c>
       <c r="AF82" s="20"/>
       <c r="AG82" s="20"/>
@@ -6123,20 +6123,20 @@
         <v>13930000</v>
       </c>
       <c r="X83" s="20">
-        <v>0</v>
+        <v>1610000</v>
       </c>
       <c r="Y83" s="20"/>
       <c r="Z83" s="20">
-        <v>13930000</v>
+        <v>15540000</v>
       </c>
       <c r="AA83" s="20"/>
       <c r="AB83" s="20"/>
       <c r="AC83" s="21">
-        <v>0.46064814814814814</v>
+        <v>0.51388888888888884</v>
       </c>
       <c r="AD83" s="21"/>
       <c r="AE83" s="20">
-        <v>16310000</v>
+        <v>14700000</v>
       </c>
       <c r="AF83" s="20"/>
       <c r="AG83" s="20"/>
@@ -6176,20 +6176,20 @@
         <v>201354000</v>
       </c>
       <c r="X84" s="20">
-        <v>0</v>
+        <v>26899000</v>
       </c>
       <c r="Y84" s="20"/>
       <c r="Z84" s="20">
-        <v>201354000</v>
+        <v>228253000</v>
       </c>
       <c r="AA84" s="20"/>
       <c r="AB84" s="20"/>
       <c r="AC84" s="21">
-        <v>0.81272401433691754</v>
+        <v>0.92129629629629628</v>
       </c>
       <c r="AD84" s="21"/>
       <c r="AE84" s="20">
-        <v>46398000</v>
+        <v>19499000</v>
       </c>
       <c r="AF84" s="20"/>
       <c r="AG84" s="20"/>
@@ -6229,20 +6229,20 @@
         <v>30709000</v>
       </c>
       <c r="X85" s="20">
-        <v>0</v>
+        <v>3239000</v>
       </c>
       <c r="Y85" s="20"/>
       <c r="Z85" s="20">
-        <v>30709000</v>
+        <v>33948000</v>
       </c>
       <c r="AA85" s="20"/>
       <c r="AB85" s="20"/>
       <c r="AC85" s="21">
-        <v>0.86689814814814814</v>
+        <v>0.95833333333333337</v>
       </c>
       <c r="AD85" s="21"/>
       <c r="AE85" s="20">
-        <v>4715000</v>
+        <v>1476000</v>
       </c>
       <c r="AF85" s="20"/>
       <c r="AG85" s="20"/>
@@ -6751,20 +6751,20 @@
         <v>136865920</v>
       </c>
       <c r="X95" s="20">
-        <v>136865920</v>
+        <v>143788036</v>
       </c>
       <c r="Y95" s="20"/>
       <c r="Z95" s="20">
-        <v>273731840</v>
+        <v>280653956</v>
       </c>
       <c r="AA95" s="20"/>
       <c r="AB95" s="20"/>
       <c r="AC95" s="21">
-        <v>2027.6432592592594</v>
+        <v>2078.9181925925927</v>
       </c>
       <c r="AD95" s="21"/>
       <c r="AE95" s="20">
-        <v>-273596840</v>
+        <v>-280518956</v>
       </c>
       <c r="AF95" s="20"/>
       <c r="AG95" s="20"/>
@@ -6806,20 +6806,20 @@
         <v>112205200</v>
       </c>
       <c r="X96" s="20">
-        <v>112205200</v>
+        <v>118612400</v>
       </c>
       <c r="Y96" s="20"/>
       <c r="Z96" s="20">
-        <v>224410400</v>
+        <v>230817600</v>
       </c>
       <c r="AA96" s="20"/>
       <c r="AB96" s="20"/>
       <c r="AC96" s="21">
-        <v>16029.314285714287</v>
+        <v>16486.971428571429</v>
       </c>
       <c r="AD96" s="21"/>
       <c r="AE96" s="20">
-        <v>-224396400</v>
+        <v>-230803600</v>
       </c>
       <c r="AF96" s="20"/>
       <c r="AG96" s="20"/>
@@ -6859,20 +6859,20 @@
         <v>112205200</v>
       </c>
       <c r="X97" s="20">
-        <v>112205200</v>
+        <v>118612400</v>
       </c>
       <c r="Y97" s="20"/>
       <c r="Z97" s="20">
-        <v>224410400</v>
+        <v>230817600</v>
       </c>
       <c r="AA97" s="20"/>
       <c r="AB97" s="20"/>
       <c r="AC97" s="21">
-        <v>18700.866666666665</v>
+        <v>19234.8</v>
       </c>
       <c r="AD97" s="21"/>
       <c r="AE97" s="20">
-        <v>-224398400</v>
+        <v>-230805600</v>
       </c>
       <c r="AF97" s="20"/>
       <c r="AG97" s="20"/>
@@ -7020,20 +7020,20 @@
         <v>2086</v>
       </c>
       <c r="X100" s="20">
-        <v>2086</v>
+        <v>2162</v>
       </c>
       <c r="Y100" s="20"/>
       <c r="Z100" s="20">
-        <v>4172</v>
+        <v>4248</v>
       </c>
       <c r="AA100" s="20"/>
       <c r="AB100" s="20"/>
       <c r="AC100" s="21">
-        <v>0.29799999999999999</v>
+        <v>0.30342857142857144</v>
       </c>
       <c r="AD100" s="21"/>
       <c r="AE100" s="20">
-        <v>9828</v>
+        <v>9752</v>
       </c>
       <c r="AF100" s="20"/>
       <c r="AG100" s="20"/>
@@ -7073,20 +7073,20 @@
         <v>2086</v>
       </c>
       <c r="X101" s="20">
-        <v>2086</v>
+        <v>2162</v>
       </c>
       <c r="Y101" s="20"/>
       <c r="Z101" s="20">
-        <v>4172</v>
+        <v>4248</v>
       </c>
       <c r="AA101" s="20"/>
       <c r="AB101" s="20"/>
       <c r="AC101" s="21">
-        <v>0.34766666666666668</v>
+        <v>0.35399999999999998</v>
       </c>
       <c r="AD101" s="21"/>
       <c r="AE101" s="20">
-        <v>7828</v>
+        <v>7752</v>
       </c>
       <c r="AF101" s="20"/>
       <c r="AG101" s="20"/>
@@ -7662,20 +7662,20 @@
         <v>7676520</v>
       </c>
       <c r="X112" s="20">
-        <v>7676520</v>
+        <v>7821360</v>
       </c>
       <c r="Y112" s="20"/>
       <c r="Z112" s="20">
-        <v>15353040</v>
+        <v>15497880</v>
       </c>
       <c r="AA112" s="20"/>
       <c r="AB112" s="20"/>
       <c r="AC112" s="21">
-        <v>1096.6457142857143</v>
+        <v>1106.9914285714285</v>
       </c>
       <c r="AD112" s="21"/>
       <c r="AE112" s="20">
-        <v>-15339040</v>
+        <v>-15483880</v>
       </c>
       <c r="AF112" s="20"/>
       <c r="AG112" s="20"/>
@@ -7715,20 +7715,20 @@
         <v>7676520</v>
       </c>
       <c r="X113" s="20">
-        <v>7676520</v>
+        <v>7821360</v>
       </c>
       <c r="Y113" s="20"/>
       <c r="Z113" s="20">
-        <v>15353040</v>
+        <v>15497880</v>
       </c>
       <c r="AA113" s="20"/>
       <c r="AB113" s="20"/>
       <c r="AC113" s="21">
-        <v>1279.42</v>
+        <v>1291.49</v>
       </c>
       <c r="AD113" s="21"/>
       <c r="AE113" s="20">
-        <v>-15341040</v>
+        <v>-15485880</v>
       </c>
       <c r="AF113" s="20"/>
       <c r="AG113" s="20"/>
@@ -8023,20 +8023,20 @@
         <v>6780000</v>
       </c>
       <c r="X119" s="20">
-        <v>6780000</v>
+        <v>7150000</v>
       </c>
       <c r="Y119" s="20"/>
       <c r="Z119" s="20">
-        <v>13560000</v>
+        <v>13930000</v>
       </c>
       <c r="AA119" s="20"/>
       <c r="AB119" s="20"/>
       <c r="AC119" s="21">
-        <v>968.57142857142856</v>
+        <v>995</v>
       </c>
       <c r="AD119" s="21"/>
       <c r="AE119" s="20">
-        <v>-13546000</v>
+        <v>-13916000</v>
       </c>
       <c r="AF119" s="20"/>
       <c r="AG119" s="20"/>
@@ -8076,20 +8076,20 @@
         <v>6780000</v>
       </c>
       <c r="X120" s="20">
-        <v>6780000</v>
+        <v>7150000</v>
       </c>
       <c r="Y120" s="20"/>
       <c r="Z120" s="20">
-        <v>13560000</v>
+        <v>13930000</v>
       </c>
       <c r="AA120" s="20"/>
       <c r="AB120" s="20"/>
       <c r="AC120" s="21">
-        <v>1130</v>
+        <v>1160.8333333333333</v>
       </c>
       <c r="AD120" s="21"/>
       <c r="AE120" s="20">
-        <v>-13548000</v>
+        <v>-13918000</v>
       </c>
       <c r="AF120" s="20"/>
       <c r="AG120" s="20"/>
@@ -8451,20 +8451,20 @@
         <v>46945779107</v>
       </c>
       <c r="X127" s="20">
-        <v>1590161054</v>
+        <v>1842950054</v>
       </c>
       <c r="Y127" s="20"/>
       <c r="Z127" s="20">
-        <v>48535940161</v>
+        <v>48788729161</v>
       </c>
       <c r="AA127" s="20"/>
       <c r="AB127" s="20"/>
       <c r="AC127" s="21">
-        <v>0.92701908640605513</v>
+        <v>0.93184726583466337</v>
       </c>
       <c r="AD127" s="21"/>
       <c r="AE127" s="20">
-        <v>3821061839</v>
+        <v>3568272839</v>
       </c>
       <c r="AF127" s="20"/>
       <c r="AG127" s="20"/>
@@ -10043,20 +10043,20 @@
         <v>1960479000</v>
       </c>
       <c r="X157" s="20">
-        <v>0</v>
+        <v>252789000</v>
       </c>
       <c r="Y157" s="20"/>
       <c r="Z157" s="20">
-        <v>1960479000</v>
+        <v>2213268000</v>
       </c>
       <c r="AA157" s="20"/>
       <c r="AB157" s="20"/>
       <c r="AC157" s="21">
-        <v>0.75977663374072213</v>
+        <v>0.8577441077441077</v>
       </c>
       <c r="AD157" s="21"/>
       <c r="AE157" s="20">
-        <v>619857000</v>
+        <v>367068000</v>
       </c>
       <c r="AF157" s="20"/>
       <c r="AG157" s="20"/>
@@ -10096,20 +10096,20 @@
         <v>174930000</v>
       </c>
       <c r="X158" s="20">
-        <v>0</v>
+        <v>24010000</v>
       </c>
       <c r="Y158" s="20"/>
       <c r="Z158" s="20">
-        <v>174930000</v>
+        <v>198940000</v>
       </c>
       <c r="AA158" s="20"/>
       <c r="AB158" s="20"/>
       <c r="AC158" s="21">
-        <v>0.68055555555555558</v>
+        <v>0.77396514161220042</v>
       </c>
       <c r="AD158" s="21"/>
       <c r="AE158" s="20">
-        <v>82110000</v>
+        <v>58100000</v>
       </c>
       <c r="AF158" s="20"/>
       <c r="AG158" s="20"/>
@@ -10149,20 +10149,20 @@
         <v>1398304000</v>
       </c>
       <c r="X159" s="20">
-        <v>0</v>
+        <v>183187000</v>
       </c>
       <c r="Y159" s="20"/>
       <c r="Z159" s="20">
-        <v>1398304000</v>
+        <v>1581491000</v>
       </c>
       <c r="AA159" s="20"/>
       <c r="AB159" s="20"/>
       <c r="AC159" s="21">
-        <v>0.78812145478812146</v>
+        <v>0.89137053720387049</v>
       </c>
       <c r="AD159" s="21"/>
       <c r="AE159" s="20">
-        <v>375920000</v>
+        <v>192733000</v>
       </c>
       <c r="AF159" s="20"/>
       <c r="AG159" s="20"/>
@@ -10202,20 +10202,20 @@
         <v>387245000</v>
       </c>
       <c r="X160" s="20">
-        <v>0</v>
+        <v>45592000</v>
       </c>
       <c r="Y160" s="20"/>
       <c r="Z160" s="20">
-        <v>387245000</v>
+        <v>432837000</v>
       </c>
       <c r="AA160" s="20"/>
       <c r="AB160" s="20"/>
       <c r="AC160" s="21">
-        <v>0.70527180406212664</v>
+        <v>0.78830645161290325</v>
       </c>
       <c r="AD160" s="21"/>
       <c r="AE160" s="20">
-        <v>161827000</v>
+        <v>116235000</v>
       </c>
       <c r="AF160" s="20"/>
       <c r="AG160" s="20"/>
@@ -10685,20 +10685,20 @@
         <v>18441056518</v>
       </c>
       <c r="X169" s="20">
-        <v>0</v>
+        <v>1390204720</v>
       </c>
       <c r="Y169" s="20"/>
       <c r="Z169" s="20">
-        <v>18441056518</v>
+        <v>19831261238</v>
       </c>
       <c r="AA169" s="20"/>
       <c r="AB169" s="20"/>
       <c r="AC169" s="21">
-        <v>1.1877562816083513</v>
+        <v>1.2772969425401071</v>
       </c>
       <c r="AD169" s="21"/>
       <c r="AE169" s="20">
-        <v>-2915096518</v>
+        <v>-4305301238</v>
       </c>
       <c r="AF169" s="20"/>
       <c r="AG169" s="20"/>
@@ -10740,20 +10740,20 @@
         <v>6960502066</v>
       </c>
       <c r="X170" s="20">
-        <v>0</v>
+        <v>1060348000</v>
       </c>
       <c r="Y170" s="20"/>
       <c r="Z170" s="20">
-        <v>6960502066</v>
+        <v>8020850066</v>
       </c>
       <c r="AA170" s="20"/>
       <c r="AB170" s="20"/>
       <c r="AC170" s="21">
-        <v>1.5592850893365586</v>
+        <v>1.7968232453819593</v>
       </c>
       <c r="AD170" s="21"/>
       <c r="AE170" s="20">
-        <v>-2496596066</v>
+        <v>-3556944066</v>
       </c>
       <c r="AF170" s="20"/>
       <c r="AG170" s="20"/>
@@ -10793,20 +10793,20 @@
         <v>5871388400</v>
       </c>
       <c r="X171" s="20">
-        <v>0</v>
+        <v>1060348000</v>
       </c>
       <c r="Y171" s="20"/>
       <c r="Z171" s="20">
-        <v>5871388400</v>
+        <v>6931736400</v>
       </c>
       <c r="AA171" s="20"/>
       <c r="AB171" s="20"/>
       <c r="AC171" s="21">
-        <v>1.7397819830839545</v>
+        <v>2.0539792768959435</v>
       </c>
       <c r="AD171" s="21"/>
       <c r="AE171" s="20">
-        <v>-2496604400</v>
+        <v>-3556952400</v>
       </c>
       <c r="AF171" s="20"/>
       <c r="AG171" s="20"/>
@@ -10993,20 +10993,20 @@
         <v>131546</v>
       </c>
       <c r="X175" s="20">
-        <v>0</v>
+        <v>5920</v>
       </c>
       <c r="Y175" s="20"/>
       <c r="Z175" s="20">
-        <v>131546</v>
+        <v>137466</v>
       </c>
       <c r="AA175" s="20"/>
       <c r="AB175" s="20"/>
       <c r="AC175" s="21">
-        <v>0.83256962025316461</v>
+        <v>0.87003797468354427</v>
       </c>
       <c r="AD175" s="21"/>
       <c r="AE175" s="20">
-        <v>26454</v>
+        <v>20534</v>
       </c>
       <c r="AF175" s="20"/>
       <c r="AG175" s="20"/>
@@ -11046,20 +11046,20 @@
         <v>118426</v>
       </c>
       <c r="X176" s="20">
-        <v>0</v>
+        <v>5920</v>
       </c>
       <c r="Y176" s="20"/>
       <c r="Z176" s="20">
-        <v>118426</v>
+        <v>124346</v>
       </c>
       <c r="AA176" s="20"/>
       <c r="AB176" s="20"/>
       <c r="AC176" s="21">
-        <v>0.82240277777777782</v>
+        <v>0.86351388888888891</v>
       </c>
       <c r="AD176" s="21"/>
       <c r="AE176" s="20">
-        <v>25574</v>
+        <v>19654</v>
       </c>
       <c r="AF176" s="20"/>
       <c r="AG176" s="20"/>
@@ -11207,20 +11207,20 @@
         <v>473036570</v>
       </c>
       <c r="X179" s="20">
-        <v>0</v>
+        <v>70065440</v>
       </c>
       <c r="Y179" s="20"/>
       <c r="Z179" s="20">
-        <v>473036570</v>
+        <v>543102010</v>
       </c>
       <c r="AA179" s="20"/>
       <c r="AB179" s="20"/>
       <c r="AC179" s="21">
-        <v>1.310111087723574</v>
+        <v>1.5041627015559482</v>
       </c>
       <c r="AD179" s="21"/>
       <c r="AE179" s="20">
-        <v>-111970570</v>
+        <v>-182036010</v>
       </c>
       <c r="AF179" s="20"/>
       <c r="AG179" s="20"/>
@@ -11260,20 +11260,20 @@
         <v>399311800</v>
       </c>
       <c r="X180" s="20">
-        <v>0</v>
+        <v>70065440</v>
       </c>
       <c r="Y180" s="20"/>
       <c r="Z180" s="20">
-        <v>399311800</v>
+        <v>469377240</v>
       </c>
       <c r="AA180" s="20"/>
       <c r="AB180" s="20"/>
       <c r="AC180" s="21">
-        <v>1.3896839980510893</v>
+        <v>1.6335255794529129</v>
       </c>
       <c r="AD180" s="21"/>
       <c r="AE180" s="20">
-        <v>-111971800</v>
+        <v>-182037240</v>
       </c>
       <c r="AF180" s="20"/>
       <c r="AG180" s="20"/>
@@ -11421,20 +11421,20 @@
         <v>141009928</v>
       </c>
       <c r="X183" s="20">
-        <v>0</v>
+        <v>20735760</v>
       </c>
       <c r="Y183" s="20"/>
       <c r="Z183" s="20">
-        <v>141009928</v>
+        <v>161745688</v>
       </c>
       <c r="AA183" s="20"/>
       <c r="AB183" s="20"/>
       <c r="AC183" s="21">
-        <v>1.2582532747974444</v>
+        <v>1.4432816504265267</v>
       </c>
       <c r="AD183" s="21"/>
       <c r="AE183" s="20">
-        <v>-28941928</v>
+        <v>-49677688</v>
       </c>
       <c r="AF183" s="20"/>
       <c r="AG183" s="20"/>
@@ -11474,20 +11474,20 @@
         <v>119127344</v>
       </c>
       <c r="X184" s="20">
-        <v>0</v>
+        <v>20735760</v>
       </c>
       <c r="Y184" s="20"/>
       <c r="Z184" s="20">
-        <v>119127344</v>
+        <v>139863104</v>
       </c>
       <c r="AA184" s="20"/>
       <c r="AB184" s="20"/>
       <c r="AC184" s="21">
-        <v>1.3209951652251053</v>
+        <v>1.5509326236416057</v>
       </c>
       <c r="AD184" s="21"/>
       <c r="AE184" s="20">
-        <v>-28947344</v>
+        <v>-49683104</v>
       </c>
       <c r="AF184" s="20"/>
       <c r="AG184" s="20"/>
@@ -11635,20 +11635,20 @@
         <v>1133130000</v>
       </c>
       <c r="X187" s="20">
-        <v>0</v>
+        <v>175320000</v>
       </c>
       <c r="Y187" s="20"/>
       <c r="Z187" s="20">
-        <v>1133130000</v>
+        <v>1308450000</v>
       </c>
       <c r="AA187" s="20"/>
       <c r="AB187" s="20"/>
       <c r="AC187" s="21">
-        <v>1.2616407241632708</v>
+        <v>1.4568441445654352</v>
       </c>
       <c r="AD187" s="21"/>
       <c r="AE187" s="20">
-        <v>-234990000</v>
+        <v>-410310000</v>
       </c>
       <c r="AF187" s="20"/>
       <c r="AG187" s="20"/>
@@ -11688,20 +11688,20 @@
         <v>955320000</v>
       </c>
       <c r="X188" s="20">
-        <v>0</v>
+        <v>175320000</v>
       </c>
       <c r="Y188" s="20"/>
       <c r="Z188" s="20">
-        <v>955320000</v>
+        <v>1130640000</v>
       </c>
       <c r="AA188" s="20"/>
       <c r="AB188" s="20"/>
       <c r="AC188" s="21">
-        <v>1.32623652689623</v>
+        <v>1.5696270011828011</v>
       </c>
       <c r="AD188" s="21"/>
       <c r="AE188" s="20">
-        <v>-234996000</v>
+        <v>-410316000</v>
       </c>
       <c r="AF188" s="20"/>
       <c r="AG188" s="20"/>
@@ -11849,20 +11849,20 @@
         <v>425745110</v>
       </c>
       <c r="X191" s="20">
-        <v>0</v>
+        <v>63729600</v>
       </c>
       <c r="Y191" s="20"/>
       <c r="Z191" s="20">
-        <v>425745110</v>
+        <v>489474710</v>
       </c>
       <c r="AA191" s="20"/>
       <c r="AB191" s="20"/>
       <c r="AC191" s="21">
-        <v>1.2872190005684085</v>
+        <v>1.4799022518654685</v>
       </c>
       <c r="AD191" s="21"/>
       <c r="AE191" s="20">
-        <v>-94997110</v>
+        <v>-158726710</v>
       </c>
       <c r="AF191" s="20"/>
       <c r="AG191" s="20"/>
@@ -11902,20 +11902,20 @@
         <v>359203200</v>
       </c>
       <c r="X192" s="20">
-        <v>0</v>
+        <v>63729600</v>
       </c>
       <c r="Y192" s="20"/>
       <c r="Z192" s="20">
-        <v>359203200</v>
+        <v>422932800</v>
       </c>
       <c r="AA192" s="20"/>
       <c r="AB192" s="20"/>
       <c r="AC192" s="21">
-        <v>1.3595676068492528</v>
+        <v>1.6007812145160558</v>
       </c>
       <c r="AD192" s="21"/>
       <c r="AE192" s="20">
-        <v>-94999200</v>
+        <v>-158728800</v>
       </c>
       <c r="AF192" s="20"/>
       <c r="AG192" s="20"/>
@@ -12477,20 +12477,20 @@
         <v>5917998846</v>
       </c>
       <c r="X203" s="31">
-        <v>9448320</v>
+        <v>83303901</v>
       </c>
       <c r="Y203" s="31"/>
       <c r="Z203" s="31">
-        <v>5927447166</v>
+        <v>6001302747</v>
       </c>
       <c r="AA203" s="31"/>
       <c r="AB203" s="31"/>
       <c r="AC203" s="32">
-        <v>0.8888986280621537</v>
+        <v>0.89997424337968945</v>
       </c>
       <c r="AD203" s="32"/>
       <c r="AE203" s="31">
-        <v>740857834</v>
+        <v>667002253</v>
       </c>
       <c r="AF203" s="31"/>
       <c r="AG203" s="31"/>
@@ -12532,20 +12532,20 @@
         <v>4659213091</v>
       </c>
       <c r="X204" s="20">
-        <v>0</v>
+        <v>23400000</v>
       </c>
       <c r="Y204" s="20"/>
       <c r="Z204" s="20">
-        <v>4659213091</v>
+        <v>4682613091</v>
       </c>
       <c r="AA204" s="20"/>
       <c r="AB204" s="20"/>
       <c r="AC204" s="21">
-        <v>0.94518676494752918</v>
+        <v>0.94993378335338308</v>
       </c>
       <c r="AD204" s="21"/>
       <c r="AE204" s="20">
-        <v>270196909</v>
+        <v>246796909</v>
       </c>
       <c r="AF204" s="20"/>
       <c r="AG204" s="20"/>
@@ -12587,20 +12587,20 @@
         <v>1700954357</v>
       </c>
       <c r="X205" s="20">
-        <v>0</v>
+        <v>23400000</v>
       </c>
       <c r="Y205" s="20"/>
       <c r="Z205" s="20">
-        <v>1700954357</v>
+        <v>1724354357</v>
       </c>
       <c r="AA205" s="20"/>
       <c r="AB205" s="20"/>
       <c r="AC205" s="21">
-        <v>0.92320896562541899</v>
+        <v>0.93590953557706447</v>
       </c>
       <c r="AD205" s="21"/>
       <c r="AE205" s="20">
-        <v>141482643</v>
+        <v>118082643</v>
       </c>
       <c r="AF205" s="20"/>
       <c r="AG205" s="20"/>
@@ -13011,20 +13011,20 @@
         <v>0</v>
       </c>
       <c r="X213" s="20">
-        <v>0</v>
+        <v>23400000</v>
       </c>
       <c r="Y213" s="20"/>
       <c r="Z213" s="20">
-        <v>0</v>
+        <v>23400000</v>
       </c>
       <c r="AA213" s="20"/>
       <c r="AB213" s="20"/>
       <c r="AC213" s="21">
-        <v>0</v>
+        <v>0.2988505747126437</v>
       </c>
       <c r="AD213" s="21"/>
       <c r="AE213" s="20">
-        <v>78300000</v>
+        <v>54900000</v>
       </c>
       <c r="AF213" s="20"/>
       <c r="AG213" s="20"/>
@@ -14014,20 +14014,20 @@
         <v>587220368</v>
       </c>
       <c r="X232" s="20">
-        <v>0</v>
+        <v>50455581</v>
       </c>
       <c r="Y232" s="20"/>
       <c r="Z232" s="20">
-        <v>587220368</v>
+        <v>637675949</v>
       </c>
       <c r="AA232" s="20"/>
       <c r="AB232" s="20"/>
       <c r="AC232" s="21">
-        <v>0.69355644163084051</v>
+        <v>0.75314870907544762</v>
       </c>
       <c r="AD232" s="21"/>
       <c r="AE232" s="20">
-        <v>259459632</v>
+        <v>209004051</v>
       </c>
       <c r="AF232" s="20"/>
       <c r="AG232" s="20"/>
@@ -14069,20 +14069,20 @@
         <v>430266392</v>
       </c>
       <c r="X233" s="20">
-        <v>0</v>
+        <v>40247519</v>
       </c>
       <c r="Y233" s="20"/>
       <c r="Z233" s="20">
-        <v>430266392</v>
+        <v>470513911</v>
       </c>
       <c r="AA233" s="20"/>
       <c r="AB233" s="20"/>
       <c r="AC233" s="21">
-        <v>0.66658361529404475</v>
+        <v>0.72893646743508711</v>
       </c>
       <c r="AD233" s="21"/>
       <c r="AE233" s="20">
-        <v>215213608</v>
+        <v>174966089</v>
       </c>
       <c r="AF233" s="20"/>
       <c r="AG233" s="20"/>
@@ -14122,20 +14122,20 @@
         <v>430266392</v>
       </c>
       <c r="X234" s="20">
-        <v>0</v>
+        <v>40247519</v>
       </c>
       <c r="Y234" s="20"/>
       <c r="Z234" s="20">
-        <v>430266392</v>
+        <v>470513911</v>
       </c>
       <c r="AA234" s="20"/>
       <c r="AB234" s="20"/>
       <c r="AC234" s="21">
-        <v>0.66658361529404475</v>
+        <v>0.72893646743508711</v>
       </c>
       <c r="AD234" s="21"/>
       <c r="AE234" s="20">
-        <v>215213608</v>
+        <v>174966089</v>
       </c>
       <c r="AF234" s="20"/>
       <c r="AG234" s="20"/>
@@ -14177,20 +14177,20 @@
         <v>5219220</v>
       </c>
       <c r="X235" s="20">
-        <v>0</v>
+        <v>266012</v>
       </c>
       <c r="Y235" s="20"/>
       <c r="Z235" s="20">
-        <v>5219220</v>
+        <v>5485232</v>
       </c>
       <c r="AA235" s="20"/>
       <c r="AB235" s="20"/>
       <c r="AC235" s="21">
-        <v>0.86987000000000003</v>
+        <v>0.91420533333333331</v>
       </c>
       <c r="AD235" s="21"/>
       <c r="AE235" s="20">
-        <v>780780</v>
+        <v>514768</v>
       </c>
       <c r="AF235" s="20"/>
       <c r="AG235" s="20"/>
@@ -14230,20 +14230,20 @@
         <v>5219220</v>
       </c>
       <c r="X236" s="20">
-        <v>0</v>
+        <v>266012</v>
       </c>
       <c r="Y236" s="20"/>
       <c r="Z236" s="20">
-        <v>5219220</v>
+        <v>5485232</v>
       </c>
       <c r="AA236" s="20"/>
       <c r="AB236" s="20"/>
       <c r="AC236" s="21">
-        <v>0.86987000000000003</v>
+        <v>0.91420533333333331</v>
       </c>
       <c r="AD236" s="21"/>
       <c r="AE236" s="20">
-        <v>780780</v>
+        <v>514768</v>
       </c>
       <c r="AF236" s="20"/>
       <c r="AG236" s="20"/>
@@ -14285,20 +14285,20 @@
         <v>29408400</v>
       </c>
       <c r="X237" s="20">
-        <v>0</v>
+        <v>691300</v>
       </c>
       <c r="Y237" s="20"/>
       <c r="Z237" s="20">
-        <v>29408400</v>
+        <v>30099700</v>
       </c>
       <c r="AA237" s="20"/>
       <c r="AB237" s="20"/>
       <c r="AC237" s="21">
-        <v>0.74263636363636365</v>
+        <v>0.76009343434343435</v>
       </c>
       <c r="AD237" s="21"/>
       <c r="AE237" s="20">
-        <v>10191600</v>
+        <v>9500300</v>
       </c>
       <c r="AF237" s="20"/>
       <c r="AG237" s="20"/>
@@ -14338,20 +14338,20 @@
         <v>29408400</v>
       </c>
       <c r="X238" s="20">
-        <v>0</v>
+        <v>691300</v>
       </c>
       <c r="Y238" s="20"/>
       <c r="Z238" s="20">
-        <v>29408400</v>
+        <v>30099700</v>
       </c>
       <c r="AA238" s="20"/>
       <c r="AB238" s="20"/>
       <c r="AC238" s="21">
-        <v>0.74263636363636365</v>
+        <v>0.76009343434343435</v>
       </c>
       <c r="AD238" s="21"/>
       <c r="AE238" s="20">
-        <v>10191600</v>
+        <v>9500300</v>
       </c>
       <c r="AF238" s="20"/>
       <c r="AG238" s="20"/>
@@ -14393,20 +14393,20 @@
         <v>122326356</v>
       </c>
       <c r="X239" s="20">
-        <v>0</v>
+        <v>9250750</v>
       </c>
       <c r="Y239" s="20"/>
       <c r="Z239" s="20">
-        <v>122326356</v>
+        <v>131577106</v>
       </c>
       <c r="AA239" s="20"/>
       <c r="AB239" s="20"/>
       <c r="AC239" s="21">
-        <v>0.78615910025706937</v>
+        <v>0.84561122107969156</v>
       </c>
       <c r="AD239" s="21"/>
       <c r="AE239" s="20">
-        <v>33273644</v>
+        <v>24022894</v>
       </c>
       <c r="AF239" s="20"/>
       <c r="AG239" s="20"/>
@@ -14446,20 +14446,20 @@
         <v>95184750</v>
       </c>
       <c r="X240" s="20">
-        <v>0</v>
+        <v>9250750</v>
       </c>
       <c r="Y240" s="20"/>
       <c r="Z240" s="20">
-        <v>95184750</v>
+        <v>104435500</v>
       </c>
       <c r="AA240" s="20"/>
       <c r="AB240" s="20"/>
       <c r="AC240" s="21">
-        <v>0.75007683215130028</v>
+        <v>0.82297478329393225</v>
       </c>
       <c r="AD240" s="21"/>
       <c r="AE240" s="20">
-        <v>31715250</v>
+        <v>22464500</v>
       </c>
       <c r="AF240" s="20"/>
       <c r="AG240" s="20"/>

</xml_diff>

<commit_message>
UP DATE REALISASI 24 NOV PKL 10
UP DATE REALISASI 24 NOV PKL 10
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B8BD4D9-BA9A-4AD3-9B9F-B8C4D70ADE32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B726F07-E42D-4E5A-81B2-FC7DCC3C45A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="600" windowWidth="14925" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="135" yWindow="165" windowWidth="14925" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GLP039_LAPORAN REALISASI SUPER " sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update realisasi per 4 Des pkl 9
Update realisasi per 4 Des pkl 9
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>9.0559784495E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>0.0</v>
+        <v>6.42836618E8</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>9.0559784495E10</v>
+        <v>9.1202621113E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.9056337261582303</v>
+        <v>0.9120623470401897</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>9.436253505E9</v>
+        <v>8.793416887E9</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>0.0</v>
+        <v>6.42836618E8</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>8.6526416455E10</v>
+        <v>8.7169253073E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.9016677558926631</v>
+        <v>0.9083665777612324</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>9.436221545E9</v>
+        <v>8.793384927E9</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>0.0</v>
+        <v>6.42836618E8</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>8.6526416455E10</v>
+        <v>8.7169253073E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.9016677558926631</v>
+        <v>0.9083665777612324</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>9.436221545E9</v>
+        <v>8.793384927E9</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>8.6525816455E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>0.0</v>
+        <v>6.42836618E8</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>8.6525816455E10</v>
+        <v>8.7168653073E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.9016671410730147</v>
+        <v>0.9083660048257833</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>9.436221545E9</v>
+        <v>8.793384927E9</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>8.6508305403E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>0.0</v>
+        <v>6.42836618E8</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>8.6508305403E10</v>
+        <v>8.7151142021E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.9016587698982197</v>
+        <v>0.9083589274325887</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>9.435202597E9</v>
+        <v>8.792365979E9</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3296,20 +3296,20 @@
         <v>8.0279551347E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>0.0</v>
+        <v>5.189E8</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
-        <v>8.0279551347E10</v>
+        <v>8.0798451347E10</v>
       </c>
       <c r="AA47" s="25" t="inlineStr"/>
       <c r="AB47" s="25" t="inlineStr"/>
       <c r="AC47" s="26" t="n">
-        <v>0.9020506445726097</v>
+        <v>0.9078811963334875</v>
       </c>
       <c r="AD47" s="26" t="inlineStr"/>
       <c r="AE47" s="25" t="n">
-        <v>8.717171653E9</v>
+        <v>8.198271653E9</v>
       </c>
       <c r="AF47" s="25" t="inlineStr"/>
       <c r="AG47" s="25" t="inlineStr"/>
@@ -3359,20 +3359,20 @@
         <v>5.831238104E9</v>
       </c>
       <c r="X48" s="14" t="n">
-        <v>0.0</v>
+        <v>2.8323E7</v>
       </c>
       <c r="Y48" s="14" t="inlineStr"/>
       <c r="Z48" s="14" t="n">
-        <v>5.831238104E9</v>
+        <v>5.859561104E9</v>
       </c>
       <c r="AA48" s="14" t="inlineStr"/>
       <c r="AB48" s="14" t="inlineStr"/>
       <c r="AC48" s="15" t="n">
-        <v>0.981210213727161</v>
+        <v>0.9859760655733292</v>
       </c>
       <c r="AD48" s="15" t="inlineStr"/>
       <c r="AE48" s="14" t="n">
-        <v>1.11665896E8</v>
+        <v>8.3342896E7</v>
       </c>
       <c r="AF48" s="14" t="inlineStr"/>
       <c r="AG48" s="14" t="inlineStr"/>
@@ -5337,20 +5337,20 @@
         <v>2.77741E8</v>
       </c>
       <c r="X82" s="14" t="n">
-        <v>0.0</v>
+        <v>2.8323E7</v>
       </c>
       <c r="Y82" s="14" t="inlineStr"/>
       <c r="Z82" s="14" t="n">
-        <v>2.77741E8</v>
+        <v>3.06064E8</v>
       </c>
       <c r="AA82" s="14" t="inlineStr"/>
       <c r="AB82" s="14" t="inlineStr"/>
       <c r="AC82" s="15" t="n">
-        <v>0.7699628520736305</v>
+        <v>0.8484808161454868</v>
       </c>
       <c r="AD82" s="15" t="inlineStr"/>
       <c r="AE82" s="14" t="n">
-        <v>8.2979E7</v>
+        <v>5.4656E7</v>
       </c>
       <c r="AF82" s="14" t="inlineStr"/>
       <c r="AG82" s="14" t="inlineStr"/>
@@ -5394,20 +5394,20 @@
         <v>1.554E7</v>
       </c>
       <c r="X83" s="14" t="n">
-        <v>0.0</v>
+        <v>1400000.0</v>
       </c>
       <c r="Y83" s="14" t="inlineStr"/>
       <c r="Z83" s="14" t="n">
-        <v>1.554E7</v>
+        <v>1.694E7</v>
       </c>
       <c r="AA83" s="14" t="inlineStr"/>
       <c r="AB83" s="14" t="inlineStr"/>
       <c r="AC83" s="15" t="n">
-        <v>0.8409090909090909</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="AD83" s="15" t="inlineStr"/>
       <c r="AE83" s="14" t="n">
-        <v>2940000.0</v>
+        <v>1540000.0</v>
       </c>
       <c r="AF83" s="14" t="inlineStr"/>
       <c r="AG83" s="14" t="inlineStr"/>
@@ -5451,20 +5451,20 @@
         <v>2.28253E8</v>
       </c>
       <c r="X84" s="14" t="n">
-        <v>0.0</v>
+        <v>2.3643E7</v>
       </c>
       <c r="Y84" s="14" t="inlineStr"/>
       <c r="Z84" s="14" t="n">
-        <v>2.28253E8</v>
+        <v>2.51896E8</v>
       </c>
       <c r="AA84" s="14" t="inlineStr"/>
       <c r="AB84" s="14" t="inlineStr"/>
       <c r="AC84" s="15" t="n">
-        <v>0.7789141414141414</v>
+        <v>0.8595959595959596</v>
       </c>
       <c r="AD84" s="15" t="inlineStr"/>
       <c r="AE84" s="14" t="n">
-        <v>6.4787E7</v>
+        <v>4.1144E7</v>
       </c>
       <c r="AF84" s="14" t="inlineStr"/>
       <c r="AG84" s="14" t="inlineStr"/>
@@ -5508,20 +5508,20 @@
         <v>3.3948E7</v>
       </c>
       <c r="X85" s="14" t="n">
-        <v>0.0</v>
+        <v>3280000.0</v>
       </c>
       <c r="Y85" s="14" t="inlineStr"/>
       <c r="Z85" s="14" t="n">
-        <v>3.3948E7</v>
+        <v>3.7228E7</v>
       </c>
       <c r="AA85" s="14" t="inlineStr"/>
       <c r="AB85" s="14" t="inlineStr"/>
       <c r="AC85" s="15" t="n">
-        <v>0.69</v>
+        <v>0.7566666666666667</v>
       </c>
       <c r="AD85" s="15" t="inlineStr"/>
       <c r="AE85" s="14" t="n">
-        <v>1.5252E7</v>
+        <v>1.1972E7</v>
       </c>
       <c r="AF85" s="14" t="inlineStr"/>
       <c r="AG85" s="14" t="inlineStr"/>
@@ -6082,20 +6082,20 @@
         <v>5.93914035E8</v>
       </c>
       <c r="X95" s="14" t="n">
-        <v>0.0</v>
+        <v>2.694E7</v>
       </c>
       <c r="Y95" s="14" t="inlineStr"/>
       <c r="Z95" s="14" t="n">
-        <v>5.93914035E8</v>
+        <v>6.20854035E8</v>
       </c>
       <c r="AA95" s="14" t="inlineStr"/>
       <c r="AB95" s="14" t="inlineStr"/>
       <c r="AC95" s="15" t="n">
-        <v>0.6139331677334524</v>
+        <v>0.6417812375955145</v>
       </c>
       <c r="AD95" s="15" t="inlineStr"/>
       <c r="AE95" s="14" t="n">
-        <v>3.73477965E8</v>
+        <v>3.46537965E8</v>
       </c>
       <c r="AF95" s="14" t="inlineStr"/>
       <c r="AG95" s="14" t="inlineStr"/>
@@ -6745,20 +6745,20 @@
         <v>3.0833E7</v>
       </c>
       <c r="X106" s="14" t="n">
-        <v>0.0</v>
+        <v>2.694E7</v>
       </c>
       <c r="Y106" s="14" t="inlineStr"/>
       <c r="Z106" s="14" t="n">
-        <v>3.0833E7</v>
+        <v>5.7773E7</v>
       </c>
       <c r="AA106" s="14" t="inlineStr"/>
       <c r="AB106" s="14" t="inlineStr"/>
       <c r="AC106" s="15" t="n">
-        <v>0.3713029865125241</v>
+        <v>0.6957249518304431</v>
       </c>
       <c r="AD106" s="15" t="inlineStr"/>
       <c r="AE106" s="14" t="n">
-        <v>5.2207E7</v>
+        <v>2.5267E7</v>
       </c>
       <c r="AF106" s="14" t="inlineStr"/>
       <c r="AG106" s="14" t="inlineStr"/>
@@ -6802,20 +6802,20 @@
         <v>8855000.0</v>
       </c>
       <c r="X107" s="14" t="n">
-        <v>0.0</v>
+        <v>7700000.0</v>
       </c>
       <c r="Y107" s="14" t="inlineStr"/>
       <c r="Z107" s="14" t="n">
-        <v>8855000.0</v>
+        <v>1.6555E7</v>
       </c>
       <c r="AA107" s="14" t="inlineStr"/>
       <c r="AB107" s="14" t="inlineStr"/>
       <c r="AC107" s="15" t="n">
-        <v>0.38333333333333336</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="AD107" s="15" t="inlineStr"/>
       <c r="AE107" s="14" t="n">
-        <v>1.4245E7</v>
+        <v>6545000.0</v>
       </c>
       <c r="AF107" s="14" t="inlineStr"/>
       <c r="AG107" s="14" t="inlineStr"/>
@@ -6859,20 +6859,20 @@
         <v>2.1978E7</v>
       </c>
       <c r="X108" s="14" t="n">
-        <v>0.0</v>
+        <v>1.924E7</v>
       </c>
       <c r="Y108" s="14" t="inlineStr"/>
       <c r="Z108" s="14" t="n">
-        <v>2.1978E7</v>
+        <v>4.1218E7</v>
       </c>
       <c r="AA108" s="14" t="inlineStr"/>
       <c r="AB108" s="14" t="inlineStr"/>
       <c r="AC108" s="15" t="n">
-        <v>0.36666666666666664</v>
+        <v>0.6876543209876543</v>
       </c>
       <c r="AD108" s="15" t="inlineStr"/>
       <c r="AE108" s="14" t="n">
-        <v>3.7962E7</v>
+        <v>1.8722E7</v>
       </c>
       <c r="AF108" s="14" t="inlineStr"/>
       <c r="AG108" s="14" t="inlineStr"/>
@@ -7162,20 +7162,20 @@
         <v>5.0689888E10</v>
       </c>
       <c r="X113" s="14" t="n">
-        <v>0.0</v>
+        <v>2.18452E8</v>
       </c>
       <c r="Y113" s="14" t="inlineStr"/>
       <c r="Z113" s="14" t="n">
-        <v>5.0689888E10</v>
+        <v>5.090834E10</v>
       </c>
       <c r="AA113" s="14" t="inlineStr"/>
       <c r="AB113" s="14" t="inlineStr"/>
       <c r="AC113" s="15" t="n">
-        <v>0.9193436738595991</v>
+        <v>0.9233056566566804</v>
       </c>
       <c r="AD113" s="15" t="inlineStr"/>
       <c r="AE113" s="14" t="n">
-        <v>4.447151E9</v>
+        <v>4.228699E9</v>
       </c>
       <c r="AF113" s="14" t="inlineStr"/>
       <c r="AG113" s="14" t="inlineStr"/>
@@ -8906,20 +8906,20 @@
         <v>2.213268E9</v>
       </c>
       <c r="X143" s="14" t="n">
-        <v>0.0</v>
+        <v>2.18452E8</v>
       </c>
       <c r="Y143" s="14" t="inlineStr"/>
       <c r="Z143" s="14" t="n">
-        <v>2.213268E9</v>
+        <v>2.43172E9</v>
       </c>
       <c r="AA143" s="14" t="inlineStr"/>
       <c r="AB143" s="14" t="inlineStr"/>
       <c r="AC143" s="15" t="n">
-        <v>0.8282097567985056</v>
+        <v>0.9099549759911868</v>
       </c>
       <c r="AD143" s="15" t="inlineStr"/>
       <c r="AE143" s="14" t="n">
-        <v>4.59084E8</v>
+        <v>2.40632E8</v>
       </c>
       <c r="AF143" s="14" t="inlineStr"/>
       <c r="AG143" s="14" t="inlineStr"/>
@@ -8963,20 +8963,20 @@
         <v>1.9894E8</v>
       </c>
       <c r="X144" s="14" t="n">
-        <v>0.0</v>
+        <v>3.0567E7</v>
       </c>
       <c r="Y144" s="14" t="inlineStr"/>
       <c r="Z144" s="14" t="n">
-        <v>1.9894E8</v>
+        <v>2.29507E8</v>
       </c>
       <c r="AA144" s="14" t="inlineStr"/>
       <c r="AB144" s="14" t="inlineStr"/>
       <c r="AC144" s="15" t="n">
-        <v>0.8166666666666667</v>
+        <v>0.9421469622331692</v>
       </c>
       <c r="AD144" s="15" t="inlineStr"/>
       <c r="AE144" s="14" t="n">
-        <v>4.466E7</v>
+        <v>1.4093E7</v>
       </c>
       <c r="AF144" s="14" t="inlineStr"/>
       <c r="AG144" s="14" t="inlineStr"/>
@@ -9063,20 +9063,20 @@
         <v>1.581491E9</v>
       </c>
       <c r="X146" s="14" t="n">
-        <v>0.0</v>
+        <v>1.59359E8</v>
       </c>
       <c r="Y146" s="14" t="inlineStr"/>
       <c r="Z146" s="14" t="n">
-        <v>1.581491E9</v>
+        <v>1.74085E9</v>
       </c>
       <c r="AA146" s="14" t="inlineStr"/>
       <c r="AB146" s="14" t="inlineStr"/>
       <c r="AC146" s="15" t="n">
-        <v>0.8283527131782946</v>
+        <v>0.9118217054263565</v>
       </c>
       <c r="AD146" s="15" t="inlineStr"/>
       <c r="AE146" s="14" t="n">
-        <v>3.27709E8</v>
+        <v>1.6835E8</v>
       </c>
       <c r="AF146" s="14" t="inlineStr"/>
       <c r="AG146" s="14" t="inlineStr"/>
@@ -9120,20 +9120,20 @@
         <v>4.32837E8</v>
       </c>
       <c r="X147" s="14" t="n">
-        <v>0.0</v>
+        <v>2.8526E7</v>
       </c>
       <c r="Y147" s="14" t="inlineStr"/>
       <c r="Z147" s="14" t="n">
-        <v>4.32837E8</v>
+        <v>4.61363E8</v>
       </c>
       <c r="AA147" s="14" t="inlineStr"/>
       <c r="AB147" s="14" t="inlineStr"/>
       <c r="AC147" s="15" t="n">
-        <v>0.8330965909090909</v>
+        <v>0.8880015859817689</v>
       </c>
       <c r="AD147" s="15" t="inlineStr"/>
       <c r="AE147" s="14" t="n">
-        <v>8.6715E7</v>
+        <v>5.8189E7</v>
       </c>
       <c r="AF147" s="14" t="inlineStr"/>
       <c r="AG147" s="14" t="inlineStr"/>
@@ -9651,20 +9651,20 @@
         <v>2.3164511208E10</v>
       </c>
       <c r="X156" s="14" t="n">
-        <v>0.0</v>
+        <v>2.45185E8</v>
       </c>
       <c r="Y156" s="14" t="inlineStr"/>
       <c r="Z156" s="14" t="n">
-        <v>2.3164511208E10</v>
+        <v>2.3409696208E10</v>
       </c>
       <c r="AA156" s="14" t="inlineStr"/>
       <c r="AB156" s="14" t="inlineStr"/>
       <c r="AC156" s="15" t="n">
-        <v>0.8595561134078443</v>
+        <v>0.8686540936662458</v>
       </c>
       <c r="AD156" s="15" t="inlineStr"/>
       <c r="AE156" s="14" t="n">
-        <v>3.784876792E9</v>
+        <v>3.539691792E9</v>
       </c>
       <c r="AF156" s="14" t="inlineStr"/>
       <c r="AG156" s="14" t="inlineStr"/>
@@ -11161,20 +11161,20 @@
         <v>1.310426E9</v>
       </c>
       <c r="X182" s="14" t="n">
-        <v>0.0</v>
+        <v>2.45185E8</v>
       </c>
       <c r="Y182" s="14" t="inlineStr"/>
       <c r="Z182" s="14" t="n">
-        <v>1.310426E9</v>
+        <v>1.555611E9</v>
       </c>
       <c r="AA182" s="14" t="inlineStr"/>
       <c r="AB182" s="14" t="inlineStr"/>
       <c r="AC182" s="15" t="n">
-        <v>0.7344778495202224</v>
+        <v>0.871901062684961</v>
       </c>
       <c r="AD182" s="15" t="inlineStr"/>
       <c r="AE182" s="14" t="n">
-        <v>4.73734E8</v>
+        <v>2.28549E8</v>
       </c>
       <c r="AF182" s="14" t="inlineStr"/>
       <c r="AG182" s="14" t="inlineStr"/>
@@ -11218,20 +11218,20 @@
         <v>1.2502E8</v>
       </c>
       <c r="X183" s="14" t="n">
-        <v>0.0</v>
+        <v>2.226E7</v>
       </c>
       <c r="Y183" s="14" t="inlineStr"/>
       <c r="Z183" s="14" t="n">
-        <v>1.2502E8</v>
+        <v>1.4728E8</v>
       </c>
       <c r="AA183" s="14" t="inlineStr"/>
       <c r="AB183" s="14" t="inlineStr"/>
       <c r="AC183" s="15" t="n">
-        <v>0.7441666666666666</v>
+        <v>0.8766666666666667</v>
       </c>
       <c r="AD183" s="15" t="inlineStr"/>
       <c r="AE183" s="14" t="n">
-        <v>4.298E7</v>
+        <v>2.072E7</v>
       </c>
       <c r="AF183" s="14" t="inlineStr"/>
       <c r="AG183" s="14" t="inlineStr"/>
@@ -11275,20 +11275,20 @@
         <v>1.185406E9</v>
       </c>
       <c r="X184" s="14" t="n">
-        <v>0.0</v>
+        <v>2.22925E8</v>
       </c>
       <c r="Y184" s="14" t="inlineStr"/>
       <c r="Z184" s="14" t="n">
-        <v>1.185406E9</v>
+        <v>1.408331E9</v>
       </c>
       <c r="AA184" s="14" t="inlineStr"/>
       <c r="AB184" s="14" t="inlineStr"/>
       <c r="AC184" s="15" t="n">
-        <v>0.7334706959706959</v>
+        <v>0.8714056776556777</v>
       </c>
       <c r="AD184" s="15" t="inlineStr"/>
       <c r="AE184" s="14" t="n">
-        <v>4.30754E8</v>
+        <v>2.07829E8</v>
       </c>
       <c r="AF184" s="14" t="inlineStr"/>
       <c r="AG184" s="14" t="inlineStr"/>
@@ -11572,20 +11572,20 @@
         <v>6.228754056E9</v>
       </c>
       <c r="X189" s="25" t="n">
-        <v>0.0</v>
+        <v>1.23936618E8</v>
       </c>
       <c r="Y189" s="25" t="inlineStr"/>
       <c r="Z189" s="25" t="n">
-        <v>6.228754056E9</v>
+        <v>6.352690674E9</v>
       </c>
       <c r="AA189" s="25" t="inlineStr"/>
       <c r="AB189" s="25" t="inlineStr"/>
       <c r="AC189" s="26" t="n">
-        <v>0.8966383810640461</v>
+        <v>0.9144792409726226</v>
       </c>
       <c r="AD189" s="26" t="inlineStr"/>
       <c r="AE189" s="25" t="n">
-        <v>7.18030944E8</v>
+        <v>5.94094326E8</v>
       </c>
       <c r="AF189" s="25" t="inlineStr"/>
       <c r="AG189" s="25" t="inlineStr"/>
@@ -11635,20 +11635,20 @@
         <v>4.783558496E9</v>
       </c>
       <c r="X190" s="14" t="n">
-        <v>0.0</v>
+        <v>9.108618E7</v>
       </c>
       <c r="Y190" s="14" t="inlineStr"/>
       <c r="Z190" s="14" t="n">
-        <v>4.783558496E9</v>
+        <v>4.874644676E9</v>
       </c>
       <c r="AA190" s="14" t="inlineStr"/>
       <c r="AB190" s="14" t="inlineStr"/>
       <c r="AC190" s="15" t="n">
-        <v>0.9567038542283953</v>
+        <v>0.9749209408482851</v>
       </c>
       <c r="AD190" s="15" t="inlineStr"/>
       <c r="AE190" s="14" t="n">
-        <v>2.16482504E8</v>
+        <v>1.25396324E8</v>
       </c>
       <c r="AF190" s="14" t="inlineStr"/>
       <c r="AG190" s="14" t="inlineStr"/>
@@ -11698,20 +11698,20 @@
         <v>1.777909494E9</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>0.0</v>
+        <v>5.2653912E7</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
-        <v>1.777909494E9</v>
+        <v>1.830563406E9</v>
       </c>
       <c r="AA191" s="14" t="inlineStr"/>
       <c r="AB191" s="14" t="inlineStr"/>
       <c r="AC191" s="15" t="n">
-        <v>0.9402863915439728</v>
+        <v>0.9681335666011042</v>
       </c>
       <c r="AD191" s="15" t="inlineStr"/>
       <c r="AE191" s="14" t="n">
-        <v>1.12907506E8</v>
+        <v>6.0253594E7</v>
       </c>
       <c r="AF191" s="14" t="inlineStr"/>
       <c r="AG191" s="14" t="inlineStr"/>
@@ -11869,20 +11869,20 @@
         <v>5.5184254E7</v>
       </c>
       <c r="X194" s="14" t="n">
-        <v>0.0</v>
+        <v>3953112.0</v>
       </c>
       <c r="Y194" s="14" t="inlineStr"/>
       <c r="Z194" s="14" t="n">
-        <v>5.5184254E7</v>
+        <v>5.9137366E7</v>
       </c>
       <c r="AA194" s="14" t="inlineStr"/>
       <c r="AB194" s="14" t="inlineStr"/>
       <c r="AC194" s="15" t="n">
-        <v>0.587504034919621</v>
+        <v>0.6295897583306718</v>
       </c>
       <c r="AD194" s="15" t="inlineStr"/>
       <c r="AE194" s="14" t="n">
-        <v>3.8745746E7</v>
+        <v>3.4792634E7</v>
       </c>
       <c r="AF194" s="14" t="inlineStr"/>
       <c r="AG194" s="14" t="inlineStr"/>
@@ -12154,20 +12154,20 @@
         <v>4.87008E7</v>
       </c>
       <c r="X199" s="14" t="n">
-        <v>0.0</v>
+        <v>4.87008E7</v>
       </c>
       <c r="Y199" s="14" t="inlineStr"/>
       <c r="Z199" s="14" t="n">
-        <v>4.87008E7</v>
+        <v>9.74016E7</v>
       </c>
       <c r="AA199" s="14" t="inlineStr"/>
       <c r="AB199" s="14" t="inlineStr"/>
       <c r="AC199" s="15" t="n">
-        <v>0.48970135746606336</v>
+        <v>0.9794027149321267</v>
       </c>
       <c r="AD199" s="15" t="inlineStr"/>
       <c r="AE199" s="14" t="n">
-        <v>5.07492E7</v>
+        <v>2048400.0</v>
       </c>
       <c r="AF199" s="14" t="inlineStr"/>
       <c r="AG199" s="14" t="inlineStr"/>
@@ -12317,20 +12317,20 @@
         <v>9417000.0</v>
       </c>
       <c r="X202" s="14" t="n">
-        <v>0.0</v>
+        <v>1380500.0</v>
       </c>
       <c r="Y202" s="14" t="inlineStr"/>
       <c r="Z202" s="14" t="n">
-        <v>9417000.0</v>
+        <v>1.07975E7</v>
       </c>
       <c r="AA202" s="14" t="inlineStr"/>
       <c r="AB202" s="14" t="inlineStr"/>
       <c r="AC202" s="15" t="n">
-        <v>0.765609756097561</v>
+        <v>0.8778455284552845</v>
       </c>
       <c r="AD202" s="15" t="inlineStr"/>
       <c r="AE202" s="14" t="n">
-        <v>2883000.0</v>
+        <v>1502500.0</v>
       </c>
       <c r="AF202" s="14" t="inlineStr"/>
       <c r="AG202" s="14" t="inlineStr"/>
@@ -12374,20 +12374,20 @@
         <v>5781000.0</v>
       </c>
       <c r="X203" s="14" t="n">
-        <v>0.0</v>
+        <v>1380500.0</v>
       </c>
       <c r="Y203" s="14" t="inlineStr"/>
       <c r="Z203" s="14" t="n">
-        <v>5781000.0</v>
+        <v>7161500.0</v>
       </c>
       <c r="AA203" s="14" t="inlineStr"/>
       <c r="AB203" s="14" t="inlineStr"/>
       <c r="AC203" s="15" t="n">
-        <v>0.7411538461538462</v>
+        <v>0.9181410256410256</v>
       </c>
       <c r="AD203" s="15" t="inlineStr"/>
       <c r="AE203" s="14" t="n">
-        <v>2019000.0</v>
+        <v>638500.0</v>
       </c>
       <c r="AF203" s="14" t="inlineStr"/>
       <c r="AG203" s="14" t="inlineStr"/>
@@ -12791,20 +12791,20 @@
         <v>2.936691192E9</v>
       </c>
       <c r="X210" s="14" t="n">
-        <v>0.0</v>
+        <v>3.7051768E7</v>
       </c>
       <c r="Y210" s="14" t="inlineStr"/>
       <c r="Z210" s="14" t="n">
-        <v>2.936691192E9</v>
+        <v>2.97374296E9</v>
       </c>
       <c r="AA210" s="14" t="inlineStr"/>
       <c r="AB210" s="14" t="inlineStr"/>
       <c r="AC210" s="15" t="n">
-        <v>0.9752016996926314</v>
+        <v>0.987505665199338</v>
       </c>
       <c r="AD210" s="15" t="inlineStr"/>
       <c r="AE210" s="14" t="n">
-        <v>7.4676808E7</v>
+        <v>3.762504E7</v>
       </c>
       <c r="AF210" s="14" t="inlineStr"/>
       <c r="AG210" s="14" t="inlineStr"/>
@@ -12905,20 +12905,20 @@
         <v>1.0331888E8</v>
       </c>
       <c r="X212" s="14" t="n">
-        <v>0.0</v>
+        <v>9468528.0</v>
       </c>
       <c r="Y212" s="14" t="inlineStr"/>
       <c r="Z212" s="14" t="n">
-        <v>1.0331888E8</v>
+        <v>1.12787408E8</v>
       </c>
       <c r="AA212" s="14" t="inlineStr"/>
       <c r="AB212" s="14" t="inlineStr"/>
       <c r="AC212" s="15" t="n">
-        <v>0.842731484502447</v>
+        <v>0.9199625448613377</v>
       </c>
       <c r="AD212" s="15" t="inlineStr"/>
       <c r="AE212" s="14" t="n">
-        <v>1.928112E7</v>
+        <v>9812592.0</v>
       </c>
       <c r="AF212" s="14" t="inlineStr"/>
       <c r="AG212" s="14" t="inlineStr"/>
@@ -13133,20 +13133,20 @@
         <v>2.2953312E7</v>
       </c>
       <c r="X216" s="14" t="n">
-        <v>0.0</v>
+        <v>2.2953312E7</v>
       </c>
       <c r="Y216" s="14" t="inlineStr"/>
       <c r="Z216" s="14" t="n">
-        <v>2.2953312E7</v>
+        <v>4.5906624E7</v>
       </c>
       <c r="AA216" s="14" t="inlineStr"/>
       <c r="AB216" s="14" t="inlineStr"/>
       <c r="AC216" s="15" t="n">
-        <v>0.33313950653120467</v>
+        <v>0.6662790130624093</v>
       </c>
       <c r="AD216" s="15" t="inlineStr"/>
       <c r="AE216" s="14" t="n">
-        <v>4.5946688E7</v>
+        <v>2.2993376E7</v>
       </c>
       <c r="AF216" s="14" t="inlineStr"/>
       <c r="AG216" s="14" t="inlineStr"/>
@@ -13190,20 +13190,20 @@
         <v>4629928.0</v>
       </c>
       <c r="X217" s="14" t="n">
-        <v>0.0</v>
+        <v>4629928.0</v>
       </c>
       <c r="Y217" s="14" t="inlineStr"/>
       <c r="Z217" s="14" t="n">
-        <v>4629928.0</v>
+        <v>9259856.0</v>
       </c>
       <c r="AA217" s="14" t="inlineStr"/>
       <c r="AB217" s="14" t="inlineStr"/>
       <c r="AC217" s="15" t="n">
-        <v>0.33332814974802016</v>
+        <v>0.6666562994960403</v>
       </c>
       <c r="AD217" s="15" t="inlineStr"/>
       <c r="AE217" s="14" t="n">
-        <v>9260072.0</v>
+        <v>4630144.0</v>
       </c>
       <c r="AF217" s="14" t="inlineStr"/>
       <c r="AG217" s="14" t="inlineStr"/>
@@ -13253,20 +13253,20 @@
         <v>6.39842407E8</v>
       </c>
       <c r="X218" s="14" t="n">
-        <v>0.0</v>
+        <v>604300.0</v>
       </c>
       <c r="Y218" s="14" t="inlineStr"/>
       <c r="Z218" s="14" t="n">
-        <v>6.39842407E8</v>
+        <v>6.40446707E8</v>
       </c>
       <c r="AA218" s="14" t="inlineStr"/>
       <c r="AB218" s="14" t="inlineStr"/>
       <c r="AC218" s="15" t="n">
-        <v>0.9138725847825591</v>
+        <v>0.9147356929431659</v>
       </c>
       <c r="AD218" s="15" t="inlineStr"/>
       <c r="AE218" s="14" t="n">
-        <v>6.0301593E7</v>
+        <v>5.9697293E7</v>
       </c>
       <c r="AF218" s="14" t="inlineStr"/>
       <c r="AG218" s="14" t="inlineStr"/>
@@ -13556,20 +13556,20 @@
         <v>3.08218E7</v>
       </c>
       <c r="X223" s="14" t="n">
-        <v>0.0</v>
+        <v>604300.0</v>
       </c>
       <c r="Y223" s="14" t="inlineStr"/>
       <c r="Z223" s="14" t="n">
-        <v>3.08218E7</v>
+        <v>3.14261E7</v>
       </c>
       <c r="AA223" s="14" t="inlineStr"/>
       <c r="AB223" s="14" t="inlineStr"/>
       <c r="AC223" s="15" t="n">
-        <v>0.9215943069010883</v>
+        <v>0.9396633177849539</v>
       </c>
       <c r="AD223" s="15" t="inlineStr"/>
       <c r="AE223" s="14" t="n">
-        <v>2622200.0</v>
+        <v>2017900.0</v>
       </c>
       <c r="AF223" s="14" t="inlineStr"/>
       <c r="AG223" s="14" t="inlineStr"/>
@@ -13613,20 +13613,20 @@
         <v>3.08218E7</v>
       </c>
       <c r="X224" s="14" t="n">
-        <v>0.0</v>
+        <v>604300.0</v>
       </c>
       <c r="Y224" s="14" t="inlineStr"/>
       <c r="Z224" s="14" t="n">
-        <v>3.08218E7</v>
+        <v>3.14261E7</v>
       </c>
       <c r="AA224" s="14" t="inlineStr"/>
       <c r="AB224" s="14" t="inlineStr"/>
       <c r="AC224" s="15" t="n">
-        <v>0.9215943069010883</v>
+        <v>0.9396633177849539</v>
       </c>
       <c r="AD224" s="15" t="inlineStr"/>
       <c r="AE224" s="14" t="n">
-        <v>2622200.0</v>
+        <v>2017900.0</v>
       </c>
       <c r="AF224" s="14" t="inlineStr"/>
       <c r="AG224" s="14" t="inlineStr"/>
@@ -13896,20 +13896,20 @@
         <v>6.74613153E8</v>
       </c>
       <c r="X229" s="14" t="n">
-        <v>0.0</v>
+        <v>3.1766138E7</v>
       </c>
       <c r="Y229" s="14" t="inlineStr"/>
       <c r="Z229" s="14" t="n">
-        <v>6.74613153E8</v>
+        <v>7.06379291E8</v>
       </c>
       <c r="AA229" s="14" t="inlineStr"/>
       <c r="AB229" s="14" t="inlineStr"/>
       <c r="AC229" s="15" t="n">
-        <v>0.6053491080562086</v>
+        <v>0.6338537454460617</v>
       </c>
       <c r="AD229" s="15" t="inlineStr"/>
       <c r="AE229" s="14" t="n">
-        <v>4.39806847E8</v>
+        <v>4.08040709E8</v>
       </c>
       <c r="AF229" s="14" t="inlineStr"/>
       <c r="AG229" s="14" t="inlineStr"/>
@@ -14256,20 +14256,20 @@
         <v>1.34221533E8</v>
       </c>
       <c r="X235" s="14" t="n">
-        <v>0.0</v>
+        <v>2.5076E7</v>
       </c>
       <c r="Y235" s="14" t="inlineStr"/>
       <c r="Z235" s="14" t="n">
-        <v>1.34221533E8</v>
+        <v>1.59297533E8</v>
       </c>
       <c r="AA235" s="14" t="inlineStr"/>
       <c r="AB235" s="14" t="inlineStr"/>
       <c r="AC235" s="15" t="n">
-        <v>0.36169536500579375</v>
+        <v>0.4292692689105069</v>
       </c>
       <c r="AD235" s="15" t="inlineStr"/>
       <c r="AE235" s="14" t="n">
-        <v>2.36868467E8</v>
+        <v>2.11792467E8</v>
       </c>
       <c r="AF235" s="14" t="inlineStr"/>
       <c r="AG235" s="14" t="inlineStr"/>
@@ -14541,20 +14541,20 @@
         <v>4421000.0</v>
       </c>
       <c r="X240" s="14" t="n">
-        <v>0.0</v>
+        <v>2.5076E7</v>
       </c>
       <c r="Y240" s="14" t="inlineStr"/>
       <c r="Z240" s="14" t="n">
-        <v>4421000.0</v>
+        <v>2.9497E7</v>
       </c>
       <c r="AA240" s="14" t="inlineStr"/>
       <c r="AB240" s="14" t="inlineStr"/>
       <c r="AC240" s="15" t="n">
-        <v>0.03296793437733035</v>
+        <v>0.2199627143922446</v>
       </c>
       <c r="AD240" s="15" t="inlineStr"/>
       <c r="AE240" s="14" t="n">
-        <v>1.29679E8</v>
+        <v>1.04603E8</v>
       </c>
       <c r="AF240" s="14" t="inlineStr"/>
       <c r="AG240" s="14" t="inlineStr"/>
@@ -15231,20 +15231,20 @@
         <v>2.11521335E8</v>
       </c>
       <c r="X252" s="14" t="n">
-        <v>0.0</v>
+        <v>6690138.0</v>
       </c>
       <c r="Y252" s="14" t="inlineStr"/>
       <c r="Z252" s="14" t="n">
-        <v>2.11521335E8</v>
+        <v>2.18211473E8</v>
       </c>
       <c r="AA252" s="14" t="inlineStr"/>
       <c r="AB252" s="14" t="inlineStr"/>
       <c r="AC252" s="15" t="n">
-        <v>0.6409737424242424</v>
+        <v>0.6612468878787878</v>
       </c>
       <c r="AD252" s="15" t="inlineStr"/>
       <c r="AE252" s="14" t="n">
-        <v>1.18478665E8</v>
+        <v>1.11788527E8</v>
       </c>
       <c r="AF252" s="14" t="inlineStr"/>
       <c r="AG252" s="14" t="inlineStr"/>
@@ -15288,20 +15288,20 @@
         <v>1.396E7</v>
       </c>
       <c r="X253" s="14" t="n">
-        <v>0.0</v>
+        <v>2890000.0</v>
       </c>
       <c r="Y253" s="14" t="inlineStr"/>
       <c r="Z253" s="14" t="n">
-        <v>1.396E7</v>
+        <v>1.685E7</v>
       </c>
       <c r="AA253" s="14" t="inlineStr"/>
       <c r="AB253" s="14" t="inlineStr"/>
       <c r="AC253" s="15" t="n">
-        <v>0.618520159503766</v>
+        <v>0.7465662383695171</v>
       </c>
       <c r="AD253" s="15" t="inlineStr"/>
       <c r="AE253" s="14" t="n">
-        <v>8610000.0</v>
+        <v>5720000.0</v>
       </c>
       <c r="AF253" s="14" t="inlineStr"/>
       <c r="AG253" s="14" t="inlineStr"/>
@@ -15502,20 +15502,20 @@
         <v>1.22043496E8</v>
       </c>
       <c r="X257" s="14" t="n">
-        <v>0.0</v>
+        <v>1490000.0</v>
       </c>
       <c r="Y257" s="14" t="inlineStr"/>
       <c r="Z257" s="14" t="n">
-        <v>1.22043496E8</v>
+        <v>1.23533496E8</v>
       </c>
       <c r="AA257" s="14" t="inlineStr"/>
       <c r="AB257" s="14" t="inlineStr"/>
       <c r="AC257" s="15" t="n">
-        <v>0.7189602120765832</v>
+        <v>0.7277378262150221</v>
       </c>
       <c r="AD257" s="15" t="inlineStr"/>
       <c r="AE257" s="14" t="n">
-        <v>4.7706504E7</v>
+        <v>4.6216504E7</v>
       </c>
       <c r="AF257" s="14" t="inlineStr"/>
       <c r="AG257" s="14" t="inlineStr"/>
@@ -15901,20 +15901,20 @@
         <v>3760846.0</v>
       </c>
       <c r="X264" s="14" t="n">
-        <v>0.0</v>
+        <v>1560138.0</v>
       </c>
       <c r="Y264" s="14" t="inlineStr"/>
       <c r="Z264" s="14" t="n">
-        <v>3760846.0</v>
+        <v>5320984.0</v>
       </c>
       <c r="AA264" s="14" t="inlineStr"/>
       <c r="AB264" s="14" t="inlineStr"/>
       <c r="AC264" s="15" t="n">
-        <v>0.24077119078104994</v>
+        <v>0.3406519846350832</v>
       </c>
       <c r="AD264" s="15" t="inlineStr"/>
       <c r="AE264" s="14" t="n">
-        <v>1.1859154E7</v>
+        <v>1.0299016E7</v>
       </c>
       <c r="AF264" s="14" t="inlineStr"/>
       <c r="AG264" s="14" t="inlineStr"/>
@@ -16129,20 +16129,20 @@
         <v>0.0</v>
       </c>
       <c r="X268" s="14" t="n">
-        <v>0.0</v>
+        <v>750000.0</v>
       </c>
       <c r="Y268" s="14" t="inlineStr"/>
       <c r="Z268" s="14" t="n">
-        <v>0.0</v>
+        <v>750000.0</v>
       </c>
       <c r="AA268" s="14" t="inlineStr"/>
       <c r="AB268" s="14" t="inlineStr"/>
       <c r="AC268" s="15" t="n">
-        <v>0.0</v>
+        <v>0.5</v>
       </c>
       <c r="AD268" s="15" t="inlineStr"/>
       <c r="AE268" s="14" t="n">
-        <v>1500000.0</v>
+        <v>750000.0</v>
       </c>
       <c r="AF268" s="14" t="inlineStr"/>
       <c r="AG268" s="14" t="inlineStr"/>
@@ -16426,20 +16426,20 @@
         <v>1.3074E8</v>
       </c>
       <c r="X273" s="14" t="n">
-        <v>0.0</v>
+        <v>480000.0</v>
       </c>
       <c r="Y273" s="14" t="inlineStr"/>
       <c r="Z273" s="14" t="n">
-        <v>1.3074E8</v>
+        <v>1.3122E8</v>
       </c>
       <c r="AA273" s="14" t="inlineStr"/>
       <c r="AB273" s="14" t="inlineStr"/>
       <c r="AC273" s="15" t="n">
-        <v>0.9891057648660917</v>
+        <v>0.9927371765773945</v>
       </c>
       <c r="AD273" s="15" t="inlineStr"/>
       <c r="AE273" s="14" t="n">
-        <v>1440000.0</v>
+        <v>960000.0</v>
       </c>
       <c r="AF273" s="14" t="inlineStr"/>
       <c r="AG273" s="14" t="inlineStr"/>
@@ -16489,20 +16489,20 @@
         <v>1.2324E8</v>
       </c>
       <c r="X274" s="14" t="n">
-        <v>0.0</v>
+        <v>480000.0</v>
       </c>
       <c r="Y274" s="14" t="inlineStr"/>
       <c r="Z274" s="14" t="n">
-        <v>1.2324E8</v>
+        <v>1.2372E8</v>
       </c>
       <c r="AA274" s="14" t="inlineStr"/>
       <c r="AB274" s="14" t="inlineStr"/>
       <c r="AC274" s="15" t="n">
-        <v>0.9884504331087585</v>
+        <v>0.9923002887391723</v>
       </c>
       <c r="AD274" s="15" t="inlineStr"/>
       <c r="AE274" s="14" t="n">
-        <v>1440000.0</v>
+        <v>960000.0</v>
       </c>
       <c r="AF274" s="14" t="inlineStr"/>
       <c r="AG274" s="14" t="inlineStr"/>
@@ -16831,20 +16831,20 @@
         <v>2700000.0</v>
       </c>
       <c r="X280" s="14" t="n">
-        <v>0.0</v>
+        <v>300000.0</v>
       </c>
       <c r="Y280" s="14" t="inlineStr"/>
       <c r="Z280" s="14" t="n">
-        <v>2700000.0</v>
+        <v>3000000.0</v>
       </c>
       <c r="AA280" s="14" t="inlineStr"/>
       <c r="AB280" s="14" t="inlineStr"/>
       <c r="AC280" s="15" t="n">
-        <v>0.75</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="AD280" s="15" t="inlineStr"/>
       <c r="AE280" s="14" t="n">
-        <v>900000.0</v>
+        <v>600000.0</v>
       </c>
       <c r="AF280" s="14" t="inlineStr"/>
       <c r="AG280" s="14" t="inlineStr"/>
@@ -16931,20 +16931,20 @@
         <v>3780000.0</v>
       </c>
       <c r="X282" s="14" t="n">
-        <v>0.0</v>
+        <v>180000.0</v>
       </c>
       <c r="Y282" s="14" t="inlineStr"/>
       <c r="Z282" s="14" t="n">
-        <v>3780000.0</v>
+        <v>3960000.0</v>
       </c>
       <c r="AA282" s="14" t="inlineStr"/>
       <c r="AB282" s="14" t="inlineStr"/>
       <c r="AC282" s="15" t="n">
-        <v>0.875</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="AD282" s="15" t="inlineStr"/>
       <c r="AE282" s="14" t="n">
-        <v>540000.0</v>
+        <v>360000.0</v>
       </c>
       <c r="AF282" s="14" t="inlineStr"/>
       <c r="AG282" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
Up date realisasi tukin nov
Up date realisasi tukin nov
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>9.0559784495E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>6.68137418E8</v>
+        <v>2.479274605E9</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>9.1227921913E10</v>
+        <v>9.30390591E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.9123153650647639</v>
+        <v>0.9304274545357487</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>8.768116087E9</v>
+        <v>6.9569789E9</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>6.68137418E8</v>
+        <v>2.479274605E9</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>8.7194553873E10</v>
+        <v>8.900569106E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.9086302303715327</v>
+        <v>0.9275035880109923</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>8.768084127E9</v>
+        <v>6.95694694E9</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>6.68137418E8</v>
+        <v>2.479274605E9</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>8.7194553873E10</v>
+        <v>8.900569106E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.9086302303715327</v>
+        <v>0.9275035880109923</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>8.768084127E9</v>
+        <v>6.95694694E9</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>8.6525816455E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>6.68137418E8</v>
+        <v>2.479274605E9</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>8.7193953873E10</v>
+        <v>8.900509106E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.9086296590845643</v>
+        <v>0.9275031347291728</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>8.768084127E9</v>
+        <v>6.95694694E9</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>8.6508305403E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>6.68137418E8</v>
+        <v>2.479274605E9</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>8.7176442821E10</v>
+        <v>8.8987580008E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.9086226326120992</v>
+        <v>0.9274997533757052</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>8.767065179E9</v>
+        <v>6.955927992E9</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3296,20 +3296,20 @@
         <v>8.0279551347E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>5.189E8</v>
+        <v>2.281636445E9</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
-        <v>8.0798451347E10</v>
+        <v>8.2561187792E10</v>
       </c>
       <c r="AA47" s="25" t="inlineStr"/>
       <c r="AB47" s="25" t="inlineStr"/>
       <c r="AC47" s="26" t="n">
-        <v>0.9078811963334875</v>
+        <v>0.9276879530946325</v>
       </c>
       <c r="AD47" s="26" t="inlineStr"/>
       <c r="AE47" s="25" t="n">
-        <v>8.198271653E9</v>
+        <v>6.435535208E9</v>
       </c>
       <c r="AF47" s="25" t="inlineStr"/>
       <c r="AG47" s="25" t="inlineStr"/>
@@ -7162,20 +7162,20 @@
         <v>5.0689888E10</v>
       </c>
       <c r="X113" s="14" t="n">
-        <v>2.18452E8</v>
+        <v>1.981188445E9</v>
       </c>
       <c r="Y113" s="14" t="inlineStr"/>
       <c r="Z113" s="14" t="n">
-        <v>5.090834E10</v>
+        <v>5.2671076445E10</v>
       </c>
       <c r="AA113" s="14" t="inlineStr"/>
       <c r="AB113" s="14" t="inlineStr"/>
       <c r="AC113" s="15" t="n">
-        <v>0.9233056566566804</v>
+        <v>0.9552757529289885</v>
       </c>
       <c r="AD113" s="15" t="inlineStr"/>
       <c r="AE113" s="14" t="n">
-        <v>4.228699E9</v>
+        <v>2.465962555E9</v>
       </c>
       <c r="AF113" s="14" t="inlineStr"/>
       <c r="AG113" s="14" t="inlineStr"/>
@@ -9417,20 +9417,20 @@
         <v>2.475555828E10</v>
       </c>
       <c r="X152" s="14" t="n">
-        <v>0.0</v>
+        <v>1.762736445E9</v>
       </c>
       <c r="Y152" s="14" t="inlineStr"/>
       <c r="Z152" s="14" t="n">
-        <v>2.475555828E10</v>
+        <v>2.6518294725E10</v>
       </c>
       <c r="AA152" s="14" t="inlineStr"/>
       <c r="AB152" s="14" t="inlineStr"/>
       <c r="AC152" s="15" t="n">
-        <v>0.8618034181440637</v>
+        <v>0.9231687194798619</v>
       </c>
       <c r="AD152" s="15" t="inlineStr"/>
       <c r="AE152" s="14" t="n">
-        <v>3.96973772E9</v>
+        <v>2.207001275E9</v>
       </c>
       <c r="AF152" s="14" t="inlineStr"/>
       <c r="AG152" s="14" t="inlineStr"/>
@@ -9474,20 +9474,20 @@
         <v>1.997827308E10</v>
       </c>
       <c r="X153" s="14" t="n">
-        <v>0.0</v>
+        <v>1.762736445E9</v>
       </c>
       <c r="Y153" s="14" t="inlineStr"/>
       <c r="Z153" s="14" t="n">
-        <v>1.997827308E10</v>
+        <v>2.1741009525E10</v>
       </c>
       <c r="AA153" s="14" t="inlineStr"/>
       <c r="AB153" s="14" t="inlineStr"/>
       <c r="AC153" s="15" t="n">
-        <v>0.8342358340523915</v>
+        <v>0.9078426919885392</v>
       </c>
       <c r="AD153" s="15" t="inlineStr"/>
       <c r="AE153" s="14" t="n">
-        <v>3.96971892E9</v>
+        <v>2.206982475E9</v>
       </c>
       <c r="AF153" s="14" t="inlineStr"/>
       <c r="AG153" s="14" t="inlineStr"/>
@@ -11572,20 +11572,20 @@
         <v>6.228754056E9</v>
       </c>
       <c r="X189" s="25" t="n">
-        <v>1.49237418E8</v>
+        <v>1.9763816E8</v>
       </c>
       <c r="Y189" s="25" t="inlineStr"/>
       <c r="Z189" s="25" t="n">
-        <v>6.377991474E9</v>
+        <v>6.426392216E9</v>
       </c>
       <c r="AA189" s="25" t="inlineStr"/>
       <c r="AB189" s="25" t="inlineStr"/>
       <c r="AC189" s="26" t="n">
-        <v>0.918121328643394</v>
+        <v>0.9250886872128617</v>
       </c>
       <c r="AD189" s="26" t="inlineStr"/>
       <c r="AE189" s="25" t="n">
-        <v>5.68793526E8</v>
+        <v>5.20392784E8</v>
       </c>
       <c r="AF189" s="25" t="inlineStr"/>
       <c r="AG189" s="25" t="inlineStr"/>
@@ -13310,20 +13310,20 @@
         <v>6.39842407E8</v>
       </c>
       <c r="X219" s="14" t="n">
-        <v>604300.0</v>
+        <v>4.9005042E7</v>
       </c>
       <c r="Y219" s="14" t="inlineStr"/>
       <c r="Z219" s="14" t="n">
-        <v>6.40446707E8</v>
+        <v>6.88847449E8</v>
       </c>
       <c r="AA219" s="14" t="inlineStr"/>
       <c r="AB219" s="14" t="inlineStr"/>
       <c r="AC219" s="15" t="n">
-        <v>0.9147356929431659</v>
+        <v>0.9838653891199525</v>
       </c>
       <c r="AD219" s="15" t="inlineStr"/>
       <c r="AE219" s="14" t="n">
-        <v>5.9697293E7</v>
+        <v>1.1296551E7</v>
       </c>
       <c r="AF219" s="14" t="inlineStr"/>
       <c r="AG219" s="14" t="inlineStr"/>
@@ -13373,20 +13373,20 @@
         <v>4.70513911E8</v>
       </c>
       <c r="X220" s="14" t="n">
-        <v>0.0</v>
+        <v>3.8886478E7</v>
       </c>
       <c r="Y220" s="14" t="inlineStr"/>
       <c r="Z220" s="14" t="n">
-        <v>4.70513911E8</v>
+        <v>5.09400389E8</v>
       </c>
       <c r="AA220" s="14" t="inlineStr"/>
       <c r="AB220" s="14" t="inlineStr"/>
       <c r="AC220" s="15" t="n">
-        <v>0.9118486647286822</v>
+        <v>0.9872100562015503</v>
       </c>
       <c r="AD220" s="15" t="inlineStr"/>
       <c r="AE220" s="14" t="n">
-        <v>4.5486089E7</v>
+        <v>6599611.0</v>
       </c>
       <c r="AF220" s="14" t="inlineStr"/>
       <c r="AG220" s="14" t="inlineStr"/>
@@ -13430,20 +13430,20 @@
         <v>4.70513911E8</v>
       </c>
       <c r="X221" s="14" t="n">
-        <v>0.0</v>
+        <v>3.8886478E7</v>
       </c>
       <c r="Y221" s="14" t="inlineStr"/>
       <c r="Z221" s="14" t="n">
-        <v>4.70513911E8</v>
+        <v>5.09400389E8</v>
       </c>
       <c r="AA221" s="14" t="inlineStr"/>
       <c r="AB221" s="14" t="inlineStr"/>
       <c r="AC221" s="15" t="n">
-        <v>0.9118486647286822</v>
+        <v>0.9872100562015503</v>
       </c>
       <c r="AD221" s="15" t="inlineStr"/>
       <c r="AE221" s="14" t="n">
-        <v>4.5486089E7</v>
+        <v>6599611.0</v>
       </c>
       <c r="AF221" s="14" t="inlineStr"/>
       <c r="AG221" s="14" t="inlineStr"/>
@@ -13493,20 +13493,20 @@
         <v>5485232.0</v>
       </c>
       <c r="X222" s="14" t="n">
-        <v>0.0</v>
+        <v>263514.0</v>
       </c>
       <c r="Y222" s="14" t="inlineStr"/>
       <c r="Z222" s="14" t="n">
-        <v>5485232.0</v>
+        <v>5748746.0</v>
       </c>
       <c r="AA222" s="14" t="inlineStr"/>
       <c r="AB222" s="14" t="inlineStr"/>
       <c r="AC222" s="15" t="n">
-        <v>0.9142053333333333</v>
+        <v>0.9581243333333334</v>
       </c>
       <c r="AD222" s="15" t="inlineStr"/>
       <c r="AE222" s="14" t="n">
-        <v>514768.0</v>
+        <v>251254.0</v>
       </c>
       <c r="AF222" s="14" t="inlineStr"/>
       <c r="AG222" s="14" t="inlineStr"/>
@@ -13550,20 +13550,20 @@
         <v>5485232.0</v>
       </c>
       <c r="X223" s="14" t="n">
-        <v>0.0</v>
+        <v>263514.0</v>
       </c>
       <c r="Y223" s="14" t="inlineStr"/>
       <c r="Z223" s="14" t="n">
-        <v>5485232.0</v>
+        <v>5748746.0</v>
       </c>
       <c r="AA223" s="14" t="inlineStr"/>
       <c r="AB223" s="14" t="inlineStr"/>
       <c r="AC223" s="15" t="n">
-        <v>0.9142053333333333</v>
+        <v>0.9581243333333334</v>
       </c>
       <c r="AD223" s="15" t="inlineStr"/>
       <c r="AE223" s="14" t="n">
-        <v>514768.0</v>
+        <v>251254.0</v>
       </c>
       <c r="AF223" s="14" t="inlineStr"/>
       <c r="AG223" s="14" t="inlineStr"/>
@@ -13733,20 +13733,20 @@
         <v>1.33021464E8</v>
       </c>
       <c r="X226" s="14" t="n">
-        <v>0.0</v>
+        <v>9250750.0</v>
       </c>
       <c r="Y226" s="14" t="inlineStr"/>
       <c r="Z226" s="14" t="n">
-        <v>1.33021464E8</v>
+        <v>1.42272214E8</v>
       </c>
       <c r="AA226" s="14" t="inlineStr"/>
       <c r="AB226" s="14" t="inlineStr"/>
       <c r="AC226" s="15" t="n">
-        <v>0.919291389080857</v>
+        <v>0.9832219350380097</v>
       </c>
       <c r="AD226" s="15" t="inlineStr"/>
       <c r="AE226" s="14" t="n">
-        <v>1.1678536E7</v>
+        <v>2427786.0</v>
       </c>
       <c r="AF226" s="14" t="inlineStr"/>
       <c r="AG226" s="14" t="inlineStr"/>
@@ -13833,20 +13833,20 @@
         <v>1.044355E8</v>
       </c>
       <c r="X228" s="14" t="n">
-        <v>0.0</v>
+        <v>9250750.0</v>
       </c>
       <c r="Y228" s="14" t="inlineStr"/>
       <c r="Z228" s="14" t="n">
-        <v>1.044355E8</v>
+        <v>1.1368625E8</v>
       </c>
       <c r="AA228" s="14" t="inlineStr"/>
       <c r="AB228" s="14" t="inlineStr"/>
       <c r="AC228" s="15" t="n">
-        <v>0.9113045375218151</v>
+        <v>0.9920266143106458</v>
       </c>
       <c r="AD228" s="15" t="inlineStr"/>
       <c r="AE228" s="14" t="n">
-        <v>1.01645E7</v>
+        <v>913750.0</v>
       </c>
       <c r="AF228" s="14" t="inlineStr"/>
       <c r="AG228" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
up date ralisasi tukin 11 des pukul 12
up date ralisasi tukin 11 des pukul 12
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>9.0559784495E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>2.479274605E9</v>
+        <v>7.709055227E9</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>9.30390591E10</v>
+        <v>9.8268839722E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.9304274545357487</v>
+        <v>0.9827273328769286</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>6.9569789E9</v>
+        <v>1.727198278E9</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>2.479274605E9</v>
+        <v>7.709055227E9</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>8.900569106E10</v>
+        <v>9.4235471682E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.9275035880109923</v>
+        <v>0.9820016794661273</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>6.95694694E9</v>
+        <v>1.727166318E9</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>2.479274605E9</v>
+        <v>7.709055227E9</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>8.900569106E10</v>
+        <v>9.4235471682E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.9275035880109923</v>
+        <v>0.9820016794661273</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>6.95694694E9</v>
+        <v>1.727166318E9</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>8.6525816455E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>2.479274605E9</v>
+        <v>7.709055227E9</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>8.900509106E10</v>
+        <v>9.4234871682E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.9275031347291728</v>
+        <v>0.9820015669321237</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>6.95694694E9</v>
+        <v>1.727166318E9</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>8.6508305403E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>2.479274605E9</v>
+        <v>7.709055227E9</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>8.8987580008E10</v>
+        <v>9.421736063E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.9274997533757052</v>
+        <v>0.9820087111052892</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>6.955927992E9</v>
+        <v>1.72614737E9</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3296,20 +3296,20 @@
         <v>8.0279551347E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>2.281636445E9</v>
+        <v>7.481889742E9</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
-        <v>8.2561187792E10</v>
+        <v>8.7761441089E10</v>
       </c>
       <c r="AA47" s="25" t="inlineStr"/>
       <c r="AB47" s="25" t="inlineStr"/>
       <c r="AC47" s="26" t="n">
-        <v>0.9276879530946325</v>
+        <v>0.9861199168985132</v>
       </c>
       <c r="AD47" s="26" t="inlineStr"/>
       <c r="AE47" s="25" t="n">
-        <v>6.435535208E9</v>
+        <v>1.235281911E9</v>
       </c>
       <c r="AF47" s="25" t="inlineStr"/>
       <c r="AG47" s="25" t="inlineStr"/>
@@ -6082,20 +6082,20 @@
         <v>5.93914035E8</v>
       </c>
       <c r="X95" s="14" t="n">
-        <v>2.694E7</v>
+        <v>3.10703762E8</v>
       </c>
       <c r="Y95" s="14" t="inlineStr"/>
       <c r="Z95" s="14" t="n">
-        <v>6.20854035E8</v>
+        <v>9.04617797E8</v>
       </c>
       <c r="AA95" s="14" t="inlineStr"/>
       <c r="AB95" s="14" t="inlineStr"/>
       <c r="AC95" s="15" t="n">
-        <v>0.6417812375955145</v>
+        <v>0.9351098592917866</v>
       </c>
       <c r="AD95" s="15" t="inlineStr"/>
       <c r="AE95" s="14" t="n">
-        <v>3.46537965E8</v>
+        <v>6.2774203E7</v>
       </c>
       <c r="AF95" s="14" t="inlineStr"/>
       <c r="AG95" s="14" t="inlineStr"/>
@@ -7042,20 +7042,20 @@
         <v>1.42100114E8</v>
       </c>
       <c r="X111" s="14" t="n">
-        <v>0.0</v>
+        <v>2.83763762E8</v>
       </c>
       <c r="Y111" s="14" t="inlineStr"/>
       <c r="Z111" s="14" t="n">
-        <v>1.42100114E8</v>
+        <v>4.25863876E8</v>
       </c>
       <c r="AA111" s="14" t="inlineStr"/>
       <c r="AB111" s="14" t="inlineStr"/>
       <c r="AC111" s="15" t="n">
-        <v>0.31577803111111113</v>
+        <v>0.9463641688888889</v>
       </c>
       <c r="AD111" s="15" t="inlineStr"/>
       <c r="AE111" s="14" t="n">
-        <v>3.07899886E8</v>
+        <v>2.4136124E7</v>
       </c>
       <c r="AF111" s="14" t="inlineStr"/>
       <c r="AG111" s="14" t="inlineStr"/>
@@ -7099,20 +7099,20 @@
         <v>1.42100114E8</v>
       </c>
       <c r="X112" s="14" t="n">
-        <v>0.0</v>
+        <v>2.83763762E8</v>
       </c>
       <c r="Y112" s="14" t="inlineStr"/>
       <c r="Z112" s="14" t="n">
-        <v>1.42100114E8</v>
+        <v>4.25863876E8</v>
       </c>
       <c r="AA112" s="14" t="inlineStr"/>
       <c r="AB112" s="14" t="inlineStr"/>
       <c r="AC112" s="15" t="n">
-        <v>0.31577803111111113</v>
+        <v>0.9463641688888889</v>
       </c>
       <c r="AD112" s="15" t="inlineStr"/>
       <c r="AE112" s="14" t="n">
-        <v>3.07899886E8</v>
+        <v>2.4136124E7</v>
       </c>
       <c r="AF112" s="14" t="inlineStr"/>
       <c r="AG112" s="14" t="inlineStr"/>
@@ -7162,20 +7162,20 @@
         <v>5.0689888E10</v>
       </c>
       <c r="X113" s="14" t="n">
-        <v>1.981188445E9</v>
+        <v>3.745299916E9</v>
       </c>
       <c r="Y113" s="14" t="inlineStr"/>
       <c r="Z113" s="14" t="n">
-        <v>5.2671076445E10</v>
+        <v>5.4435187916E10</v>
       </c>
       <c r="AA113" s="14" t="inlineStr"/>
       <c r="AB113" s="14" t="inlineStr"/>
       <c r="AC113" s="15" t="n">
-        <v>0.9552757529289885</v>
+        <v>0.9872707875372125</v>
       </c>
       <c r="AD113" s="15" t="inlineStr"/>
       <c r="AE113" s="14" t="n">
-        <v>2.465962555E9</v>
+        <v>7.01851084E8</v>
       </c>
       <c r="AF113" s="14" t="inlineStr"/>
       <c r="AG113" s="14" t="inlineStr"/>
@@ -9417,20 +9417,20 @@
         <v>2.475555828E10</v>
       </c>
       <c r="X152" s="14" t="n">
-        <v>1.762736445E9</v>
+        <v>3.526847916E9</v>
       </c>
       <c r="Y152" s="14" t="inlineStr"/>
       <c r="Z152" s="14" t="n">
-        <v>2.6518294725E10</v>
+        <v>2.8282406196E10</v>
       </c>
       <c r="AA152" s="14" t="inlineStr"/>
       <c r="AB152" s="14" t="inlineStr"/>
       <c r="AC152" s="15" t="n">
-        <v>0.9231687194798619</v>
+        <v>0.9845818889385857</v>
       </c>
       <c r="AD152" s="15" t="inlineStr"/>
       <c r="AE152" s="14" t="n">
-        <v>2.207001275E9</v>
+        <v>4.42889804E8</v>
       </c>
       <c r="AF152" s="14" t="inlineStr"/>
       <c r="AG152" s="14" t="inlineStr"/>
@@ -9474,20 +9474,20 @@
         <v>1.997827308E10</v>
       </c>
       <c r="X153" s="14" t="n">
-        <v>1.762736445E9</v>
+        <v>3.526847916E9</v>
       </c>
       <c r="Y153" s="14" t="inlineStr"/>
       <c r="Z153" s="14" t="n">
-        <v>2.1741009525E10</v>
+        <v>2.3505120996E10</v>
       </c>
       <c r="AA153" s="14" t="inlineStr"/>
       <c r="AB153" s="14" t="inlineStr"/>
       <c r="AC153" s="15" t="n">
-        <v>0.9078426919885392</v>
+        <v>0.9815069670977007</v>
       </c>
       <c r="AD153" s="15" t="inlineStr"/>
       <c r="AE153" s="14" t="n">
-        <v>2.206982475E9</v>
+        <v>4.42871004E8</v>
       </c>
       <c r="AF153" s="14" t="inlineStr"/>
       <c r="AG153" s="14" t="inlineStr"/>
@@ -9651,20 +9651,20 @@
         <v>2.3164511208E10</v>
       </c>
       <c r="X156" s="14" t="n">
-        <v>2.45185E8</v>
+        <v>3.397563064E9</v>
       </c>
       <c r="Y156" s="14" t="inlineStr"/>
       <c r="Z156" s="14" t="n">
-        <v>2.3409696208E10</v>
+        <v>2.6562074272E10</v>
       </c>
       <c r="AA156" s="14" t="inlineStr"/>
       <c r="AB156" s="14" t="inlineStr"/>
       <c r="AC156" s="15" t="n">
-        <v>0.8686540936662458</v>
+        <v>0.9856281067310323</v>
       </c>
       <c r="AD156" s="15" t="inlineStr"/>
       <c r="AE156" s="14" t="n">
-        <v>3.539691792E9</v>
+        <v>3.87313728E8</v>
       </c>
       <c r="AF156" s="14" t="inlineStr"/>
       <c r="AG156" s="14" t="inlineStr"/>
@@ -11338,20 +11338,20 @@
         <v>9.794680989E9</v>
       </c>
       <c r="X185" s="14" t="n">
-        <v>0.0</v>
+        <v>3.152378064E9</v>
       </c>
       <c r="Y185" s="14" t="inlineStr"/>
       <c r="Z185" s="14" t="n">
-        <v>9.794680989E9</v>
+        <v>1.2947059053E10</v>
       </c>
       <c r="AA185" s="14" t="inlineStr"/>
       <c r="AB185" s="14" t="inlineStr"/>
       <c r="AC185" s="15" t="n">
-        <v>0.7507542654118889</v>
+        <v>0.9923814588239839</v>
       </c>
       <c r="AD185" s="15" t="inlineStr"/>
       <c r="AE185" s="14" t="n">
-        <v>3.251773011E9</v>
+        <v>9.9394947E7</v>
       </c>
       <c r="AF185" s="14" t="inlineStr"/>
       <c r="AG185" s="14" t="inlineStr"/>
@@ -11395,20 +11395,20 @@
         <v>8.220237613E9</v>
       </c>
       <c r="X186" s="14" t="n">
-        <v>0.0</v>
+        <v>3.152378064E9</v>
       </c>
       <c r="Y186" s="14" t="inlineStr"/>
       <c r="Z186" s="14" t="n">
-        <v>8.220237613E9</v>
+        <v>1.1372615677E10</v>
       </c>
       <c r="AA186" s="14" t="inlineStr"/>
       <c r="AB186" s="14" t="inlineStr"/>
       <c r="AC186" s="15" t="n">
-        <v>0.7165479090829847</v>
+        <v>0.9913367919281729</v>
       </c>
       <c r="AD186" s="15" t="inlineStr"/>
       <c r="AE186" s="14" t="n">
-        <v>3.251762387E9</v>
+        <v>9.9384323E7</v>
       </c>
       <c r="AF186" s="14" t="inlineStr"/>
       <c r="AG186" s="14" t="inlineStr"/>
@@ -11572,20 +11572,20 @@
         <v>6.228754056E9</v>
       </c>
       <c r="X189" s="25" t="n">
-        <v>1.9763816E8</v>
+        <v>2.27165485E8</v>
       </c>
       <c r="Y189" s="25" t="inlineStr"/>
       <c r="Z189" s="25" t="n">
-        <v>6.426392216E9</v>
+        <v>6.455919541E9</v>
       </c>
       <c r="AA189" s="25" t="inlineStr"/>
       <c r="AB189" s="25" t="inlineStr"/>
       <c r="AC189" s="26" t="n">
-        <v>0.9250886872128617</v>
+        <v>0.9293391894235967</v>
       </c>
       <c r="AD189" s="26" t="inlineStr"/>
       <c r="AE189" s="25" t="n">
-        <v>5.20392784E8</v>
+        <v>4.90865459E8</v>
       </c>
       <c r="AF189" s="25" t="inlineStr"/>
       <c r="AG189" s="25" t="inlineStr"/>
@@ -11635,20 +11635,20 @@
         <v>4.783558496E9</v>
       </c>
       <c r="X190" s="14" t="n">
-        <v>1.1638698E8</v>
+        <v>1.31977006E8</v>
       </c>
       <c r="Y190" s="14" t="inlineStr"/>
       <c r="Z190" s="14" t="n">
-        <v>4.899945476E9</v>
+        <v>4.915535502E9</v>
       </c>
       <c r="AA190" s="14" t="inlineStr"/>
       <c r="AB190" s="14" t="inlineStr"/>
       <c r="AC190" s="15" t="n">
-        <v>0.9788065011852679</v>
+        <v>0.9819207437573924</v>
       </c>
       <c r="AD190" s="15" t="inlineStr"/>
       <c r="AE190" s="14" t="n">
-        <v>1.06095524E8</v>
+        <v>9.0505498E7</v>
       </c>
       <c r="AF190" s="14" t="inlineStr"/>
       <c r="AG190" s="14" t="inlineStr"/>
@@ -11698,20 +11698,20 @@
         <v>1.777909494E9</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>7.7954712E7</v>
+        <v>9.3544738E7</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
-        <v>1.855864206E9</v>
+        <v>1.871454232E9</v>
       </c>
       <c r="AA191" s="14" t="inlineStr"/>
       <c r="AB191" s="14" t="inlineStr"/>
       <c r="AC191" s="15" t="n">
-        <v>0.9815144490450425</v>
+        <v>0.9897595758870372</v>
       </c>
       <c r="AD191" s="15" t="inlineStr"/>
       <c r="AE191" s="14" t="n">
-        <v>3.4952794E7</v>
+        <v>1.9362768E7</v>
       </c>
       <c r="AF191" s="14" t="inlineStr"/>
       <c r="AG191" s="14" t="inlineStr"/>
@@ -11869,20 +11869,20 @@
         <v>5.5184254E7</v>
       </c>
       <c r="X194" s="14" t="n">
-        <v>3953112.0</v>
+        <v>1.9543138E7</v>
       </c>
       <c r="Y194" s="14" t="inlineStr"/>
       <c r="Z194" s="14" t="n">
-        <v>5.9137366E7</v>
+        <v>7.4727392E7</v>
       </c>
       <c r="AA194" s="14" t="inlineStr"/>
       <c r="AB194" s="14" t="inlineStr"/>
       <c r="AC194" s="15" t="n">
-        <v>0.6295897583306718</v>
+        <v>0.7955646971148728</v>
       </c>
       <c r="AD194" s="15" t="inlineStr"/>
       <c r="AE194" s="14" t="n">
-        <v>3.4792634E7</v>
+        <v>1.9202608E7</v>
       </c>
       <c r="AF194" s="14" t="inlineStr"/>
       <c r="AG194" s="14" t="inlineStr"/>
@@ -13953,20 +13953,20 @@
         <v>6.74613153E8</v>
       </c>
       <c r="X230" s="14" t="n">
-        <v>3.1766138E7</v>
+        <v>4.5703437E7</v>
       </c>
       <c r="Y230" s="14" t="inlineStr"/>
       <c r="Z230" s="14" t="n">
-        <v>7.06379291E8</v>
+        <v>7.2031659E8</v>
       </c>
       <c r="AA230" s="14" t="inlineStr"/>
       <c r="AB230" s="14" t="inlineStr"/>
       <c r="AC230" s="15" t="n">
-        <v>0.6372848658450768</v>
+        <v>0.6498588892297144</v>
       </c>
       <c r="AD230" s="15" t="inlineStr"/>
       <c r="AE230" s="14" t="n">
-        <v>4.02040709E8</v>
+        <v>3.8810341E8</v>
       </c>
       <c r="AF230" s="14" t="inlineStr"/>
       <c r="AG230" s="14" t="inlineStr"/>
@@ -15288,20 +15288,20 @@
         <v>2.11521335E8</v>
       </c>
       <c r="X253" s="14" t="n">
-        <v>6690138.0</v>
+        <v>2.0627437E7</v>
       </c>
       <c r="Y253" s="14" t="inlineStr"/>
       <c r="Z253" s="14" t="n">
-        <v>2.18211473E8</v>
+        <v>2.32148772E8</v>
       </c>
       <c r="AA253" s="14" t="inlineStr"/>
       <c r="AB253" s="14" t="inlineStr"/>
       <c r="AC253" s="15" t="n">
-        <v>0.6562751067669172</v>
+        <v>0.6981917954887218</v>
       </c>
       <c r="AD253" s="15" t="inlineStr"/>
       <c r="AE253" s="14" t="n">
-        <v>1.14288527E8</v>
+        <v>1.00351228E8</v>
       </c>
       <c r="AF253" s="14" t="inlineStr"/>
       <c r="AG253" s="14" t="inlineStr"/>
@@ -15559,20 +15559,20 @@
         <v>1.22043496E8</v>
       </c>
       <c r="X258" s="14" t="n">
-        <v>1490000.0</v>
+        <v>1.5139299E7</v>
       </c>
       <c r="Y258" s="14" t="inlineStr"/>
       <c r="Z258" s="14" t="n">
-        <v>1.23533496E8</v>
+        <v>1.37182795E8</v>
       </c>
       <c r="AA258" s="14" t="inlineStr"/>
       <c r="AB258" s="14" t="inlineStr"/>
       <c r="AC258" s="15" t="n">
-        <v>0.7277378262150221</v>
+        <v>0.8081460677466863</v>
       </c>
       <c r="AD258" s="15" t="inlineStr"/>
       <c r="AE258" s="14" t="n">
-        <v>4.6216504E7</v>
+        <v>3.2567205E7</v>
       </c>
       <c r="AF258" s="14" t="inlineStr"/>
       <c r="AG258" s="14" t="inlineStr"/>
@@ -15844,20 +15844,20 @@
         <v>8450284.0</v>
       </c>
       <c r="X263" s="14" t="n">
-        <v>0.0</v>
+        <v>288000.0</v>
       </c>
       <c r="Y263" s="14" t="inlineStr"/>
       <c r="Z263" s="14" t="n">
-        <v>8450284.0</v>
+        <v>8738284.0</v>
       </c>
       <c r="AA263" s="14" t="inlineStr"/>
       <c r="AB263" s="14" t="inlineStr"/>
       <c r="AC263" s="15" t="n">
-        <v>0.7041903333333334</v>
+        <v>0.7281903333333334</v>
       </c>
       <c r="AD263" s="15" t="inlineStr"/>
       <c r="AE263" s="14" t="n">
-        <v>3549716.0</v>
+        <v>3261716.0</v>
       </c>
       <c r="AF263" s="14" t="inlineStr"/>
       <c r="AG263" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
Realisasi per 22 Des, pkl 12
Realisasi per 22 Des, pkl 12, SPM LS Non Kontraktual
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>9.0559784495E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>7.709055227E9</v>
+        <v>8.096493585E9</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>9.8268839722E10</v>
+        <v>9.865627808E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.9827273328769286</v>
+        <v>0.986601869966088</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>1.727198278E9</v>
+        <v>1.33975992E9</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>7.709055227E9</v>
+        <v>8.096493585E9</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>9.4235471682E10</v>
+        <v>9.462291004E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.9820016794661273</v>
+        <v>0.9860390669960531</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>1.727166318E9</v>
+        <v>1.33972796E9</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>7.709055227E9</v>
+        <v>8.096493585E9</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>9.4235471682E10</v>
+        <v>9.462291004E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.9820016794661273</v>
+        <v>0.9860390669960531</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>1.727166318E9</v>
+        <v>1.33972796E9</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>8.6525816455E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>7.709055227E9</v>
+        <v>8.096493585E9</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>9.4234871682E10</v>
+        <v>9.462231004E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.9820015669321237</v>
+        <v>0.9860389797057041</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>1.727166318E9</v>
+        <v>1.33972796E9</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -2564,20 +2564,20 @@
         <v>1.6461052E7</v>
       </c>
       <c r="X35" s="22" t="n">
-        <v>0.0</v>
+        <v>800000.0</v>
       </c>
       <c r="Y35" s="22" t="inlineStr"/>
       <c r="Z35" s="21" t="n">
-        <v>1.6461052E7</v>
+        <v>1.7261052E7</v>
       </c>
       <c r="AA35" s="21" t="inlineStr"/>
       <c r="AB35" s="21" t="inlineStr"/>
       <c r="AC35" s="23" t="n">
-        <v>0.9417077803203662</v>
+        <v>0.9874743707093822</v>
       </c>
       <c r="AD35" s="23" t="inlineStr"/>
       <c r="AE35" s="21" t="n">
-        <v>1018948.0</v>
+        <v>218948.0</v>
       </c>
       <c r="AF35" s="21" t="inlineStr"/>
       <c r="AG35" s="21" t="inlineStr"/>
@@ -2627,20 +2627,20 @@
         <v>1.6461052E7</v>
       </c>
       <c r="X36" s="25" t="n">
-        <v>0.0</v>
+        <v>800000.0</v>
       </c>
       <c r="Y36" s="25" t="inlineStr"/>
       <c r="Z36" s="25" t="n">
-        <v>1.6461052E7</v>
+        <v>1.7261052E7</v>
       </c>
       <c r="AA36" s="25" t="inlineStr"/>
       <c r="AB36" s="25" t="inlineStr"/>
       <c r="AC36" s="26" t="n">
-        <v>0.9417077803203662</v>
+        <v>0.9874743707093822</v>
       </c>
       <c r="AD36" s="26" t="inlineStr"/>
       <c r="AE36" s="25" t="n">
-        <v>1018948.0</v>
+        <v>218948.0</v>
       </c>
       <c r="AF36" s="25" t="inlineStr"/>
       <c r="AG36" s="25" t="inlineStr"/>
@@ -2993,20 +2993,20 @@
         <v>1.4061052E7</v>
       </c>
       <c r="X42" s="14" t="n">
-        <v>0.0</v>
+        <v>800000.0</v>
       </c>
       <c r="Y42" s="14" t="inlineStr"/>
       <c r="Z42" s="14" t="n">
-        <v>1.4061052E7</v>
+        <v>1.4861052E7</v>
       </c>
       <c r="AA42" s="14" t="inlineStr"/>
       <c r="AB42" s="14" t="inlineStr"/>
       <c r="AC42" s="15" t="n">
-        <v>0.9324305039787798</v>
+        <v>0.985480901856764</v>
       </c>
       <c r="AD42" s="15" t="inlineStr"/>
       <c r="AE42" s="14" t="n">
-        <v>1018948.0</v>
+        <v>218948.0</v>
       </c>
       <c r="AF42" s="14" t="inlineStr"/>
       <c r="AG42" s="14" t="inlineStr"/>
@@ -3056,20 +3056,20 @@
         <v>1.4061052E7</v>
       </c>
       <c r="X43" s="14" t="n">
-        <v>0.0</v>
+        <v>800000.0</v>
       </c>
       <c r="Y43" s="14" t="inlineStr"/>
       <c r="Z43" s="14" t="n">
-        <v>1.4061052E7</v>
+        <v>1.4861052E7</v>
       </c>
       <c r="AA43" s="14" t="inlineStr"/>
       <c r="AB43" s="14" t="inlineStr"/>
       <c r="AC43" s="15" t="n">
-        <v>0.9324305039787798</v>
+        <v>0.985480901856764</v>
       </c>
       <c r="AD43" s="15" t="inlineStr"/>
       <c r="AE43" s="14" t="n">
-        <v>1018948.0</v>
+        <v>218948.0</v>
       </c>
       <c r="AF43" s="14" t="inlineStr"/>
       <c r="AG43" s="14" t="inlineStr"/>
@@ -3113,20 +3113,20 @@
         <v>1.3311952E7</v>
       </c>
       <c r="X44" s="14" t="n">
-        <v>0.0</v>
+        <v>800000.0</v>
       </c>
       <c r="Y44" s="14" t="inlineStr"/>
       <c r="Z44" s="14" t="n">
-        <v>1.3311952E7</v>
+        <v>1.4111952E7</v>
       </c>
       <c r="AA44" s="14" t="inlineStr"/>
       <c r="AB44" s="14" t="inlineStr"/>
       <c r="AC44" s="15" t="n">
-        <v>0.9302552061495458</v>
+        <v>0.9861601677148847</v>
       </c>
       <c r="AD44" s="15" t="inlineStr"/>
       <c r="AE44" s="14" t="n">
-        <v>998048.0</v>
+        <v>198048.0</v>
       </c>
       <c r="AF44" s="14" t="inlineStr"/>
       <c r="AG44" s="14" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>8.6508305403E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>7.709055227E9</v>
+        <v>8.095693585E9</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>9.421736063E10</v>
+        <v>9.4603998988E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.9820087111052892</v>
+        <v>0.9860385654024658</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>1.72614737E9</v>
+        <v>1.339509012E9</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3296,20 +3296,20 @@
         <v>8.0279551347E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>7.481889742E9</v>
+        <v>7.495823038E9</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
-        <v>8.7761441089E10</v>
+        <v>8.7775374385E10</v>
       </c>
       <c r="AA47" s="25" t="inlineStr"/>
       <c r="AB47" s="25" t="inlineStr"/>
       <c r="AC47" s="26" t="n">
-        <v>0.9861199168985132</v>
+        <v>0.9862764765507153</v>
       </c>
       <c r="AD47" s="26" t="inlineStr"/>
       <c r="AE47" s="25" t="n">
-        <v>1.235281911E9</v>
+        <v>1.221348615E9</v>
       </c>
       <c r="AF47" s="25" t="inlineStr"/>
       <c r="AG47" s="25" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
       <c r="O48" s="13" t="inlineStr"/>
       <c r="P48" s="13" t="inlineStr"/>
       <c r="Q48" s="14" t="n">
-        <v>5.942904E9</v>
+        <v>5.92038E9</v>
       </c>
       <c r="R48" s="14" t="inlineStr"/>
       <c r="S48" s="14" t="n">
@@ -3368,11 +3368,11 @@
       <c r="AA48" s="14" t="inlineStr"/>
       <c r="AB48" s="14" t="inlineStr"/>
       <c r="AC48" s="15" t="n">
-        <v>0.9859760655733292</v>
+        <v>0.9897271972407177</v>
       </c>
       <c r="AD48" s="15" t="inlineStr"/>
       <c r="AE48" s="14" t="n">
-        <v>8.3342896E7</v>
+        <v>6.0818896E7</v>
       </c>
       <c r="AF48" s="14" t="inlineStr"/>
       <c r="AG48" s="14" t="inlineStr"/>
@@ -5324,7 +5324,7 @@
       <c r="O82" s="13" t="inlineStr"/>
       <c r="P82" s="13" t="inlineStr"/>
       <c r="Q82" s="14" t="n">
-        <v>3.6072E8</v>
+        <v>3.38196E8</v>
       </c>
       <c r="R82" s="14" t="inlineStr"/>
       <c r="S82" s="14" t="n">
@@ -5346,11 +5346,11 @@
       <c r="AA82" s="14" t="inlineStr"/>
       <c r="AB82" s="14" t="inlineStr"/>
       <c r="AC82" s="15" t="n">
-        <v>0.8484808161454868</v>
+        <v>0.9049900057954559</v>
       </c>
       <c r="AD82" s="15" t="inlineStr"/>
       <c r="AE82" s="14" t="n">
-        <v>5.4656E7</v>
+        <v>3.2132E7</v>
       </c>
       <c r="AF82" s="14" t="inlineStr"/>
       <c r="AG82" s="14" t="inlineStr"/>
@@ -5438,7 +5438,7 @@
       <c r="O84" s="13" t="inlineStr"/>
       <c r="P84" s="13" t="inlineStr"/>
       <c r="Q84" s="14" t="n">
-        <v>2.9304E8</v>
+        <v>2.78388E8</v>
       </c>
       <c r="R84" s="14" t="inlineStr"/>
       <c r="S84" s="14" t="n">
@@ -5460,11 +5460,11 @@
       <c r="AA84" s="14" t="inlineStr"/>
       <c r="AB84" s="14" t="inlineStr"/>
       <c r="AC84" s="15" t="n">
-        <v>0.8595959595959596</v>
+        <v>0.9048378522062732</v>
       </c>
       <c r="AD84" s="15" t="inlineStr"/>
       <c r="AE84" s="14" t="n">
-        <v>4.1144E7</v>
+        <v>2.6492E7</v>
       </c>
       <c r="AF84" s="14" t="inlineStr"/>
       <c r="AG84" s="14" t="inlineStr"/>
@@ -5495,7 +5495,7 @@
       <c r="O85" s="13" t="inlineStr"/>
       <c r="P85" s="13" t="inlineStr"/>
       <c r="Q85" s="14" t="n">
-        <v>4.92E7</v>
+        <v>4.1328E7</v>
       </c>
       <c r="R85" s="14" t="inlineStr"/>
       <c r="S85" s="14" t="n">
@@ -5517,11 +5517,11 @@
       <c r="AA85" s="14" t="inlineStr"/>
       <c r="AB85" s="14" t="inlineStr"/>
       <c r="AC85" s="15" t="n">
-        <v>0.7566666666666667</v>
+        <v>0.9007936507936508</v>
       </c>
       <c r="AD85" s="15" t="inlineStr"/>
       <c r="AE85" s="14" t="n">
-        <v>1.1972E7</v>
+        <v>4100000.0</v>
       </c>
       <c r="AF85" s="14" t="inlineStr"/>
       <c r="AG85" s="14" t="inlineStr"/>
@@ -6069,7 +6069,7 @@
       <c r="O95" s="13" t="inlineStr"/>
       <c r="P95" s="13" t="inlineStr"/>
       <c r="Q95" s="14" t="n">
-        <v>9.67392E8</v>
+        <v>9.72489E8</v>
       </c>
       <c r="R95" s="14" t="inlineStr"/>
       <c r="S95" s="14" t="n">
@@ -6091,11 +6091,11 @@
       <c r="AA95" s="14" t="inlineStr"/>
       <c r="AB95" s="14" t="inlineStr"/>
       <c r="AC95" s="15" t="n">
-        <v>0.9351098592917866</v>
+        <v>0.9302087704848075</v>
       </c>
       <c r="AD95" s="15" t="inlineStr"/>
       <c r="AE95" s="14" t="n">
-        <v>6.2774203E7</v>
+        <v>6.7871203E7</v>
       </c>
       <c r="AF95" s="14" t="inlineStr"/>
       <c r="AG95" s="14" t="inlineStr"/>
@@ -6732,7 +6732,7 @@
       <c r="O106" s="13" t="inlineStr"/>
       <c r="P106" s="13" t="inlineStr"/>
       <c r="Q106" s="14" t="n">
-        <v>8.304E7</v>
+        <v>8.8137E7</v>
       </c>
       <c r="R106" s="14" t="inlineStr"/>
       <c r="S106" s="14" t="n">
@@ -6754,11 +6754,11 @@
       <c r="AA106" s="14" t="inlineStr"/>
       <c r="AB106" s="14" t="inlineStr"/>
       <c r="AC106" s="15" t="n">
-        <v>0.6957249518304431</v>
+        <v>0.6554908835108978</v>
       </c>
       <c r="AD106" s="15" t="inlineStr"/>
       <c r="AE106" s="14" t="n">
-        <v>2.5267E7</v>
+        <v>3.0364E7</v>
       </c>
       <c r="AF106" s="14" t="inlineStr"/>
       <c r="AG106" s="14" t="inlineStr"/>
@@ -6789,7 +6789,7 @@
       <c r="O107" s="13" t="inlineStr"/>
       <c r="P107" s="13" t="inlineStr"/>
       <c r="Q107" s="14" t="n">
-        <v>2.31E7</v>
+        <v>2.52E7</v>
       </c>
       <c r="R107" s="14" t="inlineStr"/>
       <c r="S107" s="14" t="n">
@@ -6811,11 +6811,11 @@
       <c r="AA107" s="14" t="inlineStr"/>
       <c r="AB107" s="14" t="inlineStr"/>
       <c r="AC107" s="15" t="n">
-        <v>0.7166666666666667</v>
+        <v>0.6569444444444444</v>
       </c>
       <c r="AD107" s="15" t="inlineStr"/>
       <c r="AE107" s="14" t="n">
-        <v>6545000.0</v>
+        <v>8645000.0</v>
       </c>
       <c r="AF107" s="14" t="inlineStr"/>
       <c r="AG107" s="14" t="inlineStr"/>
@@ -6846,7 +6846,7 @@
       <c r="O108" s="13" t="inlineStr"/>
       <c r="P108" s="13" t="inlineStr"/>
       <c r="Q108" s="14" t="n">
-        <v>5.994E7</v>
+        <v>6.2937E7</v>
       </c>
       <c r="R108" s="14" t="inlineStr"/>
       <c r="S108" s="14" t="n">
@@ -6868,11 +6868,11 @@
       <c r="AA108" s="14" t="inlineStr"/>
       <c r="AB108" s="14" t="inlineStr"/>
       <c r="AC108" s="15" t="n">
-        <v>0.6876543209876543</v>
+        <v>0.6549088771310994</v>
       </c>
       <c r="AD108" s="15" t="inlineStr"/>
       <c r="AE108" s="14" t="n">
-        <v>1.8722E7</v>
+        <v>2.1719E7</v>
       </c>
       <c r="AF108" s="14" t="inlineStr"/>
       <c r="AG108" s="14" t="inlineStr"/>
@@ -7149,7 +7149,7 @@
       <c r="O113" s="13" t="inlineStr"/>
       <c r="P113" s="13" t="inlineStr"/>
       <c r="Q113" s="14" t="n">
-        <v>5.5137039E10</v>
+        <v>5.5154319E10</v>
       </c>
       <c r="R113" s="14" t="inlineStr"/>
       <c r="S113" s="14" t="n">
@@ -7162,20 +7162,20 @@
         <v>5.0689888E10</v>
       </c>
       <c r="X113" s="14" t="n">
-        <v>3.745299916E9</v>
+        <v>3.759233212E9</v>
       </c>
       <c r="Y113" s="14" t="inlineStr"/>
       <c r="Z113" s="14" t="n">
-        <v>5.4435187916E10</v>
+        <v>5.4449121212E10</v>
       </c>
       <c r="AA113" s="14" t="inlineStr"/>
       <c r="AB113" s="14" t="inlineStr"/>
       <c r="AC113" s="15" t="n">
-        <v>0.9872707875372125</v>
+        <v>0.987214096723776</v>
       </c>
       <c r="AD113" s="15" t="inlineStr"/>
       <c r="AE113" s="14" t="n">
-        <v>7.01851084E8</v>
+        <v>7.05197788E8</v>
       </c>
       <c r="AF113" s="14" t="inlineStr"/>
       <c r="AG113" s="14" t="inlineStr"/>
@@ -7225,20 +7225,20 @@
         <v>1.70891536E10</v>
       </c>
       <c r="X114" s="14" t="n">
-        <v>0.0</v>
+        <v>3390500.0</v>
       </c>
       <c r="Y114" s="14" t="inlineStr"/>
       <c r="Z114" s="14" t="n">
-        <v>1.70891536E10</v>
+        <v>1.70925441E10</v>
       </c>
       <c r="AA114" s="14" t="inlineStr"/>
       <c r="AB114" s="14" t="inlineStr"/>
       <c r="AC114" s="15" t="n">
-        <v>0.9992991460978126</v>
+        <v>0.9994974077457648</v>
       </c>
       <c r="AD114" s="15" t="inlineStr"/>
       <c r="AE114" s="14" t="n">
-        <v>1.19854E7</v>
+        <v>8594900.0</v>
       </c>
       <c r="AF114" s="14" t="inlineStr"/>
       <c r="AG114" s="14" t="inlineStr"/>
@@ -7282,20 +7282,20 @@
         <v>1.45984002E10</v>
       </c>
       <c r="X115" s="14" t="n">
-        <v>0.0</v>
+        <v>3390500.0</v>
       </c>
       <c r="Y115" s="14" t="inlineStr"/>
       <c r="Z115" s="14" t="n">
-        <v>1.45984002E10</v>
+        <v>1.46017907E10</v>
       </c>
       <c r="AA115" s="14" t="inlineStr"/>
       <c r="AB115" s="14" t="inlineStr"/>
       <c r="AC115" s="15" t="n">
-        <v>0.9996124502364411</v>
+        <v>0.9998446117038686</v>
       </c>
       <c r="AD115" s="15" t="inlineStr"/>
       <c r="AE115" s="14" t="n">
-        <v>5659800.0</v>
+        <v>2269300.0</v>
       </c>
       <c r="AF115" s="14" t="inlineStr"/>
       <c r="AG115" s="14" t="inlineStr"/>
@@ -7502,20 +7502,20 @@
         <v>230145.0</v>
       </c>
       <c r="X119" s="14" t="n">
-        <v>0.0</v>
+        <v>76.0</v>
       </c>
       <c r="Y119" s="14" t="inlineStr"/>
       <c r="Z119" s="14" t="n">
-        <v>230145.0</v>
+        <v>230221.0</v>
       </c>
       <c r="AA119" s="14" t="inlineStr"/>
       <c r="AB119" s="14" t="inlineStr"/>
       <c r="AC119" s="15" t="n">
-        <v>0.9629497907949791</v>
+        <v>0.9632677824267782</v>
       </c>
       <c r="AD119" s="15" t="inlineStr"/>
       <c r="AE119" s="14" t="n">
-        <v>8855.0</v>
+        <v>8779.0</v>
       </c>
       <c r="AF119" s="14" t="inlineStr"/>
       <c r="AG119" s="14" t="inlineStr"/>
@@ -7559,20 +7559,20 @@
         <v>196371.0</v>
       </c>
       <c r="X120" s="14" t="n">
-        <v>0.0</v>
+        <v>76.0</v>
       </c>
       <c r="Y120" s="14" t="inlineStr"/>
       <c r="Z120" s="14" t="n">
-        <v>196371.0</v>
+        <v>196447.0</v>
       </c>
       <c r="AA120" s="14" t="inlineStr"/>
       <c r="AB120" s="14" t="inlineStr"/>
       <c r="AC120" s="15" t="n">
-        <v>0.9626029411764706</v>
+        <v>0.9629754901960784</v>
       </c>
       <c r="AD120" s="15" t="inlineStr"/>
       <c r="AE120" s="14" t="n">
-        <v>7629.0</v>
+        <v>7553.0</v>
       </c>
       <c r="AF120" s="14" t="inlineStr"/>
       <c r="AG120" s="14" t="inlineStr"/>
@@ -8204,20 +8204,20 @@
         <v>3.68345E9</v>
       </c>
       <c r="X131" s="14" t="n">
-        <v>0.0</v>
+        <v>540000.0</v>
       </c>
       <c r="Y131" s="14" t="inlineStr"/>
       <c r="Z131" s="14" t="n">
-        <v>3.68345E9</v>
+        <v>3.68399E9</v>
       </c>
       <c r="AA131" s="14" t="inlineStr"/>
       <c r="AB131" s="14" t="inlineStr"/>
       <c r="AC131" s="15" t="n">
-        <v>0.9989710472103284</v>
+        <v>0.9991174980554582</v>
       </c>
       <c r="AD131" s="15" t="inlineStr"/>
       <c r="AE131" s="14" t="n">
-        <v>3794000.0</v>
+        <v>3254000.0</v>
       </c>
       <c r="AF131" s="14" t="inlineStr"/>
       <c r="AG131" s="14" t="inlineStr"/>
@@ -8261,20 +8261,20 @@
         <v>3.14519E9</v>
       </c>
       <c r="X132" s="14" t="n">
-        <v>0.0</v>
+        <v>540000.0</v>
       </c>
       <c r="Y132" s="14" t="inlineStr"/>
       <c r="Z132" s="14" t="n">
-        <v>3.14519E9</v>
+        <v>3.14573E9</v>
       </c>
       <c r="AA132" s="14" t="inlineStr"/>
       <c r="AB132" s="14" t="inlineStr"/>
       <c r="AC132" s="15" t="n">
-        <v>0.9987964356712332</v>
+        <v>0.9989679197708464</v>
       </c>
       <c r="AD132" s="15" t="inlineStr"/>
       <c r="AE132" s="14" t="n">
-        <v>3790000.0</v>
+        <v>3250000.0</v>
       </c>
       <c r="AF132" s="14" t="inlineStr"/>
       <c r="AG132" s="14" t="inlineStr"/>
@@ -8672,20 +8672,20 @@
         <v>9.4305324E8</v>
       </c>
       <c r="X139" s="14" t="n">
-        <v>0.0</v>
+        <v>72420.0</v>
       </c>
       <c r="Y139" s="14" t="inlineStr"/>
       <c r="Z139" s="14" t="n">
-        <v>9.4305324E8</v>
+        <v>9.4312566E8</v>
       </c>
       <c r="AA139" s="14" t="inlineStr"/>
       <c r="AB139" s="14" t="inlineStr"/>
       <c r="AC139" s="15" t="n">
-        <v>0.9995307240306265</v>
+        <v>0.9996074811127975</v>
       </c>
       <c r="AD139" s="15" t="inlineStr"/>
       <c r="AE139" s="14" t="n">
-        <v>442760.0</v>
+        <v>370340.0</v>
       </c>
       <c r="AF139" s="14" t="inlineStr"/>
       <c r="AG139" s="14" t="inlineStr"/>
@@ -8729,20 +8729,20 @@
         <v>8.0632428E8</v>
       </c>
       <c r="X140" s="14" t="n">
-        <v>0.0</v>
+        <v>72420.0</v>
       </c>
       <c r="Y140" s="14" t="inlineStr"/>
       <c r="Z140" s="14" t="n">
-        <v>8.0632428E8</v>
+        <v>8.063967E8</v>
       </c>
       <c r="AA140" s="14" t="inlineStr"/>
       <c r="AB140" s="14" t="inlineStr"/>
       <c r="AC140" s="15" t="n">
-        <v>0.99945991372899</v>
+        <v>0.9995496802022906</v>
       </c>
       <c r="AD140" s="15" t="inlineStr"/>
       <c r="AE140" s="14" t="n">
-        <v>435720.0</v>
+        <v>363300.0</v>
       </c>
       <c r="AF140" s="14" t="inlineStr"/>
       <c r="AG140" s="14" t="inlineStr"/>
@@ -8893,7 +8893,7 @@
       <c r="O143" s="13" t="inlineStr"/>
       <c r="P143" s="13" t="inlineStr"/>
       <c r="Q143" s="14" t="n">
-        <v>2.672352E9</v>
+        <v>2.689632E9</v>
       </c>
       <c r="R143" s="14" t="inlineStr"/>
       <c r="S143" s="14" t="n">
@@ -8906,20 +8906,20 @@
         <v>2.213268E9</v>
       </c>
       <c r="X143" s="14" t="n">
-        <v>2.18452E8</v>
+        <v>2.19192E8</v>
       </c>
       <c r="Y143" s="14" t="inlineStr"/>
       <c r="Z143" s="14" t="n">
-        <v>2.43172E9</v>
+        <v>2.43246E9</v>
       </c>
       <c r="AA143" s="14" t="inlineStr"/>
       <c r="AB143" s="14" t="inlineStr"/>
       <c r="AC143" s="15" t="n">
-        <v>0.9099549759911868</v>
+        <v>0.904383945461684</v>
       </c>
       <c r="AD143" s="15" t="inlineStr"/>
       <c r="AE143" s="14" t="n">
-        <v>2.40632E8</v>
+        <v>2.57172E8</v>
       </c>
       <c r="AF143" s="14" t="inlineStr"/>
       <c r="AG143" s="14" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       <c r="O144" s="13" t="inlineStr"/>
       <c r="P144" s="13" t="inlineStr"/>
       <c r="Q144" s="14" t="n">
-        <v>2.436E8</v>
+        <v>2.52E8</v>
       </c>
       <c r="R144" s="14" t="inlineStr"/>
       <c r="S144" s="14" t="n">
@@ -8972,11 +8972,11 @@
       <c r="AA144" s="14" t="inlineStr"/>
       <c r="AB144" s="14" t="inlineStr"/>
       <c r="AC144" s="15" t="n">
-        <v>0.9421469622331692</v>
+        <v>0.9107420634920635</v>
       </c>
       <c r="AD144" s="15" t="inlineStr"/>
       <c r="AE144" s="14" t="n">
-        <v>1.4093E7</v>
+        <v>2.2493E7</v>
       </c>
       <c r="AF144" s="14" t="inlineStr"/>
       <c r="AG144" s="14" t="inlineStr"/>
@@ -9050,7 +9050,7 @@
       <c r="O146" s="13" t="inlineStr"/>
       <c r="P146" s="13" t="inlineStr"/>
       <c r="Q146" s="14" t="n">
-        <v>1.9092E9</v>
+        <v>1.91808E9</v>
       </c>
       <c r="R146" s="14" t="inlineStr"/>
       <c r="S146" s="14" t="n">
@@ -9063,20 +9063,20 @@
         <v>1.581491E9</v>
       </c>
       <c r="X146" s="14" t="n">
-        <v>1.59359E8</v>
+        <v>1.60099E8</v>
       </c>
       <c r="Y146" s="14" t="inlineStr"/>
       <c r="Z146" s="14" t="n">
-        <v>1.74085E9</v>
+        <v>1.74159E9</v>
       </c>
       <c r="AA146" s="14" t="inlineStr"/>
       <c r="AB146" s="14" t="inlineStr"/>
       <c r="AC146" s="15" t="n">
-        <v>0.9118217054263565</v>
+        <v>0.9079861111111112</v>
       </c>
       <c r="AD146" s="15" t="inlineStr"/>
       <c r="AE146" s="14" t="n">
-        <v>1.6835E8</v>
+        <v>1.7649E8</v>
       </c>
       <c r="AF146" s="14" t="inlineStr"/>
       <c r="AG146" s="14" t="inlineStr"/>
@@ -9417,20 +9417,20 @@
         <v>2.475555828E10</v>
       </c>
       <c r="X152" s="14" t="n">
-        <v>3.526847916E9</v>
+        <v>3.536038216E9</v>
       </c>
       <c r="Y152" s="14" t="inlineStr"/>
       <c r="Z152" s="14" t="n">
-        <v>2.8282406196E10</v>
+        <v>2.8291596496E10</v>
       </c>
       <c r="AA152" s="14" t="inlineStr"/>
       <c r="AB152" s="14" t="inlineStr"/>
       <c r="AC152" s="15" t="n">
-        <v>0.9845818889385857</v>
+        <v>0.9849018264598561</v>
       </c>
       <c r="AD152" s="15" t="inlineStr"/>
       <c r="AE152" s="14" t="n">
-        <v>4.42889804E8</v>
+        <v>4.33699504E8</v>
       </c>
       <c r="AF152" s="14" t="inlineStr"/>
       <c r="AG152" s="14" t="inlineStr"/>
@@ -9474,20 +9474,20 @@
         <v>1.997827308E10</v>
       </c>
       <c r="X153" s="14" t="n">
-        <v>3.526847916E9</v>
+        <v>3.536038216E9</v>
       </c>
       <c r="Y153" s="14" t="inlineStr"/>
       <c r="Z153" s="14" t="n">
-        <v>2.3505120996E10</v>
+        <v>2.3514311296E10</v>
       </c>
       <c r="AA153" s="14" t="inlineStr"/>
       <c r="AB153" s="14" t="inlineStr"/>
       <c r="AC153" s="15" t="n">
-        <v>0.9815069670977007</v>
+        <v>0.9818907278739696</v>
       </c>
       <c r="AD153" s="15" t="inlineStr"/>
       <c r="AE153" s="14" t="n">
-        <v>4.42871004E8</v>
+        <v>4.33680704E8</v>
       </c>
       <c r="AF153" s="14" t="inlineStr"/>
       <c r="AG153" s="14" t="inlineStr"/>
@@ -9638,7 +9638,7 @@
       <c r="O156" s="13" t="inlineStr"/>
       <c r="P156" s="13" t="inlineStr"/>
       <c r="Q156" s="14" t="n">
-        <v>2.6949388E10</v>
+        <v>2.6949535E10</v>
       </c>
       <c r="R156" s="14" t="inlineStr"/>
       <c r="S156" s="14" t="n">
@@ -9660,11 +9660,11 @@
       <c r="AA156" s="14" t="inlineStr"/>
       <c r="AB156" s="14" t="inlineStr"/>
       <c r="AC156" s="15" t="n">
-        <v>0.9856281067310323</v>
+        <v>0.9856227304849602</v>
       </c>
       <c r="AD156" s="15" t="inlineStr"/>
       <c r="AE156" s="14" t="n">
-        <v>3.87313728E8</v>
+        <v>3.87460728E8</v>
       </c>
       <c r="AF156" s="14" t="inlineStr"/>
       <c r="AG156" s="14" t="inlineStr"/>
@@ -11148,7 +11148,7 @@
       <c r="O182" s="13" t="inlineStr"/>
       <c r="P182" s="13" t="inlineStr"/>
       <c r="Q182" s="14" t="n">
-        <v>1.78416E9</v>
+        <v>1.82808E9</v>
       </c>
       <c r="R182" s="14" t="inlineStr"/>
       <c r="S182" s="14" t="n">
@@ -11170,11 +11170,11 @@
       <c r="AA182" s="14" t="inlineStr"/>
       <c r="AB182" s="14" t="inlineStr"/>
       <c r="AC182" s="15" t="n">
-        <v>0.871901062684961</v>
+        <v>0.8509534593672049</v>
       </c>
       <c r="AD182" s="15" t="inlineStr"/>
       <c r="AE182" s="14" t="n">
-        <v>2.28549E8</v>
+        <v>2.72469E8</v>
       </c>
       <c r="AF182" s="14" t="inlineStr"/>
       <c r="AG182" s="14" t="inlineStr"/>
@@ -11205,7 +11205,7 @@
       <c r="O183" s="13" t="inlineStr"/>
       <c r="P183" s="13" t="inlineStr"/>
       <c r="Q183" s="14" t="n">
-        <v>1.68E8</v>
+        <v>1.764E8</v>
       </c>
       <c r="R183" s="14" t="inlineStr"/>
       <c r="S183" s="14" t="n">
@@ -11227,11 +11227,11 @@
       <c r="AA183" s="14" t="inlineStr"/>
       <c r="AB183" s="14" t="inlineStr"/>
       <c r="AC183" s="15" t="n">
-        <v>0.8766666666666667</v>
+        <v>0.834920634920635</v>
       </c>
       <c r="AD183" s="15" t="inlineStr"/>
       <c r="AE183" s="14" t="n">
-        <v>2.072E7</v>
+        <v>2.912E7</v>
       </c>
       <c r="AF183" s="14" t="inlineStr"/>
       <c r="AG183" s="14" t="inlineStr"/>
@@ -11262,7 +11262,7 @@
       <c r="O184" s="13" t="inlineStr"/>
       <c r="P184" s="13" t="inlineStr"/>
       <c r="Q184" s="14" t="n">
-        <v>1.61616E9</v>
+        <v>1.65168E9</v>
       </c>
       <c r="R184" s="14" t="inlineStr"/>
       <c r="S184" s="14" t="n">
@@ -11284,11 +11284,11 @@
       <c r="AA184" s="14" t="inlineStr"/>
       <c r="AB184" s="14" t="inlineStr"/>
       <c r="AC184" s="15" t="n">
-        <v>0.8714056776556777</v>
+        <v>0.852665770609319</v>
       </c>
       <c r="AD184" s="15" t="inlineStr"/>
       <c r="AE184" s="14" t="n">
-        <v>2.07829E8</v>
+        <v>2.43349E8</v>
       </c>
       <c r="AF184" s="14" t="inlineStr"/>
       <c r="AG184" s="14" t="inlineStr"/>
@@ -11325,7 +11325,7 @@
       <c r="O185" s="13" t="inlineStr"/>
       <c r="P185" s="13" t="inlineStr"/>
       <c r="Q185" s="14" t="n">
-        <v>1.3046454E10</v>
+        <v>1.3002681E10</v>
       </c>
       <c r="R185" s="14" t="inlineStr"/>
       <c r="S185" s="14" t="n">
@@ -11347,11 +11347,11 @@
       <c r="AA185" s="14" t="inlineStr"/>
       <c r="AB185" s="14" t="inlineStr"/>
       <c r="AC185" s="15" t="n">
-        <v>0.9923814588239839</v>
+        <v>0.9957222708916723</v>
       </c>
       <c r="AD185" s="15" t="inlineStr"/>
       <c r="AE185" s="14" t="n">
-        <v>9.9394947E7</v>
+        <v>5.5621947E7</v>
       </c>
       <c r="AF185" s="14" t="inlineStr"/>
       <c r="AG185" s="14" t="inlineStr"/>
@@ -11382,7 +11382,7 @@
       <c r="O186" s="13" t="inlineStr"/>
       <c r="P186" s="13" t="inlineStr"/>
       <c r="Q186" s="14" t="n">
-        <v>1.1472E10</v>
+        <v>1.1428224E10</v>
       </c>
       <c r="R186" s="14" t="inlineStr"/>
       <c r="S186" s="14" t="n">
@@ -11404,11 +11404,11 @@
       <c r="AA186" s="14" t="inlineStr"/>
       <c r="AB186" s="14" t="inlineStr"/>
       <c r="AC186" s="15" t="n">
-        <v>0.9913367919281729</v>
+        <v>0.995134123814864</v>
       </c>
       <c r="AD186" s="15" t="inlineStr"/>
       <c r="AE186" s="14" t="n">
-        <v>9.9384323E7</v>
+        <v>5.5608323E7</v>
       </c>
       <c r="AF186" s="14" t="inlineStr"/>
       <c r="AG186" s="14" t="inlineStr"/>
@@ -11496,7 +11496,7 @@
       <c r="O188" s="13" t="inlineStr"/>
       <c r="P188" s="13" t="inlineStr"/>
       <c r="Q188" s="14" t="n">
-        <v>7.89135E8</v>
+        <v>7.89138E8</v>
       </c>
       <c r="R188" s="14" t="inlineStr"/>
       <c r="S188" s="14" t="n">
@@ -11518,11 +11518,11 @@
       <c r="AA188" s="14" t="inlineStr"/>
       <c r="AB188" s="14" t="inlineStr"/>
       <c r="AC188" s="15" t="n">
-        <v>0.9999994703060946</v>
+        <v>0.999995668691661</v>
       </c>
       <c r="AD188" s="15" t="inlineStr"/>
       <c r="AE188" s="14" t="n">
-        <v>418.0</v>
+        <v>3418.0</v>
       </c>
       <c r="AF188" s="14" t="inlineStr"/>
       <c r="AG188" s="14" t="inlineStr"/>
@@ -11572,20 +11572,20 @@
         <v>6.228754056E9</v>
       </c>
       <c r="X189" s="25" t="n">
-        <v>2.27165485E8</v>
+        <v>5.99870547E8</v>
       </c>
       <c r="Y189" s="25" t="inlineStr"/>
       <c r="Z189" s="25" t="n">
-        <v>6.455919541E9</v>
+        <v>6.828624603E9</v>
       </c>
       <c r="AA189" s="25" t="inlineStr"/>
       <c r="AB189" s="25" t="inlineStr"/>
       <c r="AC189" s="26" t="n">
-        <v>0.9293391894235967</v>
+        <v>0.9829906356681544</v>
       </c>
       <c r="AD189" s="26" t="inlineStr"/>
       <c r="AE189" s="25" t="n">
-        <v>4.90865459E8</v>
+        <v>1.18160397E8</v>
       </c>
       <c r="AF189" s="25" t="inlineStr"/>
       <c r="AG189" s="25" t="inlineStr"/>
@@ -11622,7 +11622,7 @@
       <c r="O190" s="13" t="inlineStr"/>
       <c r="P190" s="13" t="inlineStr"/>
       <c r="Q190" s="14" t="n">
-        <v>5.006041E9</v>
+        <v>5.008716E9</v>
       </c>
       <c r="R190" s="14" t="inlineStr"/>
       <c r="S190" s="14" t="n">
@@ -11635,20 +11635,20 @@
         <v>4.783558496E9</v>
       </c>
       <c r="X190" s="14" t="n">
-        <v>1.31977006E8</v>
+        <v>1.9710595E8</v>
       </c>
       <c r="Y190" s="14" t="inlineStr"/>
       <c r="Z190" s="14" t="n">
-        <v>4.915535502E9</v>
+        <v>4.980664446E9</v>
       </c>
       <c r="AA190" s="14" t="inlineStr"/>
       <c r="AB190" s="14" t="inlineStr"/>
       <c r="AC190" s="15" t="n">
-        <v>0.9819207437573924</v>
+        <v>0.9943994520751426</v>
       </c>
       <c r="AD190" s="15" t="inlineStr"/>
       <c r="AE190" s="14" t="n">
-        <v>9.0505498E7</v>
+        <v>2.8051554E7</v>
       </c>
       <c r="AF190" s="14" t="inlineStr"/>
       <c r="AG190" s="14" t="inlineStr"/>
@@ -11685,7 +11685,7 @@
       <c r="O191" s="13" t="inlineStr"/>
       <c r="P191" s="13" t="inlineStr"/>
       <c r="Q191" s="14" t="n">
-        <v>1.890817E9</v>
+        <v>1.892887E9</v>
       </c>
       <c r="R191" s="14" t="inlineStr"/>
       <c r="S191" s="14" t="n">
@@ -11698,20 +11698,20 @@
         <v>1.777909494E9</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>9.3544738E7</v>
+        <v>1.07421314E8</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
-        <v>1.871454232E9</v>
+        <v>1.885330808E9</v>
       </c>
       <c r="AA191" s="14" t="inlineStr"/>
       <c r="AB191" s="14" t="inlineStr"/>
       <c r="AC191" s="15" t="n">
-        <v>0.9897595758870372</v>
+        <v>0.9960081124758108</v>
       </c>
       <c r="AD191" s="15" t="inlineStr"/>
       <c r="AE191" s="14" t="n">
-        <v>1.9362768E7</v>
+        <v>7556192.0</v>
       </c>
       <c r="AF191" s="14" t="inlineStr"/>
       <c r="AG191" s="14" t="inlineStr"/>
@@ -11856,7 +11856,7 @@
       <c r="O194" s="13" t="inlineStr"/>
       <c r="P194" s="13" t="inlineStr"/>
       <c r="Q194" s="14" t="n">
-        <v>9.393E7</v>
+        <v>9.6E7</v>
       </c>
       <c r="R194" s="14" t="inlineStr"/>
       <c r="S194" s="14" t="n">
@@ -11869,20 +11869,20 @@
         <v>5.5184254E7</v>
       </c>
       <c r="X194" s="14" t="n">
-        <v>1.9543138E7</v>
+        <v>3.3419714E7</v>
       </c>
       <c r="Y194" s="14" t="inlineStr"/>
       <c r="Z194" s="14" t="n">
-        <v>7.4727392E7</v>
+        <v>8.8603968E7</v>
       </c>
       <c r="AA194" s="14" t="inlineStr"/>
       <c r="AB194" s="14" t="inlineStr"/>
       <c r="AC194" s="15" t="n">
-        <v>0.7955646971148728</v>
+        <v>0.922958</v>
       </c>
       <c r="AD194" s="15" t="inlineStr"/>
       <c r="AE194" s="14" t="n">
-        <v>1.9202608E7</v>
+        <v>7396032.0</v>
       </c>
       <c r="AF194" s="14" t="inlineStr"/>
       <c r="AG194" s="14" t="inlineStr"/>
@@ -12304,7 +12304,7 @@
       <c r="O202" s="13" t="inlineStr"/>
       <c r="P202" s="13" t="inlineStr"/>
       <c r="Q202" s="14" t="n">
-        <v>1.23E7</v>
+        <v>1.488E7</v>
       </c>
       <c r="R202" s="14" t="inlineStr"/>
       <c r="S202" s="14" t="n">
@@ -12317,20 +12317,20 @@
         <v>9417000.0</v>
       </c>
       <c r="X202" s="14" t="n">
-        <v>1380500.0</v>
+        <v>3215000.0</v>
       </c>
       <c r="Y202" s="14" t="inlineStr"/>
       <c r="Z202" s="14" t="n">
-        <v>1.07975E7</v>
+        <v>1.2632E7</v>
       </c>
       <c r="AA202" s="14" t="inlineStr"/>
       <c r="AB202" s="14" t="inlineStr"/>
       <c r="AC202" s="15" t="n">
-        <v>0.8778455284552845</v>
+        <v>0.8489247311827957</v>
       </c>
       <c r="AD202" s="15" t="inlineStr"/>
       <c r="AE202" s="14" t="n">
-        <v>1502500.0</v>
+        <v>2248000.0</v>
       </c>
       <c r="AF202" s="14" t="inlineStr"/>
       <c r="AG202" s="14" t="inlineStr"/>
@@ -12361,7 +12361,7 @@
       <c r="O203" s="13" t="inlineStr"/>
       <c r="P203" s="13" t="inlineStr"/>
       <c r="Q203" s="14" t="n">
-        <v>7800000.0</v>
+        <v>1.038E7</v>
       </c>
       <c r="R203" s="14" t="inlineStr"/>
       <c r="S203" s="14" t="n">
@@ -12374,20 +12374,20 @@
         <v>5781000.0</v>
       </c>
       <c r="X203" s="14" t="n">
-        <v>1380500.0</v>
+        <v>2407000.0</v>
       </c>
       <c r="Y203" s="14" t="inlineStr"/>
       <c r="Z203" s="14" t="n">
-        <v>7161500.0</v>
+        <v>8188000.0</v>
       </c>
       <c r="AA203" s="14" t="inlineStr"/>
       <c r="AB203" s="14" t="inlineStr"/>
       <c r="AC203" s="15" t="n">
-        <v>0.9181410256410256</v>
+        <v>0.7888246628131022</v>
       </c>
       <c r="AD203" s="15" t="inlineStr"/>
       <c r="AE203" s="14" t="n">
-        <v>638500.0</v>
+        <v>2192000.0</v>
       </c>
       <c r="AF203" s="14" t="inlineStr"/>
       <c r="AG203" s="14" t="inlineStr"/>
@@ -12431,20 +12431,20 @@
         <v>3636000.0</v>
       </c>
       <c r="X204" s="14" t="n">
-        <v>0.0</v>
+        <v>808000.0</v>
       </c>
       <c r="Y204" s="14" t="inlineStr"/>
       <c r="Z204" s="14" t="n">
-        <v>3636000.0</v>
+        <v>4444000.0</v>
       </c>
       <c r="AA204" s="14" t="inlineStr"/>
       <c r="AB204" s="14" t="inlineStr"/>
       <c r="AC204" s="15" t="n">
-        <v>0.808</v>
+        <v>0.9875555555555555</v>
       </c>
       <c r="AD204" s="15" t="inlineStr"/>
       <c r="AE204" s="14" t="n">
-        <v>864000.0</v>
+        <v>56000.0</v>
       </c>
       <c r="AF204" s="14" t="inlineStr"/>
       <c r="AG204" s="14" t="inlineStr"/>
@@ -12481,7 +12481,7 @@
       <c r="O205" s="13" t="inlineStr"/>
       <c r="P205" s="13" t="inlineStr"/>
       <c r="Q205" s="14" t="n">
-        <v>8.0556E7</v>
+        <v>7.8581E7</v>
       </c>
       <c r="R205" s="14" t="inlineStr"/>
       <c r="S205" s="14" t="n">
@@ -12494,20 +12494,20 @@
         <v>5.526601E7</v>
       </c>
       <c r="X205" s="14" t="n">
-        <v>0.0</v>
+        <v>1.23661E7</v>
       </c>
       <c r="Y205" s="14" t="inlineStr"/>
       <c r="Z205" s="14" t="n">
-        <v>5.526601E7</v>
+        <v>6.763211E7</v>
       </c>
       <c r="AA205" s="14" t="inlineStr"/>
       <c r="AB205" s="14" t="inlineStr"/>
       <c r="AC205" s="15" t="n">
-        <v>0.6860570286508764</v>
+        <v>0.8606674641452768</v>
       </c>
       <c r="AD205" s="15" t="inlineStr"/>
       <c r="AE205" s="14" t="n">
-        <v>2.528999E7</v>
+        <v>1.094889E7</v>
       </c>
       <c r="AF205" s="14" t="inlineStr"/>
       <c r="AG205" s="14" t="inlineStr"/>
@@ -12538,7 +12538,7 @@
       <c r="O206" s="13" t="inlineStr"/>
       <c r="P206" s="13" t="inlineStr"/>
       <c r="Q206" s="14" t="n">
-        <v>7.4476E7</v>
+        <v>7.2501E7</v>
       </c>
       <c r="R206" s="14" t="inlineStr"/>
       <c r="S206" s="14" t="n">
@@ -12551,20 +12551,20 @@
         <v>5.526601E7</v>
       </c>
       <c r="X206" s="14" t="n">
-        <v>0.0</v>
+        <v>9616100.0</v>
       </c>
       <c r="Y206" s="14" t="inlineStr"/>
       <c r="Z206" s="14" t="n">
-        <v>5.526601E7</v>
+        <v>6.488211E7</v>
       </c>
       <c r="AA206" s="14" t="inlineStr"/>
       <c r="AB206" s="14" t="inlineStr"/>
       <c r="AC206" s="15" t="n">
-        <v>0.7420646919813094</v>
+        <v>0.8949133115405304</v>
       </c>
       <c r="AD206" s="15" t="inlineStr"/>
       <c r="AE206" s="14" t="n">
-        <v>1.920999E7</v>
+        <v>7618890.0</v>
       </c>
       <c r="AF206" s="14" t="inlineStr"/>
       <c r="AG206" s="14" t="inlineStr"/>
@@ -12608,20 +12608,20 @@
         <v>0.0</v>
       </c>
       <c r="X207" s="14" t="n">
-        <v>0.0</v>
+        <v>2750000.0</v>
       </c>
       <c r="Y207" s="14" t="inlineStr"/>
       <c r="Z207" s="14" t="n">
-        <v>0.0</v>
+        <v>2750000.0</v>
       </c>
       <c r="AA207" s="14" t="inlineStr"/>
       <c r="AB207" s="14" t="inlineStr"/>
       <c r="AC207" s="15" t="n">
-        <v>0.0</v>
+        <v>0.45230263157894735</v>
       </c>
       <c r="AD207" s="15" t="inlineStr"/>
       <c r="AE207" s="14" t="n">
-        <v>6080000.0</v>
+        <v>3330000.0</v>
       </c>
       <c r="AF207" s="14" t="inlineStr"/>
       <c r="AG207" s="14" t="inlineStr"/>
@@ -12848,20 +12848,20 @@
         <v>2.936691192E9</v>
       </c>
       <c r="X211" s="14" t="n">
-        <v>3.7051768E7</v>
+        <v>7.4103536E7</v>
       </c>
       <c r="Y211" s="14" t="inlineStr"/>
       <c r="Z211" s="14" t="n">
-        <v>2.97374296E9</v>
+        <v>3.010794728E9</v>
       </c>
       <c r="AA211" s="14" t="inlineStr"/>
       <c r="AB211" s="14" t="inlineStr"/>
       <c r="AC211" s="15" t="n">
-        <v>0.987505665199338</v>
+        <v>0.9998096307060446</v>
       </c>
       <c r="AD211" s="15" t="inlineStr"/>
       <c r="AE211" s="14" t="n">
-        <v>3.762504E7</v>
+        <v>573272.0</v>
       </c>
       <c r="AF211" s="14" t="inlineStr"/>
       <c r="AG211" s="14" t="inlineStr"/>
@@ -12962,20 +12962,20 @@
         <v>1.0331888E8</v>
       </c>
       <c r="X213" s="14" t="n">
-        <v>9468528.0</v>
+        <v>1.8937056E7</v>
       </c>
       <c r="Y213" s="14" t="inlineStr"/>
       <c r="Z213" s="14" t="n">
-        <v>1.12787408E8</v>
+        <v>1.22255936E8</v>
       </c>
       <c r="AA213" s="14" t="inlineStr"/>
       <c r="AB213" s="14" t="inlineStr"/>
       <c r="AC213" s="15" t="n">
-        <v>0.9199625448613377</v>
+        <v>0.9971936052202284</v>
       </c>
       <c r="AD213" s="15" t="inlineStr"/>
       <c r="AE213" s="14" t="n">
-        <v>9812592.0</v>
+        <v>344064.0</v>
       </c>
       <c r="AF213" s="14" t="inlineStr"/>
       <c r="AG213" s="14" t="inlineStr"/>
@@ -13190,20 +13190,20 @@
         <v>2.2953312E7</v>
       </c>
       <c r="X217" s="14" t="n">
-        <v>2.2953312E7</v>
+        <v>4.5906624E7</v>
       </c>
       <c r="Y217" s="14" t="inlineStr"/>
       <c r="Z217" s="14" t="n">
-        <v>4.5906624E7</v>
+        <v>6.8859936E7</v>
       </c>
       <c r="AA217" s="14" t="inlineStr"/>
       <c r="AB217" s="14" t="inlineStr"/>
       <c r="AC217" s="15" t="n">
-        <v>0.6662790130624093</v>
+        <v>0.9994185195936139</v>
       </c>
       <c r="AD217" s="15" t="inlineStr"/>
       <c r="AE217" s="14" t="n">
-        <v>2.2993376E7</v>
+        <v>40064.0</v>
       </c>
       <c r="AF217" s="14" t="inlineStr"/>
       <c r="AG217" s="14" t="inlineStr"/>
@@ -13247,20 +13247,20 @@
         <v>4629928.0</v>
       </c>
       <c r="X218" s="14" t="n">
-        <v>4629928.0</v>
+        <v>9259856.0</v>
       </c>
       <c r="Y218" s="14" t="inlineStr"/>
       <c r="Z218" s="14" t="n">
-        <v>9259856.0</v>
+        <v>1.3889784E7</v>
       </c>
       <c r="AA218" s="14" t="inlineStr"/>
       <c r="AB218" s="14" t="inlineStr"/>
       <c r="AC218" s="15" t="n">
-        <v>0.6666562994960403</v>
+        <v>0.9999844492440605</v>
       </c>
       <c r="AD218" s="15" t="inlineStr"/>
       <c r="AE218" s="14" t="n">
-        <v>4630144.0</v>
+        <v>216.0</v>
       </c>
       <c r="AF218" s="14" t="inlineStr"/>
       <c r="AG218" s="14" t="inlineStr"/>
@@ -13297,7 +13297,7 @@
       <c r="O219" s="13" t="inlineStr"/>
       <c r="P219" s="13" t="inlineStr"/>
       <c r="Q219" s="14" t="n">
-        <v>7.00144E8</v>
+        <v>6.92704E8</v>
       </c>
       <c r="R219" s="14" t="inlineStr"/>
       <c r="S219" s="14" t="n">
@@ -13310,20 +13310,20 @@
         <v>6.39842407E8</v>
       </c>
       <c r="X219" s="14" t="n">
-        <v>4.9005042E7</v>
+        <v>5.2026307E7</v>
       </c>
       <c r="Y219" s="14" t="inlineStr"/>
       <c r="Z219" s="14" t="n">
-        <v>6.88847449E8</v>
+        <v>6.91868714E8</v>
       </c>
       <c r="AA219" s="14" t="inlineStr"/>
       <c r="AB219" s="14" t="inlineStr"/>
       <c r="AC219" s="15" t="n">
-        <v>0.9838653891199525</v>
+        <v>0.9987941660507229</v>
       </c>
       <c r="AD219" s="15" t="inlineStr"/>
       <c r="AE219" s="14" t="n">
-        <v>1.1296551E7</v>
+        <v>835286.0</v>
       </c>
       <c r="AF219" s="14" t="inlineStr"/>
       <c r="AG219" s="14" t="inlineStr"/>
@@ -13360,7 +13360,7 @@
       <c r="O220" s="13" t="inlineStr"/>
       <c r="P220" s="13" t="inlineStr"/>
       <c r="Q220" s="14" t="n">
-        <v>5.16E8</v>
+        <v>5.0946E8</v>
       </c>
       <c r="R220" s="14" t="inlineStr"/>
       <c r="S220" s="14" t="n">
@@ -13382,11 +13382,11 @@
       <c r="AA220" s="14" t="inlineStr"/>
       <c r="AB220" s="14" t="inlineStr"/>
       <c r="AC220" s="15" t="n">
-        <v>0.9872100562015503</v>
+        <v>0.9998829917952342</v>
       </c>
       <c r="AD220" s="15" t="inlineStr"/>
       <c r="AE220" s="14" t="n">
-        <v>6599611.0</v>
+        <v>59611.0</v>
       </c>
       <c r="AF220" s="14" t="inlineStr"/>
       <c r="AG220" s="14" t="inlineStr"/>
@@ -13417,7 +13417,7 @@
       <c r="O221" s="13" t="inlineStr"/>
       <c r="P221" s="13" t="inlineStr"/>
       <c r="Q221" s="14" t="n">
-        <v>5.16E8</v>
+        <v>5.0946E8</v>
       </c>
       <c r="R221" s="14" t="inlineStr"/>
       <c r="S221" s="14" t="n">
@@ -13439,11 +13439,11 @@
       <c r="AA221" s="14" t="inlineStr"/>
       <c r="AB221" s="14" t="inlineStr"/>
       <c r="AC221" s="15" t="n">
-        <v>0.9872100562015503</v>
+        <v>0.9998829917952342</v>
       </c>
       <c r="AD221" s="15" t="inlineStr"/>
       <c r="AE221" s="14" t="n">
-        <v>6599611.0</v>
+        <v>59611.0</v>
       </c>
       <c r="AF221" s="14" t="inlineStr"/>
       <c r="AG221" s="14" t="inlineStr"/>
@@ -13600,7 +13600,7 @@
       <c r="O224" s="13" t="inlineStr"/>
       <c r="P224" s="13" t="inlineStr"/>
       <c r="Q224" s="14" t="n">
-        <v>3.3444E7</v>
+        <v>3.2544E7</v>
       </c>
       <c r="R224" s="14" t="inlineStr"/>
       <c r="S224" s="14" t="n">
@@ -13613,20 +13613,20 @@
         <v>3.08218E7</v>
       </c>
       <c r="X224" s="14" t="n">
-        <v>604300.0</v>
+        <v>1639100.0</v>
       </c>
       <c r="Y224" s="14" t="inlineStr"/>
       <c r="Z224" s="14" t="n">
-        <v>3.14261E7</v>
+        <v>3.24609E7</v>
       </c>
       <c r="AA224" s="14" t="inlineStr"/>
       <c r="AB224" s="14" t="inlineStr"/>
       <c r="AC224" s="15" t="n">
-        <v>0.9396633177849539</v>
+        <v>0.9974465339233038</v>
       </c>
       <c r="AD224" s="15" t="inlineStr"/>
       <c r="AE224" s="14" t="n">
-        <v>2017900.0</v>
+        <v>83100.0</v>
       </c>
       <c r="AF224" s="14" t="inlineStr"/>
       <c r="AG224" s="14" t="inlineStr"/>
@@ -13657,7 +13657,7 @@
       <c r="O225" s="13" t="inlineStr"/>
       <c r="P225" s="13" t="inlineStr"/>
       <c r="Q225" s="14" t="n">
-        <v>3.3444E7</v>
+        <v>3.2544E7</v>
       </c>
       <c r="R225" s="14" t="inlineStr"/>
       <c r="S225" s="14" t="n">
@@ -13670,20 +13670,20 @@
         <v>3.08218E7</v>
       </c>
       <c r="X225" s="14" t="n">
-        <v>604300.0</v>
+        <v>1639100.0</v>
       </c>
       <c r="Y225" s="14" t="inlineStr"/>
       <c r="Z225" s="14" t="n">
-        <v>3.14261E7</v>
+        <v>3.24609E7</v>
       </c>
       <c r="AA225" s="14" t="inlineStr"/>
       <c r="AB225" s="14" t="inlineStr"/>
       <c r="AC225" s="15" t="n">
-        <v>0.9396633177849539</v>
+        <v>0.9974465339233038</v>
       </c>
       <c r="AD225" s="15" t="inlineStr"/>
       <c r="AE225" s="14" t="n">
-        <v>2017900.0</v>
+        <v>83100.0</v>
       </c>
       <c r="AF225" s="14" t="inlineStr"/>
       <c r="AG225" s="14" t="inlineStr"/>
@@ -13733,20 +13733,20 @@
         <v>1.33021464E8</v>
       </c>
       <c r="X226" s="14" t="n">
-        <v>9250750.0</v>
+        <v>1.1237215E7</v>
       </c>
       <c r="Y226" s="14" t="inlineStr"/>
       <c r="Z226" s="14" t="n">
-        <v>1.42272214E8</v>
+        <v>1.44258679E8</v>
       </c>
       <c r="AA226" s="14" t="inlineStr"/>
       <c r="AB226" s="14" t="inlineStr"/>
       <c r="AC226" s="15" t="n">
-        <v>0.9832219350380097</v>
+        <v>0.9969500967519005</v>
       </c>
       <c r="AD226" s="15" t="inlineStr"/>
       <c r="AE226" s="14" t="n">
-        <v>2427786.0</v>
+        <v>441321.0</v>
       </c>
       <c r="AF226" s="14" t="inlineStr"/>
       <c r="AG226" s="14" t="inlineStr"/>
@@ -13820,7 +13820,7 @@
       <c r="O228" s="13" t="inlineStr"/>
       <c r="P228" s="13" t="inlineStr"/>
       <c r="Q228" s="14" t="n">
-        <v>1.146E8</v>
+        <v>1.1508E8</v>
       </c>
       <c r="R228" s="14" t="inlineStr"/>
       <c r="S228" s="14" t="n">
@@ -13833,20 +13833,20 @@
         <v>1.044355E8</v>
       </c>
       <c r="X228" s="14" t="n">
-        <v>9250750.0</v>
+        <v>1.029815E7</v>
       </c>
       <c r="Y228" s="14" t="inlineStr"/>
       <c r="Z228" s="14" t="n">
-        <v>1.1368625E8</v>
+        <v>1.1473365E8</v>
       </c>
       <c r="AA228" s="14" t="inlineStr"/>
       <c r="AB228" s="14" t="inlineStr"/>
       <c r="AC228" s="15" t="n">
-        <v>0.9920266143106458</v>
+        <v>0.996990354535975</v>
       </c>
       <c r="AD228" s="15" t="inlineStr"/>
       <c r="AE228" s="14" t="n">
-        <v>913750.0</v>
+        <v>346350.0</v>
       </c>
       <c r="AF228" s="14" t="inlineStr"/>
       <c r="AG228" s="14" t="inlineStr"/>
@@ -13877,7 +13877,7 @@
       <c r="O229" s="13" t="inlineStr"/>
       <c r="P229" s="13" t="inlineStr"/>
       <c r="Q229" s="14" t="n">
-        <v>3.01E7</v>
+        <v>2.962E7</v>
       </c>
       <c r="R229" s="14" t="inlineStr"/>
       <c r="S229" s="14" t="n">
@@ -13890,20 +13890,20 @@
         <v>2.8585964E7</v>
       </c>
       <c r="X229" s="14" t="n">
-        <v>0.0</v>
+        <v>939065.0</v>
       </c>
       <c r="Y229" s="14" t="inlineStr"/>
       <c r="Z229" s="14" t="n">
-        <v>2.8585964E7</v>
+        <v>2.9525029E7</v>
       </c>
       <c r="AA229" s="14" t="inlineStr"/>
       <c r="AB229" s="14" t="inlineStr"/>
       <c r="AC229" s="15" t="n">
-        <v>0.9496998006644518</v>
+        <v>0.9967936866981769</v>
       </c>
       <c r="AD229" s="15" t="inlineStr"/>
       <c r="AE229" s="14" t="n">
-        <v>1514036.0</v>
+        <v>94971.0</v>
       </c>
       <c r="AF229" s="14" t="inlineStr"/>
       <c r="AG229" s="14" t="inlineStr"/>
@@ -13940,7 +13940,7 @@
       <c r="O230" s="13" t="inlineStr"/>
       <c r="P230" s="13" t="inlineStr"/>
       <c r="Q230" s="14" t="n">
-        <v>1.10842E9</v>
+        <v>1.093185E9</v>
       </c>
       <c r="R230" s="14" t="inlineStr"/>
       <c r="S230" s="14" t="n">
@@ -13953,20 +13953,20 @@
         <v>6.74613153E8</v>
       </c>
       <c r="X230" s="14" t="n">
-        <v>4.5703437E7</v>
+        <v>3.2949829E8</v>
       </c>
       <c r="Y230" s="14" t="inlineStr"/>
       <c r="Z230" s="14" t="n">
-        <v>7.2031659E8</v>
+        <v>1.004111443E9</v>
       </c>
       <c r="AA230" s="14" t="inlineStr"/>
       <c r="AB230" s="14" t="inlineStr"/>
       <c r="AC230" s="15" t="n">
-        <v>0.6498588892297144</v>
+        <v>0.9185192286758417</v>
       </c>
       <c r="AD230" s="15" t="inlineStr"/>
       <c r="AE230" s="14" t="n">
-        <v>3.8810341E8</v>
+        <v>8.9073557E7</v>
       </c>
       <c r="AF230" s="14" t="inlineStr"/>
       <c r="AG230" s="14" t="inlineStr"/>
@@ -14016,20 +14016,20 @@
         <v>2.179125E8</v>
       </c>
       <c r="X231" s="14" t="n">
-        <v>0.0</v>
+        <v>2.2065E7</v>
       </c>
       <c r="Y231" s="14" t="inlineStr"/>
       <c r="Z231" s="14" t="n">
-        <v>2.179125E8</v>
+        <v>2.399775E8</v>
       </c>
       <c r="AA231" s="14" t="inlineStr"/>
       <c r="AB231" s="14" t="inlineStr"/>
       <c r="AC231" s="15" t="n">
-        <v>0.90796875</v>
+        <v>0.99990625</v>
       </c>
       <c r="AD231" s="15" t="inlineStr"/>
       <c r="AE231" s="14" t="n">
-        <v>2.20875E7</v>
+        <v>22500.0</v>
       </c>
       <c r="AF231" s="14" t="inlineStr"/>
       <c r="AG231" s="14" t="inlineStr"/>
@@ -14073,20 +14073,20 @@
         <v>1.67915E8</v>
       </c>
       <c r="X232" s="14" t="n">
-        <v>0.0</v>
+        <v>1.2065E7</v>
       </c>
       <c r="Y232" s="14" t="inlineStr"/>
       <c r="Z232" s="14" t="n">
-        <v>1.67915E8</v>
+        <v>1.7998E8</v>
       </c>
       <c r="AA232" s="14" t="inlineStr"/>
       <c r="AB232" s="14" t="inlineStr"/>
       <c r="AC232" s="15" t="n">
-        <v>0.9328611111111111</v>
+        <v>0.9998888888888889</v>
       </c>
       <c r="AD232" s="15" t="inlineStr"/>
       <c r="AE232" s="14" t="n">
-        <v>1.2085E7</v>
+        <v>20000.0</v>
       </c>
       <c r="AF232" s="14" t="inlineStr"/>
       <c r="AG232" s="14" t="inlineStr"/>
@@ -14130,20 +14130,20 @@
         <v>4.99975E7</v>
       </c>
       <c r="X233" s="14" t="n">
-        <v>0.0</v>
+        <v>1.0E7</v>
       </c>
       <c r="Y233" s="14" t="inlineStr"/>
       <c r="Z233" s="14" t="n">
-        <v>4.99975E7</v>
+        <v>5.99975E7</v>
       </c>
       <c r="AA233" s="14" t="inlineStr"/>
       <c r="AB233" s="14" t="inlineStr"/>
       <c r="AC233" s="15" t="n">
-        <v>0.8332916666666667</v>
+        <v>0.9999583333333333</v>
       </c>
       <c r="AD233" s="15" t="inlineStr"/>
       <c r="AE233" s="14" t="n">
-        <v>1.00025E7</v>
+        <v>2500.0</v>
       </c>
       <c r="AF233" s="14" t="inlineStr"/>
       <c r="AG233" s="14" t="inlineStr"/>
@@ -14300,7 +14300,7 @@
       <c r="O236" s="13" t="inlineStr"/>
       <c r="P236" s="13" t="inlineStr"/>
       <c r="Q236" s="14" t="n">
-        <v>3.5259E8</v>
+        <v>3.47E8</v>
       </c>
       <c r="R236" s="14" t="inlineStr"/>
       <c r="S236" s="14" t="n">
@@ -14313,20 +14313,20 @@
         <v>1.34221533E8</v>
       </c>
       <c r="X236" s="14" t="n">
-        <v>2.5076E7</v>
+        <v>1.508445E8</v>
       </c>
       <c r="Y236" s="14" t="inlineStr"/>
       <c r="Z236" s="14" t="n">
-        <v>1.59297533E8</v>
+        <v>2.85066033E8</v>
       </c>
       <c r="AA236" s="14" t="inlineStr"/>
       <c r="AB236" s="14" t="inlineStr"/>
       <c r="AC236" s="15" t="n">
-        <v>0.4517925437476956</v>
+        <v>0.8215159452449567</v>
       </c>
       <c r="AD236" s="15" t="inlineStr"/>
       <c r="AE236" s="14" t="n">
-        <v>1.93292467E8</v>
+        <v>6.1933967E7</v>
       </c>
       <c r="AF236" s="14" t="inlineStr"/>
       <c r="AG236" s="14" t="inlineStr"/>
@@ -14427,20 +14427,20 @@
         <v>2.1347299E7</v>
       </c>
       <c r="X238" s="14" t="n">
-        <v>0.0</v>
+        <v>1.47355E7</v>
       </c>
       <c r="Y238" s="14" t="inlineStr"/>
       <c r="Z238" s="14" t="n">
-        <v>2.1347299E7</v>
+        <v>3.6082799E7</v>
       </c>
       <c r="AA238" s="14" t="inlineStr"/>
       <c r="AB238" s="14" t="inlineStr"/>
       <c r="AC238" s="15" t="n">
-        <v>0.5723136461126005</v>
+        <v>0.9673672654155496</v>
       </c>
       <c r="AD238" s="15" t="inlineStr"/>
       <c r="AE238" s="14" t="n">
-        <v>1.5952701E7</v>
+        <v>1217201.0</v>
       </c>
       <c r="AF238" s="14" t="inlineStr"/>
       <c r="AG238" s="14" t="inlineStr"/>
@@ -14484,20 +14484,20 @@
         <v>2.5327E7</v>
       </c>
       <c r="X239" s="14" t="n">
-        <v>0.0</v>
+        <v>375000.0</v>
       </c>
       <c r="Y239" s="14" t="inlineStr"/>
       <c r="Z239" s="14" t="n">
-        <v>2.5327E7</v>
+        <v>2.5702E7</v>
       </c>
       <c r="AA239" s="14" t="inlineStr"/>
       <c r="AB239" s="14" t="inlineStr"/>
       <c r="AC239" s="15" t="n">
-        <v>0.9759922928709056</v>
+        <v>0.9904431599229288</v>
       </c>
       <c r="AD239" s="15" t="inlineStr"/>
       <c r="AE239" s="14" t="n">
-        <v>623000.0</v>
+        <v>248000.0</v>
       </c>
       <c r="AF239" s="14" t="inlineStr"/>
       <c r="AG239" s="14" t="inlineStr"/>
@@ -14585,7 +14585,7 @@
       <c r="O241" s="13" t="inlineStr"/>
       <c r="P241" s="13" t="inlineStr"/>
       <c r="Q241" s="14" t="n">
-        <v>1.156E8</v>
+        <v>1.236E8</v>
       </c>
       <c r="R241" s="14" t="inlineStr"/>
       <c r="S241" s="14" t="n">
@@ -14598,20 +14598,20 @@
         <v>4421000.0</v>
       </c>
       <c r="X241" s="14" t="n">
-        <v>2.5076E7</v>
+        <v>7.4724E7</v>
       </c>
       <c r="Y241" s="14" t="inlineStr"/>
       <c r="Z241" s="14" t="n">
-        <v>2.9497E7</v>
+        <v>7.9145E7</v>
       </c>
       <c r="AA241" s="14" t="inlineStr"/>
       <c r="AB241" s="14" t="inlineStr"/>
       <c r="AC241" s="15" t="n">
-        <v>0.2551643598615917</v>
+        <v>0.640331715210356</v>
       </c>
       <c r="AD241" s="15" t="inlineStr"/>
       <c r="AE241" s="14" t="n">
-        <v>8.6103E7</v>
+        <v>4.4455E7</v>
       </c>
       <c r="AF241" s="14" t="inlineStr"/>
       <c r="AG241" s="14" t="inlineStr"/>
@@ -14642,7 +14642,7 @@
       <c r="O242" s="13" t="inlineStr"/>
       <c r="P242" s="13" t="inlineStr"/>
       <c r="Q242" s="14" t="n">
-        <v>2800000.0</v>
+        <v>1400000.0</v>
       </c>
       <c r="R242" s="14" t="inlineStr"/>
       <c r="S242" s="14" t="n">
@@ -14664,11 +14664,11 @@
       <c r="AA242" s="14" t="inlineStr"/>
       <c r="AB242" s="14" t="inlineStr"/>
       <c r="AC242" s="15" t="n">
-        <v>0.4857142857142857</v>
+        <v>0.9714285714285714</v>
       </c>
       <c r="AD242" s="15" t="inlineStr"/>
       <c r="AE242" s="14" t="n">
-        <v>1440000.0</v>
+        <v>40000.0</v>
       </c>
       <c r="AF242" s="14" t="inlineStr"/>
       <c r="AG242" s="14" t="inlineStr"/>
@@ -14699,7 +14699,7 @@
       <c r="O243" s="13" t="inlineStr"/>
       <c r="P243" s="13" t="inlineStr"/>
       <c r="Q243" s="14" t="n">
-        <v>2.66E7</v>
+        <v>1.66E7</v>
       </c>
       <c r="R243" s="14" t="inlineStr"/>
       <c r="S243" s="14" t="n">
@@ -14721,11 +14721,11 @@
       <c r="AA243" s="14" t="inlineStr"/>
       <c r="AB243" s="14" t="inlineStr"/>
       <c r="AC243" s="15" t="n">
-        <v>0.45652714285714285</v>
+        <v>0.7315434939759036</v>
       </c>
       <c r="AD243" s="15" t="inlineStr"/>
       <c r="AE243" s="14" t="n">
-        <v>1.4456378E7</v>
+        <v>4456378.0</v>
       </c>
       <c r="AF243" s="14" t="inlineStr"/>
       <c r="AG243" s="14" t="inlineStr"/>
@@ -14756,7 +14756,7 @@
       <c r="O244" s="13" t="inlineStr"/>
       <c r="P244" s="13" t="inlineStr"/>
       <c r="Q244" s="14" t="n">
-        <v>1.443E7</v>
+        <v>1.444E7</v>
       </c>
       <c r="R244" s="14" t="inlineStr"/>
       <c r="S244" s="14" t="n">
@@ -14778,11 +14778,11 @@
       <c r="AA244" s="14" t="inlineStr"/>
       <c r="AB244" s="14" t="inlineStr"/>
       <c r="AC244" s="15" t="n">
-        <v>1.0</v>
+        <v>0.9993074792243767</v>
       </c>
       <c r="AD244" s="15" t="inlineStr"/>
       <c r="AE244" s="14" t="n">
-        <v>0.0</v>
+        <v>10000.0</v>
       </c>
       <c r="AF244" s="14" t="inlineStr"/>
       <c r="AG244" s="14" t="inlineStr"/>
@@ -14826,20 +14826,20 @@
         <v>1576500.0</v>
       </c>
       <c r="X245" s="14" t="n">
-        <v>0.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="Y245" s="14" t="inlineStr"/>
       <c r="Z245" s="14" t="n">
-        <v>1576500.0</v>
+        <v>3376500.0</v>
       </c>
       <c r="AA245" s="14" t="inlineStr"/>
       <c r="AB245" s="14" t="inlineStr"/>
       <c r="AC245" s="15" t="n">
-        <v>0.37987951807228915</v>
+        <v>0.8136144578313254</v>
       </c>
       <c r="AD245" s="15" t="inlineStr"/>
       <c r="AE245" s="14" t="n">
-        <v>2573500.0</v>
+        <v>773500.0</v>
       </c>
       <c r="AF245" s="14" t="inlineStr"/>
       <c r="AG245" s="14" t="inlineStr"/>
@@ -14927,7 +14927,7 @@
       <c r="O247" s="13" t="inlineStr"/>
       <c r="P247" s="13" t="inlineStr"/>
       <c r="Q247" s="14" t="n">
-        <v>4.21E7</v>
+        <v>3.65E7</v>
       </c>
       <c r="R247" s="14" t="inlineStr"/>
       <c r="S247" s="14" t="n">
@@ -14940,20 +14940,20 @@
         <v>1.5284E7</v>
       </c>
       <c r="X247" s="14" t="n">
-        <v>0.0</v>
+        <v>2.11705E7</v>
       </c>
       <c r="Y247" s="14" t="inlineStr"/>
       <c r="Z247" s="14" t="n">
-        <v>1.5284E7</v>
+        <v>3.64545E7</v>
       </c>
       <c r="AA247" s="14" t="inlineStr"/>
       <c r="AB247" s="14" t="inlineStr"/>
       <c r="AC247" s="15" t="n">
-        <v>0.36304038004750594</v>
+        <v>0.9987534246575343</v>
       </c>
       <c r="AD247" s="15" t="inlineStr"/>
       <c r="AE247" s="14" t="n">
-        <v>2.6816E7</v>
+        <v>45500.0</v>
       </c>
       <c r="AF247" s="14" t="inlineStr"/>
       <c r="AG247" s="14" t="inlineStr"/>
@@ -14997,20 +14997,20 @@
         <v>0.0</v>
       </c>
       <c r="X248" s="14" t="n">
-        <v>0.0</v>
+        <v>3.0407E7</v>
       </c>
       <c r="Y248" s="14" t="inlineStr"/>
       <c r="Z248" s="14" t="n">
-        <v>0.0</v>
+        <v>3.0407E7</v>
       </c>
       <c r="AA248" s="14" t="inlineStr"/>
       <c r="AB248" s="14" t="inlineStr"/>
       <c r="AC248" s="15" t="n">
-        <v>0.0</v>
+        <v>0.9940176528277215</v>
       </c>
       <c r="AD248" s="15" t="inlineStr"/>
       <c r="AE248" s="14" t="n">
-        <v>3.059E7</v>
+        <v>183000.0</v>
       </c>
       <c r="AF248" s="14" t="inlineStr"/>
       <c r="AG248" s="14" t="inlineStr"/>
@@ -15111,20 +15111,20 @@
         <v>0.0</v>
       </c>
       <c r="X250" s="14" t="n">
-        <v>0.0</v>
+        <v>4300000.0</v>
       </c>
       <c r="Y250" s="14" t="inlineStr"/>
       <c r="Z250" s="14" t="n">
-        <v>0.0</v>
+        <v>4300000.0</v>
       </c>
       <c r="AA250" s="14" t="inlineStr"/>
       <c r="AB250" s="14" t="inlineStr"/>
       <c r="AC250" s="15" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="AD250" s="15" t="inlineStr"/>
       <c r="AE250" s="14" t="n">
-        <v>4300000.0</v>
+        <v>0.0</v>
       </c>
       <c r="AF250" s="14" t="inlineStr"/>
       <c r="AG250" s="14" t="inlineStr"/>
@@ -15253,29 +15253,23 @@
       <c r="E253" s="2" t="inlineStr"/>
       <c r="F253" s="2" t="inlineStr"/>
       <c r="G253" s="2" t="inlineStr"/>
-      <c r="H253" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">523121</t>
-          </r>
-        </is>
-      </c>
-      <c r="I253" s="13" t="inlineStr"/>
-      <c r="J253" s="13" t="inlineStr"/>
-      <c r="K253" s="13" t="inlineStr"/>
-      <c r="L253" s="13" t="inlineStr"/>
-      <c r="M253" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Belanja Pemeliharaan Peralatan dan Mesin</t>
-          </r>
-        </is>
-      </c>
-      <c r="N253" s="13" t="inlineStr"/>
+      <c r="H253" s="2" t="inlineStr"/>
+      <c r="I253" s="2" t="inlineStr"/>
+      <c r="J253" s="2" t="inlineStr"/>
+      <c r="K253" s="2" t="inlineStr"/>
+      <c r="L253" s="2" t="inlineStr"/>
+      <c r="M253" s="2" t="inlineStr"/>
+      <c r="N253" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000310. Pemeliharaan Gedung Lab Basah Depok</t>
+          </r>
+        </is>
+      </c>
       <c r="O253" s="13" t="inlineStr"/>
       <c r="P253" s="13" t="inlineStr"/>
       <c r="Q253" s="14" t="n">
-        <v>3.325E8</v>
+        <v>3400000.0</v>
       </c>
       <c r="R253" s="14" t="inlineStr"/>
       <c r="S253" s="14" t="n">
@@ -15285,23 +15279,23 @@
       <c r="U253" s="14" t="inlineStr"/>
       <c r="V253" s="14" t="inlineStr"/>
       <c r="W253" s="14" t="n">
-        <v>2.11521335E8</v>
+        <v>0.0</v>
       </c>
       <c r="X253" s="14" t="n">
-        <v>2.0627437E7</v>
+        <v>3332500.0</v>
       </c>
       <c r="Y253" s="14" t="inlineStr"/>
       <c r="Z253" s="14" t="n">
-        <v>2.32148772E8</v>
+        <v>3332500.0</v>
       </c>
       <c r="AA253" s="14" t="inlineStr"/>
       <c r="AB253" s="14" t="inlineStr"/>
       <c r="AC253" s="15" t="n">
-        <v>0.6981917954887218</v>
+        <v>0.9801470588235294</v>
       </c>
       <c r="AD253" s="15" t="inlineStr"/>
       <c r="AE253" s="14" t="n">
-        <v>1.00351228E8</v>
+        <v>67500.0</v>
       </c>
       <c r="AF253" s="14" t="inlineStr"/>
       <c r="AG253" s="14" t="inlineStr"/>
@@ -15359,23 +15353,29 @@
       <c r="E255" s="2" t="inlineStr"/>
       <c r="F255" s="2" t="inlineStr"/>
       <c r="G255" s="2" t="inlineStr"/>
-      <c r="H255" s="2" t="inlineStr"/>
-      <c r="I255" s="2" t="inlineStr"/>
-      <c r="J255" s="2" t="inlineStr"/>
-      <c r="K255" s="2" t="inlineStr"/>
-      <c r="L255" s="2" t="inlineStr"/>
-      <c r="M255" s="2" t="inlineStr"/>
-      <c r="N255" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">000175. Pemeliharaan AC Split</t>
-          </r>
-        </is>
-      </c>
+      <c r="H255" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">523121</t>
+          </r>
+        </is>
+      </c>
+      <c r="I255" s="13" t="inlineStr"/>
+      <c r="J255" s="13" t="inlineStr"/>
+      <c r="K255" s="13" t="inlineStr"/>
+      <c r="L255" s="13" t="inlineStr"/>
+      <c r="M255" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Belanja Pemeliharaan Peralatan dan Mesin</t>
+          </r>
+        </is>
+      </c>
+      <c r="N255" s="13" t="inlineStr"/>
       <c r="O255" s="13" t="inlineStr"/>
       <c r="P255" s="13" t="inlineStr"/>
       <c r="Q255" s="14" t="n">
-        <v>2.257E7</v>
+        <v>3.24415E8</v>
       </c>
       <c r="R255" s="14" t="inlineStr"/>
       <c r="S255" s="14" t="n">
@@ -15385,23 +15385,23 @@
       <c r="U255" s="14" t="inlineStr"/>
       <c r="V255" s="14" t="inlineStr"/>
       <c r="W255" s="14" t="n">
-        <v>1.396E7</v>
+        <v>2.11521335E8</v>
       </c>
       <c r="X255" s="14" t="n">
-        <v>2890000.0</v>
+        <v>8.661379E7</v>
       </c>
       <c r="Y255" s="14" t="inlineStr"/>
       <c r="Z255" s="14" t="n">
-        <v>1.685E7</v>
+        <v>2.98135125E8</v>
       </c>
       <c r="AA255" s="14" t="inlineStr"/>
       <c r="AB255" s="14" t="inlineStr"/>
       <c r="AC255" s="15" t="n">
-        <v>0.7465662383695171</v>
+        <v>0.918993033614352</v>
       </c>
       <c r="AD255" s="15" t="inlineStr"/>
       <c r="AE255" s="14" t="n">
-        <v>5720000.0</v>
+        <v>2.6279875E7</v>
       </c>
       <c r="AF255" s="14" t="inlineStr"/>
       <c r="AG255" s="14" t="inlineStr"/>
@@ -15425,14 +15425,14 @@
       <c r="N256" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000176. Pemeliharaan Laptop</t>
+            <t xml:space="preserve">000175. Pemeliharaan AC Split</t>
           </r>
         </is>
       </c>
       <c r="O256" s="13" t="inlineStr"/>
       <c r="P256" s="13" t="inlineStr"/>
       <c r="Q256" s="14" t="n">
-        <v>5000000.0</v>
+        <v>2.257E7</v>
       </c>
       <c r="R256" s="14" t="inlineStr"/>
       <c r="S256" s="14" t="n">
@@ -15442,23 +15442,23 @@
       <c r="U256" s="14" t="inlineStr"/>
       <c r="V256" s="14" t="inlineStr"/>
       <c r="W256" s="14" t="n">
-        <v>2487928.0</v>
+        <v>1.396E7</v>
       </c>
       <c r="X256" s="14" t="n">
-        <v>0.0</v>
+        <v>5220000.0</v>
       </c>
       <c r="Y256" s="14" t="inlineStr"/>
       <c r="Z256" s="14" t="n">
-        <v>2487928.0</v>
+        <v>1.918E7</v>
       </c>
       <c r="AA256" s="14" t="inlineStr"/>
       <c r="AB256" s="14" t="inlineStr"/>
       <c r="AC256" s="15" t="n">
-        <v>0.4975856</v>
+        <v>0.8498006202924235</v>
       </c>
       <c r="AD256" s="15" t="inlineStr"/>
       <c r="AE256" s="14" t="n">
-        <v>2512072.0</v>
+        <v>3390000.0</v>
       </c>
       <c r="AF256" s="14" t="inlineStr"/>
       <c r="AG256" s="14" t="inlineStr"/>
@@ -15482,14 +15482,14 @@
       <c r="N257" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000182. Pemeliharaan Instalasi Listrik</t>
+            <t xml:space="preserve">000176. Pemeliharaan Laptop</t>
           </r>
         </is>
       </c>
       <c r="O257" s="13" t="inlineStr"/>
       <c r="P257" s="13" t="inlineStr"/>
       <c r="Q257" s="14" t="n">
-        <v>4.5E7</v>
+        <v>5000000.0</v>
       </c>
       <c r="R257" s="14" t="inlineStr"/>
       <c r="S257" s="14" t="n">
@@ -15499,23 +15499,23 @@
       <c r="U257" s="14" t="inlineStr"/>
       <c r="V257" s="14" t="inlineStr"/>
       <c r="W257" s="14" t="n">
-        <v>2.9845218E7</v>
+        <v>2487928.0</v>
       </c>
       <c r="X257" s="14" t="n">
-        <v>0.0</v>
+        <v>2500000.0</v>
       </c>
       <c r="Y257" s="14" t="inlineStr"/>
       <c r="Z257" s="14" t="n">
-        <v>2.9845218E7</v>
+        <v>4987928.0</v>
       </c>
       <c r="AA257" s="14" t="inlineStr"/>
       <c r="AB257" s="14" t="inlineStr"/>
       <c r="AC257" s="15" t="n">
-        <v>0.6632270666666666</v>
+        <v>0.9975856</v>
       </c>
       <c r="AD257" s="15" t="inlineStr"/>
       <c r="AE257" s="14" t="n">
-        <v>1.5154782E7</v>
+        <v>12072.0</v>
       </c>
       <c r="AF257" s="14" t="inlineStr"/>
       <c r="AG257" s="14" t="inlineStr"/>
@@ -15539,14 +15539,14 @@
       <c r="N258" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000183. Pemeliharaan Kendaraan Roda 4</t>
+            <t xml:space="preserve">000182. Pemeliharaan Instalasi Listrik</t>
           </r>
         </is>
       </c>
       <c r="O258" s="13" t="inlineStr"/>
       <c r="P258" s="13" t="inlineStr"/>
       <c r="Q258" s="14" t="n">
-        <v>1.6975E8</v>
+        <v>4.5E7</v>
       </c>
       <c r="R258" s="14" t="inlineStr"/>
       <c r="S258" s="14" t="n">
@@ -15556,23 +15556,23 @@
       <c r="U258" s="14" t="inlineStr"/>
       <c r="V258" s="14" t="inlineStr"/>
       <c r="W258" s="14" t="n">
-        <v>1.22043496E8</v>
+        <v>2.9845218E7</v>
       </c>
       <c r="X258" s="14" t="n">
-        <v>1.5139299E7</v>
+        <v>1.279805E7</v>
       </c>
       <c r="Y258" s="14" t="inlineStr"/>
       <c r="Z258" s="14" t="n">
-        <v>1.37182795E8</v>
+        <v>4.2643268E7</v>
       </c>
       <c r="AA258" s="14" t="inlineStr"/>
       <c r="AB258" s="14" t="inlineStr"/>
       <c r="AC258" s="15" t="n">
-        <v>0.8081460677466863</v>
+        <v>0.9476281777777777</v>
       </c>
       <c r="AD258" s="15" t="inlineStr"/>
       <c r="AE258" s="14" t="n">
-        <v>3.2567205E7</v>
+        <v>2356732.0</v>
       </c>
       <c r="AF258" s="14" t="inlineStr"/>
       <c r="AG258" s="14" t="inlineStr"/>
@@ -15596,14 +15596,14 @@
       <c r="N259" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000184. Pemeliharaan Kendaraan Roda 2</t>
+            <t xml:space="preserve">000183. Pemeliharaan Kendaraan Roda 4</t>
           </r>
         </is>
       </c>
       <c r="O259" s="13" t="inlineStr"/>
       <c r="P259" s="13" t="inlineStr"/>
       <c r="Q259" s="14" t="n">
-        <v>4500000.0</v>
+        <v>1.74265E8</v>
       </c>
       <c r="R259" s="14" t="inlineStr"/>
       <c r="S259" s="14" t="n">
@@ -15613,23 +15613,23 @@
       <c r="U259" s="14" t="inlineStr"/>
       <c r="V259" s="14" t="inlineStr"/>
       <c r="W259" s="14" t="n">
-        <v>4147992.0</v>
+        <v>1.22043496E8</v>
       </c>
       <c r="X259" s="14" t="n">
-        <v>0.0</v>
+        <v>4.7543521E7</v>
       </c>
       <c r="Y259" s="14" t="inlineStr"/>
       <c r="Z259" s="14" t="n">
-        <v>4147992.0</v>
+        <v>1.69587017E8</v>
       </c>
       <c r="AA259" s="14" t="inlineStr"/>
       <c r="AB259" s="14" t="inlineStr"/>
       <c r="AC259" s="15" t="n">
-        <v>0.921776</v>
+        <v>0.9731559234499182</v>
       </c>
       <c r="AD259" s="15" t="inlineStr"/>
       <c r="AE259" s="14" t="n">
-        <v>352008.0</v>
+        <v>4677983.0</v>
       </c>
       <c r="AF259" s="14" t="inlineStr"/>
       <c r="AG259" s="14" t="inlineStr"/>
@@ -15653,14 +15653,14 @@
       <c r="N260" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000185. Pemeliharaan CCTV</t>
+            <t xml:space="preserve">000184. Pemeliharaan Kendaraan Roda 2</t>
           </r>
         </is>
       </c>
       <c r="O260" s="13" t="inlineStr"/>
       <c r="P260" s="13" t="inlineStr"/>
       <c r="Q260" s="14" t="n">
-        <v>2.1E7</v>
+        <v>4500000.0</v>
       </c>
       <c r="R260" s="14" t="inlineStr"/>
       <c r="S260" s="14" t="n">
@@ -15670,23 +15670,23 @@
       <c r="U260" s="14" t="inlineStr"/>
       <c r="V260" s="14" t="inlineStr"/>
       <c r="W260" s="14" t="n">
-        <v>1.4290555E7</v>
+        <v>4147992.0</v>
       </c>
       <c r="X260" s="14" t="n">
-        <v>0.0</v>
+        <v>90000.0</v>
       </c>
       <c r="Y260" s="14" t="inlineStr"/>
       <c r="Z260" s="14" t="n">
-        <v>1.4290555E7</v>
+        <v>4237992.0</v>
       </c>
       <c r="AA260" s="14" t="inlineStr"/>
       <c r="AB260" s="14" t="inlineStr"/>
       <c r="AC260" s="15" t="n">
-        <v>0.680502619047619</v>
+        <v>0.941776</v>
       </c>
       <c r="AD260" s="15" t="inlineStr"/>
       <c r="AE260" s="14" t="n">
-        <v>6709445.0</v>
+        <v>262008.0</v>
       </c>
       <c r="AF260" s="14" t="inlineStr"/>
       <c r="AG260" s="14" t="inlineStr"/>
@@ -15710,14 +15710,14 @@
       <c r="N261" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000186. Pemeliharaan Genset 250 KVA</t>
+            <t xml:space="preserve">000185. Pemeliharaan CCTV</t>
           </r>
         </is>
       </c>
       <c r="O261" s="13" t="inlineStr"/>
       <c r="P261" s="13" t="inlineStr"/>
       <c r="Q261" s="14" t="n">
-        <v>9010000.0</v>
+        <v>1.5E7</v>
       </c>
       <c r="R261" s="14" t="inlineStr"/>
       <c r="S261" s="14" t="n">
@@ -15727,23 +15727,23 @@
       <c r="U261" s="14" t="inlineStr"/>
       <c r="V261" s="14" t="inlineStr"/>
       <c r="W261" s="14" t="n">
-        <v>1000052.0</v>
+        <v>1.4290555E7</v>
       </c>
       <c r="X261" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y261" s="14" t="inlineStr"/>
       <c r="Z261" s="14" t="n">
-        <v>1000052.0</v>
+        <v>1.4290555E7</v>
       </c>
       <c r="AA261" s="14" t="inlineStr"/>
       <c r="AB261" s="14" t="inlineStr"/>
       <c r="AC261" s="15" t="n">
-        <v>0.11099356270810211</v>
+        <v>0.9527036666666666</v>
       </c>
       <c r="AD261" s="15" t="inlineStr"/>
       <c r="AE261" s="14" t="n">
-        <v>8009948.0</v>
+        <v>709445.0</v>
       </c>
       <c r="AF261" s="14" t="inlineStr"/>
       <c r="AG261" s="14" t="inlineStr"/>
@@ -15767,14 +15767,14 @@
       <c r="N262" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000187. Pemeliharaan Genset 40 KVA</t>
+            <t xml:space="preserve">000186. Pemeliharaan Genset 250 KVA</t>
           </r>
         </is>
       </c>
       <c r="O262" s="13" t="inlineStr"/>
       <c r="P262" s="13" t="inlineStr"/>
       <c r="Q262" s="14" t="n">
-        <v>4050000.0</v>
+        <v>9010000.0</v>
       </c>
       <c r="R262" s="14" t="inlineStr"/>
       <c r="S262" s="14" t="n">
@@ -15784,23 +15784,23 @@
       <c r="U262" s="14" t="inlineStr"/>
       <c r="V262" s="14" t="inlineStr"/>
       <c r="W262" s="14" t="n">
-        <v>1978406.0</v>
+        <v>1000052.0</v>
       </c>
       <c r="X262" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y262" s="14" t="inlineStr"/>
       <c r="Z262" s="14" t="n">
-        <v>1978406.0</v>
+        <v>1000052.0</v>
       </c>
       <c r="AA262" s="14" t="inlineStr"/>
       <c r="AB262" s="14" t="inlineStr"/>
       <c r="AC262" s="15" t="n">
-        <v>0.4884953086419753</v>
+        <v>0.11099356270810211</v>
       </c>
       <c r="AD262" s="15" t="inlineStr"/>
       <c r="AE262" s="14" t="n">
-        <v>2071594.0</v>
+        <v>8009948.0</v>
       </c>
       <c r="AF262" s="14" t="inlineStr"/>
       <c r="AG262" s="14" t="inlineStr"/>
@@ -15824,14 +15824,14 @@
       <c r="N263" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000190. Pemeliharaan Mesin Potong Rumput</t>
+            <t xml:space="preserve">000187. Pemeliharaan Genset 40 KVA</t>
           </r>
         </is>
       </c>
       <c r="O263" s="13" t="inlineStr"/>
       <c r="P263" s="13" t="inlineStr"/>
       <c r="Q263" s="14" t="n">
-        <v>1.2E7</v>
+        <v>3050000.0</v>
       </c>
       <c r="R263" s="14" t="inlineStr"/>
       <c r="S263" s="14" t="n">
@@ -15841,23 +15841,23 @@
       <c r="U263" s="14" t="inlineStr"/>
       <c r="V263" s="14" t="inlineStr"/>
       <c r="W263" s="14" t="n">
-        <v>8450284.0</v>
+        <v>1978406.0</v>
       </c>
       <c r="X263" s="14" t="n">
-        <v>288000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y263" s="14" t="inlineStr"/>
       <c r="Z263" s="14" t="n">
-        <v>8738284.0</v>
+        <v>1978406.0</v>
       </c>
       <c r="AA263" s="14" t="inlineStr"/>
       <c r="AB263" s="14" t="inlineStr"/>
       <c r="AC263" s="15" t="n">
-        <v>0.7281903333333334</v>
+        <v>0.6486577049180328</v>
       </c>
       <c r="AD263" s="15" t="inlineStr"/>
       <c r="AE263" s="14" t="n">
-        <v>3261716.0</v>
+        <v>1071594.0</v>
       </c>
       <c r="AF263" s="14" t="inlineStr"/>
       <c r="AG263" s="14" t="inlineStr"/>
@@ -15881,14 +15881,14 @@
       <c r="N264" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000191. Pemeliharaan Printer</t>
+            <t xml:space="preserve">000190. Pemeliharaan Mesin Potong Rumput</t>
           </r>
         </is>
       </c>
       <c r="O264" s="13" t="inlineStr"/>
       <c r="P264" s="13" t="inlineStr"/>
       <c r="Q264" s="14" t="n">
-        <v>1500000.0</v>
+        <v>1.2E7</v>
       </c>
       <c r="R264" s="14" t="inlineStr"/>
       <c r="S264" s="14" t="n">
@@ -15898,23 +15898,23 @@
       <c r="U264" s="14" t="inlineStr"/>
       <c r="V264" s="14" t="inlineStr"/>
       <c r="W264" s="14" t="n">
-        <v>1167558.0</v>
+        <v>8450284.0</v>
       </c>
       <c r="X264" s="14" t="n">
-        <v>0.0</v>
+        <v>2385941.0</v>
       </c>
       <c r="Y264" s="14" t="inlineStr"/>
       <c r="Z264" s="14" t="n">
-        <v>1167558.0</v>
+        <v>1.0836225E7</v>
       </c>
       <c r="AA264" s="14" t="inlineStr"/>
       <c r="AB264" s="14" t="inlineStr"/>
       <c r="AC264" s="15" t="n">
-        <v>0.778372</v>
+        <v>0.90301875</v>
       </c>
       <c r="AD264" s="15" t="inlineStr"/>
       <c r="AE264" s="14" t="n">
-        <v>332442.0</v>
+        <v>1163775.0</v>
       </c>
       <c r="AF264" s="14" t="inlineStr"/>
       <c r="AG264" s="14" t="inlineStr"/>
@@ -15938,14 +15938,14 @@
       <c r="N265" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000192. Pemeliharaan Komputer/PC</t>
+            <t xml:space="preserve">000191. Pemeliharaan Printer</t>
           </r>
         </is>
       </c>
       <c r="O265" s="13" t="inlineStr"/>
       <c r="P265" s="13" t="inlineStr"/>
       <c r="Q265" s="14" t="n">
-        <v>1.562E7</v>
+        <v>2000000.0</v>
       </c>
       <c r="R265" s="14" t="inlineStr"/>
       <c r="S265" s="14" t="n">
@@ -15955,23 +15955,23 @@
       <c r="U265" s="14" t="inlineStr"/>
       <c r="V265" s="14" t="inlineStr"/>
       <c r="W265" s="14" t="n">
-        <v>3760846.0</v>
+        <v>1167558.0</v>
       </c>
       <c r="X265" s="14" t="n">
-        <v>1560138.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y265" s="14" t="inlineStr"/>
       <c r="Z265" s="14" t="n">
-        <v>5320984.0</v>
+        <v>1167558.0</v>
       </c>
       <c r="AA265" s="14" t="inlineStr"/>
       <c r="AB265" s="14" t="inlineStr"/>
       <c r="AC265" s="15" t="n">
-        <v>0.3406519846350832</v>
+        <v>0.583779</v>
       </c>
       <c r="AD265" s="15" t="inlineStr"/>
       <c r="AE265" s="14" t="n">
-        <v>1.0299016E7</v>
+        <v>832442.0</v>
       </c>
       <c r="AF265" s="14" t="inlineStr"/>
       <c r="AG265" s="14" t="inlineStr"/>
@@ -15995,14 +15995,14 @@
       <c r="N266" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000283. Pemeliharaan Kulkas</t>
+            <t xml:space="preserve">000192. Pemeliharaan Komputer/PC</t>
           </r>
         </is>
       </c>
       <c r="O266" s="13" t="inlineStr"/>
       <c r="P266" s="13" t="inlineStr"/>
       <c r="Q266" s="14" t="n">
-        <v>500000.0</v>
+        <v>1.562E7</v>
       </c>
       <c r="R266" s="14" t="inlineStr"/>
       <c r="S266" s="14" t="n">
@@ -16012,23 +16012,23 @@
       <c r="U266" s="14" t="inlineStr"/>
       <c r="V266" s="14" t="inlineStr"/>
       <c r="W266" s="14" t="n">
-        <v>500000.0</v>
+        <v>3760846.0</v>
       </c>
       <c r="X266" s="14" t="n">
-        <v>0.0</v>
+        <v>9601868.0</v>
       </c>
       <c r="Y266" s="14" t="inlineStr"/>
       <c r="Z266" s="14" t="n">
-        <v>500000.0</v>
+        <v>1.3362714E7</v>
       </c>
       <c r="AA266" s="14" t="inlineStr"/>
       <c r="AB266" s="14" t="inlineStr"/>
       <c r="AC266" s="15" t="n">
-        <v>1.0</v>
+        <v>0.855487451984635</v>
       </c>
       <c r="AD266" s="15" t="inlineStr"/>
       <c r="AE266" s="14" t="n">
-        <v>0.0</v>
+        <v>2257286.0</v>
       </c>
       <c r="AF266" s="14" t="inlineStr"/>
       <c r="AG266" s="14" t="inlineStr"/>
@@ -16052,14 +16052,14 @@
       <c r="N267" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000299. Pemeliharaan Instalasi Air</t>
+            <t xml:space="preserve">000283. Pemeliharaan Kulkas</t>
           </r>
         </is>
       </c>
       <c r="O267" s="13" t="inlineStr"/>
       <c r="P267" s="13" t="inlineStr"/>
       <c r="Q267" s="14" t="n">
-        <v>1.3E7</v>
+        <v>500000.0</v>
       </c>
       <c r="R267" s="14" t="inlineStr"/>
       <c r="S267" s="14" t="n">
@@ -16069,23 +16069,23 @@
       <c r="U267" s="14" t="inlineStr"/>
       <c r="V267" s="14" t="inlineStr"/>
       <c r="W267" s="14" t="n">
-        <v>7889000.0</v>
+        <v>500000.0</v>
       </c>
       <c r="X267" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y267" s="14" t="inlineStr"/>
       <c r="Z267" s="14" t="n">
-        <v>7889000.0</v>
+        <v>500000.0</v>
       </c>
       <c r="AA267" s="14" t="inlineStr"/>
       <c r="AB267" s="14" t="inlineStr"/>
       <c r="AC267" s="15" t="n">
-        <v>0.6068461538461538</v>
+        <v>1.0</v>
       </c>
       <c r="AD267" s="15" t="inlineStr"/>
       <c r="AE267" s="14" t="n">
-        <v>5111000.0</v>
+        <v>0.0</v>
       </c>
       <c r="AF267" s="14" t="inlineStr"/>
       <c r="AG267" s="14" t="inlineStr"/>
@@ -16109,14 +16109,14 @@
       <c r="N268" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000304. Pemeliharaan Alat Laboratorium</t>
+            <t xml:space="preserve">000299. Pemeliharaan Instalasi Air</t>
           </r>
         </is>
       </c>
       <c r="O268" s="13" t="inlineStr"/>
       <c r="P268" s="13" t="inlineStr"/>
       <c r="Q268" s="14" t="n">
-        <v>2500000.0</v>
+        <v>9400000.0</v>
       </c>
       <c r="R268" s="14" t="inlineStr"/>
       <c r="S268" s="14" t="n">
@@ -16126,23 +16126,23 @@
       <c r="U268" s="14" t="inlineStr"/>
       <c r="V268" s="14" t="inlineStr"/>
       <c r="W268" s="14" t="n">
-        <v>0.0</v>
+        <v>7889000.0</v>
       </c>
       <c r="X268" s="14" t="n">
-        <v>0.0</v>
+        <v>581410.0</v>
       </c>
       <c r="Y268" s="14" t="inlineStr"/>
       <c r="Z268" s="14" t="n">
-        <v>0.0</v>
+        <v>8470410.0</v>
       </c>
       <c r="AA268" s="14" t="inlineStr"/>
       <c r="AB268" s="14" t="inlineStr"/>
       <c r="AC268" s="15" t="n">
-        <v>0.0</v>
+        <v>0.9011074468085106</v>
       </c>
       <c r="AD268" s="15" t="inlineStr"/>
       <c r="AE268" s="14" t="n">
-        <v>2500000.0</v>
+        <v>929590.0</v>
       </c>
       <c r="AF268" s="14" t="inlineStr"/>
       <c r="AG268" s="14" t="inlineStr"/>
@@ -16186,20 +16186,20 @@
         <v>0.0</v>
       </c>
       <c r="X269" s="14" t="n">
-        <v>750000.0</v>
+        <v>1450000.0</v>
       </c>
       <c r="Y269" s="14" t="inlineStr"/>
       <c r="Z269" s="14" t="n">
-        <v>750000.0</v>
+        <v>1450000.0</v>
       </c>
       <c r="AA269" s="14" t="inlineStr"/>
       <c r="AB269" s="14" t="inlineStr"/>
       <c r="AC269" s="15" t="n">
-        <v>0.5</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="AD269" s="15" t="inlineStr"/>
       <c r="AE269" s="14" t="n">
-        <v>750000.0</v>
+        <v>50000.0</v>
       </c>
       <c r="AF269" s="14" t="inlineStr"/>
       <c r="AG269" s="14" t="inlineStr"/>
@@ -16230,7 +16230,7 @@
       <c r="O270" s="13" t="inlineStr"/>
       <c r="P270" s="13" t="inlineStr"/>
       <c r="Q270" s="14" t="n">
-        <v>5000000.0</v>
+        <v>4000000.0</v>
       </c>
       <c r="R270" s="14" t="inlineStr"/>
       <c r="S270" s="14" t="n">
@@ -16243,20 +16243,20 @@
         <v>0.0</v>
       </c>
       <c r="X270" s="14" t="n">
-        <v>0.0</v>
+        <v>3955000.0</v>
       </c>
       <c r="Y270" s="14" t="inlineStr"/>
       <c r="Z270" s="14" t="n">
-        <v>0.0</v>
+        <v>3955000.0</v>
       </c>
       <c r="AA270" s="14" t="inlineStr"/>
       <c r="AB270" s="14" t="inlineStr"/>
       <c r="AC270" s="15" t="n">
-        <v>0.0</v>
+        <v>0.98875</v>
       </c>
       <c r="AD270" s="15" t="inlineStr"/>
       <c r="AE270" s="14" t="n">
-        <v>5000000.0</v>
+        <v>45000.0</v>
       </c>
       <c r="AF270" s="14" t="inlineStr"/>
       <c r="AG270" s="14" t="inlineStr"/>
@@ -16271,29 +16271,23 @@
       <c r="E271" s="2" t="inlineStr"/>
       <c r="F271" s="2" t="inlineStr"/>
       <c r="G271" s="2" t="inlineStr"/>
-      <c r="H271" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">523132</t>
-          </r>
-        </is>
-      </c>
-      <c r="I271" s="13" t="inlineStr"/>
-      <c r="J271" s="13" t="inlineStr"/>
-      <c r="K271" s="13" t="inlineStr"/>
-      <c r="L271" s="13" t="inlineStr"/>
-      <c r="M271" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Belanja Pemeliharaan Irigasi</t>
-          </r>
-        </is>
-      </c>
-      <c r="N271" s="13" t="inlineStr"/>
+      <c r="H271" s="2" t="inlineStr"/>
+      <c r="I271" s="2" t="inlineStr"/>
+      <c r="J271" s="2" t="inlineStr"/>
+      <c r="K271" s="2" t="inlineStr"/>
+      <c r="L271" s="2" t="inlineStr"/>
+      <c r="M271" s="2" t="inlineStr"/>
+      <c r="N271" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000308. Pemeliharaan Genset Portable</t>
+          </r>
+        </is>
+      </c>
       <c r="O271" s="13" t="inlineStr"/>
       <c r="P271" s="13" t="inlineStr"/>
       <c r="Q271" s="14" t="n">
-        <v>1.5292E8</v>
+        <v>1000000.0</v>
       </c>
       <c r="R271" s="14" t="inlineStr"/>
       <c r="S271" s="14" t="n">
@@ -16303,23 +16297,23 @@
       <c r="U271" s="14" t="inlineStr"/>
       <c r="V271" s="14" t="inlineStr"/>
       <c r="W271" s="14" t="n">
-        <v>8.0551E7</v>
+        <v>0.0</v>
       </c>
       <c r="X271" s="14" t="n">
-        <v>0.0</v>
+        <v>488000.0</v>
       </c>
       <c r="Y271" s="14" t="inlineStr"/>
       <c r="Z271" s="14" t="n">
-        <v>8.0551E7</v>
+        <v>488000.0</v>
       </c>
       <c r="AA271" s="14" t="inlineStr"/>
       <c r="AB271" s="14" t="inlineStr"/>
       <c r="AC271" s="15" t="n">
-        <v>0.5267525503531258</v>
+        <v>0.488</v>
       </c>
       <c r="AD271" s="15" t="inlineStr"/>
       <c r="AE271" s="14" t="n">
-        <v>7.2369E7</v>
+        <v>512000.0</v>
       </c>
       <c r="AF271" s="14" t="inlineStr"/>
       <c r="AG271" s="14" t="inlineStr"/>
@@ -16334,23 +16328,29 @@
       <c r="E272" s="2" t="inlineStr"/>
       <c r="F272" s="2" t="inlineStr"/>
       <c r="G272" s="2" t="inlineStr"/>
-      <c r="H272" s="2" t="inlineStr"/>
-      <c r="I272" s="2" t="inlineStr"/>
-      <c r="J272" s="2" t="inlineStr"/>
-      <c r="K272" s="2" t="inlineStr"/>
-      <c r="L272" s="2" t="inlineStr"/>
-      <c r="M272" s="2" t="inlineStr"/>
-      <c r="N272" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">000195. Pemeliharaan Talud Cijeruk</t>
-          </r>
-        </is>
-      </c>
+      <c r="H272" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">523132</t>
+          </r>
+        </is>
+      </c>
+      <c r="I272" s="13" t="inlineStr"/>
+      <c r="J272" s="13" t="inlineStr"/>
+      <c r="K272" s="13" t="inlineStr"/>
+      <c r="L272" s="13" t="inlineStr"/>
+      <c r="M272" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Belanja Pemeliharaan Irigasi</t>
+          </r>
+        </is>
+      </c>
+      <c r="N272" s="13" t="inlineStr"/>
       <c r="O272" s="13" t="inlineStr"/>
       <c r="P272" s="13" t="inlineStr"/>
       <c r="Q272" s="14" t="n">
-        <v>6.216E7</v>
+        <v>1.5136E8</v>
       </c>
       <c r="R272" s="14" t="inlineStr"/>
       <c r="S272" s="14" t="n">
@@ -16360,23 +16360,23 @@
       <c r="U272" s="14" t="inlineStr"/>
       <c r="V272" s="14" t="inlineStr"/>
       <c r="W272" s="14" t="n">
-        <v>3.909E7</v>
+        <v>8.0551E7</v>
       </c>
       <c r="X272" s="14" t="n">
-        <v>0.0</v>
+        <v>6.9975E7</v>
       </c>
       <c r="Y272" s="14" t="inlineStr"/>
       <c r="Z272" s="14" t="n">
-        <v>3.909E7</v>
+        <v>1.50526E8</v>
       </c>
       <c r="AA272" s="14" t="inlineStr"/>
       <c r="AB272" s="14" t="inlineStr"/>
       <c r="AC272" s="15" t="n">
-        <v>0.6288610038610039</v>
+        <v>0.9944899577167019</v>
       </c>
       <c r="AD272" s="15" t="inlineStr"/>
       <c r="AE272" s="14" t="n">
-        <v>2.307E7</v>
+        <v>834000.0</v>
       </c>
       <c r="AF272" s="14" t="inlineStr"/>
       <c r="AG272" s="14" t="inlineStr"/>
@@ -16400,14 +16400,14 @@
       <c r="N273" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000284. Pemeliharaan Talud Cibalagung</t>
+            <t xml:space="preserve">000195. Pemeliharaan Talud Cijeruk</t>
           </r>
         </is>
       </c>
       <c r="O273" s="13" t="inlineStr"/>
       <c r="P273" s="13" t="inlineStr"/>
       <c r="Q273" s="14" t="n">
-        <v>3.07E7</v>
+        <v>6.06E7</v>
       </c>
       <c r="R273" s="14" t="inlineStr"/>
       <c r="S273" s="14" t="n">
@@ -16417,23 +16417,23 @@
       <c r="U273" s="14" t="inlineStr"/>
       <c r="V273" s="14" t="inlineStr"/>
       <c r="W273" s="14" t="n">
-        <v>3.0685E7</v>
+        <v>3.909E7</v>
       </c>
       <c r="X273" s="14" t="n">
-        <v>0.0</v>
+        <v>2.1185E7</v>
       </c>
       <c r="Y273" s="14" t="inlineStr"/>
       <c r="Z273" s="14" t="n">
-        <v>3.0685E7</v>
+        <v>6.0275E7</v>
       </c>
       <c r="AA273" s="14" t="inlineStr"/>
       <c r="AB273" s="14" t="inlineStr"/>
       <c r="AC273" s="15" t="n">
-        <v>0.9995114006514658</v>
+        <v>0.9946369636963697</v>
       </c>
       <c r="AD273" s="15" t="inlineStr"/>
       <c r="AE273" s="14" t="n">
-        <v>15000.0</v>
+        <v>325000.0</v>
       </c>
       <c r="AF273" s="14" t="inlineStr"/>
       <c r="AG273" s="14" t="inlineStr"/>
@@ -16457,14 +16457,14 @@
       <c r="N274" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000285. Pemeliharaan Saluran Air Cijeruk</t>
+            <t xml:space="preserve">000284. Pemeliharaan Talud Cibalagung</t>
           </r>
         </is>
       </c>
       <c r="O274" s="13" t="inlineStr"/>
       <c r="P274" s="13" t="inlineStr"/>
       <c r="Q274" s="14" t="n">
-        <v>6.006E7</v>
+        <v>3.07E7</v>
       </c>
       <c r="R274" s="14" t="inlineStr"/>
       <c r="S274" s="14" t="n">
@@ -16474,23 +16474,23 @@
       <c r="U274" s="14" t="inlineStr"/>
       <c r="V274" s="14" t="inlineStr"/>
       <c r="W274" s="14" t="n">
-        <v>1.0776E7</v>
+        <v>3.0685E7</v>
       </c>
       <c r="X274" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y274" s="14" t="inlineStr"/>
       <c r="Z274" s="14" t="n">
-        <v>1.0776E7</v>
+        <v>3.0685E7</v>
       </c>
       <c r="AA274" s="14" t="inlineStr"/>
       <c r="AB274" s="14" t="inlineStr"/>
       <c r="AC274" s="15" t="n">
-        <v>0.17942057942057943</v>
+        <v>0.9995114006514658</v>
       </c>
       <c r="AD274" s="15" t="inlineStr"/>
       <c r="AE274" s="14" t="n">
-        <v>4.9284E7</v>
+        <v>15000.0</v>
       </c>
       <c r="AF274" s="14" t="inlineStr"/>
       <c r="AG274" s="14" t="inlineStr"/>
@@ -16503,31 +16503,25 @@
       <c r="C275" s="2" t="inlineStr"/>
       <c r="D275" s="2" t="inlineStr"/>
       <c r="E275" s="2" t="inlineStr"/>
-      <c r="F275" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">002.DD</t>
-          </r>
-        </is>
-      </c>
-      <c r="G275" s="13" t="inlineStr"/>
-      <c r="H275" s="13" t="inlineStr"/>
-      <c r="I275" s="13" t="inlineStr"/>
-      <c r="J275" s="13" t="inlineStr"/>
-      <c r="K275" s="13" t="inlineStr"/>
-      <c r="L275" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Pembayaran Terkait Pelaksanaan Operasional Kantor</t>
-          </r>
-        </is>
-      </c>
-      <c r="M275" s="13" t="inlineStr"/>
-      <c r="N275" s="13" t="inlineStr"/>
+      <c r="F275" s="2" t="inlineStr"/>
+      <c r="G275" s="2" t="inlineStr"/>
+      <c r="H275" s="2" t="inlineStr"/>
+      <c r="I275" s="2" t="inlineStr"/>
+      <c r="J275" s="2" t="inlineStr"/>
+      <c r="K275" s="2" t="inlineStr"/>
+      <c r="L275" s="2" t="inlineStr"/>
+      <c r="M275" s="2" t="inlineStr"/>
+      <c r="N275" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000285. Pemeliharaan Saluran Air Cijeruk</t>
+          </r>
+        </is>
+      </c>
       <c r="O275" s="13" t="inlineStr"/>
       <c r="P275" s="13" t="inlineStr"/>
       <c r="Q275" s="14" t="n">
-        <v>1.3218E8</v>
+        <v>6.006E7</v>
       </c>
       <c r="R275" s="14" t="inlineStr"/>
       <c r="S275" s="14" t="n">
@@ -16537,23 +16531,23 @@
       <c r="U275" s="14" t="inlineStr"/>
       <c r="V275" s="14" t="inlineStr"/>
       <c r="W275" s="14" t="n">
-        <v>1.3074E8</v>
+        <v>1.0776E7</v>
       </c>
       <c r="X275" s="14" t="n">
-        <v>480000.0</v>
+        <v>4.879E7</v>
       </c>
       <c r="Y275" s="14" t="inlineStr"/>
       <c r="Z275" s="14" t="n">
-        <v>1.3122E8</v>
+        <v>5.9566E7</v>
       </c>
       <c r="AA275" s="14" t="inlineStr"/>
       <c r="AB275" s="14" t="inlineStr"/>
       <c r="AC275" s="15" t="n">
-        <v>0.9927371765773945</v>
+        <v>0.9917748917748918</v>
       </c>
       <c r="AD275" s="15" t="inlineStr"/>
       <c r="AE275" s="14" t="n">
-        <v>960000.0</v>
+        <v>494000.0</v>
       </c>
       <c r="AF275" s="14" t="inlineStr"/>
       <c r="AG275" s="14" t="inlineStr"/>
@@ -16566,31 +16560,31 @@
       <c r="C276" s="2" t="inlineStr"/>
       <c r="D276" s="2" t="inlineStr"/>
       <c r="E276" s="2" t="inlineStr"/>
-      <c r="F276" s="2" t="inlineStr"/>
-      <c r="G276" s="2" t="inlineStr"/>
-      <c r="H276" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">521115</t>
-          </r>
-        </is>
-      </c>
+      <c r="F276" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">002.DD</t>
+          </r>
+        </is>
+      </c>
+      <c r="G276" s="13" t="inlineStr"/>
+      <c r="H276" s="13" t="inlineStr"/>
       <c r="I276" s="13" t="inlineStr"/>
       <c r="J276" s="13" t="inlineStr"/>
       <c r="K276" s="13" t="inlineStr"/>
-      <c r="L276" s="13" t="inlineStr"/>
-      <c r="M276" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Belanja Honor Operasional Satuan Kerja</t>
-          </r>
-        </is>
-      </c>
+      <c r="L276" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Pembayaran Terkait Pelaksanaan Operasional Kantor</t>
+          </r>
+        </is>
+      </c>
+      <c r="M276" s="13" t="inlineStr"/>
       <c r="N276" s="13" t="inlineStr"/>
       <c r="O276" s="13" t="inlineStr"/>
       <c r="P276" s="13" t="inlineStr"/>
       <c r="Q276" s="14" t="n">
-        <v>1.2468E8</v>
+        <v>1.5218E8</v>
       </c>
       <c r="R276" s="14" t="inlineStr"/>
       <c r="S276" s="14" t="n">
@@ -16600,23 +16594,23 @@
       <c r="U276" s="14" t="inlineStr"/>
       <c r="V276" s="14" t="inlineStr"/>
       <c r="W276" s="14" t="n">
-        <v>1.2324E8</v>
+        <v>1.3074E8</v>
       </c>
       <c r="X276" s="14" t="n">
-        <v>480000.0</v>
+        <v>2.124E7</v>
       </c>
       <c r="Y276" s="14" t="inlineStr"/>
       <c r="Z276" s="14" t="n">
-        <v>1.2372E8</v>
+        <v>1.5198E8</v>
       </c>
       <c r="AA276" s="14" t="inlineStr"/>
       <c r="AB276" s="14" t="inlineStr"/>
       <c r="AC276" s="15" t="n">
-        <v>0.9923002887391723</v>
+        <v>0.9986857668550401</v>
       </c>
       <c r="AD276" s="15" t="inlineStr"/>
       <c r="AE276" s="14" t="n">
-        <v>960000.0</v>
+        <v>200000.0</v>
       </c>
       <c r="AF276" s="14" t="inlineStr"/>
       <c r="AG276" s="14" t="inlineStr"/>
@@ -16631,23 +16625,29 @@
       <c r="E277" s="2" t="inlineStr"/>
       <c r="F277" s="2" t="inlineStr"/>
       <c r="G277" s="2" t="inlineStr"/>
-      <c r="H277" s="2" t="inlineStr"/>
-      <c r="I277" s="2" t="inlineStr"/>
-      <c r="J277" s="2" t="inlineStr"/>
-      <c r="K277" s="2" t="inlineStr"/>
-      <c r="L277" s="2" t="inlineStr"/>
-      <c r="M277" s="2" t="inlineStr"/>
-      <c r="N277" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">000197. Honorarium Pejabat Kuasa Pengguna Anggaran</t>
-          </r>
-        </is>
-      </c>
+      <c r="H277" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">521115</t>
+          </r>
+        </is>
+      </c>
+      <c r="I277" s="13" t="inlineStr"/>
+      <c r="J277" s="13" t="inlineStr"/>
+      <c r="K277" s="13" t="inlineStr"/>
+      <c r="L277" s="13" t="inlineStr"/>
+      <c r="M277" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Belanja Honor Operasional Satuan Kerja</t>
+          </r>
+        </is>
+      </c>
+      <c r="N277" s="13" t="inlineStr"/>
       <c r="O277" s="13" t="inlineStr"/>
       <c r="P277" s="13" t="inlineStr"/>
       <c r="Q277" s="14" t="n">
-        <v>3.06E7</v>
+        <v>1.2468E8</v>
       </c>
       <c r="R277" s="14" t="inlineStr"/>
       <c r="S277" s="14" t="n">
@@ -16657,14 +16657,14 @@
       <c r="U277" s="14" t="inlineStr"/>
       <c r="V277" s="14" t="inlineStr"/>
       <c r="W277" s="14" t="n">
-        <v>3.06E7</v>
+        <v>1.2324E8</v>
       </c>
       <c r="X277" s="14" t="n">
-        <v>0.0</v>
+        <v>1440000.0</v>
       </c>
       <c r="Y277" s="14" t="inlineStr"/>
       <c r="Z277" s="14" t="n">
-        <v>3.06E7</v>
+        <v>1.2468E8</v>
       </c>
       <c r="AA277" s="14" t="inlineStr"/>
       <c r="AB277" s="14" t="inlineStr"/>
@@ -16697,14 +16697,14 @@
       <c r="N278" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000198. Honorarium Pejabat Pembuat Komitmen</t>
+            <t xml:space="preserve">000197. Honorarium Pejabat Kuasa Pengguna Anggaran</t>
           </r>
         </is>
       </c>
       <c r="O278" s="13" t="inlineStr"/>
       <c r="P278" s="13" t="inlineStr"/>
       <c r="Q278" s="14" t="n">
-        <v>2.976E7</v>
+        <v>3.06E7</v>
       </c>
       <c r="R278" s="14" t="inlineStr"/>
       <c r="S278" s="14" t="n">
@@ -16714,14 +16714,14 @@
       <c r="U278" s="14" t="inlineStr"/>
       <c r="V278" s="14" t="inlineStr"/>
       <c r="W278" s="14" t="n">
-        <v>2.976E7</v>
+        <v>3.06E7</v>
       </c>
       <c r="X278" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y278" s="14" t="inlineStr"/>
       <c r="Z278" s="14" t="n">
-        <v>2.976E7</v>
+        <v>3.06E7</v>
       </c>
       <c r="AA278" s="14" t="inlineStr"/>
       <c r="AB278" s="14" t="inlineStr"/>
@@ -16737,7 +16737,7 @@
       <c r="AH278" s="14" t="inlineStr"/>
       <c r="AI278" s="14" t="inlineStr"/>
     </row>
-    <row r="279" customHeight="1" ht="18">
+    <row r="279" customHeight="1" ht="15">
       <c r="A279" s="2" t="inlineStr"/>
       <c r="B279" s="2" t="inlineStr"/>
       <c r="C279" s="2" t="inlineStr"/>
@@ -16754,14 +16754,14 @@
       <c r="N279" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000199. Honorarium Pejabat  Penguji Tagihan   Penandatangan  Spm</t>
+            <t xml:space="preserve">000198. Honorarium Pejabat Pembuat Komitmen</t>
           </r>
         </is>
       </c>
       <c r="O279" s="13" t="inlineStr"/>
       <c r="P279" s="13" t="inlineStr"/>
       <c r="Q279" s="14" t="n">
-        <v>1.476E7</v>
+        <v>2.976E7</v>
       </c>
       <c r="R279" s="14" t="inlineStr"/>
       <c r="S279" s="14" t="n">
@@ -16771,14 +16771,14 @@
       <c r="U279" s="14" t="inlineStr"/>
       <c r="V279" s="14" t="inlineStr"/>
       <c r="W279" s="14" t="n">
-        <v>1.476E7</v>
+        <v>2.976E7</v>
       </c>
       <c r="X279" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y279" s="14" t="inlineStr"/>
       <c r="Z279" s="14" t="n">
-        <v>1.476E7</v>
+        <v>2.976E7</v>
       </c>
       <c r="AA279" s="14" t="inlineStr"/>
       <c r="AB279" s="14" t="inlineStr"/>
@@ -16794,7 +16794,7 @@
       <c r="AH279" s="14" t="inlineStr"/>
       <c r="AI279" s="14" t="inlineStr"/>
     </row>
-    <row r="280" customHeight="1" ht="15">
+    <row r="280" customHeight="1" ht="18">
       <c r="A280" s="2" t="inlineStr"/>
       <c r="B280" s="2" t="inlineStr"/>
       <c r="C280" s="2" t="inlineStr"/>
@@ -16811,14 +16811,14 @@
       <c r="N280" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000200. Honorarium Bendahara  Pengeluaran</t>
+            <t xml:space="preserve">000199. Honorarium Pejabat  Penguji Tagihan   Penandatangan  Spm</t>
           </r>
         </is>
       </c>
       <c r="O280" s="13" t="inlineStr"/>
       <c r="P280" s="13" t="inlineStr"/>
       <c r="Q280" s="14" t="n">
-        <v>1.284E7</v>
+        <v>1.476E7</v>
       </c>
       <c r="R280" s="14" t="inlineStr"/>
       <c r="S280" s="14" t="n">
@@ -16828,14 +16828,14 @@
       <c r="U280" s="14" t="inlineStr"/>
       <c r="V280" s="14" t="inlineStr"/>
       <c r="W280" s="14" t="n">
-        <v>1.284E7</v>
+        <v>1.476E7</v>
       </c>
       <c r="X280" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y280" s="14" t="inlineStr"/>
       <c r="Z280" s="14" t="n">
-        <v>1.284E7</v>
+        <v>1.476E7</v>
       </c>
       <c r="AA280" s="14" t="inlineStr"/>
       <c r="AB280" s="14" t="inlineStr"/>
@@ -16911,14 +16911,14 @@
       <c r="N282" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000201. Honorarium Staf  Pengelola</t>
+            <t xml:space="preserve">000200. Honorarium Bendahara  Pengeluaran</t>
           </r>
         </is>
       </c>
       <c r="O282" s="13" t="inlineStr"/>
       <c r="P282" s="13" t="inlineStr"/>
       <c r="Q282" s="14" t="n">
-        <v>2.88E7</v>
+        <v>1.284E7</v>
       </c>
       <c r="R282" s="14" t="inlineStr"/>
       <c r="S282" s="14" t="n">
@@ -16928,14 +16928,14 @@
       <c r="U282" s="14" t="inlineStr"/>
       <c r="V282" s="14" t="inlineStr"/>
       <c r="W282" s="14" t="n">
-        <v>2.88E7</v>
+        <v>1.284E7</v>
       </c>
       <c r="X282" s="14" t="n">
         <v>0.0</v>
       </c>
       <c r="Y282" s="14" t="inlineStr"/>
       <c r="Z282" s="14" t="n">
-        <v>2.88E7</v>
+        <v>1.284E7</v>
       </c>
       <c r="AA282" s="14" t="inlineStr"/>
       <c r="AB282" s="14" t="inlineStr"/>
@@ -16968,14 +16968,14 @@
       <c r="N283" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000202. Honorarium Anggota/Petugas (UAKPA/Barang)</t>
+            <t xml:space="preserve">000201. Honorarium Staf  Pengelola</t>
           </r>
         </is>
       </c>
       <c r="O283" s="13" t="inlineStr"/>
       <c r="P283" s="13" t="inlineStr"/>
       <c r="Q283" s="14" t="n">
-        <v>3600000.0</v>
+        <v>2.88E7</v>
       </c>
       <c r="R283" s="14" t="inlineStr"/>
       <c r="S283" s="14" t="n">
@@ -16985,30 +16985,30 @@
       <c r="U283" s="14" t="inlineStr"/>
       <c r="V283" s="14" t="inlineStr"/>
       <c r="W283" s="14" t="n">
-        <v>2700000.0</v>
+        <v>2.88E7</v>
       </c>
       <c r="X283" s="14" t="n">
-        <v>300000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y283" s="14" t="inlineStr"/>
       <c r="Z283" s="14" t="n">
-        <v>3000000.0</v>
+        <v>2.88E7</v>
       </c>
       <c r="AA283" s="14" t="inlineStr"/>
       <c r="AB283" s="14" t="inlineStr"/>
       <c r="AC283" s="15" t="n">
-        <v>0.8333333333333334</v>
+        <v>1.0</v>
       </c>
       <c r="AD283" s="15" t="inlineStr"/>
       <c r="AE283" s="14" t="n">
-        <v>600000.0</v>
+        <v>0.0</v>
       </c>
       <c r="AF283" s="14" t="inlineStr"/>
       <c r="AG283" s="14" t="inlineStr"/>
       <c r="AH283" s="14" t="inlineStr"/>
       <c r="AI283" s="14" t="inlineStr"/>
     </row>
-    <row r="284" customHeight="1" ht="18">
+    <row r="284" customHeight="1" ht="15">
       <c r="A284" s="2" t="inlineStr"/>
       <c r="B284" s="2" t="inlineStr"/>
       <c r="C284" s="2" t="inlineStr"/>
@@ -17025,14 +17025,14 @@
       <c r="N284" s="13" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">000203. Honorarium Pengurus/Penyimpan Bmn Tingkat Kuasa Pengguna Barang</t>
+            <t xml:space="preserve">000202. Honorarium Anggota/Petugas (UAKPA/Barang)</t>
           </r>
         </is>
       </c>
       <c r="O284" s="13" t="inlineStr"/>
       <c r="P284" s="13" t="inlineStr"/>
       <c r="Q284" s="14" t="n">
-        <v>4320000.0</v>
+        <v>3600000.0</v>
       </c>
       <c r="R284" s="14" t="inlineStr"/>
       <c r="S284" s="14" t="n">
@@ -17042,30 +17042,30 @@
       <c r="U284" s="14" t="inlineStr"/>
       <c r="V284" s="14" t="inlineStr"/>
       <c r="W284" s="14" t="n">
-        <v>3780000.0</v>
+        <v>2700000.0</v>
       </c>
       <c r="X284" s="14" t="n">
-        <v>180000.0</v>
+        <v>900000.0</v>
       </c>
       <c r="Y284" s="14" t="inlineStr"/>
       <c r="Z284" s="14" t="n">
-        <v>3960000.0</v>
+        <v>3600000.0</v>
       </c>
       <c r="AA284" s="14" t="inlineStr"/>
       <c r="AB284" s="14" t="inlineStr"/>
       <c r="AC284" s="15" t="n">
-        <v>0.9166666666666666</v>
+        <v>1.0</v>
       </c>
       <c r="AD284" s="15" t="inlineStr"/>
       <c r="AE284" s="14" t="n">
-        <v>360000.0</v>
+        <v>0.0</v>
       </c>
       <c r="AF284" s="14" t="inlineStr"/>
       <c r="AG284" s="14" t="inlineStr"/>
       <c r="AH284" s="14" t="inlineStr"/>
       <c r="AI284" s="14" t="inlineStr"/>
     </row>
-    <row r="285" customHeight="1" ht="15">
+    <row r="285" customHeight="1" ht="18">
       <c r="A285" s="2" t="inlineStr"/>
       <c r="B285" s="2" t="inlineStr"/>
       <c r="C285" s="2" t="inlineStr"/>
@@ -17073,29 +17073,23 @@
       <c r="E285" s="2" t="inlineStr"/>
       <c r="F285" s="2" t="inlineStr"/>
       <c r="G285" s="2" t="inlineStr"/>
-      <c r="H285" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">521119</t>
-          </r>
-        </is>
-      </c>
-      <c r="I285" s="13" t="inlineStr"/>
-      <c r="J285" s="13" t="inlineStr"/>
-      <c r="K285" s="13" t="inlineStr"/>
-      <c r="L285" s="13" t="inlineStr"/>
-      <c r="M285" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Belanja Barang Operasional Lainnya</t>
-          </r>
-        </is>
-      </c>
-      <c r="N285" s="13" t="inlineStr"/>
+      <c r="H285" s="2" t="inlineStr"/>
+      <c r="I285" s="2" t="inlineStr"/>
+      <c r="J285" s="2" t="inlineStr"/>
+      <c r="K285" s="2" t="inlineStr"/>
+      <c r="L285" s="2" t="inlineStr"/>
+      <c r="M285" s="2" t="inlineStr"/>
+      <c r="N285" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000203. Honorarium Pengurus/Penyimpan Bmn Tingkat Kuasa Pengguna Barang</t>
+          </r>
+        </is>
+      </c>
       <c r="O285" s="13" t="inlineStr"/>
       <c r="P285" s="13" t="inlineStr"/>
       <c r="Q285" s="14" t="n">
-        <v>7500000.0</v>
+        <v>4320000.0</v>
       </c>
       <c r="R285" s="14" t="inlineStr"/>
       <c r="S285" s="14" t="n">
@@ -17105,14 +17099,14 @@
       <c r="U285" s="14" t="inlineStr"/>
       <c r="V285" s="14" t="inlineStr"/>
       <c r="W285" s="14" t="n">
-        <v>7500000.0</v>
+        <v>3780000.0</v>
       </c>
       <c r="X285" s="14" t="n">
-        <v>0.0</v>
+        <v>540000.0</v>
       </c>
       <c r="Y285" s="14" t="inlineStr"/>
       <c r="Z285" s="14" t="n">
-        <v>7500000.0</v>
+        <v>4320000.0</v>
       </c>
       <c r="AA285" s="14" t="inlineStr"/>
       <c r="AB285" s="14" t="inlineStr"/>
@@ -17136,23 +17130,29 @@
       <c r="E286" s="2" t="inlineStr"/>
       <c r="F286" s="2" t="inlineStr"/>
       <c r="G286" s="2" t="inlineStr"/>
-      <c r="H286" s="2" t="inlineStr"/>
-      <c r="I286" s="2" t="inlineStr"/>
-      <c r="J286" s="2" t="inlineStr"/>
-      <c r="K286" s="2" t="inlineStr"/>
-      <c r="L286" s="2" t="inlineStr"/>
-      <c r="M286" s="2" t="inlineStr"/>
-      <c r="N286" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">000243. Pakaian Kerja PJLP</t>
-          </r>
-        </is>
-      </c>
+      <c r="H286" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">521119</t>
+          </r>
+        </is>
+      </c>
+      <c r="I286" s="13" t="inlineStr"/>
+      <c r="J286" s="13" t="inlineStr"/>
+      <c r="K286" s="13" t="inlineStr"/>
+      <c r="L286" s="13" t="inlineStr"/>
+      <c r="M286" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Belanja Barang Operasional Lainnya</t>
+          </r>
+        </is>
+      </c>
+      <c r="N286" s="13" t="inlineStr"/>
       <c r="O286" s="13" t="inlineStr"/>
       <c r="P286" s="13" t="inlineStr"/>
       <c r="Q286" s="14" t="n">
-        <v>7500000.0</v>
+        <v>2.75E7</v>
       </c>
       <c r="R286" s="14" t="inlineStr"/>
       <c r="S286" s="14" t="n">
@@ -17165,20 +17165,20 @@
         <v>7500000.0</v>
       </c>
       <c r="X286" s="14" t="n">
-        <v>0.0</v>
+        <v>1.98E7</v>
       </c>
       <c r="Y286" s="14" t="inlineStr"/>
       <c r="Z286" s="14" t="n">
-        <v>7500000.0</v>
+        <v>2.73E7</v>
       </c>
       <c r="AA286" s="14" t="inlineStr"/>
       <c r="AB286" s="14" t="inlineStr"/>
       <c r="AC286" s="15" t="n">
-        <v>1.0</v>
+        <v>0.9927272727272727</v>
       </c>
       <c r="AD286" s="15" t="inlineStr"/>
       <c r="AE286" s="14" t="n">
-        <v>0.0</v>
+        <v>200000.0</v>
       </c>
       <c r="AF286" s="14" t="inlineStr"/>
       <c r="AG286" s="14" t="inlineStr"/>
@@ -17188,317 +17188,305 @@
     <row r="287" customHeight="1" ht="15">
       <c r="A287" s="2" t="inlineStr"/>
       <c r="B287" s="2" t="inlineStr"/>
-      <c r="C287" s="16" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">EBD</t>
-          </r>
-        </is>
-      </c>
-      <c r="D287" s="16" t="inlineStr"/>
-      <c r="E287" s="16" t="inlineStr"/>
-      <c r="F287" s="16" t="inlineStr"/>
-      <c r="G287" s="16" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Layanan Manajemen Kinerja Internal</t>
-          </r>
-        </is>
-      </c>
-      <c r="H287" s="16" t="inlineStr"/>
-      <c r="I287" s="16" t="inlineStr"/>
-      <c r="J287" s="16" t="inlineStr"/>
-      <c r="K287" s="16" t="inlineStr"/>
-      <c r="L287" s="16" t="inlineStr"/>
-      <c r="M287" s="16" t="inlineStr"/>
-      <c r="N287" s="16" t="inlineStr"/>
-      <c r="O287" s="16" t="inlineStr"/>
-      <c r="P287" s="16" t="inlineStr"/>
-      <c r="Q287" s="17" t="n">
-        <v>600000.0</v>
-      </c>
-      <c r="R287" s="17" t="inlineStr"/>
-      <c r="S287" s="17" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="T287" s="17" t="inlineStr"/>
-      <c r="U287" s="17" t="inlineStr"/>
-      <c r="V287" s="17" t="inlineStr"/>
-      <c r="W287" s="17" t="n">
-        <v>600000.0</v>
-      </c>
-      <c r="X287" s="17" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Y287" s="17" t="inlineStr"/>
-      <c r="Z287" s="17" t="n">
-        <v>600000.0</v>
-      </c>
-      <c r="AA287" s="17" t="inlineStr"/>
-      <c r="AB287" s="17" t="inlineStr"/>
-      <c r="AC287" s="18" t="n">
+      <c r="C287" s="2" t="inlineStr"/>
+      <c r="D287" s="2" t="inlineStr"/>
+      <c r="E287" s="2" t="inlineStr"/>
+      <c r="F287" s="2" t="inlineStr"/>
+      <c r="G287" s="2" t="inlineStr"/>
+      <c r="H287" s="2" t="inlineStr"/>
+      <c r="I287" s="2" t="inlineStr"/>
+      <c r="J287" s="2" t="inlineStr"/>
+      <c r="K287" s="2" t="inlineStr"/>
+      <c r="L287" s="2" t="inlineStr"/>
+      <c r="M287" s="2" t="inlineStr"/>
+      <c r="N287" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000243. Pakaian Kerja PJLP</t>
+          </r>
+        </is>
+      </c>
+      <c r="O287" s="13" t="inlineStr"/>
+      <c r="P287" s="13" t="inlineStr"/>
+      <c r="Q287" s="14" t="n">
+        <v>7500000.0</v>
+      </c>
+      <c r="R287" s="14" t="inlineStr"/>
+      <c r="S287" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T287" s="14" t="inlineStr"/>
+      <c r="U287" s="14" t="inlineStr"/>
+      <c r="V287" s="14" t="inlineStr"/>
+      <c r="W287" s="14" t="n">
+        <v>7500000.0</v>
+      </c>
+      <c r="X287" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y287" s="14" t="inlineStr"/>
+      <c r="Z287" s="14" t="n">
+        <v>7500000.0</v>
+      </c>
+      <c r="AA287" s="14" t="inlineStr"/>
+      <c r="AB287" s="14" t="inlineStr"/>
+      <c r="AC287" s="15" t="n">
         <v>1.0</v>
       </c>
-      <c r="AD287" s="18" t="inlineStr"/>
-      <c r="AE287" s="17" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="AF287" s="17" t="inlineStr"/>
-      <c r="AG287" s="17" t="inlineStr"/>
-      <c r="AH287" s="17" t="inlineStr"/>
-      <c r="AI287" s="17" t="inlineStr"/>
+      <c r="AD287" s="15" t="inlineStr"/>
+      <c r="AE287" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF287" s="14" t="inlineStr"/>
+      <c r="AG287" s="14" t="inlineStr"/>
+      <c r="AH287" s="14" t="inlineStr"/>
+      <c r="AI287" s="14" t="inlineStr"/>
     </row>
     <row r="288" customHeight="1" ht="15">
       <c r="A288" s="2" t="inlineStr"/>
       <c r="B288" s="2" t="inlineStr"/>
-      <c r="C288" s="28" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">EBD.955</t>
-          </r>
-        </is>
-      </c>
-      <c r="D288" s="28" t="inlineStr"/>
-      <c r="E288" s="28" t="inlineStr"/>
-      <c r="F288" s="28" t="inlineStr"/>
-      <c r="G288" s="28" t="inlineStr"/>
-      <c r="H288" s="28" t="inlineStr"/>
-      <c r="I288" s="28" t="inlineStr"/>
-      <c r="J288" s="28" t="inlineStr"/>
-      <c r="K288" s="20" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Layanan Manajemen Keuangan</t>
-          </r>
-        </is>
-      </c>
-      <c r="L288" s="20" t="inlineStr"/>
-      <c r="M288" s="20" t="inlineStr"/>
-      <c r="N288" s="20" t="inlineStr"/>
-      <c r="O288" s="20" t="inlineStr"/>
-      <c r="P288" s="20" t="inlineStr"/>
-      <c r="Q288" s="21" t="n">
-        <v>600000.0</v>
-      </c>
-      <c r="R288" s="21" t="inlineStr"/>
-      <c r="S288" s="21" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="T288" s="21" t="inlineStr"/>
-      <c r="U288" s="21" t="inlineStr"/>
-      <c r="V288" s="21" t="inlineStr"/>
-      <c r="W288" s="22" t="n">
-        <v>600000.0</v>
-      </c>
-      <c r="X288" s="22" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Y288" s="22" t="inlineStr"/>
-      <c r="Z288" s="21" t="n">
-        <v>600000.0</v>
-      </c>
-      <c r="AA288" s="21" t="inlineStr"/>
-      <c r="AB288" s="21" t="inlineStr"/>
-      <c r="AC288" s="23" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="AD288" s="23" t="inlineStr"/>
-      <c r="AE288" s="21" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="AF288" s="21" t="inlineStr"/>
-      <c r="AG288" s="21" t="inlineStr"/>
-      <c r="AH288" s="21" t="inlineStr"/>
-      <c r="AI288" s="21" t="inlineStr"/>
+      <c r="C288" s="2" t="inlineStr"/>
+      <c r="D288" s="2" t="inlineStr"/>
+      <c r="E288" s="2" t="inlineStr"/>
+      <c r="F288" s="2" t="inlineStr"/>
+      <c r="G288" s="2" t="inlineStr"/>
+      <c r="H288" s="2" t="inlineStr"/>
+      <c r="I288" s="2" t="inlineStr"/>
+      <c r="J288" s="2" t="inlineStr"/>
+      <c r="K288" s="2" t="inlineStr"/>
+      <c r="L288" s="2" t="inlineStr"/>
+      <c r="M288" s="2" t="inlineStr"/>
+      <c r="N288" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000309. Pakaian Lapangan</t>
+          </r>
+        </is>
+      </c>
+      <c r="O288" s="13" t="inlineStr"/>
+      <c r="P288" s="13" t="inlineStr"/>
+      <c r="Q288" s="14" t="n">
+        <v>2.0E7</v>
+      </c>
+      <c r="R288" s="14" t="inlineStr"/>
+      <c r="S288" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T288" s="14" t="inlineStr"/>
+      <c r="U288" s="14" t="inlineStr"/>
+      <c r="V288" s="14" t="inlineStr"/>
+      <c r="W288" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="X288" s="14" t="n">
+        <v>1.98E7</v>
+      </c>
+      <c r="Y288" s="14" t="inlineStr"/>
+      <c r="Z288" s="14" t="n">
+        <v>1.98E7</v>
+      </c>
+      <c r="AA288" s="14" t="inlineStr"/>
+      <c r="AB288" s="14" t="inlineStr"/>
+      <c r="AC288" s="15" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AD288" s="15" t="inlineStr"/>
+      <c r="AE288" s="14" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="AF288" s="14" t="inlineStr"/>
+      <c r="AG288" s="14" t="inlineStr"/>
+      <c r="AH288" s="14" t="inlineStr"/>
+      <c r="AI288" s="14" t="inlineStr"/>
     </row>
     <row r="289" customHeight="1" ht="15">
       <c r="A289" s="2" t="inlineStr"/>
       <c r="B289" s="2" t="inlineStr"/>
-      <c r="C289" s="2" t="inlineStr"/>
-      <c r="D289" s="2" t="inlineStr"/>
-      <c r="E289" s="24" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">201</t>
-          </r>
-        </is>
-      </c>
-      <c r="F289" s="24" t="inlineStr"/>
-      <c r="G289" s="24" t="inlineStr"/>
-      <c r="H289" s="24" t="inlineStr"/>
-      <c r="I289" s="24" t="inlineStr"/>
-      <c r="J289" s="24" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Pelayanan Keuangan Penyuluhan Kelautan dan Perikanan</t>
-          </r>
-        </is>
-      </c>
-      <c r="K289" s="24" t="inlineStr"/>
-      <c r="L289" s="24" t="inlineStr"/>
-      <c r="M289" s="24" t="inlineStr"/>
-      <c r="N289" s="24" t="inlineStr"/>
-      <c r="O289" s="24" t="inlineStr"/>
-      <c r="P289" s="24" t="inlineStr"/>
-      <c r="Q289" s="25" t="n">
+      <c r="C289" s="16" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">EBD</t>
+          </r>
+        </is>
+      </c>
+      <c r="D289" s="16" t="inlineStr"/>
+      <c r="E289" s="16" t="inlineStr"/>
+      <c r="F289" s="16" t="inlineStr"/>
+      <c r="G289" s="16" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Layanan Manajemen Kinerja Internal</t>
+          </r>
+        </is>
+      </c>
+      <c r="H289" s="16" t="inlineStr"/>
+      <c r="I289" s="16" t="inlineStr"/>
+      <c r="J289" s="16" t="inlineStr"/>
+      <c r="K289" s="16" t="inlineStr"/>
+      <c r="L289" s="16" t="inlineStr"/>
+      <c r="M289" s="16" t="inlineStr"/>
+      <c r="N289" s="16" t="inlineStr"/>
+      <c r="O289" s="16" t="inlineStr"/>
+      <c r="P289" s="16" t="inlineStr"/>
+      <c r="Q289" s="17" t="n">
         <v>600000.0</v>
       </c>
-      <c r="R289" s="25" t="inlineStr"/>
-      <c r="S289" s="25" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="T289" s="25" t="inlineStr"/>
-      <c r="U289" s="25" t="inlineStr"/>
-      <c r="V289" s="25" t="inlineStr"/>
-      <c r="W289" s="25" t="n">
+      <c r="R289" s="17" t="inlineStr"/>
+      <c r="S289" s="17" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T289" s="17" t="inlineStr"/>
+      <c r="U289" s="17" t="inlineStr"/>
+      <c r="V289" s="17" t="inlineStr"/>
+      <c r="W289" s="17" t="n">
         <v>600000.0</v>
       </c>
-      <c r="X289" s="25" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Y289" s="25" t="inlineStr"/>
-      <c r="Z289" s="25" t="n">
+      <c r="X289" s="17" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y289" s="17" t="inlineStr"/>
+      <c r="Z289" s="17" t="n">
         <v>600000.0</v>
       </c>
-      <c r="AA289" s="25" t="inlineStr"/>
-      <c r="AB289" s="25" t="inlineStr"/>
-      <c r="AC289" s="26" t="n">
+      <c r="AA289" s="17" t="inlineStr"/>
+      <c r="AB289" s="17" t="inlineStr"/>
+      <c r="AC289" s="18" t="n">
         <v>1.0</v>
       </c>
-      <c r="AD289" s="26" t="inlineStr"/>
-      <c r="AE289" s="25" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="AF289" s="25" t="inlineStr"/>
-      <c r="AG289" s="25" t="inlineStr"/>
-      <c r="AH289" s="25" t="inlineStr"/>
-      <c r="AI289" s="25" t="inlineStr"/>
+      <c r="AD289" s="18" t="inlineStr"/>
+      <c r="AE289" s="17" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF289" s="17" t="inlineStr"/>
+      <c r="AG289" s="17" t="inlineStr"/>
+      <c r="AH289" s="17" t="inlineStr"/>
+      <c r="AI289" s="17" t="inlineStr"/>
     </row>
     <row r="290" customHeight="1" ht="15">
       <c r="A290" s="2" t="inlineStr"/>
       <c r="B290" s="2" t="inlineStr"/>
-      <c r="C290" s="2" t="inlineStr"/>
-      <c r="D290" s="2" t="inlineStr"/>
-      <c r="E290" s="2" t="inlineStr"/>
-      <c r="F290" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">201.DA</t>
-          </r>
-        </is>
-      </c>
-      <c r="G290" s="13" t="inlineStr"/>
-      <c r="H290" s="13" t="inlineStr"/>
-      <c r="I290" s="13" t="inlineStr"/>
-      <c r="J290" s="13" t="inlineStr"/>
-      <c r="K290" s="13" t="inlineStr"/>
-      <c r="L290" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Layanan Keuangan</t>
-          </r>
-        </is>
-      </c>
-      <c r="M290" s="13" t="inlineStr"/>
-      <c r="N290" s="13" t="inlineStr"/>
-      <c r="O290" s="13" t="inlineStr"/>
-      <c r="P290" s="13" t="inlineStr"/>
-      <c r="Q290" s="14" t="n">
+      <c r="C290" s="28" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">EBD.955</t>
+          </r>
+        </is>
+      </c>
+      <c r="D290" s="28" t="inlineStr"/>
+      <c r="E290" s="28" t="inlineStr"/>
+      <c r="F290" s="28" t="inlineStr"/>
+      <c r="G290" s="28" t="inlineStr"/>
+      <c r="H290" s="28" t="inlineStr"/>
+      <c r="I290" s="28" t="inlineStr"/>
+      <c r="J290" s="28" t="inlineStr"/>
+      <c r="K290" s="20" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Layanan Manajemen Keuangan</t>
+          </r>
+        </is>
+      </c>
+      <c r="L290" s="20" t="inlineStr"/>
+      <c r="M290" s="20" t="inlineStr"/>
+      <c r="N290" s="20" t="inlineStr"/>
+      <c r="O290" s="20" t="inlineStr"/>
+      <c r="P290" s="20" t="inlineStr"/>
+      <c r="Q290" s="21" t="n">
         <v>600000.0</v>
       </c>
-      <c r="R290" s="14" t="inlineStr"/>
-      <c r="S290" s="14" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="T290" s="14" t="inlineStr"/>
-      <c r="U290" s="14" t="inlineStr"/>
-      <c r="V290" s="14" t="inlineStr"/>
-      <c r="W290" s="14" t="n">
+      <c r="R290" s="21" t="inlineStr"/>
+      <c r="S290" s="21" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T290" s="21" t="inlineStr"/>
+      <c r="U290" s="21" t="inlineStr"/>
+      <c r="V290" s="21" t="inlineStr"/>
+      <c r="W290" s="22" t="n">
         <v>600000.0</v>
       </c>
-      <c r="X290" s="14" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Y290" s="14" t="inlineStr"/>
-      <c r="Z290" s="14" t="n">
+      <c r="X290" s="22" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y290" s="22" t="inlineStr"/>
+      <c r="Z290" s="21" t="n">
         <v>600000.0</v>
       </c>
-      <c r="AA290" s="14" t="inlineStr"/>
-      <c r="AB290" s="14" t="inlineStr"/>
-      <c r="AC290" s="15" t="n">
+      <c r="AA290" s="21" t="inlineStr"/>
+      <c r="AB290" s="21" t="inlineStr"/>
+      <c r="AC290" s="23" t="n">
         <v>1.0</v>
       </c>
-      <c r="AD290" s="15" t="inlineStr"/>
-      <c r="AE290" s="14" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="AF290" s="14" t="inlineStr"/>
-      <c r="AG290" s="14" t="inlineStr"/>
-      <c r="AH290" s="14" t="inlineStr"/>
-      <c r="AI290" s="14" t="inlineStr"/>
+      <c r="AD290" s="23" t="inlineStr"/>
+      <c r="AE290" s="21" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF290" s="21" t="inlineStr"/>
+      <c r="AG290" s="21" t="inlineStr"/>
+      <c r="AH290" s="21" t="inlineStr"/>
+      <c r="AI290" s="21" t="inlineStr"/>
     </row>
     <row r="291" customHeight="1" ht="15">
       <c r="A291" s="2" t="inlineStr"/>
       <c r="B291" s="2" t="inlineStr"/>
       <c r="C291" s="2" t="inlineStr"/>
       <c r="D291" s="2" t="inlineStr"/>
-      <c r="E291" s="2" t="inlineStr"/>
-      <c r="F291" s="2" t="inlineStr"/>
-      <c r="G291" s="2" t="inlineStr"/>
-      <c r="H291" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">524111</t>
-          </r>
-        </is>
-      </c>
-      <c r="I291" s="13" t="inlineStr"/>
-      <c r="J291" s="13" t="inlineStr"/>
-      <c r="K291" s="13" t="inlineStr"/>
-      <c r="L291" s="13" t="inlineStr"/>
-      <c r="M291" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">Belanja Perjalanan Dinas Biasa</t>
-          </r>
-        </is>
-      </c>
-      <c r="N291" s="13" t="inlineStr"/>
-      <c r="O291" s="13" t="inlineStr"/>
-      <c r="P291" s="13" t="inlineStr"/>
-      <c r="Q291" s="14" t="n">
+      <c r="E291" s="24" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">201</t>
+          </r>
+        </is>
+      </c>
+      <c r="F291" s="24" t="inlineStr"/>
+      <c r="G291" s="24" t="inlineStr"/>
+      <c r="H291" s="24" t="inlineStr"/>
+      <c r="I291" s="24" t="inlineStr"/>
+      <c r="J291" s="24" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Pelayanan Keuangan Penyuluhan Kelautan dan Perikanan</t>
+          </r>
+        </is>
+      </c>
+      <c r="K291" s="24" t="inlineStr"/>
+      <c r="L291" s="24" t="inlineStr"/>
+      <c r="M291" s="24" t="inlineStr"/>
+      <c r="N291" s="24" t="inlineStr"/>
+      <c r="O291" s="24" t="inlineStr"/>
+      <c r="P291" s="24" t="inlineStr"/>
+      <c r="Q291" s="25" t="n">
         <v>600000.0</v>
       </c>
-      <c r="R291" s="14" t="inlineStr"/>
-      <c r="S291" s="14" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="T291" s="14" t="inlineStr"/>
-      <c r="U291" s="14" t="inlineStr"/>
-      <c r="V291" s="14" t="inlineStr"/>
-      <c r="W291" s="14" t="n">
+      <c r="R291" s="25" t="inlineStr"/>
+      <c r="S291" s="25" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T291" s="25" t="inlineStr"/>
+      <c r="U291" s="25" t="inlineStr"/>
+      <c r="V291" s="25" t="inlineStr"/>
+      <c r="W291" s="25" t="n">
         <v>600000.0</v>
       </c>
-      <c r="X291" s="14" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="Y291" s="14" t="inlineStr"/>
-      <c r="Z291" s="14" t="n">
+      <c r="X291" s="25" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y291" s="25" t="inlineStr"/>
+      <c r="Z291" s="25" t="n">
         <v>600000.0</v>
       </c>
-      <c r="AA291" s="14" t="inlineStr"/>
-      <c r="AB291" s="14" t="inlineStr"/>
-      <c r="AC291" s="15" t="n">
+      <c r="AA291" s="25" t="inlineStr"/>
+      <c r="AB291" s="25" t="inlineStr"/>
+      <c r="AC291" s="26" t="n">
         <v>1.0</v>
       </c>
-      <c r="AD291" s="15" t="inlineStr"/>
-      <c r="AE291" s="14" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="AF291" s="14" t="inlineStr"/>
-      <c r="AG291" s="14" t="inlineStr"/>
-      <c r="AH291" s="14" t="inlineStr"/>
-      <c r="AI291" s="14" t="inlineStr"/>
+      <c r="AD291" s="26" t="inlineStr"/>
+      <c r="AE291" s="25" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF291" s="25" t="inlineStr"/>
+      <c r="AG291" s="25" t="inlineStr"/>
+      <c r="AH291" s="25" t="inlineStr"/>
+      <c r="AI291" s="25" t="inlineStr"/>
     </row>
     <row r="292" customHeight="1" ht="15">
       <c r="A292" s="2" t="inlineStr"/>
@@ -17506,21 +17494,27 @@
       <c r="C292" s="2" t="inlineStr"/>
       <c r="D292" s="2" t="inlineStr"/>
       <c r="E292" s="2" t="inlineStr"/>
-      <c r="F292" s="2" t="inlineStr"/>
-      <c r="G292" s="2" t="inlineStr"/>
-      <c r="H292" s="2" t="inlineStr"/>
-      <c r="I292" s="2" t="inlineStr"/>
-      <c r="J292" s="2" t="inlineStr"/>
-      <c r="K292" s="2" t="inlineStr"/>
-      <c r="L292" s="2" t="inlineStr"/>
-      <c r="M292" s="2" t="inlineStr"/>
-      <c r="N292" s="13" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">000231. Uang Harian</t>
-          </r>
-        </is>
-      </c>
+      <c r="F292" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">201.DA</t>
+          </r>
+        </is>
+      </c>
+      <c r="G292" s="13" t="inlineStr"/>
+      <c r="H292" s="13" t="inlineStr"/>
+      <c r="I292" s="13" t="inlineStr"/>
+      <c r="J292" s="13" t="inlineStr"/>
+      <c r="K292" s="13" t="inlineStr"/>
+      <c r="L292" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Layanan Keuangan</t>
+          </r>
+        </is>
+      </c>
+      <c r="M292" s="13" t="inlineStr"/>
+      <c r="N292" s="13" t="inlineStr"/>
       <c r="O292" s="13" t="inlineStr"/>
       <c r="P292" s="13" t="inlineStr"/>
       <c r="Q292" s="14" t="n">
@@ -17557,48 +17551,168 @@
       <c r="AH292" s="14" t="inlineStr"/>
       <c r="AI292" s="14" t="inlineStr"/>
     </row>
-    <row r="293" customHeight="1" ht="12">
+    <row r="293" customHeight="1" ht="15">
       <c r="A293" s="2" t="inlineStr"/>
-      <c r="B293" s="27" t="inlineStr">
+      <c r="B293" s="2" t="inlineStr"/>
+      <c r="C293" s="2" t="inlineStr"/>
+      <c r="D293" s="2" t="inlineStr"/>
+      <c r="E293" s="2" t="inlineStr"/>
+      <c r="F293" s="2" t="inlineStr"/>
+      <c r="G293" s="2" t="inlineStr"/>
+      <c r="H293" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">524111</t>
+          </r>
+        </is>
+      </c>
+      <c r="I293" s="13" t="inlineStr"/>
+      <c r="J293" s="13" t="inlineStr"/>
+      <c r="K293" s="13" t="inlineStr"/>
+      <c r="L293" s="13" t="inlineStr"/>
+      <c r="M293" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Belanja Perjalanan Dinas Biasa</t>
+          </r>
+        </is>
+      </c>
+      <c r="N293" s="13" t="inlineStr"/>
+      <c r="O293" s="13" t="inlineStr"/>
+      <c r="P293" s="13" t="inlineStr"/>
+      <c r="Q293" s="14" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="R293" s="14" t="inlineStr"/>
+      <c r="S293" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T293" s="14" t="inlineStr"/>
+      <c r="U293" s="14" t="inlineStr"/>
+      <c r="V293" s="14" t="inlineStr"/>
+      <c r="W293" s="14" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="X293" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y293" s="14" t="inlineStr"/>
+      <c r="Z293" s="14" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="AA293" s="14" t="inlineStr"/>
+      <c r="AB293" s="14" t="inlineStr"/>
+      <c r="AC293" s="15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AD293" s="15" t="inlineStr"/>
+      <c r="AE293" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF293" s="14" t="inlineStr"/>
+      <c r="AG293" s="14" t="inlineStr"/>
+      <c r="AH293" s="14" t="inlineStr"/>
+      <c r="AI293" s="14" t="inlineStr"/>
+    </row>
+    <row r="294" customHeight="1" ht="15">
+      <c r="A294" s="2" t="inlineStr"/>
+      <c r="B294" s="2" t="inlineStr"/>
+      <c r="C294" s="2" t="inlineStr"/>
+      <c r="D294" s="2" t="inlineStr"/>
+      <c r="E294" s="2" t="inlineStr"/>
+      <c r="F294" s="2" t="inlineStr"/>
+      <c r="G294" s="2" t="inlineStr"/>
+      <c r="H294" s="2" t="inlineStr"/>
+      <c r="I294" s="2" t="inlineStr"/>
+      <c r="J294" s="2" t="inlineStr"/>
+      <c r="K294" s="2" t="inlineStr"/>
+      <c r="L294" s="2" t="inlineStr"/>
+      <c r="M294" s="2" t="inlineStr"/>
+      <c r="N294" s="13" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">000231. Uang Harian</t>
+          </r>
+        </is>
+      </c>
+      <c r="O294" s="13" t="inlineStr"/>
+      <c r="P294" s="13" t="inlineStr"/>
+      <c r="Q294" s="14" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="R294" s="14" t="inlineStr"/>
+      <c r="S294" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T294" s="14" t="inlineStr"/>
+      <c r="U294" s="14" t="inlineStr"/>
+      <c r="V294" s="14" t="inlineStr"/>
+      <c r="W294" s="14" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="X294" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y294" s="14" t="inlineStr"/>
+      <c r="Z294" s="14" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="AA294" s="14" t="inlineStr"/>
+      <c r="AB294" s="14" t="inlineStr"/>
+      <c r="AC294" s="15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AD294" s="15" t="inlineStr"/>
+      <c r="AE294" s="14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF294" s="14" t="inlineStr"/>
+      <c r="AG294" s="14" t="inlineStr"/>
+      <c r="AH294" s="14" t="inlineStr"/>
+      <c r="AI294" s="14" t="inlineStr"/>
+    </row>
+    <row r="295" customHeight="1" ht="12">
+      <c r="A295" s="2" t="inlineStr"/>
+      <c r="B295" s="27" t="inlineStr">
         <is>
           <r>
             <t xml:space="preserve">*Lock Pagu adalah jumlah pagu yang sedang dalam proses usulan revisi DIPA atau POK. Lock pagu akan hilang setelah usulan revisi DIPA/POK selesai menjadi DIPA.</t>
           </r>
         </is>
       </c>
-      <c r="C293" s="27" t="inlineStr"/>
-      <c r="D293" s="27" t="inlineStr"/>
-      <c r="E293" s="27" t="inlineStr"/>
-      <c r="F293" s="27" t="inlineStr"/>
-      <c r="G293" s="27" t="inlineStr"/>
-      <c r="H293" s="27" t="inlineStr"/>
-      <c r="I293" s="27" t="inlineStr"/>
-      <c r="J293" s="27" t="inlineStr"/>
-      <c r="K293" s="27" t="inlineStr"/>
-      <c r="L293" s="27" t="inlineStr"/>
-      <c r="M293" s="27" t="inlineStr"/>
-      <c r="N293" s="27" t="inlineStr"/>
-      <c r="O293" s="27" t="inlineStr"/>
-      <c r="P293" s="27" t="inlineStr"/>
-      <c r="Q293" s="27" t="inlineStr"/>
-      <c r="R293" s="27" t="inlineStr"/>
-      <c r="S293" s="27" t="inlineStr"/>
-      <c r="T293" s="27" t="inlineStr"/>
-      <c r="U293" s="27" t="inlineStr"/>
-      <c r="V293" s="27" t="inlineStr"/>
-      <c r="W293" s="27" t="inlineStr"/>
-      <c r="X293" s="27" t="inlineStr"/>
-      <c r="Y293" s="27" t="inlineStr"/>
-      <c r="Z293" s="27" t="inlineStr"/>
-      <c r="AA293" s="27" t="inlineStr"/>
-      <c r="AB293" s="27" t="inlineStr"/>
-      <c r="AC293" s="27" t="inlineStr"/>
-      <c r="AD293" s="27" t="inlineStr"/>
-      <c r="AE293" s="27" t="inlineStr"/>
-      <c r="AF293" s="27" t="inlineStr"/>
-      <c r="AG293" s="2" t="inlineStr"/>
-      <c r="AH293" s="2" t="inlineStr"/>
-      <c r="AI293" s="2" t="inlineStr"/>
+      <c r="C295" s="27" t="inlineStr"/>
+      <c r="D295" s="27" t="inlineStr"/>
+      <c r="E295" s="27" t="inlineStr"/>
+      <c r="F295" s="27" t="inlineStr"/>
+      <c r="G295" s="27" t="inlineStr"/>
+      <c r="H295" s="27" t="inlineStr"/>
+      <c r="I295" s="27" t="inlineStr"/>
+      <c r="J295" s="27" t="inlineStr"/>
+      <c r="K295" s="27" t="inlineStr"/>
+      <c r="L295" s="27" t="inlineStr"/>
+      <c r="M295" s="27" t="inlineStr"/>
+      <c r="N295" s="27" t="inlineStr"/>
+      <c r="O295" s="27" t="inlineStr"/>
+      <c r="P295" s="27" t="inlineStr"/>
+      <c r="Q295" s="27" t="inlineStr"/>
+      <c r="R295" s="27" t="inlineStr"/>
+      <c r="S295" s="27" t="inlineStr"/>
+      <c r="T295" s="27" t="inlineStr"/>
+      <c r="U295" s="27" t="inlineStr"/>
+      <c r="V295" s="27" t="inlineStr"/>
+      <c r="W295" s="27" t="inlineStr"/>
+      <c r="X295" s="27" t="inlineStr"/>
+      <c r="Y295" s="27" t="inlineStr"/>
+      <c r="Z295" s="27" t="inlineStr"/>
+      <c r="AA295" s="27" t="inlineStr"/>
+      <c r="AB295" s="27" t="inlineStr"/>
+      <c r="AC295" s="27" t="inlineStr"/>
+      <c r="AD295" s="27" t="inlineStr"/>
+      <c r="AE295" s="27" t="inlineStr"/>
+      <c r="AF295" s="27" t="inlineStr"/>
+      <c r="AG295" s="2" t="inlineStr"/>
+      <c r="AH295" s="2" t="inlineStr"/>
+      <c r="AI295" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -19361,8 +19475,7 @@
     <mergeCell ref="Z252:AB252"/>
     <mergeCell ref="AC252:AD252"/>
     <mergeCell ref="AE252:AI252"/>
-    <mergeCell ref="H253:L253"/>
-    <mergeCell ref="M253:P253"/>
+    <mergeCell ref="N253:P253"/>
     <mergeCell ref="Q253:R253"/>
     <mergeCell ref="S253:V253"/>
     <mergeCell ref="X253:Y253"/>
@@ -19370,7 +19483,8 @@
     <mergeCell ref="AC253:AD253"/>
     <mergeCell ref="AE253:AI253"/>
     <mergeCell ref="B254:AF254"/>
-    <mergeCell ref="N255:P255"/>
+    <mergeCell ref="H255:L255"/>
+    <mergeCell ref="M255:P255"/>
     <mergeCell ref="Q255:R255"/>
     <mergeCell ref="S255:V255"/>
     <mergeCell ref="X255:Y255"/>
@@ -19482,15 +19596,15 @@
     <mergeCell ref="Z270:AB270"/>
     <mergeCell ref="AC270:AD270"/>
     <mergeCell ref="AE270:AI270"/>
-    <mergeCell ref="H271:L271"/>
-    <mergeCell ref="M271:P271"/>
+    <mergeCell ref="N271:P271"/>
     <mergeCell ref="Q271:R271"/>
     <mergeCell ref="S271:V271"/>
     <mergeCell ref="X271:Y271"/>
     <mergeCell ref="Z271:AB271"/>
     <mergeCell ref="AC271:AD271"/>
     <mergeCell ref="AE271:AI271"/>
-    <mergeCell ref="N272:P272"/>
+    <mergeCell ref="H272:L272"/>
+    <mergeCell ref="M272:P272"/>
     <mergeCell ref="Q272:R272"/>
     <mergeCell ref="S272:V272"/>
     <mergeCell ref="X272:Y272"/>
@@ -19511,23 +19625,23 @@
     <mergeCell ref="Z274:AB274"/>
     <mergeCell ref="AC274:AD274"/>
     <mergeCell ref="AE274:AI274"/>
-    <mergeCell ref="F275:K275"/>
-    <mergeCell ref="L275:P275"/>
+    <mergeCell ref="N275:P275"/>
     <mergeCell ref="Q275:R275"/>
     <mergeCell ref="S275:V275"/>
     <mergeCell ref="X275:Y275"/>
     <mergeCell ref="Z275:AB275"/>
     <mergeCell ref="AC275:AD275"/>
     <mergeCell ref="AE275:AI275"/>
-    <mergeCell ref="H276:L276"/>
-    <mergeCell ref="M276:P276"/>
+    <mergeCell ref="F276:K276"/>
+    <mergeCell ref="L276:P276"/>
     <mergeCell ref="Q276:R276"/>
     <mergeCell ref="S276:V276"/>
     <mergeCell ref="X276:Y276"/>
     <mergeCell ref="Z276:AB276"/>
     <mergeCell ref="AC276:AD276"/>
     <mergeCell ref="AE276:AI276"/>
-    <mergeCell ref="N277:P277"/>
+    <mergeCell ref="H277:L277"/>
+    <mergeCell ref="M277:P277"/>
     <mergeCell ref="Q277:R277"/>
     <mergeCell ref="S277:V277"/>
     <mergeCell ref="X277:Y277"/>
@@ -19577,69 +19691,83 @@
     <mergeCell ref="Z284:AB284"/>
     <mergeCell ref="AC284:AD284"/>
     <mergeCell ref="AE284:AI284"/>
-    <mergeCell ref="H285:L285"/>
-    <mergeCell ref="M285:P285"/>
+    <mergeCell ref="N285:P285"/>
     <mergeCell ref="Q285:R285"/>
     <mergeCell ref="S285:V285"/>
     <mergeCell ref="X285:Y285"/>
     <mergeCell ref="Z285:AB285"/>
     <mergeCell ref="AC285:AD285"/>
     <mergeCell ref="AE285:AI285"/>
-    <mergeCell ref="N286:P286"/>
+    <mergeCell ref="H286:L286"/>
+    <mergeCell ref="M286:P286"/>
     <mergeCell ref="Q286:R286"/>
     <mergeCell ref="S286:V286"/>
     <mergeCell ref="X286:Y286"/>
     <mergeCell ref="Z286:AB286"/>
     <mergeCell ref="AC286:AD286"/>
     <mergeCell ref="AE286:AI286"/>
-    <mergeCell ref="C287:F287"/>
-    <mergeCell ref="G287:P287"/>
+    <mergeCell ref="N287:P287"/>
     <mergeCell ref="Q287:R287"/>
     <mergeCell ref="S287:V287"/>
     <mergeCell ref="X287:Y287"/>
     <mergeCell ref="Z287:AB287"/>
     <mergeCell ref="AC287:AD287"/>
     <mergeCell ref="AE287:AI287"/>
-    <mergeCell ref="C288:J288"/>
-    <mergeCell ref="K288:P288"/>
+    <mergeCell ref="N288:P288"/>
     <mergeCell ref="Q288:R288"/>
     <mergeCell ref="S288:V288"/>
     <mergeCell ref="X288:Y288"/>
     <mergeCell ref="Z288:AB288"/>
     <mergeCell ref="AC288:AD288"/>
     <mergeCell ref="AE288:AI288"/>
-    <mergeCell ref="E289:I289"/>
-    <mergeCell ref="J289:P289"/>
+    <mergeCell ref="C289:F289"/>
+    <mergeCell ref="G289:P289"/>
     <mergeCell ref="Q289:R289"/>
     <mergeCell ref="S289:V289"/>
     <mergeCell ref="X289:Y289"/>
     <mergeCell ref="Z289:AB289"/>
     <mergeCell ref="AC289:AD289"/>
     <mergeCell ref="AE289:AI289"/>
-    <mergeCell ref="F290:K290"/>
-    <mergeCell ref="L290:P290"/>
+    <mergeCell ref="C290:J290"/>
+    <mergeCell ref="K290:P290"/>
     <mergeCell ref="Q290:R290"/>
     <mergeCell ref="S290:V290"/>
     <mergeCell ref="X290:Y290"/>
     <mergeCell ref="Z290:AB290"/>
     <mergeCell ref="AC290:AD290"/>
     <mergeCell ref="AE290:AI290"/>
-    <mergeCell ref="H291:L291"/>
-    <mergeCell ref="M291:P291"/>
+    <mergeCell ref="E291:I291"/>
+    <mergeCell ref="J291:P291"/>
     <mergeCell ref="Q291:R291"/>
     <mergeCell ref="S291:V291"/>
     <mergeCell ref="X291:Y291"/>
     <mergeCell ref="Z291:AB291"/>
     <mergeCell ref="AC291:AD291"/>
     <mergeCell ref="AE291:AI291"/>
-    <mergeCell ref="N292:P292"/>
+    <mergeCell ref="F292:K292"/>
+    <mergeCell ref="L292:P292"/>
     <mergeCell ref="Q292:R292"/>
     <mergeCell ref="S292:V292"/>
     <mergeCell ref="X292:Y292"/>
     <mergeCell ref="Z292:AB292"/>
     <mergeCell ref="AC292:AD292"/>
     <mergeCell ref="AE292:AI292"/>
-    <mergeCell ref="B293:AF293"/>
+    <mergeCell ref="H293:L293"/>
+    <mergeCell ref="M293:P293"/>
+    <mergeCell ref="Q293:R293"/>
+    <mergeCell ref="S293:V293"/>
+    <mergeCell ref="X293:Y293"/>
+    <mergeCell ref="Z293:AB293"/>
+    <mergeCell ref="AC293:AD293"/>
+    <mergeCell ref="AE293:AI293"/>
+    <mergeCell ref="N294:P294"/>
+    <mergeCell ref="Q294:R294"/>
+    <mergeCell ref="S294:V294"/>
+    <mergeCell ref="X294:Y294"/>
+    <mergeCell ref="Z294:AB294"/>
+    <mergeCell ref="AC294:AD294"/>
+    <mergeCell ref="AE294:AI294"/>
+    <mergeCell ref="B295:AF295"/>
   </mergeCells>
   <pageMargins left="0.0" right="0.0" top="0.0" bottom="0.00" header="0.0" footer="0.0"/>
   <pageSetup orientation="landscape" paperSize="9"/>

</xml_diff>

<commit_message>
DIPA REV 11 dan update realisasi
DIPA REV 11 dan update realisasi
</commit_message>
<xml_diff>
--- a/Database/Akrual.xlsx
+++ b/Database/Akrual.xlsx
@@ -982,19 +982,19 @@
         <v>9.0559784495E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>8.096493585E9</v>
+        <v>8.742642945E9</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>9.865627808E10</v>
+        <v>9.930242744E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.986601869966088</v>
+        <v>0.9930636195806077</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>1.33975992E9</v>
+        <v>6.9361056E8</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1714,20 +1714,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X21" s="14" t="n">
-        <v>8.096493585E9</v>
+        <v>8.742642945E9</v>
       </c>
       <c r="Y21" s="14" t="inlineStr"/>
       <c r="Z21" s="14" t="n">
-        <v>9.462291004E10</v>
+        <v>9.52690594E10</v>
       </c>
       <c r="AA21" s="14" t="inlineStr"/>
       <c r="AB21" s="14" t="inlineStr"/>
       <c r="AC21" s="15" t="n">
-        <v>0.9860390669960531</v>
+        <v>0.9927724100289949</v>
       </c>
       <c r="AD21" s="15" t="inlineStr"/>
       <c r="AE21" s="14" t="n">
-        <v>1.33972796E9</v>
+        <v>6.935786E8</v>
       </c>
       <c r="AF21" s="14" t="inlineStr"/>
       <c r="AG21" s="14" t="inlineStr"/>
@@ -1777,20 +1777,20 @@
         <v>8.6526416455E10</v>
       </c>
       <c r="X22" s="14" t="n">
-        <v>8.096493585E9</v>
+        <v>8.742642945E9</v>
       </c>
       <c r="Y22" s="14" t="inlineStr"/>
       <c r="Z22" s="14" t="n">
-        <v>9.462291004E10</v>
+        <v>9.52690594E10</v>
       </c>
       <c r="AA22" s="14" t="inlineStr"/>
       <c r="AB22" s="14" t="inlineStr"/>
       <c r="AC22" s="15" t="n">
-        <v>0.9860390669960531</v>
+        <v>0.9927724100289949</v>
       </c>
       <c r="AD22" s="15" t="inlineStr"/>
       <c r="AE22" s="14" t="n">
-        <v>1.33972796E9</v>
+        <v>6.935786E8</v>
       </c>
       <c r="AF22" s="14" t="inlineStr"/>
       <c r="AG22" s="14" t="inlineStr"/>
@@ -1840,20 +1840,20 @@
         <v>8.6525816455E10</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>8.096493585E9</v>
+        <v>8.742642945E9</v>
       </c>
       <c r="Y23" s="17" t="inlineStr"/>
       <c r="Z23" s="17" t="n">
-        <v>9.462231004E10</v>
+        <v>9.52684594E10</v>
       </c>
       <c r="AA23" s="17" t="inlineStr"/>
       <c r="AB23" s="17" t="inlineStr"/>
       <c r="AC23" s="18" t="n">
-        <v>0.9860389797057041</v>
+        <v>0.9927723648386876</v>
       </c>
       <c r="AD23" s="18" t="inlineStr"/>
       <c r="AE23" s="17" t="n">
-        <v>1.33972796E9</v>
+        <v>6.935786E8</v>
       </c>
       <c r="AF23" s="17" t="inlineStr"/>
       <c r="AG23" s="17" t="inlineStr"/>
@@ -3233,20 +3233,20 @@
         <v>8.6508305403E10</v>
       </c>
       <c r="X46" s="22" t="n">
-        <v>8.095693585E9</v>
+        <v>8.741842945E9</v>
       </c>
       <c r="Y46" s="22" t="inlineStr"/>
       <c r="Z46" s="21" t="n">
-        <v>9.4603998988E10</v>
+        <v>9.5250148348E10</v>
       </c>
       <c r="AA46" s="21" t="inlineStr"/>
       <c r="AB46" s="21" t="inlineStr"/>
       <c r="AC46" s="23" t="n">
-        <v>0.9860385654024658</v>
+        <v>0.9927732509843188</v>
       </c>
       <c r="AD46" s="23" t="inlineStr"/>
       <c r="AE46" s="21" t="n">
-        <v>1.339509012E9</v>
+        <v>6.93359652E8</v>
       </c>
       <c r="AF46" s="21" t="inlineStr"/>
       <c r="AG46" s="21" t="inlineStr"/>
@@ -3296,20 +3296,20 @@
         <v>8.0279551347E10</v>
       </c>
       <c r="X47" s="25" t="n">
-        <v>7.495823038E9</v>
+        <v>8.034845038E9</v>
       </c>
       <c r="Y47" s="25" t="inlineStr"/>
       <c r="Z47" s="25" t="n">
-        <v>8.7775374385E10</v>
+        <v>8.8314396385E10</v>
       </c>
       <c r="AA47" s="25" t="inlineStr"/>
       <c r="AB47" s="25" t="inlineStr"/>
       <c r="AC47" s="26" t="n">
-        <v>0.9862764765507153</v>
+        <v>0.9923331265242205</v>
       </c>
       <c r="AD47" s="26" t="inlineStr"/>
       <c r="AE47" s="25" t="n">
-        <v>1.221348615E9</v>
+        <v>6.82326615E8</v>
       </c>
       <c r="AF47" s="25" t="inlineStr"/>
       <c r="AG47" s="25" t="inlineStr"/>
@@ -3359,20 +3359,20 @@
         <v>5.831238104E9</v>
       </c>
       <c r="X48" s="14" t="n">
-        <v>2.8323E7</v>
+        <v>5.3354E7</v>
       </c>
       <c r="Y48" s="14" t="inlineStr"/>
       <c r="Z48" s="14" t="n">
-        <v>5.859561104E9</v>
+        <v>5.884592104E9</v>
       </c>
       <c r="AA48" s="14" t="inlineStr"/>
       <c r="AB48" s="14" t="inlineStr"/>
       <c r="AC48" s="15" t="n">
-        <v>0.9897271972407177</v>
+        <v>0.9939551353122603</v>
       </c>
       <c r="AD48" s="15" t="inlineStr"/>
       <c r="AE48" s="14" t="n">
-        <v>6.0818896E7</v>
+        <v>3.5787896E7</v>
       </c>
       <c r="AF48" s="14" t="inlineStr"/>
       <c r="AG48" s="14" t="inlineStr"/>
@@ -5337,20 +5337,20 @@
         <v>2.77741E8</v>
       </c>
       <c r="X82" s="14" t="n">
-        <v>2.8323E7</v>
+        <v>5.3354E7</v>
       </c>
       <c r="Y82" s="14" t="inlineStr"/>
       <c r="Z82" s="14" t="n">
-        <v>3.06064E8</v>
+        <v>3.31095E8</v>
       </c>
       <c r="AA82" s="14" t="inlineStr"/>
       <c r="AB82" s="14" t="inlineStr"/>
       <c r="AC82" s="15" t="n">
-        <v>0.9049900057954559</v>
+        <v>0.9790032998616187</v>
       </c>
       <c r="AD82" s="15" t="inlineStr"/>
       <c r="AE82" s="14" t="n">
-        <v>3.2132E7</v>
+        <v>7101000.0</v>
       </c>
       <c r="AF82" s="14" t="inlineStr"/>
       <c r="AG82" s="14" t="inlineStr"/>
@@ -5394,20 +5394,20 @@
         <v>1.554E7</v>
       </c>
       <c r="X83" s="14" t="n">
-        <v>1400000.0</v>
+        <v>2870000.0</v>
       </c>
       <c r="Y83" s="14" t="inlineStr"/>
       <c r="Z83" s="14" t="n">
-        <v>1.694E7</v>
+        <v>1.841E7</v>
       </c>
       <c r="AA83" s="14" t="inlineStr"/>
       <c r="AB83" s="14" t="inlineStr"/>
       <c r="AC83" s="15" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9962121212121212</v>
       </c>
       <c r="AD83" s="15" t="inlineStr"/>
       <c r="AE83" s="14" t="n">
-        <v>1540000.0</v>
+        <v>70000.0</v>
       </c>
       <c r="AF83" s="14" t="inlineStr"/>
       <c r="AG83" s="14" t="inlineStr"/>
@@ -5451,20 +5451,20 @@
         <v>2.28253E8</v>
       </c>
       <c r="X84" s="14" t="n">
-        <v>2.3643E7</v>
+        <v>4.5769E7</v>
       </c>
       <c r="Y84" s="14" t="inlineStr"/>
       <c r="Z84" s="14" t="n">
-        <v>2.51896E8</v>
+        <v>2.74022E8</v>
       </c>
       <c r="AA84" s="14" t="inlineStr"/>
       <c r="AB84" s="14" t="inlineStr"/>
       <c r="AC84" s="15" t="n">
-        <v>0.9048378522062732</v>
+        <v>0.9843168527379054</v>
       </c>
       <c r="AD84" s="15" t="inlineStr"/>
       <c r="AE84" s="14" t="n">
-        <v>2.6492E7</v>
+        <v>4366000.0</v>
       </c>
       <c r="AF84" s="14" t="inlineStr"/>
       <c r="AG84" s="14" t="inlineStr"/>
@@ -5508,20 +5508,20 @@
         <v>3.3948E7</v>
       </c>
       <c r="X85" s="14" t="n">
-        <v>3280000.0</v>
+        <v>4715000.0</v>
       </c>
       <c r="Y85" s="14" t="inlineStr"/>
       <c r="Z85" s="14" t="n">
-        <v>3.7228E7</v>
+        <v>3.8663E7</v>
       </c>
       <c r="AA85" s="14" t="inlineStr"/>
       <c r="AB85" s="14" t="inlineStr"/>
       <c r="AC85" s="15" t="n">
-        <v>0.9007936507936508</v>
+        <v>0.935515873015873</v>
       </c>
       <c r="AD85" s="15" t="inlineStr"/>
       <c r="AE85" s="14" t="n">
-        <v>4100000.0</v>
+        <v>2665000.0</v>
       </c>
       <c r="AF85" s="14" t="inlineStr"/>
       <c r="AG85" s="14" t="inlineStr"/>
@@ -6082,20 +6082,20 @@
         <v>5.93914035E8</v>
       </c>
       <c r="X95" s="14" t="n">
-        <v>3.10703762E8</v>
+        <v>3.39619762E8</v>
       </c>
       <c r="Y95" s="14" t="inlineStr"/>
       <c r="Z95" s="14" t="n">
-        <v>9.04617797E8</v>
+        <v>9.33533797E8</v>
       </c>
       <c r="AA95" s="14" t="inlineStr"/>
       <c r="AB95" s="14" t="inlineStr"/>
       <c r="AC95" s="15" t="n">
-        <v>0.9302087704848075</v>
+        <v>0.9599427829003722</v>
       </c>
       <c r="AD95" s="15" t="inlineStr"/>
       <c r="AE95" s="14" t="n">
-        <v>6.7871203E7</v>
+        <v>3.8955203E7</v>
       </c>
       <c r="AF95" s="14" t="inlineStr"/>
       <c r="AG95" s="14" t="inlineStr"/>
@@ -6745,20 +6745,20 @@
         <v>3.0833E7</v>
       </c>
       <c r="X106" s="14" t="n">
-        <v>2.694E7</v>
+        <v>5.5856E7</v>
       </c>
       <c r="Y106" s="14" t="inlineStr"/>
       <c r="Z106" s="14" t="n">
-        <v>5.7773E7</v>
+        <v>8.6689E7</v>
       </c>
       <c r="AA106" s="14" t="inlineStr"/>
       <c r="AB106" s="14" t="inlineStr"/>
       <c r="AC106" s="15" t="n">
-        <v>0.6554908835108978</v>
+        <v>0.9835710314623825</v>
       </c>
       <c r="AD106" s="15" t="inlineStr"/>
       <c r="AE106" s="14" t="n">
-        <v>3.0364E7</v>
+        <v>1448000.0</v>
       </c>
       <c r="AF106" s="14" t="inlineStr"/>
       <c r="AG106" s="14" t="inlineStr"/>
@@ -6802,20 +6802,20 @@
         <v>8855000.0</v>
       </c>
       <c r="X107" s="14" t="n">
-        <v>7700000.0</v>
+        <v>1.5785E7</v>
       </c>
       <c r="Y107" s="14" t="inlineStr"/>
       <c r="Z107" s="14" t="n">
-        <v>1.6555E7</v>
+        <v>2.464E7</v>
       </c>
       <c r="AA107" s="14" t="inlineStr"/>
       <c r="AB107" s="14" t="inlineStr"/>
       <c r="AC107" s="15" t="n">
-        <v>0.6569444444444444</v>
+        <v>0.9777777777777777</v>
       </c>
       <c r="AD107" s="15" t="inlineStr"/>
       <c r="AE107" s="14" t="n">
-        <v>8645000.0</v>
+        <v>560000.0</v>
       </c>
       <c r="AF107" s="14" t="inlineStr"/>
       <c r="AG107" s="14" t="inlineStr"/>
@@ -6859,20 +6859,20 @@
         <v>2.1978E7</v>
       </c>
       <c r="X108" s="14" t="n">
-        <v>1.924E7</v>
+        <v>4.0071E7</v>
       </c>
       <c r="Y108" s="14" t="inlineStr"/>
       <c r="Z108" s="14" t="n">
-        <v>4.1218E7</v>
+        <v>6.2049E7</v>
       </c>
       <c r="AA108" s="14" t="inlineStr"/>
       <c r="AB108" s="14" t="inlineStr"/>
       <c r="AC108" s="15" t="n">
-        <v>0.6549088771310994</v>
+        <v>0.9858906525573192</v>
       </c>
       <c r="AD108" s="15" t="inlineStr"/>
       <c r="AE108" s="14" t="n">
-        <v>2.1719E7</v>
+        <v>888000.0</v>
       </c>
       <c r="AF108" s="14" t="inlineStr"/>
       <c r="AG108" s="14" t="inlineStr"/>
@@ -7162,20 +7162,20 @@
         <v>5.0689888E10</v>
       </c>
       <c r="X113" s="14" t="n">
-        <v>3.759233212E9</v>
+        <v>3.988527212E9</v>
       </c>
       <c r="Y113" s="14" t="inlineStr"/>
       <c r="Z113" s="14" t="n">
-        <v>5.4449121212E10</v>
+        <v>5.4678415212E10</v>
       </c>
       <c r="AA113" s="14" t="inlineStr"/>
       <c r="AB113" s="14" t="inlineStr"/>
       <c r="AC113" s="15" t="n">
-        <v>0.987214096723776</v>
+        <v>0.9913714139413089</v>
       </c>
       <c r="AD113" s="15" t="inlineStr"/>
       <c r="AE113" s="14" t="n">
-        <v>7.05197788E8</v>
+        <v>4.75903788E8</v>
       </c>
       <c r="AF113" s="14" t="inlineStr"/>
       <c r="AG113" s="14" t="inlineStr"/>
@@ -8906,20 +8906,20 @@
         <v>2.213268E9</v>
       </c>
       <c r="X143" s="14" t="n">
-        <v>2.19192E8</v>
+        <v>4.48486E8</v>
       </c>
       <c r="Y143" s="14" t="inlineStr"/>
       <c r="Z143" s="14" t="n">
-        <v>2.43246E9</v>
+        <v>2.661754E9</v>
       </c>
       <c r="AA143" s="14" t="inlineStr"/>
       <c r="AB143" s="14" t="inlineStr"/>
       <c r="AC143" s="15" t="n">
-        <v>0.904383945461684</v>
+        <v>0.9896350132657553</v>
       </c>
       <c r="AD143" s="15" t="inlineStr"/>
       <c r="AE143" s="14" t="n">
-        <v>2.57172E8</v>
+        <v>2.7878E7</v>
       </c>
       <c r="AF143" s="14" t="inlineStr"/>
       <c r="AG143" s="14" t="inlineStr"/>
@@ -8963,20 +8963,20 @@
         <v>1.9894E8</v>
       </c>
       <c r="X144" s="14" t="n">
-        <v>3.0567E7</v>
+        <v>5.1952E7</v>
       </c>
       <c r="Y144" s="14" t="inlineStr"/>
       <c r="Z144" s="14" t="n">
-        <v>2.29507E8</v>
+        <v>2.50892E8</v>
       </c>
       <c r="AA144" s="14" t="inlineStr"/>
       <c r="AB144" s="14" t="inlineStr"/>
       <c r="AC144" s="15" t="n">
-        <v>0.9107420634920635</v>
+        <v>0.9956031746031746</v>
       </c>
       <c r="AD144" s="15" t="inlineStr"/>
       <c r="AE144" s="14" t="n">
-        <v>2.2493E7</v>
+        <v>1108000.0</v>
       </c>
       <c r="AF144" s="14" t="inlineStr"/>
       <c r="AG144" s="14" t="inlineStr"/>
@@ -9063,20 +9063,20 @@
         <v>1.581491E9</v>
       </c>
       <c r="X146" s="14" t="n">
-        <v>1.60099E8</v>
+        <v>3.29263E8</v>
       </c>
       <c r="Y146" s="14" t="inlineStr"/>
       <c r="Z146" s="14" t="n">
-        <v>1.74159E9</v>
+        <v>1.910754E9</v>
       </c>
       <c r="AA146" s="14" t="inlineStr"/>
       <c r="AB146" s="14" t="inlineStr"/>
       <c r="AC146" s="15" t="n">
-        <v>0.9079861111111112</v>
+        <v>0.9961805555555555</v>
       </c>
       <c r="AD146" s="15" t="inlineStr"/>
       <c r="AE146" s="14" t="n">
-        <v>1.7649E8</v>
+        <v>7326000.0</v>
       </c>
       <c r="AF146" s="14" t="inlineStr"/>
       <c r="AG146" s="14" t="inlineStr"/>
@@ -9120,20 +9120,20 @@
         <v>4.32837E8</v>
       </c>
       <c r="X147" s="14" t="n">
-        <v>2.8526E7</v>
+        <v>6.7271E7</v>
       </c>
       <c r="Y147" s="14" t="inlineStr"/>
       <c r="Z147" s="14" t="n">
-        <v>4.61363E8</v>
+        <v>5.00108E8</v>
       </c>
       <c r="AA147" s="14" t="inlineStr"/>
       <c r="AB147" s="14" t="inlineStr"/>
       <c r="AC147" s="15" t="n">
-        <v>0.8880015859817689</v>
+        <v>0.9625754496181326</v>
       </c>
       <c r="AD147" s="15" t="inlineStr"/>
       <c r="AE147" s="14" t="n">
-        <v>5.8189E7</v>
+        <v>1.9444E7</v>
       </c>
       <c r="AF147" s="14" t="inlineStr"/>
       <c r="AG147" s="14" t="inlineStr"/>
@@ -9651,20 +9651,20 @@
         <v>2.3164511208E10</v>
       </c>
       <c r="X156" s="14" t="n">
-        <v>3.397563064E9</v>
+        <v>3.653344064E9</v>
       </c>
       <c r="Y156" s="14" t="inlineStr"/>
       <c r="Z156" s="14" t="n">
-        <v>2.6562074272E10</v>
+        <v>2.6817855272E10</v>
       </c>
       <c r="AA156" s="14" t="inlineStr"/>
       <c r="AB156" s="14" t="inlineStr"/>
       <c r="AC156" s="15" t="n">
-        <v>0.9856227304849602</v>
+        <v>0.9951138404428871</v>
       </c>
       <c r="AD156" s="15" t="inlineStr"/>
       <c r="AE156" s="14" t="n">
-        <v>3.87460728E8</v>
+        <v>1.31679728E8</v>
       </c>
       <c r="AF156" s="14" t="inlineStr"/>
       <c r="AG156" s="14" t="inlineStr"/>
@@ -11161,20 +11161,20 @@
         <v>1.310426E9</v>
       </c>
       <c r="X182" s="14" t="n">
-        <v>2.45185E8</v>
+        <v>5.00966E8</v>
       </c>
       <c r="Y182" s="14" t="inlineStr"/>
       <c r="Z182" s="14" t="n">
-        <v>1.555611E9</v>
+        <v>1.811392E9</v>
       </c>
       <c r="AA182" s="14" t="inlineStr"/>
       <c r="AB182" s="14" t="inlineStr"/>
       <c r="AC182" s="15" t="n">
-        <v>0.8509534593672049</v>
+        <v>0.9908712966609776</v>
       </c>
       <c r="AD182" s="15" t="inlineStr"/>
       <c r="AE182" s="14" t="n">
-        <v>2.72469E8</v>
+        <v>1.6688E7</v>
       </c>
       <c r="AF182" s="14" t="inlineStr"/>
       <c r="AG182" s="14" t="inlineStr"/>
@@ -11218,20 +11218,20 @@
         <v>1.2502E8</v>
       </c>
       <c r="X183" s="14" t="n">
-        <v>2.226E7</v>
+        <v>4.557E7</v>
       </c>
       <c r="Y183" s="14" t="inlineStr"/>
       <c r="Z183" s="14" t="n">
-        <v>1.4728E8</v>
+        <v>1.7059E8</v>
       </c>
       <c r="AA183" s="14" t="inlineStr"/>
       <c r="AB183" s="14" t="inlineStr"/>
       <c r="AC183" s="15" t="n">
-        <v>0.834920634920635</v>
+        <v>0.9670634920634921</v>
       </c>
       <c r="AD183" s="15" t="inlineStr"/>
       <c r="AE183" s="14" t="n">
-        <v>2.912E7</v>
+        <v>5810000.0</v>
       </c>
       <c r="AF183" s="14" t="inlineStr"/>
       <c r="AG183" s="14" t="inlineStr"/>
@@ -11275,20 +11275,20 @@
         <v>1.185406E9</v>
       </c>
       <c r="X184" s="14" t="n">
-        <v>2.22925E8</v>
+        <v>4.55396E8</v>
       </c>
       <c r="Y184" s="14" t="inlineStr"/>
       <c r="Z184" s="14" t="n">
-        <v>1.408331E9</v>
+        <v>1.640802E9</v>
       </c>
       <c r="AA184" s="14" t="inlineStr"/>
       <c r="AB184" s="14" t="inlineStr"/>
       <c r="AC184" s="15" t="n">
-        <v>0.852665770609319</v>
+        <v>0.9934139784946237</v>
       </c>
       <c r="AD184" s="15" t="inlineStr"/>
       <c r="AE184" s="14" t="n">
-        <v>2.43349E8</v>
+        <v>1.0878E7</v>
       </c>
       <c r="AF184" s="14" t="inlineStr"/>
       <c r="AG184" s="14" t="inlineStr"/>
@@ -11572,20 +11572,20 @@
         <v>6.228754056E9</v>
       </c>
       <c r="X189" s="25" t="n">
-        <v>5.99870547E8</v>
+        <v>7.06997907E8</v>
       </c>
       <c r="Y189" s="25" t="inlineStr"/>
       <c r="Z189" s="25" t="n">
-        <v>6.828624603E9</v>
+        <v>6.935751963E9</v>
       </c>
       <c r="AA189" s="25" t="inlineStr"/>
       <c r="AB189" s="25" t="inlineStr"/>
       <c r="AC189" s="26" t="n">
-        <v>0.9829906356681544</v>
+        <v>0.9984117779663543</v>
       </c>
       <c r="AD189" s="26" t="inlineStr"/>
       <c r="AE189" s="25" t="n">
-        <v>1.18160397E8</v>
+        <v>1.1033037E7</v>
       </c>
       <c r="AF189" s="25" t="inlineStr"/>
       <c r="AG189" s="25" t="inlineStr"/>
@@ -11635,20 +11635,20 @@
         <v>4.783558496E9</v>
       </c>
       <c r="X190" s="14" t="n">
-        <v>1.9710595E8</v>
+        <v>2.21112562E8</v>
       </c>
       <c r="Y190" s="14" t="inlineStr"/>
       <c r="Z190" s="14" t="n">
-        <v>4.980664446E9</v>
+        <v>5.004671058E9</v>
       </c>
       <c r="AA190" s="14" t="inlineStr"/>
       <c r="AB190" s="14" t="inlineStr"/>
       <c r="AC190" s="15" t="n">
-        <v>0.9943994520751426</v>
+        <v>0.9991924193745463</v>
       </c>
       <c r="AD190" s="15" t="inlineStr"/>
       <c r="AE190" s="14" t="n">
-        <v>2.8051554E7</v>
+        <v>4044942.0</v>
       </c>
       <c r="AF190" s="14" t="inlineStr"/>
       <c r="AG190" s="14" t="inlineStr"/>
@@ -11698,20 +11698,20 @@
         <v>1.777909494E9</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>1.07421314E8</v>
+        <v>1.14587926E8</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
-        <v>1.885330808E9</v>
+        <v>1.89249742E9</v>
       </c>
       <c r="AA191" s="14" t="inlineStr"/>
       <c r="AB191" s="14" t="inlineStr"/>
       <c r="AC191" s="15" t="n">
-        <v>0.9960081124758108</v>
+        <v>0.9997941873973459</v>
       </c>
       <c r="AD191" s="15" t="inlineStr"/>
       <c r="AE191" s="14" t="n">
-        <v>7556192.0</v>
+        <v>389580.0</v>
       </c>
       <c r="AF191" s="14" t="inlineStr"/>
       <c r="AG191" s="14" t="inlineStr"/>
@@ -11869,20 +11869,20 @@
         <v>5.5184254E7</v>
       </c>
       <c r="X194" s="14" t="n">
-        <v>3.3419714E7</v>
+        <v>4.0586326E7</v>
       </c>
       <c r="Y194" s="14" t="inlineStr"/>
       <c r="Z194" s="14" t="n">
-        <v>8.8603968E7</v>
+        <v>9.577058E7</v>
       </c>
       <c r="AA194" s="14" t="inlineStr"/>
       <c r="AB194" s="14" t="inlineStr"/>
       <c r="AC194" s="15" t="n">
-        <v>0.922958</v>
+        <v>0.9976102083333334</v>
       </c>
       <c r="AD194" s="15" t="inlineStr"/>
       <c r="AE194" s="14" t="n">
-        <v>7396032.0</v>
+        <v>229420.0</v>
       </c>
       <c r="AF194" s="14" t="inlineStr"/>
       <c r="AG194" s="14" t="inlineStr"/>
@@ -12317,20 +12317,20 @@
         <v>9417000.0</v>
       </c>
       <c r="X202" s="14" t="n">
-        <v>3215000.0</v>
+        <v>4155500.0</v>
       </c>
       <c r="Y202" s="14" t="inlineStr"/>
       <c r="Z202" s="14" t="n">
-        <v>1.2632E7</v>
+        <v>1.35725E7</v>
       </c>
       <c r="AA202" s="14" t="inlineStr"/>
       <c r="AB202" s="14" t="inlineStr"/>
       <c r="AC202" s="15" t="n">
-        <v>0.8489247311827957</v>
+        <v>0.912130376344086</v>
       </c>
       <c r="AD202" s="15" t="inlineStr"/>
       <c r="AE202" s="14" t="n">
-        <v>2248000.0</v>
+        <v>1307500.0</v>
       </c>
       <c r="AF202" s="14" t="inlineStr"/>
       <c r="AG202" s="14" t="inlineStr"/>
@@ -12374,20 +12374,20 @@
         <v>5781000.0</v>
       </c>
       <c r="X203" s="14" t="n">
-        <v>2407000.0</v>
+        <v>3347500.0</v>
       </c>
       <c r="Y203" s="14" t="inlineStr"/>
       <c r="Z203" s="14" t="n">
-        <v>8188000.0</v>
+        <v>9128500.0</v>
       </c>
       <c r="AA203" s="14" t="inlineStr"/>
       <c r="AB203" s="14" t="inlineStr"/>
       <c r="AC203" s="15" t="n">
-        <v>0.7888246628131022</v>
+        <v>0.879431599229287</v>
       </c>
       <c r="AD203" s="15" t="inlineStr"/>
       <c r="AE203" s="14" t="n">
-        <v>2192000.0</v>
+        <v>1251500.0</v>
       </c>
       <c r="AF203" s="14" t="inlineStr"/>
       <c r="AG203" s="14" t="inlineStr"/>
@@ -12494,20 +12494,20 @@
         <v>5.526601E7</v>
       </c>
       <c r="X205" s="14" t="n">
-        <v>1.23661E7</v>
+        <v>2.15411E7</v>
       </c>
       <c r="Y205" s="14" t="inlineStr"/>
       <c r="Z205" s="14" t="n">
-        <v>6.763211E7</v>
+        <v>7.680711E7</v>
       </c>
       <c r="AA205" s="14" t="inlineStr"/>
       <c r="AB205" s="14" t="inlineStr"/>
       <c r="AC205" s="15" t="n">
-        <v>0.8606674641452768</v>
+        <v>0.9774259681093395</v>
       </c>
       <c r="AD205" s="15" t="inlineStr"/>
       <c r="AE205" s="14" t="n">
-        <v>1.094889E7</v>
+        <v>1773890.0</v>
       </c>
       <c r="AF205" s="14" t="inlineStr"/>
       <c r="AG205" s="14" t="inlineStr"/>
@@ -12551,20 +12551,20 @@
         <v>5.526601E7</v>
       </c>
       <c r="X206" s="14" t="n">
-        <v>9616100.0</v>
+        <v>1.57661E7</v>
       </c>
       <c r="Y206" s="14" t="inlineStr"/>
       <c r="Z206" s="14" t="n">
-        <v>6.488211E7</v>
+        <v>7.103211E7</v>
       </c>
       <c r="AA206" s="14" t="inlineStr"/>
       <c r="AB206" s="14" t="inlineStr"/>
       <c r="AC206" s="15" t="n">
-        <v>0.8949133115405304</v>
+        <v>0.9797397277278934</v>
       </c>
       <c r="AD206" s="15" t="inlineStr"/>
       <c r="AE206" s="14" t="n">
-        <v>7618890.0</v>
+        <v>1468890.0</v>
       </c>
       <c r="AF206" s="14" t="inlineStr"/>
       <c r="AG206" s="14" t="inlineStr"/>
@@ -12608,20 +12608,20 @@
         <v>0.0</v>
       </c>
       <c r="X207" s="14" t="n">
-        <v>2750000.0</v>
+        <v>5775000.0</v>
       </c>
       <c r="Y207" s="14" t="inlineStr"/>
       <c r="Z207" s="14" t="n">
-        <v>2750000.0</v>
+        <v>5775000.0</v>
       </c>
       <c r="AA207" s="14" t="inlineStr"/>
       <c r="AB207" s="14" t="inlineStr"/>
       <c r="AC207" s="15" t="n">
-        <v>0.45230263157894735</v>
+        <v>0.9498355263157895</v>
       </c>
       <c r="AD207" s="15" t="inlineStr"/>
       <c r="AE207" s="14" t="n">
-        <v>3330000.0</v>
+        <v>305000.0</v>
       </c>
       <c r="AF207" s="14" t="inlineStr"/>
       <c r="AG207" s="14" t="inlineStr"/>
@@ -12671,20 +12671,20 @@
         <v>4274800.0</v>
       </c>
       <c r="X208" s="14" t="n">
-        <v>0.0</v>
+        <v>6724500.0</v>
       </c>
       <c r="Y208" s="14" t="inlineStr"/>
       <c r="Z208" s="14" t="n">
-        <v>4274800.0</v>
+        <v>1.09993E7</v>
       </c>
       <c r="AA208" s="14" t="inlineStr"/>
       <c r="AB208" s="14" t="inlineStr"/>
       <c r="AC208" s="15" t="n">
-        <v>0.3886181818181818</v>
+        <v>0.9999363636363636</v>
       </c>
       <c r="AD208" s="15" t="inlineStr"/>
       <c r="AE208" s="14" t="n">
-        <v>6725200.0</v>
+        <v>700.0</v>
       </c>
       <c r="AF208" s="14" t="inlineStr"/>
       <c r="AG208" s="14" t="inlineStr"/>
@@ -12728,20 +12728,20 @@
         <v>3964800.0</v>
       </c>
       <c r="X209" s="14" t="n">
-        <v>0.0</v>
+        <v>5035000.0</v>
       </c>
       <c r="Y209" s="14" t="inlineStr"/>
       <c r="Z209" s="14" t="n">
-        <v>3964800.0</v>
+        <v>8999800.0</v>
       </c>
       <c r="AA209" s="14" t="inlineStr"/>
       <c r="AB209" s="14" t="inlineStr"/>
       <c r="AC209" s="15" t="n">
-        <v>0.44053333333333333</v>
+        <v>0.9999777777777777</v>
       </c>
       <c r="AD209" s="15" t="inlineStr"/>
       <c r="AE209" s="14" t="n">
-        <v>5035200.0</v>
+        <v>200.0</v>
       </c>
       <c r="AF209" s="14" t="inlineStr"/>
       <c r="AG209" s="14" t="inlineStr"/>
@@ -12785,20 +12785,20 @@
         <v>310000.0</v>
       </c>
       <c r="X210" s="14" t="n">
-        <v>0.0</v>
+        <v>1689500.0</v>
       </c>
       <c r="Y210" s="14" t="inlineStr"/>
       <c r="Z210" s="14" t="n">
-        <v>310000.0</v>
+        <v>1999500.0</v>
       </c>
       <c r="AA210" s="14" t="inlineStr"/>
       <c r="AB210" s="14" t="inlineStr"/>
       <c r="AC210" s="15" t="n">
-        <v>0.155</v>
+        <v>0.99975</v>
       </c>
       <c r="AD210" s="15" t="inlineStr"/>
       <c r="AE210" s="14" t="n">
-        <v>1690000.0</v>
+        <v>500.0</v>
       </c>
       <c r="AF210" s="14" t="inlineStr"/>
       <c r="AG210" s="14" t="inlineStr"/>
@@ -13953,20 +13953,20 @@
         <v>6.74613153E8</v>
       </c>
       <c r="X230" s="14" t="n">
-        <v>3.2949829E8</v>
+        <v>4.12619038E8</v>
       </c>
       <c r="Y230" s="14" t="inlineStr"/>
       <c r="Z230" s="14" t="n">
-        <v>1.004111443E9</v>
+        <v>1.087232191E9</v>
       </c>
       <c r="AA230" s="14" t="inlineStr"/>
       <c r="AB230" s="14" t="inlineStr"/>
       <c r="AC230" s="15" t="n">
-        <v>0.9185192286758417</v>
+        <v>0.9945546188431053</v>
       </c>
       <c r="AD230" s="15" t="inlineStr"/>
       <c r="AE230" s="14" t="n">
-        <v>8.9073557E7</v>
+        <v>5952809.0</v>
       </c>
       <c r="AF230" s="14" t="inlineStr"/>
       <c r="AG230" s="14" t="inlineStr"/>
@@ -14313,20 +14313,20 @@
         <v>1.34221533E8</v>
       </c>
       <c r="X236" s="14" t="n">
-        <v>1.508445E8</v>
+        <v>2.1079542E8</v>
       </c>
       <c r="Y236" s="14" t="inlineStr"/>
       <c r="Z236" s="14" t="n">
-        <v>2.85066033E8</v>
+        <v>3.45016953E8</v>
       </c>
       <c r="AA236" s="14" t="inlineStr"/>
       <c r="AB236" s="14" t="inlineStr"/>
       <c r="AC236" s="15" t="n">
-        <v>0.8215159452449567</v>
+        <v>0.994285167146974</v>
       </c>
       <c r="AD236" s="15" t="inlineStr"/>
       <c r="AE236" s="14" t="n">
-        <v>6.1933967E7</v>
+        <v>1983047.0</v>
       </c>
       <c r="AF236" s="14" t="inlineStr"/>
       <c r="AG236" s="14" t="inlineStr"/>
@@ -14427,20 +14427,20 @@
         <v>2.1347299E7</v>
       </c>
       <c r="X238" s="14" t="n">
-        <v>1.47355E7</v>
+        <v>1.57755E7</v>
       </c>
       <c r="Y238" s="14" t="inlineStr"/>
       <c r="Z238" s="14" t="n">
-        <v>3.6082799E7</v>
+        <v>3.7122799E7</v>
       </c>
       <c r="AA238" s="14" t="inlineStr"/>
       <c r="AB238" s="14" t="inlineStr"/>
       <c r="AC238" s="15" t="n">
-        <v>0.9673672654155496</v>
+        <v>0.9952493029490617</v>
       </c>
       <c r="AD238" s="15" t="inlineStr"/>
       <c r="AE238" s="14" t="n">
-        <v>1217201.0</v>
+        <v>177201.0</v>
       </c>
       <c r="AF238" s="14" t="inlineStr"/>
       <c r="AG238" s="14" t="inlineStr"/>
@@ -14484,20 +14484,20 @@
         <v>2.5327E7</v>
       </c>
       <c r="X239" s="14" t="n">
-        <v>375000.0</v>
+        <v>595920.0</v>
       </c>
       <c r="Y239" s="14" t="inlineStr"/>
       <c r="Z239" s="14" t="n">
-        <v>2.5702E7</v>
+        <v>2.592292E7</v>
       </c>
       <c r="AA239" s="14" t="inlineStr"/>
       <c r="AB239" s="14" t="inlineStr"/>
       <c r="AC239" s="15" t="n">
-        <v>0.9904431599229288</v>
+        <v>0.9989564547206166</v>
       </c>
       <c r="AD239" s="15" t="inlineStr"/>
       <c r="AE239" s="14" t="n">
-        <v>248000.0</v>
+        <v>27080.0</v>
       </c>
       <c r="AF239" s="14" t="inlineStr"/>
       <c r="AG239" s="14" t="inlineStr"/>
@@ -14598,20 +14598,20 @@
         <v>4421000.0</v>
       </c>
       <c r="X241" s="14" t="n">
-        <v>7.4724E7</v>
+        <v>1.18724E8</v>
       </c>
       <c r="Y241" s="14" t="inlineStr"/>
       <c r="Z241" s="14" t="n">
-        <v>7.9145E7</v>
+        <v>1.23145E8</v>
       </c>
       <c r="AA241" s="14" t="inlineStr"/>
       <c r="AB241" s="14" t="inlineStr"/>
       <c r="AC241" s="15" t="n">
-        <v>0.640331715210356</v>
+        <v>0.9963187702265373</v>
       </c>
       <c r="AD241" s="15" t="inlineStr"/>
       <c r="AE241" s="14" t="n">
-        <v>4.4455E7</v>
+        <v>455000.0</v>
       </c>
       <c r="AF241" s="14" t="inlineStr"/>
       <c r="AG241" s="14" t="inlineStr"/>
@@ -14712,20 +14712,20 @@
         <v>1.2143622E7</v>
       </c>
       <c r="X243" s="14" t="n">
-        <v>0.0</v>
+        <v>4395000.0</v>
       </c>
       <c r="Y243" s="14" t="inlineStr"/>
       <c r="Z243" s="14" t="n">
-        <v>1.2143622E7</v>
+        <v>1.6538622E7</v>
       </c>
       <c r="AA243" s="14" t="inlineStr"/>
       <c r="AB243" s="14" t="inlineStr"/>
       <c r="AC243" s="15" t="n">
-        <v>0.7315434939759036</v>
+        <v>0.996302530120482</v>
       </c>
       <c r="AD243" s="15" t="inlineStr"/>
       <c r="AE243" s="14" t="n">
-        <v>4456378.0</v>
+        <v>61378.0</v>
       </c>
       <c r="AF243" s="14" t="inlineStr"/>
       <c r="AG243" s="14" t="inlineStr"/>
@@ -14826,20 +14826,20 @@
         <v>1576500.0</v>
       </c>
       <c r="X245" s="14" t="n">
-        <v>1800000.0</v>
+        <v>2400000.0</v>
       </c>
       <c r="Y245" s="14" t="inlineStr"/>
       <c r="Z245" s="14" t="n">
-        <v>3376500.0</v>
+        <v>3976500.0</v>
       </c>
       <c r="AA245" s="14" t="inlineStr"/>
       <c r="AB245" s="14" t="inlineStr"/>
       <c r="AC245" s="15" t="n">
-        <v>0.8136144578313254</v>
+        <v>0.9581927710843373</v>
       </c>
       <c r="AD245" s="15" t="inlineStr"/>
       <c r="AE245" s="14" t="n">
-        <v>773500.0</v>
+        <v>173500.0</v>
       </c>
       <c r="AF245" s="14" t="inlineStr"/>
       <c r="AG245" s="14" t="inlineStr"/>
@@ -15168,20 +15168,20 @@
         <v>0.0</v>
       </c>
       <c r="X251" s="14" t="n">
-        <v>0.0</v>
+        <v>5695000.0</v>
       </c>
       <c r="Y251" s="14" t="inlineStr"/>
       <c r="Z251" s="14" t="n">
-        <v>0.0</v>
+        <v>5695000.0</v>
       </c>
       <c r="AA251" s="14" t="inlineStr"/>
       <c r="AB251" s="14" t="inlineStr"/>
       <c r="AC251" s="15" t="n">
-        <v>0.0</v>
+        <v>0.9991228070175439</v>
       </c>
       <c r="AD251" s="15" t="inlineStr"/>
       <c r="AE251" s="14" t="n">
-        <v>5700000.0</v>
+        <v>5000.0</v>
       </c>
       <c r="AF251" s="14" t="inlineStr"/>
       <c r="AG251" s="14" t="inlineStr"/>
@@ -15225,20 +15225,20 @@
         <v>5413000.0</v>
       </c>
       <c r="X252" s="14" t="n">
-        <v>0.0</v>
+        <v>4000000.0</v>
       </c>
       <c r="Y252" s="14" t="inlineStr"/>
       <c r="Z252" s="14" t="n">
-        <v>5413000.0</v>
+        <v>9413000.0</v>
       </c>
       <c r="AA252" s="14" t="inlineStr"/>
       <c r="AB252" s="14" t="inlineStr"/>
       <c r="AC252" s="15" t="n">
-        <v>0.5697894736842105</v>
+        <v>0.9908421052631579</v>
       </c>
       <c r="AD252" s="15" t="inlineStr"/>
       <c r="AE252" s="14" t="n">
-        <v>4087000.0</v>
+        <v>87000.0</v>
       </c>
       <c r="AF252" s="14" t="inlineStr"/>
       <c r="AG252" s="14" t="inlineStr"/>
@@ -15388,20 +15388,20 @@
         <v>2.11521335E8</v>
       </c>
       <c r="X255" s="14" t="n">
-        <v>8.661379E7</v>
+        <v>1.09783618E8</v>
       </c>
       <c r="Y255" s="14" t="inlineStr"/>
       <c r="Z255" s="14" t="n">
-        <v>2.98135125E8</v>
+        <v>3.21304953E8</v>
       </c>
       <c r="AA255" s="14" t="inlineStr"/>
       <c r="AB255" s="14" t="inlineStr"/>
       <c r="AC255" s="15" t="n">
-        <v>0.918993033614352</v>
+        <v>0.9904133686790069</v>
       </c>
       <c r="AD255" s="15" t="inlineStr"/>
       <c r="AE255" s="14" t="n">
-        <v>2.6279875E7</v>
+        <v>3110047.0</v>
       </c>
       <c r="AF255" s="14" t="inlineStr"/>
       <c r="AG255" s="14" t="inlineStr"/>
@@ -15445,20 +15445,20 @@
         <v>1.396E7</v>
       </c>
       <c r="X256" s="14" t="n">
-        <v>5220000.0</v>
+        <v>8440000.0</v>
       </c>
       <c r="Y256" s="14" t="inlineStr"/>
       <c r="Z256" s="14" t="n">
-        <v>1.918E7</v>
+        <v>2.24E7</v>
       </c>
       <c r="AA256" s="14" t="inlineStr"/>
       <c r="AB256" s="14" t="inlineStr"/>
       <c r="AC256" s="15" t="n">
-        <v>0.8498006202924235</v>
+        <v>0.9924678777137793</v>
       </c>
       <c r="AD256" s="15" t="inlineStr"/>
       <c r="AE256" s="14" t="n">
-        <v>3390000.0</v>
+        <v>170000.0</v>
       </c>
       <c r="AF256" s="14" t="inlineStr"/>
       <c r="AG256" s="14" t="inlineStr"/>
@@ -15559,20 +15559,20 @@
         <v>2.9845218E7</v>
       </c>
       <c r="X258" s="14" t="n">
-        <v>1.279805E7</v>
+        <v>1.510805E7</v>
       </c>
       <c r="Y258" s="14" t="inlineStr"/>
       <c r="Z258" s="14" t="n">
-        <v>4.2643268E7</v>
+        <v>4.4953268E7</v>
       </c>
       <c r="AA258" s="14" t="inlineStr"/>
       <c r="AB258" s="14" t="inlineStr"/>
       <c r="AC258" s="15" t="n">
-        <v>0.9476281777777777</v>
+        <v>0.9989615111111111</v>
       </c>
       <c r="AD258" s="15" t="inlineStr"/>
       <c r="AE258" s="14" t="n">
-        <v>2356732.0</v>
+        <v>46732.0</v>
       </c>
       <c r="AF258" s="14" t="inlineStr"/>
       <c r="AG258" s="14" t="inlineStr"/>
@@ -15616,20 +15616,20 @@
         <v>1.22043496E8</v>
       </c>
       <c r="X259" s="14" t="n">
-        <v>4.7543521E7</v>
+        <v>5.1816623E7</v>
       </c>
       <c r="Y259" s="14" t="inlineStr"/>
       <c r="Z259" s="14" t="n">
-        <v>1.69587017E8</v>
+        <v>1.73860119E8</v>
       </c>
       <c r="AA259" s="14" t="inlineStr"/>
       <c r="AB259" s="14" t="inlineStr"/>
       <c r="AC259" s="15" t="n">
-        <v>0.9731559234499182</v>
+        <v>0.9976766361575761</v>
       </c>
       <c r="AD259" s="15" t="inlineStr"/>
       <c r="AE259" s="14" t="n">
-        <v>4677983.0</v>
+        <v>404881.0</v>
       </c>
       <c r="AF259" s="14" t="inlineStr"/>
       <c r="AG259" s="14" t="inlineStr"/>
@@ -15673,20 +15673,20 @@
         <v>4147992.0</v>
       </c>
       <c r="X260" s="14" t="n">
-        <v>90000.0</v>
+        <v>225000.0</v>
       </c>
       <c r="Y260" s="14" t="inlineStr"/>
       <c r="Z260" s="14" t="n">
-        <v>4237992.0</v>
+        <v>4372992.0</v>
       </c>
       <c r="AA260" s="14" t="inlineStr"/>
       <c r="AB260" s="14" t="inlineStr"/>
       <c r="AC260" s="15" t="n">
-        <v>0.941776</v>
+        <v>0.971776</v>
       </c>
       <c r="AD260" s="15" t="inlineStr"/>
       <c r="AE260" s="14" t="n">
-        <v>262008.0</v>
+        <v>127008.0</v>
       </c>
       <c r="AF260" s="14" t="inlineStr"/>
       <c r="AG260" s="14" t="inlineStr"/>
@@ -15787,20 +15787,20 @@
         <v>1000052.0</v>
       </c>
       <c r="X262" s="14" t="n">
-        <v>0.0</v>
+        <v>7986000.0</v>
       </c>
       <c r="Y262" s="14" t="inlineStr"/>
       <c r="Z262" s="14" t="n">
-        <v>1000052.0</v>
+        <v>8986052.0</v>
       </c>
       <c r="AA262" s="14" t="inlineStr"/>
       <c r="AB262" s="14" t="inlineStr"/>
       <c r="AC262" s="15" t="n">
-        <v>0.11099356270810211</v>
+        <v>0.997342064372919</v>
       </c>
       <c r="AD262" s="15" t="inlineStr"/>
       <c r="AE262" s="14" t="n">
-        <v>8009948.0</v>
+        <v>23948.0</v>
       </c>
       <c r="AF262" s="14" t="inlineStr"/>
       <c r="AG262" s="14" t="inlineStr"/>
@@ -15844,20 +15844,20 @@
         <v>1978406.0</v>
       </c>
       <c r="X263" s="14" t="n">
-        <v>0.0</v>
+        <v>1000000.0</v>
       </c>
       <c r="Y263" s="14" t="inlineStr"/>
       <c r="Z263" s="14" t="n">
-        <v>1978406.0</v>
+        <v>2978406.0</v>
       </c>
       <c r="AA263" s="14" t="inlineStr"/>
       <c r="AB263" s="14" t="inlineStr"/>
       <c r="AC263" s="15" t="n">
-        <v>0.6486577049180328</v>
+        <v>0.9765265573770492</v>
       </c>
       <c r="AD263" s="15" t="inlineStr"/>
       <c r="AE263" s="14" t="n">
-        <v>1071594.0</v>
+        <v>71594.0</v>
       </c>
       <c r="AF263" s="14" t="inlineStr"/>
       <c r="AG263" s="14" t="inlineStr"/>
@@ -15901,20 +15901,20 @@
         <v>8450284.0</v>
       </c>
       <c r="X264" s="14" t="n">
-        <v>2385941.0</v>
+        <v>3365941.0</v>
       </c>
       <c r="Y264" s="14" t="inlineStr"/>
       <c r="Z264" s="14" t="n">
-        <v>1.0836225E7</v>
+        <v>1.1816225E7</v>
       </c>
       <c r="AA264" s="14" t="inlineStr"/>
       <c r="AB264" s="14" t="inlineStr"/>
       <c r="AC264" s="15" t="n">
-        <v>0.90301875</v>
+        <v>0.9846854166666666</v>
       </c>
       <c r="AD264" s="15" t="inlineStr"/>
       <c r="AE264" s="14" t="n">
-        <v>1163775.0</v>
+        <v>183775.0</v>
       </c>
       <c r="AF264" s="14" t="inlineStr"/>
       <c r="AG264" s="14" t="inlineStr"/>
@@ -15958,20 +15958,20 @@
         <v>1167558.0</v>
       </c>
       <c r="X265" s="14" t="n">
-        <v>0.0</v>
+        <v>500000.0</v>
       </c>
       <c r="Y265" s="14" t="inlineStr"/>
       <c r="Z265" s="14" t="n">
-        <v>1167558.0</v>
+        <v>1667558.0</v>
       </c>
       <c r="AA265" s="14" t="inlineStr"/>
       <c r="AB265" s="14" t="inlineStr"/>
       <c r="AC265" s="15" t="n">
-        <v>0.583779</v>
+        <v>0.833779</v>
       </c>
       <c r="AD265" s="15" t="inlineStr"/>
       <c r="AE265" s="14" t="n">
-        <v>832442.0</v>
+        <v>332442.0</v>
       </c>
       <c r="AF265" s="14" t="inlineStr"/>
       <c r="AG265" s="14" t="inlineStr"/>
@@ -16015,20 +16015,20 @@
         <v>3760846.0</v>
       </c>
       <c r="X266" s="14" t="n">
-        <v>9601868.0</v>
+        <v>1.1772594E7</v>
       </c>
       <c r="Y266" s="14" t="inlineStr"/>
       <c r="Z266" s="14" t="n">
-        <v>1.3362714E7</v>
+        <v>1.553344E7</v>
       </c>
       <c r="AA266" s="14" t="inlineStr"/>
       <c r="AB266" s="14" t="inlineStr"/>
       <c r="AC266" s="15" t="n">
-        <v>0.855487451984635</v>
+        <v>0.9944583866837388</v>
       </c>
       <c r="AD266" s="15" t="inlineStr"/>
       <c r="AE266" s="14" t="n">
-        <v>2257286.0</v>
+        <v>86560.0</v>
       </c>
       <c r="AF266" s="14" t="inlineStr"/>
       <c r="AG266" s="14" t="inlineStr"/>
@@ -16129,20 +16129,20 @@
         <v>7889000.0</v>
       </c>
       <c r="X268" s="14" t="n">
-        <v>581410.0</v>
+        <v>666410.0</v>
       </c>
       <c r="Y268" s="14" t="inlineStr"/>
       <c r="Z268" s="14" t="n">
-        <v>8470410.0</v>
+        <v>8555410.0</v>
       </c>
       <c r="AA268" s="14" t="inlineStr"/>
       <c r="AB268" s="14" t="inlineStr"/>
       <c r="AC268" s="15" t="n">
-        <v>0.9011074468085106</v>
+        <v>0.91015</v>
       </c>
       <c r="AD268" s="15" t="inlineStr"/>
       <c r="AE268" s="14" t="n">
-        <v>929590.0</v>
+        <v>844590.0</v>
       </c>
       <c r="AF268" s="14" t="inlineStr"/>
       <c r="AG268" s="14" t="inlineStr"/>
@@ -16300,20 +16300,20 @@
         <v>0.0</v>
       </c>
       <c r="X271" s="14" t="n">
-        <v>488000.0</v>
+        <v>998000.0</v>
       </c>
       <c r="Y271" s="14" t="inlineStr"/>
       <c r="Z271" s="14" t="n">
-        <v>488000.0</v>
+        <v>998000.0</v>
       </c>
       <c r="AA271" s="14" t="inlineStr"/>
       <c r="AB271" s="14" t="inlineStr"/>
       <c r="AC271" s="15" t="n">
-        <v>0.488</v>
+        <v>0.998</v>
       </c>
       <c r="AD271" s="15" t="inlineStr"/>
       <c r="AE271" s="14" t="n">
-        <v>512000.0</v>
+        <v>2000.0</v>
       </c>
       <c r="AF271" s="14" t="inlineStr"/>
       <c r="AG271" s="14" t="inlineStr"/>

</xml_diff>